<commit_message>
docs: add DEC-014..016 and sync status workbook
Methodology re-review against newly added meta-analysis methods
papers (Stanley et al. 2024/2025; van Aert 2023; van Aert & van
Assen 2026; Pustejovsky & Tipton 2022).

- DEC-014: cluster-robust (CR2) inference for FAT-PET-PEESE and all
  meta-regressions, not only the headline pooled mean. Table 7/8
  standard errors were invalid under effect-size dependence.
- DEC-015: correlation small-sample bias. Retain Fisher's z, add
  UWLS+3/HS robustness, report the n-distribution (37% of effects
  n<200), use PCC degrees of freedom n-k-3, add bivariate-only check.
- DEC-016: selection-model secondary publication-bias check
  (3PSM / p-uniform*) at study level; PET-PEESE remains primary.

Status workbook: Roadmap themes #14-16, Tasks T0.4/T4/T5/T7,
DecisionLog index (count 13->16), Setup update trail.
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -123,7 +123,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -145,11 +145,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -251,6 +295,8 @@
     <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -633,7 +679,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Update 2026-06-29(b): DEC-Log FINALISIERT (DEC-001..013 aktiv) + DECISION_LOG.md erzeugt — #6–9 zu DECs ausformuliert, #11/#12 bleiben Tasks.  (a): SOMA-Handoff integriert (Verifier, Review-Gate, Source-Pointer, Commit-Ritual, gitignore); DEC-Log auf Methodik-only getrimmt.</t>
+          <t>Update 2026-06-30: Methodik-Re-Review gegen neue PK-Methoden-Paper (Stanley et al. 2024/2025 Korrelations-Bias; van Aert 2023 PCC; van Aert &amp; van Assen 2026 p-uniform*; Pustejovsky &amp; Tipton 2022 RVE). +DEC-014..016: (014) CR2-SE fuer FAT-PET-PEESE &amp; Meta-Reg; (015) Korrelations-Small-Sample-Bias → UWLS+3/HS-Robustheit + n-Reporting + PCC-df; (016) Selektionsmodell sekundaer. Roadmap #14–16 ergaenzt.  Update 2026-06-29(b): DEC-Log FINALISIERT (DEC-001..013 aktiv) + DECISION_LOG.md erzeugt — #6–9 zu DECs ausformuliert, #11/#12 bleiben Tasks.  (a): SOMA-Handoff integriert (Verifier, Review-Gate, Source-Pointer, Commit-Ritual, gitignore); DEC-Log auf Methodik-only getrimmt.</t>
         </is>
       </c>
     </row>
@@ -643,7 +689,7 @@
           <t>1 — WERKZEUG-ROLLEN</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n"/>
+      <c r="B3" s="35" t="n"/>
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -687,7 +733,7 @@
           <t>2 — ARBEITSFLUSS (Hand-off-Loop)</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n"/>
+      <c r="B7" s="35" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -755,7 +801,7 @@
           <t>3 — REVIEW-GATE (Hybrid — macht Pfad a vertrauenswuerdig)</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n"/>
+      <c r="B13" s="35" t="n"/>
     </row>
     <row r="14" ht="34" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -787,7 +833,7 @@
           <t>4 — VERIFIER-DISZIPLIN (das Sicherheitsnetz)</t>
         </is>
       </c>
-      <c r="B16" s="4" t="n"/>
+      <c r="B16" s="35" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -843,7 +889,7 @@
           <t>5 — ARTEFAKT-OEKOSYSTEM (verzahnt ueber DEC-IDs + Source-Pointer)</t>
         </is>
       </c>
-      <c r="B21" s="4" t="n"/>
+      <c r="B21" s="35" t="n"/>
     </row>
     <row r="22" ht="28" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -853,7 +899,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>Das WARUM: 8-Feld-Eintraege (s. §7). Nur reviewer-verteidigbare Methodik. [noch zu erstellen]</t>
+          <t>Das WARUM: 8-Feld-Eintraege (s. §7). Nur reviewer-verteidigbare Methodik. [aktiv: DEC-001..016]</t>
         </is>
       </c>
     </row>
@@ -923,7 +969,7 @@
           <t>6 — REPO, ENVIRONMENT &amp; COMMIT (vor erster Analyse einfrieren)</t>
         </is>
       </c>
-      <c r="B28" s="4" t="n"/>
+      <c r="B28" s="35" t="n"/>
     </row>
     <row r="29" ht="34" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
@@ -1003,7 +1049,7 @@
           <t>7 — KERN-KONVENTIONEN</t>
         </is>
       </c>
-      <c r="B35" s="4" t="n"/>
+      <c r="B35" s="35" t="n"/>
     </row>
     <row r="36" ht="32" customHeight="1">
       <c r="A36" s="5" t="inlineStr">
@@ -1107,7 +1153,7 @@
           <t>8 — TAB-INDEX DIESES WORKBOOKS</t>
         </is>
       </c>
-      <c r="B44" s="4" t="n"/>
+      <c r="B44" s="35" t="n"/>
     </row>
     <row r="45" ht="24" customHeight="1">
       <c r="A45" s="5" t="inlineStr">
@@ -1129,7 +1175,7 @@
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>13 Themen (strategischer Layer): Kritik → geplante Aenderung → Status → DEC-Ref.</t>
+          <t>16 Themen (strategischer Layer): Kritik → geplante Aenderung → Status → DEC-Ref.</t>
         </is>
       </c>
     </row>
@@ -1177,15 +1223,15 @@
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>DEC-ID-Register (Methodik-only, 9 Eintraege; Pointer auf DECISION_LOG.md). IDs derzeit VORLAEUFIG.</t>
+          <t>DEC-ID-Register (Methodik-only, 16 Eintraege; Pointer auf DECISION_LOG.md). IDs aktiv.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A16:B16"/>
     <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A16:B16"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A13:B13"/>
@@ -1204,7 +1250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1599,7 +1645,7 @@
       </c>
       <c r="H10" s="12" t="inlineStr">
         <is>
-          <t>DEC-010</t>
+          <t>DEC-010, DEC-014, DEC-016</t>
         </is>
       </c>
       <c r="I10" s="12" t="inlineStr"/>
@@ -1865,6 +1911,147 @@
         </is>
       </c>
       <c r="I16" s="15" t="inlineStr"/>
+    </row>
+    <row r="17" ht="56" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Cluster-robuste Inferenz (alle Regressionen)</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>FAT-PET-PEESE &amp; Meta-Reg poolen 1.306 abh. ES als unabhaengig → SE/Sterne in Tab. 7/8 ungueltig</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>CR2-SE (clubSandwich), geclustert auf study, ueber T5 UND T7 — nicht nur Headline (T1)</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Entschieden</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>#1, #6</t>
+        </is>
+      </c>
+      <c r="H17" s="9" t="inlineStr">
+        <is>
+          <t>DEC-014</t>
+        </is>
+      </c>
+      <c r="I17" s="9" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="56" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Korrelations-Small-Sample-Bias</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>RE-IVW auf r/Fisher-z rest-verzerrt (Stanley 2024/25); 37% n&lt;200; Headline r=−0,020</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>Fisher-z behalten; WLS/RVE-Headline mit Stanley begruenden; UWLS+3/HS-Robustheit; n-Verteilung berichten; PCC-df (n−k−3)</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>Entschieden</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="inlineStr">
+        <is>
+          <t>#1, #5</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>DEC-015</t>
+        </is>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="56" customHeight="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Selektionsmodell (Pub-Bias-Triangulation)</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>Bias-Evidenz nur eine Methodenfamilie (FAT-PET-PEESE)</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>3PSM/p-uniform* sekundaer auf Studienebene (k=66); PET-PEESE bleibt primaer</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>Entschieden</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>#6</t>
+        </is>
+      </c>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>DEC-016</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2136,12 +2323,12 @@
       </c>
       <c r="D7" s="23" t="inlineStr">
         <is>
-          <t>ZWINGEND: kont. Jahresvar. (Start/End/Midpoint) — Blocker fuer T8 Moves 1–2. Regul.-Codebook. n&lt;10/non-integer n. Drago/Devalle verifizieren.</t>
+          <t>ZWINGEND: kont. Jahresvar. (Start/End/Midpoint) — Blocker fuer T8 Moves 1–2. Regul.-Codebook. n&lt;10/non-integer n. Drago/Devalle verifizieren. + n-Verteilung dokumentieren (Median 289; 37% n&lt;200) [DEC-015].</t>
         </is>
       </c>
       <c r="E7" s="22" t="inlineStr">
         <is>
-          <t>#3,#9</t>
+          <t>#3,#9,#15</t>
         </is>
       </c>
       <c r="F7" s="23" t="inlineStr">
@@ -2344,12 +2531,12 @@
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>Leave-one-out · Outlier (rstudent) · winsor/unwinsor · one-effect-per-study · r-Typ · CER-Typ · Journal-Q · Event-Coding · Paris-Lags — Long-CSV mit spec-Spalte.</t>
+          <t>Leave-one-out · Outlier (rstudent) · winsor/unwinsor · one-effect-per-study · r-Typ · CER-Typ · Journal-Q · Event-Coding · Paris-Lags — Long-CSV mit spec-Spalte. · UWLS+3/HS (Korrelations-Bias) [DEC-015] · Bivariat-only (drop 36 P) [DEC-004/015].</t>
         </is>
       </c>
       <c r="E11" s="25" t="inlineStr">
         <is>
-          <t>#5,#3,#9</t>
+          <t>#5,#3,#9,#15</t>
         </is>
       </c>
       <c r="F11" s="26" t="inlineStr">
@@ -2396,17 +2583,17 @@
       </c>
       <c r="D12" s="26" t="inlineStr">
         <is>
-          <t>FAT-PET-PEESE konsistent ueber ALLE Subgruppen; PET-PEESE-Entscheidungsregel; ggf. selection model sekundaer.</t>
+          <t>FAT-PET-PEESE konsistent ueber ALLE Subgruppen, MIT CR2-SE (geclustert auf study) [DEC-014]; PET-PEESE-Entscheidungsregel; 3PSM/p-uniform* sekundaer auf Studienebene (k=66) [DEC-016].</t>
         </is>
       </c>
       <c r="E12" s="25" t="inlineStr">
         <is>
-          <t>#6</t>
+          <t>#6,#14,#16</t>
         </is>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>FAT-PET-PEESE</t>
+          <t>FAT-PET-PEESE + CR2; 3PSM/p-uniform*</t>
         </is>
       </c>
       <c r="G12" s="25" t="inlineStr">
@@ -2500,12 +2687,12 @@
       </c>
       <c r="D14" s="26" t="inlineStr">
         <is>
-          <t>CER–COD ~ Pre/Post + Paris×Moderator + Moderatoren + method. Artefakte; RVE-SEs; loest alte Modell-10-Multikollinearitaet.</t>
+          <t>CER–COD ~ Pre/Post + Paris×Moderator + Moderatoren + method. Artefakte; RVE-SEs; loest alte Modell-10-Multikollinearitaet. (CR2-SE bestaetigt [DEC-014].)</t>
         </is>
       </c>
       <c r="E14" s="25" t="inlineStr">
         <is>
-          <t>#1,#10</t>
+          <t>#1,#10,#14</t>
         </is>
       </c>
       <c r="F14" s="26" t="inlineStr">
@@ -2983,8 +3170,8 @@
           <t>Phase 2 — Core (T1–T3)</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
+      <c r="B4" s="36" t="n"/>
+      <c r="C4" s="35" t="n"/>
     </row>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -3043,8 +3230,8 @@
           <t>Phase 2 — Identifikation &amp; Robustheit (T2, T8, T5, T4)</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
+      <c r="B8" s="36" t="n"/>
+      <c r="C8" s="35" t="n"/>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -3120,8 +3307,8 @@
           <t>Phase 2 — Moderatoren (T6, T7)</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
+      <c r="B13" s="36" t="n"/>
+      <c r="C13" s="35" t="n"/>
     </row>
     <row r="14" ht="26" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -3175,7 +3362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3197,7 +3384,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>13 aktive Methodik-DECs (DEC-001..013). Volleintraege im DECISION_LOG.md (8-Feld-Schema inkl. gespaltenem Reviewer-Risk). Setup/Prozess → Tab 'Setup'; Reporting/Polish (#11/#12) = Tasks, keine DEC.</t>
+          <t>16 aktive Methodik-DECs (DEC-001..016). Volleintraege im DECISION_LOG.md (8-Feld-Schema inkl. gespaltenem Reviewer-Risk). Setup/Prozess → Tab 'Setup'; Reporting/Polish (#11/#12) = Tasks, keine DEC.</t>
         </is>
       </c>
     </row>
@@ -3719,24 +3906,135 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="44" customHeight="1">
-      <c r="A17" s="34" t="inlineStr">
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="33" t="inlineStr">
+        <is>
+          <t>DEC-014</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Cluster-robuste Bias-/Meta-Regression (CR2)</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>#14,#6 / T5,T7</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>FAT-PET-PEESE &amp; Meta-Reg mit CR2-SE (geclustert auf study, Satterthwaite-df); 1.306 abh. ES nicht als unabhaengig. Tab. 7/8 neu.</t>
+        </is>
+      </c>
+      <c r="G17" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="33" t="inlineStr">
+        <is>
+          <t>DEC-015</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Korrelations-Small-Sample-Bias / UWLS+3</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>#15,#1,#5 / T4,T0.4</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Fisher-z behalten (Stanley 2024/25: r-IVW rest-verzerrt, 37% n&lt;200); WLS/RVE-Headline begruenden; UWLS+3/HS-Robustheit; n-Verteilung; PCC-df (n−k−3); Bivariat-only.</t>
+        </is>
+      </c>
+      <c r="G18" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="33" t="inlineStr">
+        <is>
+          <t>DEC-016</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Selektionsmodell sekundaer (3PSM/p-uniform*)</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>#16,#6 / T5</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>3PSM/p-uniform* (van Aert &amp; van Assen 2026) sekundaer auf Studienebene (k=66); PET-PEESE bleibt primaer (Stanley 2025). Triangulation.</t>
+        </is>
+      </c>
+      <c r="G19" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="44" customHeight="1">
+      <c r="A20" s="34" t="inlineStr">
         <is>
           <t>Pending/Conditional DECs (im DECISION_LOG.md): Pending-A Headline-Event-Coding (nach T2) · Pending-B Transform-Doku (#11) · Pending-C Framing A vs. C (nach T1–T3 + T8).  Setup/Prozess-Entscheidungen → Tab 'Setup' (keine DECs). #11/#12 = Tasks.</t>
         </is>
       </c>
-      <c r="B17" s="4" t="n"/>
-      <c r="C17" s="4" t="n"/>
-      <c r="D17" s="4" t="n"/>
-      <c r="E17" s="4" t="n"/>
-      <c r="F17" s="4" t="n"/>
-      <c r="G17" s="4" t="n"/>
+      <c r="B20" s="36" t="n"/>
+      <c r="C20" s="36" t="n"/>
+      <c r="D20" s="36" t="n"/>
+      <c r="E20" s="36" t="n"/>
+      <c r="F20" s="36" t="n"/>
+      <c r="G20" s="35" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A20:G20"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A17:G17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: T0.1 analysis plan + DEC-017 (rho working correlation)
Add docs/analysis_plan.md: canonical executable spec operationalizing
DEC-002..017 (3LMA-RVE rma.mv signature, V via impute_covariance_matrix
rho=0.6, CR2 on all regressions, headline-vs-robustness a priori).

- DEC-017: within-study working correlation rho=0.6, sensitivity
  0.4/0.6/0.8; operationalizes DEC-002.
- Tracker: T0.1 and T0.2 -> DONE; T4 rho-sensitivity spec;
  Roadmap #1 and DecisionLog index updated (17 DECs).
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -679,7 +679,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Update 2026-06-30: Methodik-Re-Review gegen neue PK-Methoden-Paper (Stanley et al. 2024/2025 Korrelations-Bias; van Aert 2023 PCC; van Aert &amp; van Assen 2026 p-uniform*; Pustejovsky &amp; Tipton 2022 RVE). +DEC-014..016: (014) CR2-SE fuer FAT-PET-PEESE &amp; Meta-Reg; (015) Korrelations-Small-Sample-Bias → UWLS+3/HS-Robustheit + n-Reporting + PCC-df; (016) Selektionsmodell sekundaer. Roadmap #14–16 ergaenzt.  Update 2026-06-29(b): DEC-Log FINALISIERT (DEC-001..013 aktiv) + DECISION_LOG.md erzeugt — #6–9 zu DECs ausformuliert, #11/#12 bleiben Tasks.  (a): SOMA-Handoff integriert (Verifier, Review-Gate, Source-Pointer, Commit-Ritual, gitignore); DEC-Log auf Methodik-only getrimmt.</t>
+          <t>Update 2026-06-30(b): T0.1 abgeschlossen — docs/analysis_plan.md (kanonische HOW-Spec) geschrieben; +DEC-017 (rho=0,6 working correlation, Sensitivitaet 0,4/0,6/0,8); E1–E6 gelockt; T0.1/T0.2 → DONE. puniform 0.2.8 installiert (Lock-Snapshot ausstehend).  Update 2026-06-30: Methodik-Re-Review gegen neue PK-Methoden-Paper (Stanley et al. 2024/2025 Korrelations-Bias; van Aert 2023 PCC; van Aert &amp; van Assen 2026 p-uniform*; Pustejovsky &amp; Tipton 2022 RVE). +DEC-014..016: (014) CR2-SE fuer FAT-PET-PEESE &amp; Meta-Reg; (015) Korrelations-Small-Sample-Bias → UWLS+3/HS-Robustheit + n-Reporting + PCC-df; (016) Selektionsmodell sekundaer. Roadmap #14–16 ergaenzt.  Update 2026-06-29(b): DEC-Log FINALISIERT (DEC-001..013 aktiv) + DECISION_LOG.md erzeugt — #6–9 zu DECs ausformuliert, #11/#12 bleiben Tasks.  (a): SOMA-Handoff integriert (Verifier, Review-Gate, Source-Pointer, Commit-Ritual, gitignore); DEC-Log auf Methodik-only getrimmt.</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>DEC-ID-Register (Methodik-only, 16 Eintraege; Pointer auf DECISION_LOG.md). IDs aktiv.</t>
+          <t>DEC-ID-Register (Methodik-only, 17 Eintraege; Pointer auf DECISION_LOG.md). IDs aktiv.</t>
         </is>
       </c>
     </row>
@@ -1363,7 +1363,7 @@
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
-          <t>DEC-002,003</t>
+          <t>DEC-002,003,017</t>
         </is>
       </c>
       <c r="I4" s="9" t="inlineStr">
@@ -2187,17 +2187,17 @@
       </c>
       <c r="H4" s="19" t="inlineStr">
         <is>
-          <t>IN ARBEIT</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="I4" s="20" t="inlineStr">
         <is>
-          <t>Architektur entschieden (DEC-002/003/009)</t>
+          <t>DONE: analysis_plan.md geschrieben — rma.mv-Signatur, V via impute_covariance_matrix(r=0.6) [DEC-017], CR2 ueber alle Reg [DEC-014], Headline-vs-Robustness a priori (§10). E1–E6 gelockt. → Commit + Hash nachtragen.</t>
         </is>
       </c>
       <c r="J4" s="20" t="inlineStr">
         <is>
-          <t>docs/analysis_plan.md (geplant)</t>
+          <t>docs/analysis_plan.md</t>
         </is>
       </c>
     </row>
@@ -2239,17 +2239,17 @@
       </c>
       <c r="H5" s="19" t="inlineStr">
         <is>
-          <t>OFFEN</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="I5" s="20" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DONE: a priori fixiert in analysis_plan.md §10/§6/§2 — Headline=3LMA-RVE pooled; Identifikation=Meta-Reg; Event-Coding &amp; r-Typ a priori. → Commit + Hash nachtragen.</t>
         </is>
       </c>
       <c r="J5" s="20" t="inlineStr">
         <is>
-          <t>docs/analysis_plan.md (geplant)</t>
+          <t>docs/analysis_plan.md</t>
         </is>
       </c>
     </row>
@@ -2531,12 +2531,12 @@
       </c>
       <c r="D11" s="26" t="inlineStr">
         <is>
-          <t>Leave-one-out · Outlier (rstudent) · winsor/unwinsor · one-effect-per-study · r-Typ · CER-Typ · Journal-Q · Event-Coding · Paris-Lags — Long-CSV mit spec-Spalte. · UWLS+3/HS (Korrelations-Bias) [DEC-015] · Bivariat-only (drop 36 P) [DEC-004/015].</t>
+          <t>Leave-one-out · Outlier (rstudent) · winsor/unwinsor · one-effect-per-study · r-Typ · CER-Typ · Journal-Q · Event-Coding · Paris-Lags — Long-CSV mit spec-Spalte. · UWLS+3/HS (Korrelations-Bias) [DEC-015] · Bivariat-only (drop 36 P) [DEC-004/015]. · rho-Sensitivitaet 0,4/0,6/0,8 [DEC-017].</t>
         </is>
       </c>
       <c r="E11" s="25" t="inlineStr">
         <is>
-          <t>#5,#3,#9,#15</t>
+          <t>#5,#3,#9,#15,#1</t>
         </is>
       </c>
       <c r="F11" s="26" t="inlineStr">
@@ -3362,7 +3362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3384,7 +3384,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>16 aktive Methodik-DECs (DEC-001..016). Volleintraege im DECISION_LOG.md (8-Feld-Schema inkl. gespaltenem Reviewer-Risk). Setup/Prozess → Tab 'Setup'; Reporting/Polish (#11/#12) = Tasks, keine DEC.</t>
+          <t>17 aktive Methodik-DECs (DEC-001..017). Volleintraege im DECISION_LOG.md (8-Feld-Schema inkl. gespaltenem Reviewer-Risk). Setup/Prozess → Tab 'Setup'; Reporting/Polish (#11/#12) = Tasks, keine DEC.</t>
         </is>
       </c>
     </row>
@@ -4017,22 +4017,59 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="44" customHeight="1">
-      <c r="A20" s="34" t="inlineStr">
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>DEC-017</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>rho working correlation (CE/CHE-Kovarianz)</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>#1 / T1,T4</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>rho=0,6 default, Sensitivitaet 0,4/0,6/0,8; operationalisiert DEC-002. impute_covariance_matrix(r=0.6); CR2 macht Punktschaetzer rho-robust. spec rho_0.4/rho_0.8 in T4.</t>
+        </is>
+      </c>
+      <c r="G20" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="44" customHeight="1">
+      <c r="A21" s="34" t="inlineStr">
         <is>
           <t>Pending/Conditional DECs (im DECISION_LOG.md): Pending-A Headline-Event-Coding (nach T2) · Pending-B Transform-Doku (#11) · Pending-C Framing A vs. C (nach T1–T3 + T8).  Setup/Prozess-Entscheidungen → Tab 'Setup' (keine DECs). #11/#12 = Tasks.</t>
         </is>
       </c>
-      <c r="B20" s="36" t="n"/>
-      <c r="C20" s="36" t="n"/>
-      <c r="D20" s="36" t="n"/>
-      <c r="E20" s="36" t="n"/>
-      <c r="F20" s="36" t="n"/>
-      <c r="G20" s="35" t="n"/>
+      <c r="B21" s="36" t="n"/>
+      <c r="C21" s="36" t="n"/>
+      <c r="D21" s="36" t="n"/>
+      <c r="E21" s="36" t="n"/>
+      <c r="F21" s="36" t="n"/>
+      <c r="G21" s="35" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A21:G21"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>

</xml_diff>

<commit_message>
docs: add Datenagenda tab (13 open data questions/requirements)
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -10,9 +10,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aufgaben" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifikation" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key_Results" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DecisionLog_Index" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datenagenda" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifikation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key_Results" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DecisionLog_Index" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,6 +64,15 @@
       <name val="Arial"/>
       <color rgb="00000000"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="12">
@@ -193,7 +203,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -297,6 +307,21 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -662,7 +687,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B50"/>
+  <dimension ref="A1:B51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -679,7 +704,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Update 2026-06-30(b): T0.1 abgeschlossen — docs/analysis_plan.md (kanonische HOW-Spec) geschrieben; +DEC-017 (rho=0,6 working correlation, Sensitivitaet 0,4/0,6/0,8); E1–E6 gelockt; T0.1/T0.2 → DONE. puniform 0.2.8 installiert (Lock-Snapshot ausstehend).  Update 2026-06-30: Methodik-Re-Review gegen neue PK-Methoden-Paper (Stanley et al. 2024/2025 Korrelations-Bias; van Aert 2023 PCC; van Aert &amp; van Assen 2026 p-uniform*; Pustejovsky &amp; Tipton 2022 RVE). +DEC-014..016: (014) CR2-SE fuer FAT-PET-PEESE &amp; Meta-Reg; (015) Korrelations-Small-Sample-Bias → UWLS+3/HS-Robustheit + n-Reporting + PCC-df; (016) Selektionsmodell sekundaer. Roadmap #14–16 ergaenzt.  Update 2026-06-29(b): DEC-Log FINALISIERT (DEC-001..013 aktiv) + DECISION_LOG.md erzeugt — #6–9 zu DECs ausformuliert, #11/#12 bleiben Tasks.  (a): SOMA-Handoff integriert (Verifier, Review-Gate, Source-Pointer, Commit-Ritual, gitignore); DEC-Log auf Methodik-only getrimmt.</t>
+          <t>Update 2026-06-30(c): Tab 'Datenagenda' ergänzt — 13 offene Datenfragen/-anforderungen aus Abgleich Daten↔analysis_plan (n-Regel, Regulierung 0/1/9, Sample-Jahre, COE-Overlap, Methoden-Artefakt-Moderator …); Volker-Agenda + Beschaffungs-Backlog.  Update 2026-06-30(b): T0.1 abgeschlossen — docs/analysis_plan.md (kanonische HOW-Spec) geschrieben; +DEC-017 (rho=0,6 working correlation, Sensitivitaet 0,4/0,6/0,8); E1–E6 gelockt; T0.1/T0.2 → DONE. puniform 0.2.8 installiert (Lock-Snapshot ausstehend).  Update 2026-06-30: Methodik-Re-Review gegen neue PK-Methoden-Paper (Stanley et al. 2024/2025 Korrelations-Bias; van Aert 2023 PCC; van Aert &amp; van Assen 2026 p-uniform*; Pustejovsky &amp; Tipton 2022 RVE). +DEC-014..016: (014) CR2-SE fuer FAT-PET-PEESE &amp; Meta-Reg; (015) Korrelations-Small-Sample-Bias → UWLS+3/HS-Robustheit + n-Reporting + PCC-df; (016) Selektionsmodell sekundaer. Roadmap #14–16 ergaenzt.  Update 2026-06-29(b): DEC-Log FINALISIERT (DEC-001..013 aktiv) + DECISION_LOG.md erzeugt — #6–9 zu DECs ausformuliert, #11/#12 bleiben Tasks.  (a): SOMA-Handoff integriert (Verifier, Review-Gate, Source-Pointer, Commit-Ritual, gitignore); DEC-Log auf Methodik-only getrimmt.</t>
         </is>
       </c>
     </row>
@@ -1224,6 +1249,18 @@
       <c r="B50" s="6" t="inlineStr">
         <is>
           <t>DEC-ID-Register (Methodik-only, 17 Eintraege; Pointer auf DECISION_LOG.md). IDs aktiv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="24" customHeight="1">
+      <c r="A51" s="37" t="inlineStr">
+        <is>
+          <t>Datenagenda</t>
+        </is>
+      </c>
+      <c r="B51" s="38" t="inlineStr">
+        <is>
+          <t>Offene Datenfragen &amp; -anforderungen (Nr/Typ/Titel/Beschreibung/Quelle/Status/Antwort); Volker-Agenda + Beschaffungs-Backlog.</t>
         </is>
       </c>
     </row>
@@ -2788,327 +2825,471 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Identifikation: Bruch vs. Trend — Werkzeugkasten gegen den Saekulartrend-Confound (#13 / T8)</t>
+          <t>Datenagenda — offene Datenfragen &amp; -anforderungen (Abgleich Daten ↔ analysis_plan)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Problem: Pre/Post-Dummy trennt Bruch nicht von Drift. Daten zeigen Drift (Pre-median r=−0,025 vs. Post r=−0,019). Strategie: Trend modellieren, Paris muss DARUEBER HINAUS liefern.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Move</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Staerke-Tier</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Was es testet / leistet</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>Methode</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>Datenabhaengigkeit</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>Praezedenz / Anker</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="A2" s="39" t="inlineStr">
+        <is>
+          <t>Typ: Frage (Semantik/Regel bestehender Daten) · Daten (fehlt, neu zu beschaffen).  Quelle: Volker = Extraktions-Sheet/Codebook · extern · Design (wir).  Kritisch (gating): 1, 2, 3, 10, 11.  Items 1/2/6/8/10/13 löst Volkers Sheet in einem Zug.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="40" t="inlineStr">
+        <is>
+          <t>Nr</t>
+        </is>
+      </c>
+      <c r="B3" s="40" t="inlineStr">
+        <is>
+          <t>Typ</t>
+        </is>
+      </c>
+      <c r="C3" s="40" t="inlineStr">
+        <is>
+          <t>Titel</t>
+        </is>
+      </c>
+      <c r="D3" s="40" t="inlineStr">
+        <is>
+          <t>Beschreibung</t>
+        </is>
+      </c>
+      <c r="E3" s="40" t="inlineStr">
+        <is>
+          <t>Quelle</t>
+        </is>
+      </c>
+      <c r="F3" s="40" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="84" customHeight="1">
-      <c r="A4" s="27" t="inlineStr">
-        <is>
-          <t>1. Trend-vs-Bruch-Wettrennen</t>
-        </is>
-      </c>
-      <c r="B4" s="28" t="inlineStr">
-        <is>
-          <t>Tier 1 — essenziell, sofort</t>
-        </is>
-      </c>
-      <c r="C4" s="27" t="inlineStr">
-        <is>
-          <t>Trennt glatte Drift vom diskreten Level-Sprung. Dummy weg → nur Drift; ueberlebt → echte Diskontinuitaet</t>
-        </is>
-      </c>
-      <c r="D4" s="27" t="inlineStr">
-        <is>
-          <t>Kont. Zeit (zentr. Midpoint) + Paris-Dummy im SELBEN sparsamen Modell</t>
-        </is>
-      </c>
-      <c r="E4" s="27" t="inlineStr">
-        <is>
-          <t>Sofort — sobald T0.4 kont. Zeit liefert</t>
-        </is>
-      </c>
-      <c r="F4" s="27" t="inlineStr">
-        <is>
-          <t>Huang 2020 (pub-year-Control neben GFC)</t>
-        </is>
-      </c>
-      <c r="G4" s="27" t="inlineStr">
-        <is>
-          <t>OFFEN (T0.4-abh.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="84" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
-        <is>
-          <t>2. Segmentierte Meta-Regression (ITS)</t>
-        </is>
-      </c>
-      <c r="B5" s="28" t="inlineStr">
-        <is>
-          <t>Tier 1 — essenziell, sofort</t>
-        </is>
-      </c>
-      <c r="C5" s="27" t="inlineStr">
-        <is>
-          <t>β₂ Level-Sprung, β₃ Slope-Aenderung. Nistet reinen Trend vs. Bruch als testbare Spezialfaelle</t>
-        </is>
-      </c>
-      <c r="D5" s="27" t="inlineStr">
-        <is>
-          <t>effect ~ β₀+β₁·Zeit+β₂·post+β₃·(Zeit×post); RVE</t>
-        </is>
-      </c>
-      <c r="E5" s="27" t="inlineStr">
-        <is>
-          <t>Sofort — T0.4-abh.</t>
-        </is>
-      </c>
-      <c r="F5" s="27" t="inlineStr">
-        <is>
-          <t>ITS-Standard; COVID-Wellen-Analogon</t>
-        </is>
-      </c>
-      <c r="G5" s="27" t="inlineStr">
-        <is>
-          <t>OFFEN (T0.4-abh.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="84" customHeight="1">
-      <c r="A6" s="29" t="inlineStr">
-        <is>
-          <t>3. Placebo-/Falsifikations-Bruchdaten</t>
-        </is>
-      </c>
-      <c r="B6" s="30" t="inlineStr">
-        <is>
-          <t>Tier 2 — stark</t>
-        </is>
-      </c>
-      <c r="C6" s="29" t="inlineStr">
-        <is>
-          <t>Bruch an Nicht-Paris-Jahren (2012/13/17/18). Ueberall → kein Paris-Bruch; nur 2015/16 → echt. DEUTET LAG1–3 ZU FALSIFIKATION UM</t>
-        </is>
-      </c>
-      <c r="D6" s="29" t="inlineStr">
-        <is>
-          <t>Bruch-Magnitude je Cutoff; Lokalisierungs-Vergleich</t>
-        </is>
-      </c>
-      <c r="E6" s="29" t="inlineStr">
-        <is>
-          <t>Sofort — T0.4-abh.</t>
-        </is>
-      </c>
-      <c r="F6" s="29" t="inlineStr">
-        <is>
-          <t>Placebo-Test-Standard</t>
-        </is>
-      </c>
-      <c r="G6" s="29" t="inlineStr">
-        <is>
-          <t>OFFEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="84" customHeight="1">
-      <c r="A7" s="29" t="inlineStr">
-        <is>
-          <t>4. Kompositions-Kontrolle</t>
-        </is>
-      </c>
-      <c r="B7" s="30" t="inlineStr">
-        <is>
-          <t>Tier 2 — stark, sofort</t>
-        </is>
-      </c>
-      <c r="C7" s="29" t="inlineStr">
-        <is>
-          <t>Haelt Studien-/Laender-/Instrument-Mix konstant; Within-Stratum-Check. Nur im Aggregat → kompositorisch</t>
-        </is>
-      </c>
-      <c r="D7" s="29" t="inlineStr">
-        <is>
-          <t>Paris-Term + Moderatoren als Kovariaten (= T7); Within-Stratum</t>
-        </is>
-      </c>
-      <c r="E7" s="29" t="inlineStr">
-        <is>
-          <t>Sofort (= T7)</t>
-        </is>
-      </c>
-      <c r="F7" s="29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G7" s="29" t="inlineStr">
-        <is>
-          <t>OFFEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="84" customHeight="1">
-      <c r="A8" s="29" t="inlineStr">
-        <is>
-          <t>5. Differential-Exposure (DiD-artig)</t>
-        </is>
-      </c>
-      <c r="B8" s="30" t="inlineStr">
-        <is>
-          <t>Tier 2 — stark</t>
-        </is>
-      </c>
-      <c r="C8" s="29" t="inlineStr">
-        <is>
-          <t>(post−pre) High-Exposure minus (post−pre) Low: gemeinsamer Trend differenziert sich heraus</t>
-        </is>
-      </c>
-      <c r="D8" s="29" t="inlineStr">
-        <is>
-          <t>post × High-Exposure (carbon-intensiv / Carbon-Pricing); Pre-Trend-Check</t>
-        </is>
-      </c>
-      <c r="E8" s="29" t="inlineStr">
-        <is>
-          <t>Sofort; Pre-Trend datenabh.</t>
-        </is>
-      </c>
-      <c r="F8" s="29" t="inlineStr">
-        <is>
-          <t>DiD-Logik. CAVEAT: Parallel-Trends unpruefbar</t>
-        </is>
-      </c>
-      <c r="G8" s="29" t="inlineStr">
-        <is>
-          <t>OFFEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="84" customHeight="1">
-      <c r="A9" s="31" t="inlineStr">
-        <is>
-          <t>6. Within-Study-Identifikation</t>
-        </is>
-      </c>
-      <c r="B9" s="32" t="inlineStr">
-        <is>
-          <t>Tier 3 — Goldstandard, DATENBEDINGT TOT</t>
-        </is>
-      </c>
-      <c r="C9" s="31" t="inlineStr">
-        <is>
-          <t>Studien, die Bruch SELBST ueberspannen + separate Pre/Post. Haelt alle between-Confounder konstant</t>
-        </is>
-      </c>
-      <c r="D9" s="31" t="inlineStr">
-        <is>
-          <t>Within-Study-Pre/Post-Kontrast</t>
-        </is>
-      </c>
-      <c r="E9" s="31" t="inlineStr">
-        <is>
-          <t>NICHT VERFUEGBAR — nur 1–3/66 Studien ueberspannen</t>
-        </is>
-      </c>
-      <c r="F9" s="31" t="inlineStr">
-        <is>
-          <t>COVID within-cohort (Sun, Robinson)</t>
-        </is>
-      </c>
-      <c r="G9" s="31" t="inlineStr">
-        <is>
-          <t>ENTFAELLT (Datenbefund T0.3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="84" customHeight="1">
-      <c r="A10" s="17" t="inlineStr">
-        <is>
-          <t>7. Sensitivitaets-Schranke (Bounding)</t>
-        </is>
-      </c>
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>Tier 4 — Schlussklammer</t>
-        </is>
-      </c>
-      <c r="C10" s="17" t="inlineStr">
-        <is>
-          <t>Wie gross muesste ein Trend sein, um verbleibenden Paris-Dummy zu erklaeren. Begrenzt Confound explizit</t>
-        </is>
-      </c>
-      <c r="D10" s="17" t="inlineStr">
-        <is>
-          <t>Oster-Bounds / E-Value auf finales Modell</t>
-        </is>
-      </c>
-      <c r="E10" s="17" t="inlineStr">
-        <is>
-          <t>Sofort (nach Hauptmodell)</t>
-        </is>
-      </c>
-      <c r="F10" s="17" t="inlineStr">
-        <is>
-          <t>Oster 2019; E-Value (VanderWeele 2017)</t>
-        </is>
-      </c>
-      <c r="G10" s="17" t="inlineStr">
-        <is>
-          <t>OFFEN</t>
-        </is>
-      </c>
+      <c r="G3" s="40" t="inlineStr">
+        <is>
+          <t>Antwort</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="44" customHeight="1">
+      <c r="A4" s="41" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="41" t="inlineStr">
+        <is>
+          <t>Frage</t>
+        </is>
+      </c>
+      <c r="C4" s="41" t="inlineStr">
+        <is>
+          <t>n-Ableitungsregel</t>
+        </is>
+      </c>
+      <c r="D4" s="41" t="inlineStr">
+        <is>
+          <t>699/1.306 n nicht-ganzzahlig (ratio-artig). Gesamt-N über Effekte geteilt? Bestimmt vz/Gewichte → T1-Headline. Korrekt unter RVE: volle Studien-N pro Effekt.</t>
+        </is>
+      </c>
+      <c r="E4" s="41" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="F4" s="41" t="inlineStr">
+        <is>
+          <t>offen · kritisch</t>
+        </is>
+      </c>
+      <c r="G4" s="41" t="inlineStr"/>
+    </row>
+    <row r="5" ht="44" customHeight="1">
+      <c r="A5" s="41" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="41" t="inlineStr">
+        <is>
+          <t>Frage</t>
+        </is>
+      </c>
+      <c r="C5" s="41" t="inlineStr">
+        <is>
+          <t>Regulierungs-Kodierung</t>
+        </is>
+      </c>
+      <c r="D5" s="41" t="inlineStr">
+        <is>
+          <t>Bedeutung 0/1/9/NA in regulation_start/_end; warum start (1=746) &gt; end (1=337)? Nötig für Regulierungs-Moderator (§7).</t>
+        </is>
+      </c>
+      <c r="E5" s="41" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="F5" s="41" t="inlineStr">
+        <is>
+          <t>offen · kritisch</t>
+        </is>
+      </c>
+      <c r="G5" s="41" t="inlineStr"/>
+    </row>
+    <row r="6" ht="44" customHeight="1">
+      <c r="A6" s="41" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" s="41" t="inlineStr">
+        <is>
+          <t>Frage</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="inlineStr">
+        <is>
+          <t>Methoden-Artefakt-Moderator</t>
+        </is>
+      </c>
+      <c r="D6" s="41" t="inlineStr">
+        <is>
+          <t>Plan §7 nutzt method_artefacts — keine Spalte mappt darauf. Welche Variablen (Endogenitäts-Behandlung, Modelltyp)? Design-Entscheidung bei uns.</t>
+        </is>
+      </c>
+      <c r="E6" s="41" t="inlineStr">
+        <is>
+          <t>Design (wir)</t>
+        </is>
+      </c>
+      <c r="F6" s="41" t="inlineStr">
+        <is>
+          <t>offen · kritisch</t>
+        </is>
+      </c>
+      <c r="G6" s="41" t="inlineStr"/>
+    </row>
+    <row r="7" ht="44" customHeight="1">
+      <c r="A7" s="41" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" s="41" t="inlineStr">
+        <is>
+          <t>Frage</t>
+        </is>
+      </c>
+      <c r="C7" s="41" t="inlineStr">
+        <is>
+          <t>COD-Instrument-Kategorien</t>
+        </is>
+      </c>
+      <c r="D7" s="41" t="inlineStr">
+        <is>
+          <t>cod_measure = interest/rating/yields/derivativ (4). Mapping auf H3-Instrumenttypen? Label „derivativ“? Für §7 + H3.</t>
+        </is>
+      </c>
+      <c r="E7" s="41" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="F7" s="41" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="G7" s="41" t="inlineStr"/>
+    </row>
+    <row r="8" ht="44" customHeight="1">
+      <c r="A8" s="41" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="41" t="inlineStr">
+        <is>
+          <t>Frage</t>
+        </is>
+      </c>
+      <c r="C8" s="41" t="inlineStr">
+        <is>
+          <t>Industrie-Richtung</t>
+        </is>
+      </c>
+      <c r="D8" s="41" t="inlineStr">
+        <is>
+          <t>industry: 1=185, 0=1.121. Ist 1 = emissionsintensiv/„sensitive“? Für Industrie-Moderator (§7).</t>
+        </is>
+      </c>
+      <c r="E8" s="41" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="F8" s="41" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="G8" s="41" t="inlineStr"/>
+    </row>
+    <row r="9" ht="44" customHeight="1">
+      <c r="A9" s="41" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="41" t="inlineStr">
+        <is>
+          <t>Frage</t>
+        </is>
+      </c>
+      <c r="C9" s="41" t="inlineStr">
+        <is>
+          <t>CER-Operationalisierung</t>
+        </is>
+      </c>
+      <c r="D9" s="41" t="inlineStr">
+        <is>
+          <t>cer_measure = Performance (1.063)/Disclosure (243). Bestätigen als die zwei CER-Konstrukte (cer_type).</t>
+        </is>
+      </c>
+      <c r="E9" s="41" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="F9" s="41" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="G9" s="41" t="inlineStr"/>
+    </row>
+    <row r="10" ht="44" customHeight="1">
+      <c r="A10" s="41" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="41" t="inlineStr">
+        <is>
+          <t>Frage</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>Publikationsstatus</t>
+        </is>
+      </c>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>peer-reviewed vs. Working Paper kodiert? journal_q für alle 1.306 gesetzt → alle publiziert? Für Pub-Bias + Grey-Lit-Claim.</t>
+        </is>
+      </c>
+      <c r="E10" s="41" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="F10" s="41" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="G10" s="41" t="inlineStr"/>
+    </row>
+    <row r="11" ht="44" customHeight="1">
+      <c r="A11" s="41" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="41" t="inlineStr">
+        <is>
+          <t>Frage</t>
+        </is>
+      </c>
+      <c r="C11" s="41" t="inlineStr">
+        <is>
+          <t>journal_q-Schwelle</t>
+        </is>
+      </c>
+      <c r="D11" s="41" t="inlineStr">
+        <is>
+          <t>LOW (755)/HIGH (551): welches Ranking/Cutoff? Für Journal-Q-Robustheit (§9).</t>
+        </is>
+      </c>
+      <c r="E11" s="41" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="F11" s="41" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="G11" s="41" t="inlineStr"/>
+    </row>
+    <row r="12" ht="44" customHeight="1">
+      <c r="A12" s="41" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="41" t="inlineStr">
+        <is>
+          <t>Frage</t>
+        </is>
+      </c>
+      <c r="C12" s="41" t="inlineStr">
+        <is>
+          <t>outcome-Spalte</t>
+        </is>
+      </c>
+      <c r="D12" s="41" t="inlineStr">
+        <is>
+          <t>Was kodiert outcome (1,2,3,…) — Effekt-Index je Studie oder Outcome-Typ? Für esid/Struktur.</t>
+        </is>
+      </c>
+      <c r="E12" s="41" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="F12" s="41" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="G12" s="41" t="inlineStr"/>
+    </row>
+    <row r="13" ht="44" customHeight="1">
+      <c r="A13" s="41" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="41" t="inlineStr">
+        <is>
+          <t>Daten</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>Sample-Zeitraum-Jahre</t>
+        </is>
+      </c>
+      <c r="D13" s="41" t="inlineStr">
+        <is>
+          <t>Start-/Endjahr (oder Mittelpunkt) der Stichprobenperiode je Effekt/Studie. Blocker für Identifikation (§4/T8). Interim: pub_year.</t>
+        </is>
+      </c>
+      <c r="E13" s="41" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="F13" s="41" t="inlineStr">
+        <is>
+          <t>offen · kritisch</t>
+        </is>
+      </c>
+      <c r="G13" s="41" t="inlineStr"/>
+    </row>
+    <row r="14" ht="44" customHeight="1">
+      <c r="A14" s="41" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="41" t="inlineStr">
+        <is>
+          <t>Daten</t>
+        </is>
+      </c>
+      <c r="C14" s="41" t="inlineStr">
+        <is>
+          <t>COE-Companion-Studienliste</t>
+        </is>
+      </c>
+      <c r="D14" s="41" t="inlineStr">
+        <is>
+          <t>Welche der 66 COD-Studien überlappen mit der akzeptierten COE-MA? Für Selbstüberlappungs-Verteidigung (DEC-011, Desk-Reject).</t>
+        </is>
+      </c>
+      <c r="E14" s="41" t="inlineStr">
+        <is>
+          <t>extern</t>
+        </is>
+      </c>
+      <c r="F14" s="41" t="inlineStr">
+        <is>
+          <t>offen · kritisch</t>
+        </is>
+      </c>
+      <c r="G14" s="41" t="inlineStr"/>
+    </row>
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="41" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="41" t="inlineStr">
+        <is>
+          <t>Daten</t>
+        </is>
+      </c>
+      <c r="C15" s="41" t="inlineStr">
+        <is>
+          <t>Extremwert-Quellwerte</t>
+        </is>
+      </c>
+      <c r="D15" s="41" t="inlineStr">
+        <is>
+          <t>Originalwerte Drago (r=−0,9977, n=184) + Devalle (r=+0,9998, n=56) aus Primärquellen — verifizieren (DEC-013).</t>
+        </is>
+      </c>
+      <c r="E15" s="41" t="inlineStr">
+        <is>
+          <t>extern</t>
+        </is>
+      </c>
+      <c r="F15" s="41" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="G15" s="41" t="inlineStr"/>
+    </row>
+    <row r="16" ht="44" customHeight="1">
+      <c r="A16" s="41" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="41" t="inlineStr">
+        <is>
+          <t>Daten</t>
+        </is>
+      </c>
+      <c r="C16" s="41" t="inlineStr">
+        <is>
+          <t>Kontrollvariablen-Zahl (k)</t>
+        </is>
+      </c>
+      <c r="D16" s="41" t="inlineStr">
+        <is>
+          <t>Anzahl Kontrollvariablen je der 36 Partials — für exakte PCC-df (n−k−3). Optional: E5 nutzt n−3.</t>
+        </is>
+      </c>
+      <c r="E16" s="41" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="F16" s="41" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="G16" s="41" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3125,6 +3306,343 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Identifikation: Bruch vs. Trend — Werkzeugkasten gegen den Saekulartrend-Confound (#13 / T8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Problem: Pre/Post-Dummy trennt Bruch nicht von Drift. Daten zeigen Drift (Pre-median r=−0,025 vs. Post r=−0,019). Strategie: Trend modellieren, Paris muss DARUEBER HINAUS liefern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Move</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Staerke-Tier</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Was es testet / leistet</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Methode</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Datenabhaengigkeit</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Praezedenz / Anker</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="84" customHeight="1">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>1. Trend-vs-Bruch-Wettrennen</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Tier 1 — essenziell, sofort</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>Trennt glatte Drift vom diskreten Level-Sprung. Dummy weg → nur Drift; ueberlebt → echte Diskontinuitaet</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>Kont. Zeit (zentr. Midpoint) + Paris-Dummy im SELBEN sparsamen Modell</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>Sofort — sobald T0.4 kont. Zeit liefert</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>Huang 2020 (pub-year-Control neben GFC)</t>
+        </is>
+      </c>
+      <c r="G4" s="27" t="inlineStr">
+        <is>
+          <t>OFFEN (T0.4-abh.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="84" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>2. Segmentierte Meta-Regression (ITS)</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>Tier 1 — essenziell, sofort</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>β₂ Level-Sprung, β₃ Slope-Aenderung. Nistet reinen Trend vs. Bruch als testbare Spezialfaelle</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>effect ~ β₀+β₁·Zeit+β₂·post+β₃·(Zeit×post); RVE</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>Sofort — T0.4-abh.</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>ITS-Standard; COVID-Wellen-Analogon</t>
+        </is>
+      </c>
+      <c r="G5" s="27" t="inlineStr">
+        <is>
+          <t>OFFEN (T0.4-abh.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="84" customHeight="1">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>3. Placebo-/Falsifikations-Bruchdaten</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>Tier 2 — stark</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="inlineStr">
+        <is>
+          <t>Bruch an Nicht-Paris-Jahren (2012/13/17/18). Ueberall → kein Paris-Bruch; nur 2015/16 → echt. DEUTET LAG1–3 ZU FALSIFIKATION UM</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="inlineStr">
+        <is>
+          <t>Bruch-Magnitude je Cutoff; Lokalisierungs-Vergleich</t>
+        </is>
+      </c>
+      <c r="E6" s="29" t="inlineStr">
+        <is>
+          <t>Sofort — T0.4-abh.</t>
+        </is>
+      </c>
+      <c r="F6" s="29" t="inlineStr">
+        <is>
+          <t>Placebo-Test-Standard</t>
+        </is>
+      </c>
+      <c r="G6" s="29" t="inlineStr">
+        <is>
+          <t>OFFEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="84" customHeight="1">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>4. Kompositions-Kontrolle</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>Tier 2 — stark, sofort</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>Haelt Studien-/Laender-/Instrument-Mix konstant; Within-Stratum-Check. Nur im Aggregat → kompositorisch</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="inlineStr">
+        <is>
+          <t>Paris-Term + Moderatoren als Kovariaten (= T7); Within-Stratum</t>
+        </is>
+      </c>
+      <c r="E7" s="29" t="inlineStr">
+        <is>
+          <t>Sofort (= T7)</t>
+        </is>
+      </c>
+      <c r="F7" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" s="29" t="inlineStr">
+        <is>
+          <t>OFFEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="84" customHeight="1">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>5. Differential-Exposure (DiD-artig)</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>Tier 2 — stark</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>(post−pre) High-Exposure minus (post−pre) Low: gemeinsamer Trend differenziert sich heraus</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="inlineStr">
+        <is>
+          <t>post × High-Exposure (carbon-intensiv / Carbon-Pricing); Pre-Trend-Check</t>
+        </is>
+      </c>
+      <c r="E8" s="29" t="inlineStr">
+        <is>
+          <t>Sofort; Pre-Trend datenabh.</t>
+        </is>
+      </c>
+      <c r="F8" s="29" t="inlineStr">
+        <is>
+          <t>DiD-Logik. CAVEAT: Parallel-Trends unpruefbar</t>
+        </is>
+      </c>
+      <c r="G8" s="29" t="inlineStr">
+        <is>
+          <t>OFFEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="84" customHeight="1">
+      <c r="A9" s="31" t="inlineStr">
+        <is>
+          <t>6. Within-Study-Identifikation</t>
+        </is>
+      </c>
+      <c r="B9" s="32" t="inlineStr">
+        <is>
+          <t>Tier 3 — Goldstandard, DATENBEDINGT TOT</t>
+        </is>
+      </c>
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>Studien, die Bruch SELBST ueberspannen + separate Pre/Post. Haelt alle between-Confounder konstant</t>
+        </is>
+      </c>
+      <c r="D9" s="31" t="inlineStr">
+        <is>
+          <t>Within-Study-Pre/Post-Kontrast</t>
+        </is>
+      </c>
+      <c r="E9" s="31" t="inlineStr">
+        <is>
+          <t>NICHT VERFUEGBAR — nur 1–3/66 Studien ueberspannen</t>
+        </is>
+      </c>
+      <c r="F9" s="31" t="inlineStr">
+        <is>
+          <t>COVID within-cohort (Sun, Robinson)</t>
+        </is>
+      </c>
+      <c r="G9" s="31" t="inlineStr">
+        <is>
+          <t>ENTFAELLT (Datenbefund T0.3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="84" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>7. Sensitivitaets-Schranke (Bounding)</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Tier 4 — Schlussklammer</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>Wie gross muesste ein Trend sein, um verbleibenden Paris-Dummy zu erklaeren. Begrenzt Confound explizit</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>Oster-Bounds / E-Value auf finales Modell</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>Sofort (nach Hauptmodell)</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>Oster 2019; E-Value (VanderWeele 2017)</t>
+        </is>
+      </c>
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>OFFEN</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3356,7 +3874,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
feat: T0.4 provisional data prep + verifier; DEC-018
Add R/01_prep.R (foundational, diff-reviewed) + R/01_verify_outputs.R
(paired verifier, O1-O12 + row conservation) + docs/data_dictionary.md.
Audit run: 13/13 PASS; flags surfaced (699 non-integer n, 2 extremes
Drago/Devalle, 9 with n<10). data/processed/ gitignored; no analysis run.

- DEC-018 (E8): interim publication-year time axis (pub_year),
  provisional; superseded by sample year (Datenagenda #10).
- analysis_plan.md: data-path fix (data/CER-COD_data_v1.xlsx); §4 axis.
- Tracker: T0.4 -> skript fertig / Lauf gated; T0.1/T0.2 hash backfill.

T1 and all downstream analysis remain GATED until the final dataset
(F2 n-rule + sample year, pending Volker).
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -704,7 +704,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Update 2026-06-30(c): Tab 'Datenagenda' ergänzt — 13 offene Datenfragen/-anforderungen aus Abgleich Daten↔analysis_plan (n-Regel, Regulierung 0/1/9, Sample-Jahre, COE-Overlap, Methoden-Artefakt-Moderator …); Volker-Agenda + Beschaffungs-Backlog.  Update 2026-06-30(b): T0.1 abgeschlossen — docs/analysis_plan.md (kanonische HOW-Spec) geschrieben; +DEC-017 (rho=0,6 working correlation, Sensitivitaet 0,4/0,6/0,8); E1–E6 gelockt; T0.1/T0.2 → DONE. puniform 0.2.8 installiert (Lock-Snapshot ausstehend).  Update 2026-06-30: Methodik-Re-Review gegen neue PK-Methoden-Paper (Stanley et al. 2024/2025 Korrelations-Bias; van Aert 2023 PCC; van Aert &amp; van Assen 2026 p-uniform*; Pustejovsky &amp; Tipton 2022 RVE). +DEC-014..016: (014) CR2-SE fuer FAT-PET-PEESE &amp; Meta-Reg; (015) Korrelations-Small-Sample-Bias → UWLS+3/HS-Robustheit + n-Reporting + PCC-df; (016) Selektionsmodell sekundaer. Roadmap #14–16 ergaenzt.  Update 2026-06-29(b): DEC-Log FINALISIERT (DEC-001..013 aktiv) + DECISION_LOG.md erzeugt — #6–9 zu DECs ausformuliert, #11/#12 bleiben Tasks.  (a): SOMA-Handoff integriert (Verifier, Review-Gate, Source-Pointer, Commit-Ritual, gitignore); DEC-Log auf Methodik-only getrimmt.</t>
+          <t>Update 2026-06-30(d): T0.4 Skript+Verifier gebaut, Audit-Lauf 13/13 PASS (3 FLAGs: 699 non-int n, 2 Extreme, 9x n&lt;10). +DEC-018 (E8: pub_year Interim-Zeitachse). analysis_plan.md §1 Datenpfad-Fix (data/CER-COD_data_v1.xlsx). T0.4 → Skript fertig/Lauf gated; T0.1/T0.2 Hash c5e328a nachgetragen. T1 GATED bis finale Daten.  Update 2026-06-30(c): Tab 'Datenagenda' ergänzt — 13 offene Datenfragen/-anforderungen aus Abgleich Daten↔analysis_plan (n-Regel, Regulierung 0/1/9, Sample-Jahre, COE-Overlap, Methoden-Artefakt-Moderator …); Volker-Agenda + Beschaffungs-Backlog.  Update 2026-06-30(b): T0.1 abgeschlossen — docs/analysis_plan.md (kanonische HOW-Spec) geschrieben; +DEC-017 (rho=0,6 working correlation, Sensitivitaet 0,4/0,6/0,8); E1–E6 gelockt; T0.1/T0.2 → DONE. puniform 0.2.8 installiert (Lock-Snapshot ausstehend).  Update 2026-06-30: Methodik-Re-Review gegen neue PK-Methoden-Paper (Stanley et al. 2024/2025 Korrelations-Bias; van Aert 2023 PCC; van Aert &amp; van Assen 2026 p-uniform*; Pustejovsky &amp; Tipton 2022 RVE). +DEC-014..016: (014) CR2-SE fuer FAT-PET-PEESE &amp; Meta-Reg; (015) Korrelations-Small-Sample-Bias → UWLS+3/HS-Robustheit + n-Reporting + PCC-df; (016) Selektionsmodell sekundaer. Roadmap #14–16 ergaenzt.  Update 2026-06-29(b): DEC-Log FINALISIERT (DEC-001..013 aktiv) + DECISION_LOG.md erzeugt — #6–9 zu DECs ausformuliert, #11/#12 bleiben Tasks.  (a): SOMA-Handoff integriert (Verifier, Review-Gate, Source-Pointer, Commit-Ritual, gitignore); DEC-Log auf Methodik-only getrimmt.</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>DEC-ID-Register (Methodik-only, 17 Eintraege; Pointer auf DECISION_LOG.md). IDs aktiv.</t>
+          <t>DEC-ID-Register (Methodik-only, 18 Eintraege; Pointer auf DECISION_LOG.md). IDs aktiv.</t>
         </is>
       </c>
     </row>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>DEC-007,008</t>
+          <t>DEC-007,008,018</t>
         </is>
       </c>
       <c r="I8" s="9" t="inlineStr">
@@ -2229,7 +2229,7 @@
       </c>
       <c r="I4" s="20" t="inlineStr">
         <is>
-          <t>DONE: analysis_plan.md geschrieben — rma.mv-Signatur, V via impute_covariance_matrix(r=0.6) [DEC-017], CR2 ueber alle Reg [DEC-014], Headline-vs-Robustness a priori (§10). E1–E6 gelockt. → Commit + Hash nachtragen.</t>
+          <t>DONE: analysis_plan.md geschrieben — rma.mv-Signatur, V via impute_covariance_matrix(r=0.6) [DEC-017], CR2 ueber alle Reg [DEC-014], Headline-vs-Robustness a priori (§10). E1–E6 gelockt. → [commit c5e328a].</t>
         </is>
       </c>
       <c r="J4" s="20" t="inlineStr">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="I5" s="20" t="inlineStr">
         <is>
-          <t>DONE: a priori fixiert in analysis_plan.md §10/§6/§2 — Headline=3LMA-RVE pooled; Identifikation=Meta-Reg; Event-Coding &amp; r-Typ a priori. → Commit + Hash nachtragen.</t>
+          <t>DONE: a priori fixiert in analysis_plan.md §10/§6/§2 — Headline=3LMA-RVE pooled; Identifikation=Meta-Reg; Event-Coding &amp; r-Typ a priori. → [commit c5e328a].</t>
         </is>
       </c>
       <c r="J5" s="20" t="inlineStr">
@@ -2380,17 +2380,17 @@
       </c>
       <c r="H7" s="22" t="inlineStr">
         <is>
-          <t>OFFEN — BLOCKER</t>
+          <t>Skript fertig · Lauf gated</t>
         </is>
       </c>
       <c r="I7" s="23" t="inlineStr">
         <is>
-          <t>kont. Zeit fehlt → blockiert Identifikation; Regul.-Richtung 0/1/9 unklar</t>
+          <t>13/13 PASS (R/01_prep.R + Verifier) · FLAGS: O7 (699 non-int n) · O8 (2 Extreme: Drago esid414 / Devalle esid409) · O9 (9x n&lt;10). Keine FAILs. 1306 Zeilen erhalten. LAUF+COMMIT gebaut, aber T1 GATED bis finale Daten (F2 n-Regel + Sample-Jahr via Volker); pub_year = Interim-Achse [DEC-018].</t>
         </is>
       </c>
       <c r="J7" s="23" t="inlineStr">
         <is>
-          <t>R/NN_prep + _verify · data/processed/ (geplant)</t>
+          <t>R/01_prep.R + R/01_verify_outputs.R · docs/data_dictionary.md</t>
         </is>
       </c>
     </row>
@@ -3880,7 +3880,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3902,7 +3902,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>17 aktive Methodik-DECs (DEC-001..017). Volleintraege im DECISION_LOG.md (8-Feld-Schema inkl. gespaltenem Reviewer-Risk). Setup/Prozess → Tab 'Setup'; Reporting/Polish (#11/#12) = Tasks, keine DEC.</t>
+          <t>18 aktive Methodik-DECs (DEC-001..018). Volleintraege im DECISION_LOG.md (8-Feld-Schema inkl. gespaltenem Reviewer-Risk). Setup/Prozess → Tab 'Setup'; Reporting/Polish (#11/#12) = Tasks, keine DEC.</t>
         </is>
       </c>
     </row>
@@ -4572,23 +4572,60 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="44" customHeight="1">
-      <c r="A21" s="34" t="inlineStr">
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="33" t="inlineStr">
+        <is>
+          <t>DEC-018</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Interim-Zeitachse pub_year (E8)</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>#13 / T0.4,T8</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Kont. Zeit fehlt im Datensatz; pub_year aus study geparst (alle 66, 2010-2024) als PROVISORISCHE Interim-Achse. Sample-Jahr (Datenagenda #10) ersetzt sie. T8 re-zentriert aus rohem pub_year.</t>
+        </is>
+      </c>
+      <c r="G21" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="44" customHeight="1">
+      <c r="A22" s="34" t="inlineStr">
         <is>
           <t>Pending/Conditional DECs (im DECISION_LOG.md): Pending-A Headline-Event-Coding (nach T2) · Pending-B Transform-Doku (#11) · Pending-C Framing A vs. C (nach T1–T3 + T8).  Setup/Prozess-Entscheidungen → Tab 'Setup' (keine DECs). #11/#12 = Tasks.</t>
         </is>
       </c>
-      <c r="B21" s="36" t="n"/>
-      <c r="C21" s="36" t="n"/>
-      <c r="D21" s="36" t="n"/>
-      <c r="E21" s="36" t="n"/>
-      <c r="F21" s="36" t="n"/>
-      <c r="G21" s="35" t="n"/>
+      <c r="B22" s="36" t="n"/>
+      <c r="C22" s="36" t="n"/>
+      <c r="D22" s="36" t="n"/>
+      <c r="E22" s="36" t="n"/>
+      <c r="F22" s="36" t="n"/>
+      <c r="G22" s="35" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A21:G21"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: add Ablauf tab (master execution plan, 11 steps + guardrails)
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -8,12 +8,13 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Setup" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aufgaben" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datenagenda" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifikation" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key_Results" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DecisionLog_Index" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ablauf" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aufgaben" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datenagenda" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifikation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key_Results" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DecisionLog_Index" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,6 +74,12 @@
     <font>
       <name val="Arial"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="12">
@@ -203,7 +210,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -322,6 +329,10 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -687,7 +698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B51"/>
+  <dimension ref="A1:B79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -704,7 +715,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Update 2026-06-30(d): T0.4 Skript+Verifier gebaut, Audit-Lauf 13/13 PASS (3 FLAGs: 699 non-int n, 2 Extreme, 9x n&lt;10). +DEC-018 (E8: pub_year Interim-Zeitachse). analysis_plan.md §1 Datenpfad-Fix (data/CER-COD_data_v1.xlsx). T0.4 → Skript fertig/Lauf gated; T0.1/T0.2 Hash c5e328a nachgetragen. T1 GATED bis finale Daten.  Update 2026-06-30(c): Tab 'Datenagenda' ergänzt — 13 offene Datenfragen/-anforderungen aus Abgleich Daten↔analysis_plan (n-Regel, Regulierung 0/1/9, Sample-Jahre, COE-Overlap, Methoden-Artefakt-Moderator …); Volker-Agenda + Beschaffungs-Backlog.  Update 2026-06-30(b): T0.1 abgeschlossen — docs/analysis_plan.md (kanonische HOW-Spec) geschrieben; +DEC-017 (rho=0,6 working correlation, Sensitivitaet 0,4/0,6/0,8); E1–E6 gelockt; T0.1/T0.2 → DONE. puniform 0.2.8 installiert (Lock-Snapshot ausstehend).  Update 2026-06-30: Methodik-Re-Review gegen neue PK-Methoden-Paper (Stanley et al. 2024/2025 Korrelations-Bias; van Aert 2023 PCC; van Aert &amp; van Assen 2026 p-uniform*; Pustejovsky &amp; Tipton 2022 RVE). +DEC-014..016: (014) CR2-SE fuer FAT-PET-PEESE &amp; Meta-Reg; (015) Korrelations-Small-Sample-Bias → UWLS+3/HS-Robustheit + n-Reporting + PCC-df; (016) Selektionsmodell sekundaer. Roadmap #14–16 ergaenzt.  Update 2026-06-29(b): DEC-Log FINALISIERT (DEC-001..013 aktiv) + DECISION_LOG.md erzeugt — #6–9 zu DECs ausformuliert, #11/#12 bleiben Tasks.  (a): SOMA-Handoff integriert (Verifier, Review-Gate, Source-Pointer, Commit-Ritual, gitignore); DEC-Log auf Methodik-only getrimmt.</t>
+          <t>Update 2026-06-30(e): Tab 'Ablauf' ergänzt (Position 1) — Master-Ausführungsplan 11 Schritte + 5 Guardrails; Sequenz Datenaudit→Methodik(Fable5)→Datenset→Analysen→A-vs-C→Positionierung→Kapitel.  Update 2026-06-30(d): T0.4 Skript+Verifier gebaut, Audit-Lauf 13/13 PASS (3 FLAGs: 699 non-int n, 2 Extreme, 9x n&lt;10). +DEC-018 (E8: pub_year Interim-Zeitachse). analysis_plan.md §1 Datenpfad-Fix (data/CER-COD_data_v1.xlsx). T0.4 → Skript fertig/Lauf gated; T0.1/T0.2 Hash c5e328a nachgetragen. T1 GATED bis finale Daten.  Update 2026-06-30(c): Tab 'Datenagenda' ergänzt — 13 offene Datenfragen/-anforderungen aus Abgleich Daten↔analysis_plan (n-Regel, Regulierung 0/1/9, Sample-Jahre, COE-Overlap, Methoden-Artefakt-Moderator …); Volker-Agenda + Beschaffungs-Backlog.  Update 2026-06-30(b): T0.1 abgeschlossen — docs/analysis_plan.md (kanonische HOW-Spec) geschrieben; +DEC-017 (rho=0,6 working correlation, Sensitivitaet 0,4/0,6/0,8); E1–E6 gelockt; T0.1/T0.2 → DONE. puniform 0.2.8 installiert (Lock-Snapshot ausstehend).  Update 2026-06-30: Methodik-Re-Review gegen neue PK-Methoden-Paper (Stanley et al. 2024/2025 Korrelations-Bias; van Aert 2023 PCC; van Aert &amp; van Assen 2026 p-uniform*; Pustejovsky &amp; Tipton 2022 RVE). +DEC-014..016: (014) CR2-SE fuer FAT-PET-PEESE &amp; Meta-Reg; (015) Korrelations-Small-Sample-Bias → UWLS+3/HS-Robustheit + n-Reporting + PCC-df; (016) Selektionsmodell sekundaer. Roadmap #14–16 ergaenzt.  Update 2026-06-29(b): DEC-Log FINALISIERT (DEC-001..013 aktiv) + DECISION_LOG.md erzeugt — #6–9 zu DECs ausformuliert, #11/#12 bleiben Tasks.  (a): SOMA-Handoff integriert (Verifier, Review-Gate, Source-Pointer, Commit-Ritual, gitignore); DEC-Log auf Methodik-only getrimmt.</t>
         </is>
       </c>
     </row>
@@ -1264,6 +1275,45 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="37" t="inlineStr">
+        <is>
+          <t>Ablauf</t>
+        </is>
+      </c>
+      <c r="B52" s="38" t="inlineStr">
+        <is>
+          <t>Master-Ablaufplan (11 Schritte + Guardrails): Datenaudit → Methodik (Fable 5) → Datenset → Analysen → A-vs-C → Positionierung → Kapitel. Nr/Block/Schritt/Beschreibung/Gate/Ort/Status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A21:B21"/>
@@ -1287,6 +1337,604 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="42" t="inlineStr">
+        <is>
+          <t>Ausführungsplan — CER–COD FOMA (verfeinerte Sequenz, Stand 2026-06-30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="40" t="inlineStr">
+        <is>
+          <t>Nr</t>
+        </is>
+      </c>
+      <c r="B2" s="40" t="inlineStr">
+        <is>
+          <t>Block</t>
+        </is>
+      </c>
+      <c r="C2" s="40" t="inlineStr">
+        <is>
+          <t>Schritt</t>
+        </is>
+      </c>
+      <c r="D2" s="40" t="inlineStr">
+        <is>
+          <t>Kurzbeschreibung</t>
+        </is>
+      </c>
+      <c r="E2" s="40" t="inlineStr">
+        <is>
+          <t>Gate / Abhängigkeit</t>
+        </is>
+      </c>
+      <c r="F2" s="40" t="inlineStr">
+        <is>
+          <t>Ort</t>
+        </is>
+      </c>
+      <c r="G2" s="40" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="46" customHeight="1">
+      <c r="A3" s="41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="B3" s="41" t="inlineStr">
+        <is>
+          <t>Daten &amp; Methodik</t>
+        </is>
+      </c>
+      <c r="C3" s="41" t="inlineStr">
+        <is>
+          <t>Volker-Daten-Audit</t>
+        </is>
+      </c>
+      <c r="D3" s="41" t="inlineStr">
+        <is>
+          <t>Volkers Lieferung gegen Datenagenda prüfen (kritisch: 1 n-Regel, 2 Regulierung, 10 Sample-Jahre; Klärung: 4/5/7) + COE-Overlap (#11). Ergebnis: was gelöst / offen / ändert Methodik.</t>
+        </is>
+      </c>
+      <c r="E3" s="41" t="inlineStr">
+        <is>
+          <t>Volker-Daten erhalten ✓</t>
+        </is>
+      </c>
+      <c r="F3" s="41" t="inlineStr">
+        <is>
+          <t>dieser Chat</t>
+        </is>
+      </c>
+      <c r="G3" s="41" t="inlineStr">
+        <is>
+          <t>jetzt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="46" customHeight="1">
+      <c r="A4" s="41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" s="41" t="inlineStr">
+        <is>
+          <t>Daten &amp; Methodik</t>
+        </is>
+      </c>
+      <c r="C4" s="41" t="inlineStr">
+        <is>
+          <t>Methodik finalisieren</t>
+        </is>
+      </c>
+      <c r="D4" s="41" t="inlineStr">
+        <is>
+          <t>Geplante Methodik (DEC-001..018) gegen Audit-Ergebnis validieren + offene Items schließen. Ergebnis: finaler analysis_plan.</t>
+        </is>
+      </c>
+      <c r="E4" s="41" t="inlineStr">
+        <is>
+          <t>Schritt 0</t>
+        </is>
+      </c>
+      <c r="F4" s="41" t="inlineStr">
+        <is>
+          <t>neuer Chat · Fable 5</t>
+        </is>
+      </c>
+      <c r="G4" s="41" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="41" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" s="41" t="inlineStr">
+        <is>
+          <t>Daten &amp; Methodik</t>
+        </is>
+      </c>
+      <c r="C5" s="41" t="inlineStr">
+        <is>
+          <t>Finales Datenset bauen</t>
+        </is>
+      </c>
+      <c r="D5" s="41" t="inlineStr">
+        <is>
+          <t>Re-prep (R/01_prep.R) gegen finale Volker-Daten; n-Regel + Sample-Jahr + Regulierung final. Öffnet das T1-Gate.</t>
+        </is>
+      </c>
+      <c r="E5" s="41" t="inlineStr">
+        <is>
+          <t>Schritt 1 + Volker-Antworten</t>
+        </is>
+      </c>
+      <c r="F5" s="41" t="inlineStr">
+        <is>
+          <t>CC / RStudio</t>
+        </is>
+      </c>
+      <c r="G5" s="41" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="41" t="inlineStr">
+        <is>
+          <t>Analysen</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="inlineStr">
+        <is>
+          <t>Alle Analysen</t>
+        </is>
+      </c>
+      <c r="D6" s="41" t="inlineStr">
+        <is>
+          <t>T1 (3LMA-RVE) · T4 (Robustheit) · T5 (Pub-Bias) · T7 (unified MR) · T8 (Identifikation). Je Skript + Verifier.</t>
+        </is>
+      </c>
+      <c r="E6" s="41" t="inlineStr">
+        <is>
+          <t>finales Datenset (Schritt 2)</t>
+        </is>
+      </c>
+      <c r="F6" s="41" t="inlineStr">
+        <is>
+          <t>CC / RStudio</t>
+        </is>
+      </c>
+      <c r="G6" s="41" t="inlineStr">
+        <is>
+          <t>gated</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="41" t="inlineStr">
+        <is>
+          <t>3b</t>
+        </is>
+      </c>
+      <c r="B7" s="41" t="inlineStr">
+        <is>
+          <t>Analysen</t>
+        </is>
+      </c>
+      <c r="C7" s="41" t="inlineStr">
+        <is>
+          <t>Ergebnisse + A-vs-C entscheiden</t>
+        </is>
+      </c>
+      <c r="D7" s="41" t="inlineStr">
+        <is>
+          <t>Finalen Paris-Befund interpretieren; strategische Weiche Pfad A (Nullbefund/Debunking) vs. C (kontingenter Effekt). Determiniert 4–6.</t>
+        </is>
+      </c>
+      <c r="E7" s="41" t="inlineStr">
+        <is>
+          <t>Schritt 3</t>
+        </is>
+      </c>
+      <c r="F7" s="41" t="inlineStr">
+        <is>
+          <t>dieser Chat</t>
+        </is>
+      </c>
+      <c r="G7" s="41" t="inlineStr">
+        <is>
+          <t>gated</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="A8" s="41" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" s="41" t="inlineStr">
+        <is>
+          <t>Positionierung</t>
+        </is>
+      </c>
+      <c r="C8" s="41" t="inlineStr">
+        <is>
+          <t>Narrativer roter Faden</t>
+        </is>
+      </c>
+      <c r="D8" s="41" t="inlineStr">
+        <is>
+          <t>Intro→RQ→Beitrag; Claim–Evidence-Abgleich (Paris-Framing an Befund). GEKOPPELT mit 5/6, iterativ.</t>
+        </is>
+      </c>
+      <c r="E8" s="41" t="inlineStr">
+        <is>
+          <t>A-vs-C (3b)</t>
+        </is>
+      </c>
+      <c r="F8" s="41" t="inlineStr">
+        <is>
+          <t>dieser Chat</t>
+        </is>
+      </c>
+      <c r="G8" s="41" t="inlineStr">
+        <is>
+          <t>gated</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
+      <c r="A9" s="41" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B9" s="41" t="inlineStr">
+        <is>
+          <t>Positionierung</t>
+        </is>
+      </c>
+      <c r="C9" s="41" t="inlineStr">
+        <is>
+          <t>Hypothesen</t>
+        </is>
+      </c>
+      <c r="D9" s="41" t="inlineStr">
+        <is>
+          <t>H2/H3-Renumber, RQ↔H-Mapping, Formulierung an A-vs-C. GEKOPPELT mit 4/6.</t>
+        </is>
+      </c>
+      <c r="E9" s="41" t="inlineStr">
+        <is>
+          <t>A-vs-C (3b)</t>
+        </is>
+      </c>
+      <c r="F9" s="41" t="inlineStr">
+        <is>
+          <t>dieser Chat</t>
+        </is>
+      </c>
+      <c r="G9" s="41" t="inlineStr">
+        <is>
+          <t>gated</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="46" customHeight="1">
+      <c r="A10" s="41" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B10" s="41" t="inlineStr">
+        <is>
+          <t>Positionierung</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>Theorie / Konstrukt</t>
+        </is>
+      </c>
+      <c r="D10" s="41" t="inlineStr">
+        <is>
+          <t>Transition-Risk-Repricing als integrierende Klammer; Theorie-Architektur an Befund. GEKOPPELT mit 4/5.</t>
+        </is>
+      </c>
+      <c r="E10" s="41" t="inlineStr">
+        <is>
+          <t>A-vs-C (3b)</t>
+        </is>
+      </c>
+      <c r="F10" s="41" t="inlineStr">
+        <is>
+          <t>dieser Chat</t>
+        </is>
+      </c>
+      <c r="G10" s="41" t="inlineStr">
+        <is>
+          <t>gated</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
+      <c r="A11" s="41" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="B11" s="41" t="inlineStr">
+        <is>
+          <t>Schreiben</t>
+        </is>
+      </c>
+      <c r="C11" s="41" t="inlineStr">
+        <is>
+          <t>Ch 2 — Literatur &amp; Hypothesen</t>
+        </is>
+      </c>
+      <c r="D11" s="41" t="inlineStr">
+        <is>
+          <t>Schreiben/finalisieren; Novelty/Positionierung (Zarea/Witte, COE-Abgrenzung DEC-011).</t>
+        </is>
+      </c>
+      <c r="E11" s="41" t="inlineStr">
+        <is>
+          <t>Positionierung (4–6)</t>
+        </is>
+      </c>
+      <c r="F11" s="41" t="inlineStr">
+        <is>
+          <t>dieser Chat</t>
+        </is>
+      </c>
+      <c r="G11" s="41" t="inlineStr">
+        <is>
+          <t>gated</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
+      <c r="A12" s="41" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="B12" s="41" t="inlineStr">
+        <is>
+          <t>Schreiben</t>
+        </is>
+      </c>
+      <c r="C12" s="41" t="inlineStr">
+        <is>
+          <t>Ch 3 — Methodik</t>
+        </is>
+      </c>
+      <c r="D12" s="41" t="inlineStr">
+        <is>
+          <t>Schreiben/finalisieren gegen finale Methodik + Analysen.</t>
+        </is>
+      </c>
+      <c r="E12" s="41" t="inlineStr">
+        <is>
+          <t>Schritt 1 + 3</t>
+        </is>
+      </c>
+      <c r="F12" s="41" t="inlineStr">
+        <is>
+          <t>dieser Chat</t>
+        </is>
+      </c>
+      <c r="G12" s="41" t="inlineStr">
+        <is>
+          <t>gated</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="46" customHeight="1">
+      <c r="A13" s="41" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B13" s="41" t="inlineStr">
+        <is>
+          <t>Schreiben</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>Ch 4 — Results &amp; Diskussion</t>
+        </is>
+      </c>
+      <c r="D13" s="41" t="inlineStr">
+        <is>
+          <t>Schreiben/finalisieren gegen Analysen + A-vs-C.</t>
+        </is>
+      </c>
+      <c r="E13" s="41" t="inlineStr">
+        <is>
+          <t>Schritt 3 + 3b</t>
+        </is>
+      </c>
+      <c r="F13" s="41" t="inlineStr">
+        <is>
+          <t>dieser Chat</t>
+        </is>
+      </c>
+      <c r="G13" s="41" t="inlineStr">
+        <is>
+          <t>gated</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="46" customHeight="1">
+      <c r="A14" s="41" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B14" s="41" t="inlineStr">
+        <is>
+          <t>Schreiben</t>
+        </is>
+      </c>
+      <c r="C14" s="41" t="inlineStr">
+        <is>
+          <t>Ch 1 — Einleitung</t>
+        </is>
+      </c>
+      <c r="D14" s="41" t="inlineStr">
+        <is>
+          <t>Schreiben/finalisieren zuletzt, aus finalem Framing.</t>
+        </is>
+      </c>
+      <c r="E14" s="41" t="inlineStr">
+        <is>
+          <t>Ch 2–4 (7–9)</t>
+        </is>
+      </c>
+      <c r="F14" s="41" t="inlineStr">
+        <is>
+          <t>dieser Chat</t>
+        </is>
+      </c>
+      <c r="G14" s="41" t="inlineStr">
+        <is>
+          <t>gated</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="46" customHeight="1">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B15" s="41" t="inlineStr">
+        <is>
+          <t>Schreiben</t>
+        </is>
+      </c>
+      <c r="C15" s="41" t="inlineStr">
+        <is>
+          <t>Ch 5 — Conclusion + Abstract</t>
+        </is>
+      </c>
+      <c r="D15" s="41" t="inlineStr">
+        <is>
+          <t>Schreiben/finalisieren; Abstract ganz am Ende.</t>
+        </is>
+      </c>
+      <c r="E15" s="41" t="inlineStr">
+        <is>
+          <t>Ch 1–4</t>
+        </is>
+      </c>
+      <c r="F15" s="41" t="inlineStr">
+        <is>
+          <t>dieser Chat</t>
+        </is>
+      </c>
+      <c r="G15" s="41" t="inlineStr">
+        <is>
+          <t>gated</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="43" t="inlineStr">
+        <is>
+          <t>Guardrails / Hinweise</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="41" t="inlineStr">
+        <is>
+          <t>G1 — PK vor Schritt 1 aktuell: DEC-018, analysis_plan.md, Status-xlsx, data_dictionary.md — und die T0.4-Skripte (01_prep.R, 01_verify_outputs.R) mit hochladen, damit Fable 5 die reale Prep-Logik sieht, nicht nur die Spec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="41" t="inlineStr">
+        <is>
+          <t>G2 — Scope in Fable-5 binden: offene Items schließen + Plan validieren; die 18 DECs NICHT grundlos neu aufrollen (verteidigte Entscheidungen → sonst Churn).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>G3 — Fordert Fable 5 einen DEC heraus: auf Merit prüfen + loggen — weder automatisch übernehmen noch abtun. Begründete Kritik bleibt, bis entkräftet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="41" t="inlineStr">
+        <is>
+          <t>G4 — Schritte 4–6 sind ein gekoppelter, iterativer Positionierungs-Block (Primärordnung Narrativ→Hyp→Theorie), kein starrer Einmal-Lock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>G5 — COE-Selbstüberlappung (#11) ist Desk-Reject-Risiko: klären im Audit (0) oder spätestens bei Ch 2 (7).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A19:G19"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2099,7 +2747,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2819,7 +3467,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3300,7 +3948,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3637,7 +4285,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3874,7 +4522,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
data: finalize dataset v4 + DEC-019..023
Add CER-COD_data_v4.xlsx (final: 40 cols + country_lookup + source_lookup)
as the analysis source. Effect-size set identical to v1; adds derived
Pre/Post, country (region/dev/culture/legal), and quality moderators.

- DEC-019 n=no_firms · DEC-020 Pre/Post suite + headline shift (end->mid/
  continuous) · DEC-021 sample_mid time axis (retires DEC-018) ·
  DEC-022 country moderators (IMF/DST/La Porta, parse-homogeneous->NCE) ·
  DEC-023 quality moderators (VHB/JIF/field; CIT dropped).
- Datenagenda resolved; Analysen tab added.

Open for methodology finalization: headline-cut choice; VHB/JIF-for-
working-papers basis; COE self-overlap (Datenagenda #11).
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -11,10 +11,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ablauf" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aufgaben" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datenagenda" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifikation" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key_Results" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DecisionLog_Index" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysen" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datenagenda" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifikation" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key_Results" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DecisionLog_Index" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -210,7 +211,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -333,6 +334,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -698,7 +702,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B79"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -715,7 +719,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Update 2026-06-30(e): Tab 'Ablauf' ergänzt (Position 1) — Master-Ausführungsplan 11 Schritte + 5 Guardrails; Sequenz Datenaudit→Methodik(Fable5)→Datenset→Analysen→A-vs-C→Positionierung→Kapitel.  Update 2026-06-30(d): T0.4 Skript+Verifier gebaut, Audit-Lauf 13/13 PASS (3 FLAGs: 699 non-int n, 2 Extreme, 9x n&lt;10). +DEC-018 (E8: pub_year Interim-Zeitachse). analysis_plan.md §1 Datenpfad-Fix (data/CER-COD_data_v1.xlsx). T0.4 → Skript fertig/Lauf gated; T0.1/T0.2 Hash c5e328a nachgetragen. T1 GATED bis finale Daten.  Update 2026-06-30(c): Tab 'Datenagenda' ergänzt — 13 offene Datenfragen/-anforderungen aus Abgleich Daten↔analysis_plan (n-Regel, Regulierung 0/1/9, Sample-Jahre, COE-Overlap, Methoden-Artefakt-Moderator …); Volker-Agenda + Beschaffungs-Backlog.  Update 2026-06-30(b): T0.1 abgeschlossen — docs/analysis_plan.md (kanonische HOW-Spec) geschrieben; +DEC-017 (rho=0,6 working correlation, Sensitivitaet 0,4/0,6/0,8); E1–E6 gelockt; T0.1/T0.2 → DONE. puniform 0.2.8 installiert (Lock-Snapshot ausstehend).  Update 2026-06-30: Methodik-Re-Review gegen neue PK-Methoden-Paper (Stanley et al. 2024/2025 Korrelations-Bias; van Aert 2023 PCC; van Aert &amp; van Assen 2026 p-uniform*; Pustejovsky &amp; Tipton 2022 RVE). +DEC-014..016: (014) CR2-SE fuer FAT-PET-PEESE &amp; Meta-Reg; (015) Korrelations-Small-Sample-Bias → UWLS+3/HS-Robustheit + n-Reporting + PCC-df; (016) Selektionsmodell sekundaer. Roadmap #14–16 ergaenzt.  Update 2026-06-29(b): DEC-Log FINALISIERT (DEC-001..013 aktiv) + DECISION_LOG.md erzeugt — #6–9 zu DECs ausformuliert, #11/#12 bleiben Tasks.  (a): SOMA-Handoff integriert (Verifier, Review-Gate, Source-Pointer, Commit-Ritual, gitignore); DEC-Log auf Methodik-only getrimmt.</t>
+          <t>Update 2026-07-03: Datenphase abgeschlossen — v4 final (40 Sp. + country_lookup + source_lookup). +DEC-019–023 (n=no_firms; Pre/Post-Suite+Headline-Cut; sample_mid löst DEC-018 ab; country×4; quality, CIT gestrichen). Datenagenda gelöst (offen: #11 COE, #12 Quellprüfung, VHB/JIF-WP). Tab 'Analysen' ergänzt. Offen für Fable-5: Headline-Cut.  Update 2026-06-30(e): Tab 'Ablauf' ergänzt (Position 1) — Master-Ausführungsplan 11 Schritte + 5 Guardrails; Sequenz Datenaudit→Methodik(Fable5)→Datenset→Analysen→A-vs-C→Positionierung→Kapitel.  Update 2026-06-30(d): T0.4 Skript+Verifier gebaut, Audit-Lauf 13/13 PASS (3 FLAGs: 699 non-int n, 2 Extreme, 9x n&lt;10). +DEC-018 (E8: pub_year Interim-Zeitachse). analysis_plan.md §1 Datenpfad-Fix (data/CER-COD_data_v1.xlsx). T0.4 → Skript fertig/Lauf gated; T0.1/T0.2 Hash c5e328a nachgetragen. T1 GATED bis finale Daten.  Update 2026-06-30(c): Tab 'Datenagenda' ergänzt — 13 offene Datenfragen/-anforderungen aus Abgleich Daten↔analysis_plan (n-Regel, Regulierung 0/1/9, Sample-Jahre, COE-Overlap, Methoden-Artefakt-Moderator …); Volker-Agenda + Beschaffungs-Backlog.  Update 2026-06-30(b): T0.1 abgeschlossen — docs/analysis_plan.md (kanonische HOW-Spec) geschrieben; +DEC-017 (rho=0,6 working correlation, Sensitivitaet 0,4/0,6/0,8); E1–E6 gelockt; T0.1/T0.2 → DONE. puniform 0.2.8 installiert (Lock-Snapshot ausstehend).  Update 2026-06-30: Methodik-Re-Review gegen neue PK-Methoden-Paper (Stanley et al. 2024/2025 Korrelations-Bias; van Aert 2023 PCC; van Aert &amp; van Assen 2026 p-uniform*; Pustejovsky &amp; Tipton 2022 RVE). +DEC-014..016: (014) CR2-SE fuer FAT-PET-PEESE &amp; Meta-Reg; (015) Korrelations-Small-Sample-Bias → UWLS+3/HS-Robustheit + n-Reporting + PCC-df; (016) Selektionsmodell sekundaer. Roadmap #14–16 ergaenzt.  Update 2026-06-29(b): DEC-Log FINALISIERT (DEC-001..013 aktiv) + DECISION_LOG.md erzeugt — #6–9 zu DECs ausformuliert, #11/#12 bleiben Tasks.  (a): SOMA-Handoff integriert (Verifier, Review-Gate, Source-Pointer, Commit-Ritual, gitignore); DEC-Log auf Methodik-only getrimmt.</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1263,7 @@
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>DEC-ID-Register (Methodik-only, 18 Eintraege; Pointer auf DECISION_LOG.md). IDs aktiv.</t>
+          <t>DEC-ID-Register (Methodik-only, 23 Eintraege; Pointer auf DECISION_LOG.md). IDs aktiv.</t>
         </is>
       </c>
     </row>
@@ -1287,33 +1291,6 @@
         </is>
       </c>
     </row>
-    <row r="53"/>
-    <row r="54"/>
-    <row r="55"/>
-    <row r="56"/>
-    <row r="57"/>
-    <row r="58"/>
-    <row r="59"/>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
-    <row r="76"/>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A21:B21"/>
@@ -1411,7 +1388,7 @@
       </c>
       <c r="D3" s="41" t="inlineStr">
         <is>
-          <t>Volkers Lieferung gegen Datenagenda prüfen (kritisch: 1 n-Regel, 2 Regulierung, 10 Sample-Jahre; Klärung: 4/5/7) + COE-Overlap (#11). Ergebnis: was gelöst / offen / ändert Methodik.</t>
+          <t>Volkers Lieferung gegen Datenagenda prüfen (kritisch: 1 n-Regel, 2 Regulierung, 10 Sample-Jahre; Klärung: 4/5/7) + COE-Overlap (#11). Ergebnis: was gelöst / offen / ändert Methodik. [ERLEDIGT: v4 final, DEC-019–023; Lookups country+source; Headline-Cut + VHB/JIF-WP offen für Step 1]</t>
         </is>
       </c>
       <c r="E3" s="41" t="inlineStr">
@@ -1426,7 +1403,7 @@
       </c>
       <c r="G3" s="41" t="inlineStr">
         <is>
-          <t>jetzt</t>
+          <t>erledigt</t>
         </is>
       </c>
     </row>
@@ -3473,6 +3450,440 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="42" t="inlineStr">
+        <is>
+          <t>Analysen-Übersicht — CER–COD FOMA (aus analysen.xlsx; Daten-Status v4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1">
+      <c r="A2" s="44" t="inlineStr">
+        <is>
+          <t>Block / Analyse</t>
+        </is>
+      </c>
+      <c r="B2" s="44" t="inlineStr">
+        <is>
+          <t>Split</t>
+        </is>
+      </c>
+      <c r="C2" s="44" t="inlineStr">
+        <is>
+          <t>Status (Daten v4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="43" t="inlineStr">
+        <is>
+          <t>1 — Main</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="41" t="inlineStr">
+        <is>
+          <t>Forest Plot</t>
+        </is>
+      </c>
+      <c r="B4" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C4" s="41" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="41" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="B5" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C5" s="41" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="41" t="inlineStr">
+        <is>
+          <t>Overall Pre/Post</t>
+        </is>
+      </c>
+      <c r="B6" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="43" t="inlineStr">
+        <is>
+          <t>2 — Robustheit: Parametrisierung</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="41" t="inlineStr">
+        <is>
+          <t>Pre/Post Lag 1/2/3</t>
+        </is>
+      </c>
+      <c r="B8" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C8" s="41" t="inlineStr">
+        <is>
+          <t>ready (pp_share_lag1–3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="41" t="inlineStr">
+        <is>
+          <t>Event-Cut: median / end / start</t>
+        </is>
+      </c>
+      <c r="B9" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C9" s="41" t="inlineStr">
+        <is>
+          <t>ready (pp_median/end/start)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="41" t="inlineStr">
+        <is>
+          <t>Outlier: drop-outliers/-contributors · cap · SAMD(2×,3×) · SD · winsor · trim</t>
+        </is>
+      </c>
+      <c r="B10" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C10" s="41" t="inlineStr">
+        <is>
+          <t>ready (R)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="41" t="inlineStr">
+        <is>
+          <t>Effektgröße: drop bivariate</t>
+        </is>
+      </c>
+      <c r="B11" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C11" s="41" t="inlineStr">
+        <is>
+          <t>ready (ES_measure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="41" t="inlineStr">
+        <is>
+          <t>Modell-Spez. (FE/RE/…)</t>
+        </is>
+      </c>
+      <c r="B12" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C12" s="41" t="inlineStr">
+        <is>
+          <t>ready (R)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="28" customHeight="1">
+      <c r="A13" s="41" t="inlineStr">
+        <is>
+          <t>Study-Level</t>
+        </is>
+      </c>
+      <c r="B13" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>ready (R-Aggregation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="41" t="inlineStr">
+        <is>
+          <t>Firm-Years</t>
+        </is>
+      </c>
+      <c r="B14" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C14" s="41" t="inlineStr">
+        <is>
+          <t>ready (no_firm-years)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="41" t="inlineStr">
+        <is>
+          <t>Quality: Status / VHB / JIF / Field</t>
+        </is>
+      </c>
+      <c r="B15" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C15" s="41" t="inlineStr">
+        <is>
+          <t>ready (v4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="41" t="inlineStr">
+        <is>
+          <t>Quality: CIT</t>
+        </is>
+      </c>
+      <c r="B16" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C16" s="41" t="inlineStr">
+        <is>
+          <t>GESTRICHEN (DEC-023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="43" t="inlineStr">
+        <is>
+          <t>3 — Robustheit: Underlying Trend (T8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="41" t="inlineStr">
+        <is>
+          <t>Secular-Trend / Identifikation</t>
+        </is>
+      </c>
+      <c r="B18" s="41" t="inlineStr">
+        <is>
+          <t>kont. Zeit</t>
+        </is>
+      </c>
+      <c r="C18" s="41" t="inlineStr">
+        <is>
+          <t>ready (sample_mid, DEC-021)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="43" t="inlineStr">
+        <is>
+          <t>4 — Publication Bias</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="41" t="inlineStr">
+        <is>
+          <t>Funnel · FAT-PET-PEESE · Trim&amp;Fill · 3PSM · p-curve/p-uniform · RoBMA</t>
+        </is>
+      </c>
+      <c r="B20" s="41" t="inlineStr">
+        <is>
+          <t>overall/subgruppen</t>
+        </is>
+      </c>
+      <c r="C20" s="41" t="inlineStr">
+        <is>
+          <t>ready (R; RoBMA-Paket)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="43" t="inlineStr">
+        <is>
+          <t>5 — Moderatoren</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>CER-Measure (perf/discl)</t>
+        </is>
+      </c>
+      <c r="B22" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C22" s="41" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="41" t="inlineStr">
+        <is>
+          <t>COD-Instrument (loan/rating/bond/deriv)</t>
+        </is>
+      </c>
+      <c r="B23" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C23" s="41" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="41" t="inlineStr">
+        <is>
+          <t>Industrie (sensitive/non-sensitive)</t>
+        </is>
+      </c>
+      <c r="B24" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C24" s="41" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="41" t="inlineStr">
+        <is>
+          <t>Country: Region · Development · Culture · Legal</t>
+        </is>
+      </c>
+      <c r="B25" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C25" s="41" t="inlineStr">
+        <is>
+          <t>ready (v4, 4 Schemata + NCE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="41" t="inlineStr">
+        <is>
+          <t>Regulierung (ETS/CT)</t>
+        </is>
+      </c>
+      <c r="B26" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C26" s="41" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="43" t="inlineStr">
+        <is>
+          <t>6 — Regression (T7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="41" t="inlineStr">
+        <is>
+          <t>Unified Meta-Regression</t>
+        </is>
+      </c>
+      <c r="B28" s="41" t="inlineStr">
+        <is>
+          <t>kont. + Interaktionen</t>
+        </is>
+      </c>
+      <c r="C28" s="41" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A7:C7"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3562,7 +3973,7 @@
       </c>
       <c r="F4" s="41" t="inlineStr">
         <is>
-          <t>offen · kritisch</t>
+          <t>gelöst (DEC-019: no_firms/firm-years)</t>
         </is>
       </c>
       <c r="G4" s="41" t="inlineStr"/>
@@ -3593,7 +4004,7 @@
       </c>
       <c r="F5" s="41" t="inlineStr">
         <is>
-          <t>offen · kritisch</t>
+          <t>gelöst (ETS/CT-Semantik)</t>
         </is>
       </c>
       <c r="G5" s="41" t="inlineStr"/>
@@ -3624,7 +4035,7 @@
       </c>
       <c r="F6" s="41" t="inlineStr">
         <is>
-          <t>offen · kritisch</t>
+          <t>offen · Design (Fable-5)</t>
         </is>
       </c>
       <c r="G6" s="41" t="inlineStr"/>
@@ -3655,7 +4066,7 @@
       </c>
       <c r="F7" s="41" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>gelöst (loan/rating/bond/deriv)</t>
         </is>
       </c>
       <c r="G7" s="41" t="inlineStr"/>
@@ -3686,7 +4097,7 @@
       </c>
       <c r="F8" s="41" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>gelöst (sensitive/non-sensitive)</t>
         </is>
       </c>
       <c r="G8" s="41" t="inlineStr"/>
@@ -3717,7 +4128,7 @@
       </c>
       <c r="F9" s="41" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>gelöst (perf/disclosure)</t>
         </is>
       </c>
       <c r="G9" s="41" t="inlineStr"/>
@@ -3748,7 +4159,7 @@
       </c>
       <c r="F10" s="41" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>gelöst (q_status)</t>
         </is>
       </c>
       <c r="G10" s="41" t="inlineStr"/>
@@ -3779,7 +4190,7 @@
       </c>
       <c r="F11" s="41" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>gelöst → VHB/JIF-Tiers (DEC-023)</t>
         </is>
       </c>
       <c r="G11" s="41" t="inlineStr"/>
@@ -3810,7 +4221,7 @@
       </c>
       <c r="F12" s="41" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>minor (Effekt-Index)</t>
         </is>
       </c>
       <c r="G12" s="41" t="inlineStr"/>
@@ -3841,7 +4252,7 @@
       </c>
       <c r="F13" s="41" t="inlineStr">
         <is>
-          <t>offen · kritisch</t>
+          <t>gelöst (DEC-021: sample_mid)</t>
         </is>
       </c>
       <c r="G13" s="41" t="inlineStr"/>
@@ -3872,7 +4283,7 @@
       </c>
       <c r="F14" s="41" t="inlineStr">
         <is>
-          <t>offen · kritisch</t>
+          <t>offen · extern (COE-Liste)</t>
         </is>
       </c>
       <c r="G14" s="41" t="inlineStr"/>
@@ -3903,7 +4314,7 @@
       </c>
       <c r="F15" s="41" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>offen · Quellprüfung Drago/Devalle</t>
         </is>
       </c>
       <c r="G15" s="41" t="inlineStr"/>
@@ -3934,7 +4345,7 @@
       </c>
       <c r="F16" s="41" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>gelöst → E5 (n−3) / CIT gestrichen</t>
         </is>
       </c>
       <c r="G16" s="41" t="inlineStr"/>
@@ -3948,7 +4359,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4285,7 +4696,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4522,13 +4933,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4550,7 +4961,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>18 aktive Methodik-DECs (DEC-001..018). Volleintraege im DECISION_LOG.md (8-Feld-Schema inkl. gespaltenem Reviewer-Risk). Setup/Prozess → Tab 'Setup'; Reporting/Polish (#11/#12) = Tasks, keine DEC.</t>
+          <t>23 aktive Methodik-DECs (DEC-001..023). Volleintraege im DECISION_LOG.md (8-Feld-Schema inkl. gespaltenem Reviewer-Risk). Setup/Prozess → Tab 'Setup'; Reporting/Polish (#11/#12) = Tasks, keine DEC.</t>
         </is>
       </c>
     </row>
@@ -5257,23 +5668,208 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="44" customHeight="1">
-      <c r="A22" s="34" t="inlineStr">
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="33" t="inlineStr">
+        <is>
+          <t>DEC-019</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>n-Definition = no_firms (headline)</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>T1,T4</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>no_firms als Gewichts-Basis; no_firm-years + study-level = Robustheit. [E14]</t>
+        </is>
+      </c>
+      <c r="G22" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>DEC-020</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Pre/Post-Operationalisierung + Headline-Cut</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>T1,T4,T8</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Suite (share/mid/end/start/median/tertil/window_class); Headline mid/kont., end→Robustheit (81% Kontamination); Cut-Entscheidung an Fable-5. Löst DEC-005-end ab.</t>
+        </is>
+      </c>
+      <c r="G23" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="33" t="inlineStr">
+        <is>
+          <t>DEC-021</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>sample_mid = Zeitachse (löst DEC-018 ab)</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>T8</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Sample-Jahre vorhanden → sample_mid statt pub_year; Datenagenda #10 gelöst.</t>
+        </is>
+      </c>
+      <c r="G24" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="33" t="inlineStr">
+        <is>
+          <t>DEC-022</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Country-Moderatoren (region/dev/culture/legal)</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>IMF Advanced · DST Western · La Porta common/civil · Region; parse-homogen → NCE; dominant gestrichen (E21).</t>
+        </is>
+      </c>
+      <c r="G25" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="33" t="inlineStr">
+        <is>
+          <t>DEC-023</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Quality-Moderatoren (status/VHB/JIF/field)</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>source_lookup; CIT gestrichen. Offen: VHB/JIF für 536 Working Paper.</t>
+        </is>
+      </c>
+      <c r="G26" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="33" t="inlineStr">
         <is>
           <t>Pending/Conditional DECs (im DECISION_LOG.md): Pending-A Headline-Event-Coding (nach T2) · Pending-B Transform-Doku (#11) · Pending-C Framing A vs. C (nach T1–T3 + T8).  Setup/Prozess-Entscheidungen → Tab 'Setup' (keine DECs). #11/#12 = Tasks.</t>
         </is>
       </c>
-      <c r="B22" s="36" t="n"/>
-      <c r="C22" s="36" t="n"/>
-      <c r="D22" s="36" t="n"/>
-      <c r="E22" s="36" t="n"/>
-      <c r="F22" s="36" t="n"/>
-      <c r="G22" s="35" t="n"/>
+      <c r="B27" s="36" t="n"/>
+      <c r="C27" s="36" t="n"/>
+      <c r="D27" s="36" t="n"/>
+      <c r="E27" s="36" t="n"/>
+      <c r="F27" s="36" t="n"/>
+      <c r="G27" s="35" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A27:G27"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A22:G22"/>
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Step 1 methodology finalization: DEC-024-027 logged; analysis_plan on v8 basis
- DECISION_LOG.md: DEC-024 (headline Paris cut pp_share_lag0 + inference-transfer
  rule; Pending-A resolved), DEC-025 (q_status + q_VHB; q_JIF retired), DEC-026
  (publication-status correction, 7 studies; version policy; full source audit),
  DEC-027 (n = no_firms validated; E14 -> n_obs); DEC-013 closed (extremes
  verified at source)
- analysis_plan.md: source -> data/CERCOD_data_v8.xlsx; sections 1/2/4/6/7/9
  replaced; open-items block rewritten; changelog 2026-07-03 (b)
- CERCOD_Status.xlsx: Ablauf step 1 done; DecisionLog_Index +DEC-024..027;
  Datenagenda #11/#12 closed, #14-#17 added
- data: remove v1/v4 (retrievable from history; lineage in plan sec. 1);
  add CERCOD_data_v8.xlsx as the analysis source; gitignore .claude/
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1329,7 +1329,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="42" t="inlineStr">
         <is>
-          <t>Ausführungsplan — CER–COD FOMA (verfeinerte Sequenz, Stand 2026-06-30)</t>
+          <t>Ausführungsplan — CER–COD FOMA (verfeinerte Sequenz, Stand 2026-07-03)</t>
         </is>
       </c>
     </row>
@@ -1425,7 +1425,7 @@
       </c>
       <c r="D4" s="41" t="inlineStr">
         <is>
-          <t>Geplante Methodik (DEC-001..018) gegen Audit-Ergebnis validieren + offene Items schließen. Ergebnis: finaler analysis_plan.</t>
+          <t>Geplante Methodik (DEC-001..018) gegen Audit-Ergebnis validieren + offene Items schließen. [ERLEDIGT 2026-07-03: DEC-024–027 geloggt; Pending-A gelöst; Headline pp_share_lag0 + Inference-Transfer-Regel; q_JIF gestrichen; Status-Korrektur 7 Studien; n validiert/E14→n_obs; Datenbasis v8; #11/#12 geschlossen]</t>
         </is>
       </c>
       <c r="E4" s="41" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="G4" s="41" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt</t>
         </is>
       </c>
     </row>
@@ -1462,12 +1462,12 @@
       </c>
       <c r="D5" s="41" t="inlineStr">
         <is>
-          <t>Re-prep (R/01_prep.R) gegen finale Volker-Daten; n-Regel + Sample-Jahr + Regulierung final. Öffnet das T1-Gate.</t>
+          <t>Re-prep (R/01_prep.R) gegen CERCOD_data_v8.xlsx; Verifier erweitert um DEC-024/025/026/027-Checks (pp_start≥2016, Identitäten, Lookup-Anti-Join, df-Berechnung Transfer-Regel). Öffnet das T1-Gate.</t>
         </is>
       </c>
       <c r="E5" s="41" t="inlineStr">
         <is>
-          <t>Schritt 1 + Volker-Antworten</t>
+          <t>Schritt 1 ✓</t>
         </is>
       </c>
       <c r="F5" s="41" t="inlineStr">
@@ -3884,7 +3884,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3976,7 +3976,11 @@
           <t>gelöst (DEC-019: no_firms/firm-years)</t>
         </is>
       </c>
-      <c r="G4" s="41" t="inlineStr"/>
+      <c r="G4" s="41" t="inlineStr">
+        <is>
+          <t>DEC-027: Ableitungsregel round(n_obs/T) dokumentiert (85,1% konsistent; alle 9 n&lt;10); reported-vs-derived-Flag → V4</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="44" customHeight="1">
       <c r="A5" s="41" t="n">
@@ -4035,10 +4039,14 @@
       </c>
       <c r="F6" s="41" t="inlineStr">
         <is>
-          <t>offen · Design (Fable-5)</t>
-        </is>
-      </c>
-      <c r="G6" s="41" t="inlineStr"/>
+          <t>offen · an V5/Pending-B gekoppelt</t>
+        </is>
+      </c>
+      <c r="G6" s="41" t="inlineStr">
+        <is>
+          <t>method_artefacts = r-Konversions-/Extraktionsartefakt-Flag; Operationalisierung mit V5 (r-Transformations-Doku)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="44" customHeight="1">
       <c r="A7" s="41" t="n">
@@ -4283,10 +4291,14 @@
       </c>
       <c r="F14" s="41" t="inlineStr">
         <is>
-          <t>offen · extern (COE-Liste)</t>
-        </is>
-      </c>
-      <c r="G14" s="41" t="inlineStr"/>
+          <t>gelöst (2026-07-03, DEC-026-Anhang)</t>
+        </is>
+      </c>
+      <c r="G14" s="41" t="inlineStr">
+        <is>
+          <t>Overlap = 5/66 Studien (Chava 2014 · Chen&amp;Gao 2011 · Li 2014 · Shad · Lemma) = 42/1.306 Eff. (3,2%); Effektgrößen disjunkt (beidseitige Extraktionsregeln, COE-Kriterium ii); Cover-Letter-Baustein liegt vor</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="44" customHeight="1">
       <c r="A15" s="41" t="n">
@@ -4314,10 +4326,14 @@
       </c>
       <c r="F15" s="41" t="inlineStr">
         <is>
-          <t>offen · Quellprüfung Drago/Devalle</t>
-        </is>
-      </c>
-      <c r="G15" s="41" t="inlineStr"/>
+          <t>gelöst (V2, 2026-07-03)</t>
+        </is>
+      </c>
+      <c r="G15" s="41" t="inlineStr">
+        <is>
+          <t>Quellwerte bestätigt — keine Extraktionsfehler; verbleiben; rstudent/LOSO/winsor trägt Einfluss (DEC-013 geschlossen)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="44" customHeight="1">
       <c r="A16" s="41" t="n">
@@ -4349,6 +4365,130 @@
         </is>
       </c>
       <c r="G16" s="41" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>14</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Daten</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>reported-vs-derived-Flag (no_firms)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Je Studie kennzeichnen: n direkt berichtet vs. round(n_obs/T) abgeleitet (DEC-027)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>offen (V4, vor Ch. 3)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>15</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Frage</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>r-Transformations-Doku + k der 36 PCCs</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Exakte Konversionsformel (Peterson–Brown / t-Konversion) + k falls trivial; operationalisiert method_artefacts (#3); Pending-B</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>offen (V5, vor Ch. 3)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>16</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Daten</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>PRISMA-Basics</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Suchdatum, Datenbanken, Treffer-/Screening-Zahlen, Inter-Coder-Angaben (Roadmap #11)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>offen (V6, vor Ch. 3)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>17</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Daten</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Lookup-Pflege + Sharfman-Begründung</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Shad-Jahr (Key 2022 vs ESPR 2020) · Lemma-Jahr-Konvention · Li-Doppelzeile konsolidieren · reference_verified-Header + 7 Leerzeilen · F16: Ausschlussgrund Sharfman&amp;Fernando 2008 (im COE-Korpus, berichtet COD)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>offen (nicht blockierend)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -4939,7 +5079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4961,7 +5101,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>23 aktive Methodik-DECs (DEC-001..023). Volleintraege im DECISION_LOG.md (8-Feld-Schema inkl. gespaltenem Reviewer-Risk). Setup/Prozess → Tab 'Setup'; Reporting/Polish (#11/#12) = Tasks, keine DEC.</t>
+          <t>27 aktive Methodik-DECs (DEC-001..027). Volleinträge im DECISION_LOG.md (append-only).</t>
         </is>
       </c>
     </row>
@@ -5854,17 +5994,165 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="33" t="inlineStr">
-        <is>
-          <t>Pending/Conditional DECs (im DECISION_LOG.md): Pending-A Headline-Event-Coding (nach T2) · Pending-B Transform-Doku (#11) · Pending-C Framing A vs. C (nach T1–T3 + T8).  Setup/Prozess-Entscheidungen → Tab 'Setup' (keine DECs). #11/#12 = Tasks.</t>
-        </is>
-      </c>
-      <c r="B27" s="36" t="n"/>
-      <c r="C27" s="36" t="n"/>
-      <c r="D27" s="36" t="n"/>
-      <c r="E27" s="36" t="n"/>
-      <c r="F27" s="36" t="n"/>
-      <c r="G27" s="35" t="n"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>DEC-024</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Headline-Paris-Cut + Inference-Transfer-Regel</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>#3 / T1,T2,T7,T8</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>pp_share_lag0 (Ties→Post) Headline; Dose→T8 Move 5; end = any-exposure-Bound; Lag-Panels a priori platziert; präregistrierte df-Regel; Pending-A gelöst; DEC-020-Corrigendum</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>DEC-025</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Quality-Moderatoren konsolidiert; q_JIF gestrichen</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>q_status + q_VHB (published-only, Referenzzellen-Kodierung); univariate VHB-Panels nur published; JIF analytisch tot (Roh im Lookup); DEC-023-Offenpunkt geschlossen</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DEC-026</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Daten</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Publikationsstatus-Korrektur + Versions-Regel + Voll-Audit</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>source_lookup / T5,T7</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>7 Studien (229 Eff.) → published (Stand 2026-07-03); Effekte bleiben as-coded (Triage: keine materiellen Abweichungen); 66-Zeilen-Audit; spec status_as_extracted; Feld-Semantik journal/year=as coded, reference_verified=VoR</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DEC-027</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>n-Definition validiert; E14 → n_obs</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>#1 / T1,T2,T4</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>no_firms bestätigt (konservativ; CR2-working-weights); Ableitungsregel round(n_obs/T) dokumentiert (85% konsistent, alle 9 n&lt;10); E14 umbenannt n_obs (81 Eff./3 Studien sub-annual/loan-level)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="33" t="inlineStr">
+        <is>
+          <t>Pending/Conditional DECs (im DECISION_LOG.md): Pending-A GELÖST → DEC-024 (2026-07-03) · Pending-B r-from-regression-Transformation (offen, V5) · Pending-C A-vs-C-Framing (offen, nach T8).</t>
+        </is>
+      </c>
+      <c r="B31" s="36" t="n"/>
+      <c r="C31" s="36" t="n"/>
+      <c r="D31" s="36" t="n"/>
+      <c r="E31" s="36" t="n"/>
+      <c r="F31" s="36" t="n"/>
+      <c r="G31" s="35" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
docs: apply canonical data filename CER-COD_data_v8.xlsx in LOG/plan/status (completes bbb8377 message)
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1462,7 +1462,7 @@
       </c>
       <c r="D5" s="41" t="inlineStr">
         <is>
-          <t>Re-prep (R/01_prep.R) gegen CERCOD_data_v8.xlsx; Verifier erweitert um DEC-024/025/026/027-Checks (pp_start≥2016, Identitäten, Lookup-Anti-Join, df-Berechnung Transfer-Regel). Öffnet das T1-Gate.</t>
+          <t>Re-prep (R/01_prep.R) gegen CER-COD_data_v8.xlsx; Verifier erweitert um DEC-024/025/026/027-Checks (pp_start≥2016, Identitäten, Lookup-Anti-Join, df-Berechnung Transfer-Regel). Öffnet das T1-Gate.</t>
         </is>
       </c>
       <c r="E5" s="41" t="inlineStr">
@@ -4395,7 +4395,6 @@
           <t>offen (V4, vor Ch. 3)</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -4426,7 +4425,6 @@
           <t>offen (V5, vor Ch. 3)</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -4457,7 +4455,6 @@
           <t>offen (V6, vor Ch. 3)</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -4488,7 +4485,6 @@
           <t>offen (nicht blockierend)</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5999,36 +5995,6 @@
           <t>DEC-024</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Headline-Paris-Cut + Inference-Transfer-Regel</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>#3 / T1,T2,T7,T8</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>pp_share_lag0 (Ties→Post) Headline; Dose→T8 Move 5; end = any-exposure-Bound; Lag-Panels a priori platziert; präregistrierte df-Regel; Pending-A gelöst; DEC-020-Corrigendum</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">

</xml_diff>

<commit_message>
Data closure v10 + null battery: DEC-028/029 logged; Pending-B resolved
DEC-028: v10 canonical (formula sheet, source flags, ES-type fix 36 bivariate/1270 PCC, df~n_obs convention, ES_source factor, Li key rename). DEC-029: null-robustness battery N1-N15 all adopted a priori; DEC-008 partially reopened (descriptive). Plan sec 1/2/7/9/13 updated; status workbook: Datenagenda 3/14/15 closed, battery decisions set.
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -12,10 +12,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aufgaben" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysen" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datenagenda" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifikation" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key_Results" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DecisionLog_Index" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Null_Battery" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datenagenda" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifikation" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key_Results" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DecisionLog_Index" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +26,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -81,6 +82,9 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="12">
@@ -211,7 +215,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -336,6 +340,10 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1308,6 +1316,1141 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="53" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Decision-Log Index — DEC-ID-Register (Methodik-only; Pointer auf DECISION_LOG.md) (v1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="40" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>29 aktive Methodik-DECs (DEC-001..029). Volleinträge im DECISION_LOG.md (append-only).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>DEC-ID</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Kategorie</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Titel</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Betrifft (#/Task)</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Kurzfassung</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="33" t="inlineStr">
+        <is>
+          <t>DEC-001</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Strategie</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Arbeitshypothese: Design bleibt</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>— / alle</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>FOMA CER–COD mit Paris als durchgaengiger Linse ueber alle Moderatoren.</t>
+        </is>
+      </c>
+      <c r="G4" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>DEC-002</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Dependence: 3LMA-RVE + Meta-Regression</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>#1,#2 / T1,T7</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Multilevel/CE working model + RVE-CR2 als Headline + unified Meta-Regression — eine Pipeline, zwei Sichten.</t>
+        </is>
+      </c>
+      <c r="G5" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t>DEC-003</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Headline-Rollenteilung</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>#1,#13 / T1,T7</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>3LMA-RVE traegt die Magnitude; Meta-Regression traegt die Identifikation (Bruch vs. Trend).</t>
+        </is>
+      </c>
+      <c r="G6" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>DEC-004</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Effektgroessen-Mischung</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>#5 / T4</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>Bivariat+partiell mischen, offenlegen, Literatur, Robustheit. Daten: nur 36 P → partial-only infeasibel, bivariat-only trivial.</t>
+        </is>
+      </c>
+      <c r="G7" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t>DEC-005</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Event-Coding: Compute-then-Select</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>#3 / T2</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>Varianten rechnen (End/Median/Mean/Lags/Stringency); Headline a priori. Konkrete Headline-Wahl = Pending-A (nach T2).</t>
+        </is>
+      </c>
+      <c r="G8" s="33" t="inlineStr">
+        <is>
+          <t>aktiv (Detail offen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>DEC-006</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Framing</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Kausalsprache abschwaechen</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>#4 / —</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>'structural break/exogenous shock' → 'temporal policy moderator'; Forschheit auf Debunking/Kontingenz umlenken.</t>
+        </is>
+      </c>
+      <c r="G9" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>DEC-007</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>Identifikation: 7-Move-Werkzeugkasten</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>#13 / T8</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Trend-Race · segm. MR · Placebo · Komposition · Diff-Exposure · Within-Study · Bounding.</t>
+        </is>
+      </c>
+      <c r="G10" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t>DEC-008</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Datenbefund</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Within-Study tot; Moves 1–2 brauchen kont. Zeit</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>#13 / T8,T0.4</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Move 6 entfaellt (1–3/66 Studien ueberspannen). Identifikation ruht auf Moves 1–5; Moves 1–2 erfordern kont. Jahresvar. (T0.4).</t>
+        </is>
+      </c>
+      <c r="G11" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="33" t="inlineStr">
+        <is>
+          <t>DEC-009</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Moderator×Paris: Interaktion statt Subgruppen</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>#10 / T6,T7</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Unified Interaktion (T7) statt genesteter Subgruppen — erzwungen durch duenne Cluster-Zellen (RVE-Mindest-Cluster unterschritten).</t>
+        </is>
+      </c>
+      <c r="G12" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>DEC-010</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Publikationsbias: PET-PEESE konsistent</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>#6 / T5</t>
+        </is>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>PET-PEESE-Entscheidungsregel ueber ALLE Subgruppen; PET n.s. → kein Effekt jenseits Bias. Industrie/No-pricing-Claims tempern.</t>
+        </is>
+      </c>
+      <c r="G13" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t>DEC-011</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Framing</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Novelty: Zarea/Witte zitieren + abgrenzen</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>#7 / —</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>'erste mit Paris' tot (Zarea H5). Novelty auf Debt-Kanal + Kanal-Dekomposition (Bank/Bond/CDS/Rating). Self-Overlap mit COE-Sibling adressieren.</t>
+        </is>
+      </c>
+      <c r="G14" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="33" t="inlineStr">
+        <is>
+          <t>DEC-012</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>Oekonomische Signifikanz in Basispunkten</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>#8 / —</t>
+        </is>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>r → bp Credit-Spread; ehrliche Magnitude (r=−0,020 unter 0,07-Schwelle, Doucouliagos 2011); ~5× kleiner als Zarea.</t>
+        </is>
+      </c>
+      <c r="G15" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="33" t="inlineStr">
+        <is>
+          <t>DEC-013</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Outlier: 2 Extremwerte verifizieren statt winsorisieren</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>#9 / T0.4,T4</t>
+        </is>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>Drago (−0,998) + Devalle (+0,9998) als Kodierfehler-Verdacht an der Quelle pruefen; rstudent.rma.mv + drop-refit statt blankem Winsorizing.</t>
+        </is>
+      </c>
+      <c r="G16" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="33" t="inlineStr">
+        <is>
+          <t>DEC-014</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Cluster-robuste Bias-/Meta-Regression (CR2)</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>#14,#6 / T5,T7</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>FAT-PET-PEESE &amp; Meta-Reg mit CR2-SE (geclustert auf study, Satterthwaite-df); 1.306 abh. ES nicht als unabhaengig. Tab. 7/8 neu.</t>
+        </is>
+      </c>
+      <c r="G17" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="33" t="inlineStr">
+        <is>
+          <t>DEC-015</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>Korrelations-Small-Sample-Bias / UWLS+3</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>#15,#1,#5 / T4,T0.4</t>
+        </is>
+      </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>Fisher-z behalten (Stanley 2024/25: r-IVW rest-verzerrt, 37% n&lt;200); WLS/RVE-Headline begruenden; UWLS+3/HS-Robustheit; n-Verteilung; PCC-df (n−k−3); Bivariat-only.</t>
+        </is>
+      </c>
+      <c r="G18" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="40" customHeight="1">
+      <c r="A19" s="33" t="inlineStr">
+        <is>
+          <t>DEC-016</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Selektionsmodell sekundaer (3PSM/p-uniform*)</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>#16,#6 / T5</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>3PSM/p-uniform* (van Aert &amp; van Assen 2026) sekundaer auf Studienebene (k=66); PET-PEESE bleibt primaer (Stanley 2025). Triangulation.</t>
+        </is>
+      </c>
+      <c r="G19" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="40" customHeight="1">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>DEC-017</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>rho working correlation (CE/CHE-Kovarianz)</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>#1 / T1,T4</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>rho=0,6 default, Sensitivitaet 0,4/0,6/0,8; operationalisiert DEC-002. impute_covariance_matrix(r=0.6); CR2 macht Punktschaetzer rho-robust. spec rho_0.4/rho_0.8 in T4.</t>
+        </is>
+      </c>
+      <c r="G20" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="40" customHeight="1">
+      <c r="A21" s="33" t="inlineStr">
+        <is>
+          <t>DEC-018</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Interim-Zeitachse pub_year (E8)</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>#13 / T0.4,T8</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>Kont. Zeit fehlt im Datensatz; pub_year aus study geparst (alle 66, 2010-2024) als PROVISORISCHE Interim-Achse. Sample-Jahr (Datenagenda #10) ersetzt sie. T8 re-zentriert aus rohem pub_year.</t>
+        </is>
+      </c>
+      <c r="G21" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="40" customHeight="1">
+      <c r="A22" s="33" t="inlineStr">
+        <is>
+          <t>DEC-019</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>n-Definition = no_firms (headline)</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>T1,T4</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>no_firms als Gewichts-Basis; no_firm-years + study-level = Robustheit. [E14]</t>
+        </is>
+      </c>
+      <c r="G22" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40" customHeight="1">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>DEC-020</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Pre/Post-Operationalisierung + Headline-Cut</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>T1,T4,T8</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>Suite (share/mid/end/start/median/tertil/window_class); Headline mid/kont., end→Robustheit (81% Kontamination); Cut-Entscheidung an Fable-5. Löst DEC-005-end ab.</t>
+        </is>
+      </c>
+      <c r="G23" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="40" customHeight="1">
+      <c r="A24" s="33" t="inlineStr">
+        <is>
+          <t>DEC-021</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>sample_mid = Zeitachse (löst DEC-018 ab)</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>T8</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>Sample-Jahre vorhanden → sample_mid statt pub_year; Datenagenda #10 gelöst.</t>
+        </is>
+      </c>
+      <c r="G24" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="40" customHeight="1">
+      <c r="A25" s="33" t="inlineStr">
+        <is>
+          <t>DEC-022</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Country-Moderatoren (region/dev/culture/legal)</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>IMF Advanced · DST Western · La Porta common/civil · Region; parse-homogen → NCE; dominant gestrichen (E21).</t>
+        </is>
+      </c>
+      <c r="G25" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="40" customHeight="1">
+      <c r="A26" s="33" t="inlineStr">
+        <is>
+          <t>DEC-023</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>Quality-Moderatoren (status/VHB/JIF/field)</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="F26" s="6" t="inlineStr">
+        <is>
+          <t>source_lookup; CIT gestrichen. Offen: VHB/JIF für 536 Working Paper.</t>
+        </is>
+      </c>
+      <c r="G26" s="33" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>DEC-024</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>DEC-025</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Quality-Moderatoren konsolidiert; q_JIF gestrichen</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>q_status + q_VHB (published-only, Referenzzellen-Kodierung); univariate VHB-Panels nur published; JIF analytisch tot (Roh im Lookup); DEC-023-Offenpunkt geschlossen</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DEC-026</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Daten</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Publikationsstatus-Korrektur + Versions-Regel + Voll-Audit</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>source_lookup / T5,T7</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>7 Studien (229 Eff.) → published (Stand 2026-07-03); Effekte bleiben as-coded (Triage: keine materiellen Abweichungen); 66-Zeilen-Audit; spec status_as_extracted; Feld-Semantik journal/year=as coded, reference_verified=VoR</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DEC-027</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>n-Definition validiert; E14 → n_obs</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>#1 / T1,T2,T4</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>no_firms bestätigt (konservativ; CR2-working-weights); Ableitungsregel round(n_obs/T) dokumentiert (85% konsistent, alle 9 n&lt;10); E14 umbenannt n_obs (81 Eff./3 Studien sub-annual/loan-level)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>DEC-028</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Daten</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Daten-Doku-Abschluss v9/v10; Pending-B gelöst</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>data/lookup · §§1/2/7/9</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>v10 kanonisch; formula-Sheet dokumentiert 4 Konversionsrouten; ES-Typ korrigiert (36 bivariat / 1.270 PCC); df≈n_obs-Konvention + pcc_df_k-Sensitivität; ES_source ersetzt es_type/method_artefacts; V4-Flags autoritativ (calculated 54,6%); Li-Key-Rename 2021→2022; Shad-Kreuznotiz (F22)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>DEC-029</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Null-Battery a priori designiert (N1–N15, alle)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Null_Battery · §§9/13 · T1-Gate</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Alle 15 GO; Platzierungen fixiert; N13 konditional (≥5-Regel); N15 deskriptiv mit DEC-008-Teil-Reopen; Inputs (SESOI/F18, Priors, Faktorraum, Grids, Fensterparameter) VOR T1 zu fixieren; Paper-Beschaffung: Lakens, Simonsohn 2020, WAAP</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="33" t="inlineStr">
+        <is>
+          <t>Pending/Conditional DECs (im DECISION_LOG.md): Pending-A GELÖST → DEC-024 · Pending-B GELÖST → DEC-028 (2026-07-04) · Pending-C A-vs-C-Framing (offen, nach T8).</t>
+        </is>
+      </c>
+      <c r="B33" s="36" t="n"/>
+      <c r="C33" s="36" t="n"/>
+      <c r="D33" s="36" t="n"/>
+      <c r="E33" s="36" t="n"/>
+      <c r="F33" s="36" t="n"/>
+      <c r="G33" s="35" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -1329,7 +2472,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="42" t="inlineStr">
         <is>
-          <t>Ausführungsplan — CER–COD FOMA (verfeinerte Sequenz, Stand 2026-07-03)</t>
+          <t>Ausführungsplan — CER–COD FOMA (verfeinerte Sequenz, Stand 2026-07-04)</t>
         </is>
       </c>
     </row>
@@ -1462,7 +2605,7 @@
       </c>
       <c r="D5" s="41" t="inlineStr">
         <is>
-          <t>Re-prep (R/01_prep.R) gegen CER-COD_data_v8.xlsx; Verifier erweitert um DEC-024/025/026/027-Checks (pp_start≥2016, Identitäten, Lookup-Anti-Join, df-Berechnung Transfer-Regel). Öffnet das T1-Gate.</t>
+          <t>Re-prep (R/01_prep.R) gegen CER-COD_data_v10.xlsx; Verifier erweitert um DEC-024..028-Checks (pp_start≥2016, Identitäten, Lookup-Anti-Join, ES_source×ES_measure-Diagonale, Formel-Spotcheck, df-Berechnung Transfer-Regel). Vorab: DEC-029-Battery-Inputs fixieren (SESOI, Priors, Faktorraum, Grids). Öffnet das T1-Gate.</t>
         </is>
       </c>
       <c r="E5" s="41" t="inlineStr">
@@ -3884,6 +5027,1195 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:N17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Null-Battery — Kandidaten-Analysen zur Absicherung des Null-Befunds (Paris). Stand 2026-07-03. Auswahl → DEC-028 (a priori, VOR T1 zu designieren, DEC-005-Disziplin). Linien: A = Zufall/Power · B = Spezifikationsraum · C = Zeitachse · D = Benchmark/Erwartung. Kernbefund der Daten-Checks: ALLE 15 Analysen laufen auf CER-COD_data_v8.xlsx — keine neue Datenerhebung nötig. | ENTSCHEIDUNG: ALLE 15 GO per DEC-029 (2026-07-04); Inputs-Fixierung vor T1 (Battery-Prep).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="45" t="inlineStr">
+        <is>
+          <t>Nr</t>
+        </is>
+      </c>
+      <c r="B2" s="45" t="inlineStr">
+        <is>
+          <t>Linie</t>
+        </is>
+      </c>
+      <c r="C2" s="45" t="inlineStr">
+        <is>
+          <t>Analyse</t>
+        </is>
+      </c>
+      <c r="D2" s="45" t="inlineStr">
+        <is>
+          <t>Ziel (was zeigt sie)</t>
+        </is>
+      </c>
+      <c r="E2" s="45" t="inlineStr">
+        <is>
+          <t>Vorgehen (was wird gemacht)</t>
+        </is>
+      </c>
+      <c r="F2" s="45" t="inlineStr">
+        <is>
+          <t>Daten in v8?</t>
+        </is>
+      </c>
+      <c r="G2" s="45" t="inlineStr">
+        <is>
+          <t>Zusätzliche Inputs (Annahmen/Cutoffs/externe Werte)</t>
+        </is>
+      </c>
+      <c r="H2" s="45" t="inlineStr">
+        <is>
+          <t>Methodik-Paper nötig?</t>
+        </is>
+      </c>
+      <c r="I2" s="45" t="inlineStr">
+        <is>
+          <t>Quellen-Anker</t>
+        </is>
+      </c>
+      <c r="J2" s="45" t="inlineStr">
+        <is>
+          <t>Ertrag</t>
+        </is>
+      </c>
+      <c r="K2" s="45" t="inlineStr">
+        <is>
+          <t>Aufwand</t>
+        </is>
+      </c>
+      <c r="L2" s="45" t="inlineStr">
+        <is>
+          <t>DEC-Berührung</t>
+        </is>
+      </c>
+      <c r="M2" s="45" t="inlineStr">
+        <is>
+          <t>Prio-Vorschlag</t>
+        </is>
+      </c>
+      <c r="N2" s="45" t="inlineStr">
+        <is>
+          <t>Entscheidung (RW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="46" t="inlineStr">
+        <is>
+          <t>N1</t>
+        </is>
+      </c>
+      <c r="B3" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C3" s="46" t="inlineStr">
+        <is>
+          <t>Äquivalenztest (TOST) auf Paris-Kontrast</t>
+        </is>
+      </c>
+      <c r="D3" s="46" t="inlineStr">
+        <is>
+          <t>Dreht die Beweislast: statt "nicht signifikant" wird aktiv gezeigt, dass der Paris-Effekt kleiner ist als jeder ökonomisch relevante Effekt. Macht den Null zum positiven Befund.</t>
+        </is>
+      </c>
+      <c r="E3" s="46" t="inlineStr">
+        <is>
+          <t>A priori kleinsten relevanten Effekt (SESOI, ±δ) festlegen; zwei einseitige Tests auf den CR2-Paris-Koeffizienten; äquivalent: liegt das 90%-CI vollständig in [−δ,+δ]? Ausweis neben dem NHST-Ergebnis.</t>
+        </is>
+      </c>
+      <c r="F3" s="46" t="inlineStr">
+        <is>
+          <t>ja (nutzt T1/T7-Modelle, keine neuen Spalten)</t>
+        </is>
+      </c>
+      <c r="G3" s="46" t="inlineStr">
+        <is>
+          <t>SESOI-Wert = DIE Annahme (F18): Zarea-Post-Effekt (aus PK-PDF extrahierbar) und/oder Konvention |Δr|=0,05; a priori in DEC-028 fixieren</t>
+        </is>
+      </c>
+      <c r="H3" s="46" t="inlineStr">
+        <is>
+          <t>Lücke: Lakens (2017/2018) TOST-Primer nicht im PK — beschaffen</t>
+        </is>
+      </c>
+      <c r="I3" s="46" t="inlineStr">
+        <is>
+          <t>Lakens 2017 (fehlt); CR2-Inferenz: Tipton &amp; Pustejovsky 2015 (PK)</t>
+        </is>
+      </c>
+      <c r="J3" s="46" t="inlineStr">
+        <is>
+          <t>hoch — direkt die Kernaussage</t>
+        </is>
+      </c>
+      <c r="K3" s="46" t="inlineStr">
+        <is>
+          <t>niedrig</t>
+        </is>
+      </c>
+      <c r="L3" s="46" t="inlineStr">
+        <is>
+          <t>DEC-028 (SESOI a priori)</t>
+        </is>
+      </c>
+      <c r="M3" s="46" t="inlineStr">
+        <is>
+          <t>HAUPTTEXT</t>
+        </is>
+      </c>
+      <c r="N3" s="46" t="inlineStr">
+        <is>
+          <t>GO (RW 2026-07-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="46" t="inlineStr">
+        <is>
+          <t>N2</t>
+        </is>
+      </c>
+      <c r="B4" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C4" s="46" t="inlineStr">
+        <is>
+          <t>Design-basierte Power-/MDE-Simulation</t>
+        </is>
+      </c>
+      <c r="D4" s="46" t="inlineStr">
+        <is>
+          <t>Zeigt ergebnisblind, welchen Paris-Effekt unser Design mit 80% Power entdeckt hätte (MDE). Liegt der MDE unter dem literaturerwarteten Effekt, ist der Null informativ, kein Powermangel.</t>
+        </is>
+      </c>
+      <c r="E4" s="46" t="inlineStr">
+        <is>
+          <t>Monte-Carlo mit exakter Datenstruktur (66 Studien, 11 Post-Cluster, reale n, ρ=0,6, τ²-Grid bzw. COE-Companion-Werte); Effekt δ injizieren, Anteil signifikanter CR2-Tests → Powerkurve + MDE.</t>
+        </is>
+      </c>
+      <c r="F4" s="46" t="inlineStr">
+        <is>
+          <t>ja (reine Designspalten; design-only = ergebnisblind)</t>
+        </is>
+      </c>
+      <c r="G4" s="46" t="inlineStr">
+        <is>
+          <t>τ²/ω²-Annahmen (Grid oder COE-Werte); δ-Grid; Seed; Anschluss an df-Transfer-Regel im T2-Verifier</t>
+        </is>
+      </c>
+      <c r="H4" s="46" t="inlineStr">
+        <is>
+          <t>nein (Standard-MC; Rahmen im PK vorhanden)</t>
+        </is>
+      </c>
+      <c r="I4" s="46" t="inlineStr">
+        <is>
+          <t>Tipton &amp; Pustejovsky 2015; Pustejovsky &amp; Tipton 2022 (beide PK)</t>
+        </is>
+      </c>
+      <c r="J4" s="46" t="inlineStr">
+        <is>
+          <t>hoch — entkräftet Power-Einwand ex ante</t>
+        </is>
+      </c>
+      <c r="K4" s="46" t="inlineStr">
+        <is>
+          <t>mittel (Simulationsskript, CC-geeignet)</t>
+        </is>
+      </c>
+      <c r="L4" s="46" t="inlineStr">
+        <is>
+          <t>DEC-028; koppelt an DEC-024-Transferregel</t>
+        </is>
+      </c>
+      <c r="M4" s="46" t="inlineStr">
+        <is>
+          <t>HAUPTTEXT (Zahl; Kurve → Appendix)</t>
+        </is>
+      </c>
+      <c r="N4" s="46" t="inlineStr">
+        <is>
+          <t>GO (RW 2026-07-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="46" t="inlineStr">
+        <is>
+          <t>N3</t>
+        </is>
+      </c>
+      <c r="B5" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C5" s="46" t="inlineStr">
+        <is>
+          <t>Bayes-Faktor / Robust Bayesian MA (RoBMA)</t>
+        </is>
+      </c>
+      <c r="D5" s="46" t="inlineStr">
+        <is>
+          <t>Quantifiziert Evidenz FÜR die Null: BF01 sagt, wie viel wahrscheinlicher die Daten ohne Paris-Shift sind als mit dem erwarteten Effekt — inkl. Modellmittelung über Publikationsbias.</t>
+        </is>
+      </c>
+      <c r="E5" s="46" t="inlineStr">
+        <is>
+          <t>RoBMA auf den Pre/Post-Kontrast; Priors: Default + informierter Prior aus Zarea-Effekt; BF01 + Posterior für δ berichten. Dependence-Handling nötig (Aggregation auf Studienebene o. cluster-robuste Variante).</t>
+        </is>
+      </c>
+      <c r="F5" s="46" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G5" s="46" t="inlineStr">
+        <is>
+          <t>Prior-Spezifikation a priori (default vs. Zarea-informiert); RoBMA-Package in renv; Entscheidung Dependence-Handling</t>
+        </is>
+      </c>
+      <c r="H5" s="46" t="inlineStr">
+        <is>
+          <t>nein — Bartoš et al. 2022 zweifach im PK</t>
+        </is>
+      </c>
+      <c r="I5" s="46" t="inlineStr">
+        <is>
+          <t>Bartoš et al. 2022 (JASP/R + robust BMA)</t>
+        </is>
+      </c>
+      <c r="J5" s="46" t="inlineStr">
+        <is>
+          <t>hoch — moderne, BSE-taugliche Evidenzsprache</t>
+        </is>
+      </c>
+      <c r="K5" s="46" t="inlineStr">
+        <is>
+          <t>mittel-hoch (neues Package, Dependence)</t>
+        </is>
+      </c>
+      <c r="L5" s="46" t="inlineStr">
+        <is>
+          <t>DEC-028</t>
+        </is>
+      </c>
+      <c r="M5" s="46" t="inlineStr">
+        <is>
+          <t>HAUPTTEXT kompakt; Details Appendix</t>
+        </is>
+      </c>
+      <c r="N5" s="46" t="inlineStr">
+        <is>
+          <t>GO (RW 2026-07-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="46" t="inlineStr">
+        <is>
+          <t>N4</t>
+        </is>
+      </c>
+      <c r="B6" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C6" s="46" t="inlineStr">
+        <is>
+          <t>Prädiktionsintervalle pre vs. post</t>
+        </is>
+      </c>
+      <c r="D6" s="46" t="inlineStr">
+        <is>
+          <t>Zeigt auf Verteilungsebene, dass die plausiblen wahren Effekte pre und post praktisch deckungsgleich sind — kein Regimewechsel auch jenseits des Mittelwerts.</t>
+        </is>
+      </c>
+      <c r="E6" s="46" t="inlineStr">
+        <is>
+          <t>95%-PI je Periode aus dem 3LMA (μ ± t·√(τ²+ω²+SE²)); Overlap-Grafik/Forest-Panel.</t>
+        </is>
+      </c>
+      <c r="F6" s="46" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G6" s="46" t="inlineStr">
+        <is>
+          <t>keine</t>
+        </is>
+      </c>
+      <c r="H6" s="46" t="inlineStr">
+        <is>
+          <t>nein — Borenstein et al. 2017 im PK</t>
+        </is>
+      </c>
+      <c r="I6" s="46" t="inlineStr">
+        <is>
+          <t>Borenstein et al. 2017; Borenstein 2009</t>
+        </is>
+      </c>
+      <c r="J6" s="46" t="inlineStr">
+        <is>
+          <t>mittel — billig, reviewer-vertraut</t>
+        </is>
+      </c>
+      <c r="K6" s="46" t="inlineStr">
+        <is>
+          <t>sehr niedrig</t>
+        </is>
+      </c>
+      <c r="L6" s="46" t="inlineStr">
+        <is>
+          <t>keiner (Reporting)</t>
+        </is>
+      </c>
+      <c r="M6" s="46" t="inlineStr">
+        <is>
+          <t>HAUPTTEXT (Grafik)</t>
+        </is>
+      </c>
+      <c r="N6" s="46" t="inlineStr">
+        <is>
+          <t>GO (RW 2026-07-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="46" t="inlineStr">
+        <is>
+          <t>N5</t>
+        </is>
+      </c>
+      <c r="B7" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C7" s="46" t="inlineStr">
+        <is>
+          <t>Multiverse-/Spezifikationskurven-Analyse</t>
+        </is>
+      </c>
+      <c r="D7" s="46" t="inlineStr">
+        <is>
+          <t>Das Dach gegen "genau eure Analysen": alle vertretbaren Analysepfade werden systematisch gekreuzt; gezeigt wird, dass der Null über den gesamten Spezifikationsraum stabil ist.</t>
+        </is>
+      </c>
+      <c r="E7" s="46" t="inlineStr">
+        <is>
+          <t>Faktorraum a priori definieren (Paris-Coding ×  Schätzer × n-Definition × Outlier × ρ × Subsample aus §9); alle Kombinationen schätzen; Spezifikationskurve, Verteilungsstatistik, optional Permutations-Jointtest.</t>
+        </is>
+      </c>
+      <c r="F7" s="46" t="inlineStr">
+        <is>
+          <t>ja (alles §9-Zutaten)</t>
+        </is>
+      </c>
+      <c r="G7" s="46" t="inlineStr">
+        <is>
+          <t>Faktorraum-Abgrenzung a priori (welche Faktoren zählen als vertretbar) — gehört in DEC-028; Rechenzeit</t>
+        </is>
+      </c>
+      <c r="H7" s="46" t="inlineStr">
+        <is>
+          <t>Lücke: Simonsohn et al. 2020 (Spec-Curve) / Steegen et al. 2016 (Multiverse) nicht im PK</t>
+        </is>
+      </c>
+      <c r="I7" s="46" t="inlineStr">
+        <is>
+          <t>Simonsohn et al. 2020 (fehlt); §9-Katalog [DEC-004]</t>
+        </is>
+      </c>
+      <c r="J7" s="46" t="inlineStr">
+        <is>
+          <t>sehr hoch — strukturelles Gegenargument</t>
+        </is>
+      </c>
+      <c r="K7" s="46" t="inlineStr">
+        <is>
+          <t>mittel (Loop über bestehende Specs; Jointtest +)</t>
+        </is>
+      </c>
+      <c r="L7" s="46" t="inlineStr">
+        <is>
+          <t>DEC-028 (Faktorraum a priori)</t>
+        </is>
+      </c>
+      <c r="M7" s="46" t="inlineStr">
+        <is>
+          <t>HAUPTTEXT (Kern-Abbildung)</t>
+        </is>
+      </c>
+      <c r="N7" s="46" t="inlineStr">
+        <is>
+          <t>GO (RW 2026-07-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="46" t="inlineStr">
+        <is>
+          <t>N6</t>
+        </is>
+      </c>
+      <c r="B8" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C8" s="46" t="inlineStr">
+        <is>
+          <t>Sup-Break-Test (datengewählter Bruchpunkt)</t>
+        </is>
+      </c>
+      <c r="D8" s="46" t="inlineStr">
+        <is>
+          <t>Schließt aus, dass 2015/16 günstig gewählt ist: selbst der bestmögliche, datengewählte Bruchpunkt über die gesamte Zeitachse zeigt keinen Effekt.</t>
+        </is>
+      </c>
+      <c r="E8" s="46" t="inlineStr">
+        <is>
+          <t>Segmentiertes Modell für jedes Kandidatenjahr (Grid auf sample_mid); sup-|t| über alle Jahre; Inferenz via Permutation/Bootstrap statt asymptotischer kritischer Werte (MA-Kontext, CR2).</t>
+        </is>
+      </c>
+      <c r="F8" s="46" t="inlineStr">
+        <is>
+          <t>ja (sample_mid)</t>
+        </is>
+      </c>
+      <c r="G8" s="46" t="inlineStr">
+        <is>
+          <t>Kandidatenjahr-Grid; Inferenzweg (Permutation — teilt Maschinerie mit N7)</t>
+        </is>
+      </c>
+      <c r="H8" s="46" t="inlineStr">
+        <is>
+          <t>vermeidbar (permutationsbasiert gerahmt); klassisch wäre Andrews 1993 (fehlt)</t>
+        </is>
+      </c>
+      <c r="I8" s="46" t="inlineStr">
+        <is>
+          <t>T8-Placebo-Grid [DEC-024] als Basis</t>
+        </is>
+      </c>
+      <c r="J8" s="46" t="inlineStr">
+        <is>
+          <t>hoch — tötet den Cutoff-Wahl-Einwand beidseitig</t>
+        </is>
+      </c>
+      <c r="K8" s="46" t="inlineStr">
+        <is>
+          <t>niedrig-mittel (Erweiterung des Placebo-Grids)</t>
+        </is>
+      </c>
+      <c r="L8" s="46" t="inlineStr">
+        <is>
+          <t>DEC-028 (formalisiert Placebo zu Jointtest)</t>
+        </is>
+      </c>
+      <c r="M8" s="46" t="inlineStr">
+        <is>
+          <t>HAUPTTEXT (eine Statistik); Grid-Grafik Appendix</t>
+        </is>
+      </c>
+      <c r="N8" s="46" t="inlineStr">
+        <is>
+          <t>GO (RW 2026-07-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="46" t="inlineStr">
+        <is>
+          <t>N7</t>
+        </is>
+      </c>
+      <c r="B9" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C9" s="46" t="inlineStr">
+        <is>
+          <t>Permutationsinferenz auf dem Paris-Label</t>
+        </is>
+      </c>
+      <c r="D9" s="46" t="inlineStr">
+        <is>
+          <t>Verteilungsfreie Inferenz für den Paris-Koeffizienten — bei nur 11 Post-Clustern robuster als Asymptotik; formalisiert die Placebos zu einem echten Test.</t>
+        </is>
+      </c>
+      <c r="E9" s="46" t="inlineStr">
+        <is>
+          <t>Post-Label auf Studienebene B-fach permutieren (strukturerhaltend: 11 Studien ziehen); Modell je Permutation; empirischer p-Wert = Rangposition des beobachteten Koeffizienten.</t>
+        </is>
+      </c>
+      <c r="F9" s="46" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G9" s="46" t="inlineStr">
+        <is>
+          <t>B (z. B. 5.000); Permutationsschema (studienweise; optional regionsblockweise) a priori</t>
+        </is>
+      </c>
+      <c r="H9" s="46" t="inlineStr">
+        <is>
+          <t>nein (Fisher-Randomisierung, Standard)</t>
+        </is>
+      </c>
+      <c r="I9" s="46" t="inlineStr">
+        <is>
+          <t>generisch; bündeln mit N6</t>
+        </is>
+      </c>
+      <c r="J9" s="46" t="inlineStr">
+        <is>
+          <t>mittel-hoch</t>
+        </is>
+      </c>
+      <c r="K9" s="46" t="inlineStr">
+        <is>
+          <t>niedrig (Loop; teilt Code mit N6)</t>
+        </is>
+      </c>
+      <c r="L9" s="46" t="inlineStr">
+        <is>
+          <t>DEC-028</t>
+        </is>
+      </c>
+      <c r="M9" s="46" t="inlineStr">
+        <is>
+          <t>HAUPTTEXT-Zeile (p_perm neben p_CR2); Details Appendix</t>
+        </is>
+      </c>
+      <c r="N9" s="46" t="inlineStr">
+        <is>
+          <t>GO (RW 2026-07-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="46" t="inlineStr">
+        <is>
+          <t>N8</t>
+        </is>
+      </c>
+      <c r="B10" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C10" s="46" t="inlineStr">
+        <is>
+          <t>Zarea-Spezifikations-Transplantation</t>
+        </is>
+      </c>
+      <c r="D10" s="46" t="inlineStr">
+        <is>
+          <t>Rhetorisch das schärfste Einzelstück: Der Null bleibt auch unter der Spezifikation des stärksten positiven Präzedenzfalls bestehen — entkräftet "andere Analysen, anderes Ergebnis" maximal.</t>
+        </is>
+      </c>
+      <c r="E10" s="46" t="inlineStr">
+        <is>
+          <t>Zareas Paris-Setup exakt nachbauen (Midpoint-Split MIT Tie-Exklusion, 3-Level-REML, deren Subgruppen-/Moderatorlogik, soweit dokumentiert) und auf unsere Daten anwenden; neben Zareas berichtetem Post-Effekt ausweisen.</t>
+        </is>
+      </c>
+      <c r="F10" s="46" t="inlineStr">
+        <is>
+          <t>ja (pp_mid + Exklusion der 2 Tie-Effekte)</t>
+        </is>
+      </c>
+      <c r="G10" s="46" t="inlineStr">
+        <is>
+          <t>Zarea-Spezifikationsdetails aus dem PDF extrahieren (PK vorhanden); Unschärfen dokumentieren</t>
+        </is>
+      </c>
+      <c r="H10" s="46" t="inlineStr">
+        <is>
+          <t>nein — Zarea im PK</t>
+        </is>
+      </c>
+      <c r="I10" s="46" t="inlineStr">
+        <is>
+          <t>Zarea et al. 2026 (PK)</t>
+        </is>
+      </c>
+      <c r="J10" s="46" t="inlineStr">
+        <is>
+          <t>sehr hoch (rhetorisch)</t>
+        </is>
+      </c>
+      <c r="K10" s="46" t="inlineStr">
+        <is>
+          <t>niedrig</t>
+        </is>
+      </c>
+      <c r="L10" s="46" t="inlineStr">
+        <is>
+          <t>DEC-028; berührt DEC-024 nicht (Zusatzspec)</t>
+        </is>
+      </c>
+      <c r="M10" s="46" t="inlineStr">
+        <is>
+          <t>HAUPTTEXT</t>
+        </is>
+      </c>
+      <c r="N10" s="46" t="inlineStr">
+        <is>
+          <t>GO (RW 2026-07-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="46" t="inlineStr">
+        <is>
+          <t>N9</t>
+        </is>
+      </c>
+      <c r="B11" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C11" s="46" t="inlineStr">
+        <is>
+          <t>Alternative Schätztraditionen: Hunter-Schmidt (+ optional WAAP)</t>
+        </is>
+      </c>
+      <c r="D11" s="46" t="inlineStr">
+        <is>
+          <t>Schließt die Gewichtungsphilosophie als Freiheitsgrad: Null auch unter psychometrischer Tradition (HS bare-bones) und optional unter WAAP (nur adäquat gepowerte Studien).</t>
+        </is>
+      </c>
+      <c r="E11" s="46" t="inlineStr">
+        <is>
+          <t>HS-Random-Effects auf r-Ebene (bare-bones; Dependence via Studienaggregation); WAAP: nur Studien mit Power ≥ 80% relativ zum WLS-Mittel poolen.</t>
+        </is>
+      </c>
+      <c r="F11" s="46" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G11" s="46" t="inlineStr">
+        <is>
+          <t>HS-Dependence-Konvention festlegen; WAAP-Powerregel</t>
+        </is>
+      </c>
+      <c r="H11" s="46" t="inlineStr">
+        <is>
+          <t>HS: nein (H&amp;S 2004 im PK). WAAP: Lücke — Stanley/Doucouliagos/Ioannidis 2017 fehlt</t>
+        </is>
+      </c>
+      <c r="I11" s="46" t="inlineStr">
+        <is>
+          <t>Hunter &amp; Schmidt 2004 (PK); Stanley &amp; Doucouliagos 2012/2017 (PK)</t>
+        </is>
+      </c>
+      <c r="J11" s="46" t="inlineStr">
+        <is>
+          <t>mittel — bedient Management-Flanke</t>
+        </is>
+      </c>
+      <c r="K11" s="46" t="inlineStr">
+        <is>
+          <t>niedrig</t>
+        </is>
+      </c>
+      <c r="L11" s="46" t="inlineStr">
+        <is>
+          <t>Upgrade des E2-Deferred-Status (Notiz in DEC-028)</t>
+        </is>
+      </c>
+      <c r="M11" s="46" t="inlineStr">
+        <is>
+          <t>APPENDIX (bzw. Multiverse-Faktor in N5)</t>
+        </is>
+      </c>
+      <c r="N11" s="46" t="inlineStr">
+        <is>
+          <t>GO — Appendix</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="46" t="inlineStr">
+        <is>
+          <t>N10</t>
+        </is>
+      </c>
+      <c r="B12" s="46" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C12" s="46" t="inlineStr">
+        <is>
+          <t>Kumulative Meta-Analyse über die Zeit</t>
+        </is>
+      </c>
+      <c r="D12" s="46" t="inlineStr">
+        <is>
+          <t>Visuell sofort verständlich: Der gepoolte Effekt driftet beim chronologischen Auffüllen der Evidenz nie in Richtung des erwarteten Paris-Shifts.</t>
+        </is>
+      </c>
+      <c r="E12" s="46" t="inlineStr">
+        <is>
+          <t>Studien nach sample_mid sortieren; sequentiell poolen (Studienebene oder 3LMA-Refits); Trajektorie mit CI-Band, Markierung 2015/16.</t>
+        </is>
+      </c>
+      <c r="F12" s="46" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G12" s="46" t="inlineStr">
+        <is>
+          <t>Sortier-/Aggregationskonvention</t>
+        </is>
+      </c>
+      <c r="H12" s="46" t="inlineStr">
+        <is>
+          <t>nein — Borenstein 2009 im PK</t>
+        </is>
+      </c>
+      <c r="I12" s="46" t="inlineStr">
+        <is>
+          <t>Borenstein et al. 2009</t>
+        </is>
+      </c>
+      <c r="J12" s="46" t="inlineStr">
+        <is>
+          <t>mittel (stark visuell)</t>
+        </is>
+      </c>
+      <c r="K12" s="46" t="inlineStr">
+        <is>
+          <t>niedrig</t>
+        </is>
+      </c>
+      <c r="L12" s="46" t="inlineStr">
+        <is>
+          <t>keiner (Display)</t>
+        </is>
+      </c>
+      <c r="M12" s="46" t="inlineStr">
+        <is>
+          <t>HAUPTTEXT-Grafik (alternativ N11 → nur eine der beiden Zeitgrafiken in den Haupttext)</t>
+        </is>
+      </c>
+      <c r="N12" s="46" t="inlineStr">
+        <is>
+          <t>GO (RW 2026-07-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="46" t="inlineStr">
+        <is>
+          <t>N11</t>
+        </is>
+      </c>
+      <c r="B13" s="46" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C13" s="46" t="inlineStr">
+        <is>
+          <t>Rolling-Window-Trajektorie</t>
+        </is>
+      </c>
+      <c r="D13" s="46" t="inlineStr">
+        <is>
+          <t>Zeigt die gesamte Zeitform des Zusammenhangs nichtparametrisch — keine versteckte Nichtlinearität, die ein Ein-Punkt-Break übersieht.</t>
+        </is>
+      </c>
+      <c r="E13" s="46" t="inlineStr">
+        <is>
+          <t>Gleitende Fenster über sample_mid (z. B. 7 Jahre, Schritt 1) oder Jahres-Bins; Effekt + CI je Fenster; Plot neben der segmentierten Regression.</t>
+        </is>
+      </c>
+      <c r="F13" s="46" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G13" s="46" t="inlineStr">
+        <is>
+          <t>Fensterbreite/Schritt a priori (+ Sensitivität)</t>
+        </is>
+      </c>
+      <c r="H13" s="46" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="I13" s="46" t="inlineStr">
+        <is>
+          <t>deskriptiv / T8</t>
+        </is>
+      </c>
+      <c r="J13" s="46" t="inlineStr">
+        <is>
+          <t>mittel</t>
+        </is>
+      </c>
+      <c r="K13" s="46" t="inlineStr">
+        <is>
+          <t>niedrig</t>
+        </is>
+      </c>
+      <c r="L13" s="46" t="inlineStr">
+        <is>
+          <t>DEC-028 (Fensterparameter)</t>
+        </is>
+      </c>
+      <c r="M13" s="46" t="inlineStr">
+        <is>
+          <t>APPENDIX (redundant zu N10 + Dose im Haupttext)</t>
+        </is>
+      </c>
+      <c r="N13" s="46" t="inlineStr">
+        <is>
+          <t>GO — Appendix</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="46" t="inlineStr">
+        <is>
+          <t>N12</t>
+        </is>
+      </c>
+      <c r="B14" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C14" s="46" t="inlineStr">
+        <is>
+          <t>Formaler Differenztest gegen externe Effekte (Zarea; ggf. COE)</t>
+        </is>
+      </c>
+      <c r="D14" s="46" t="inlineStr">
+        <is>
+          <t>Macht "unser Null ≠ deren Effekt" quantitativ: Differenz unseres Paris-Kontrasts zum berichteten Zarea-Post-Effekt wird beziffert und getestet statt nur erzählt.</t>
+        </is>
+      </c>
+      <c r="E14" s="46" t="inlineStr">
+        <is>
+          <t>z-Differenztest zweier unabhängiger Schätzer (unser CR2-Kontrast vs. Zarea-Punkt+SE aus dem Paper); Metrik-Harmonisierung (r/z/deren ES) dokumentieren; als Kontext-, nicht Identitätstest framen (Banken vs. alle Firmen).</t>
+        </is>
+      </c>
+      <c r="F14" s="46" t="inlineStr">
+        <is>
+          <t>ja + externe Werte</t>
+        </is>
+      </c>
+      <c r="G14" s="46" t="inlineStr">
+        <is>
+          <t>Zarea Punkt + SE extrahieren (PK); COE-Companion: verifizieren, ob dort ein Paris-Moderator existiert</t>
+        </is>
+      </c>
+      <c r="H14" s="46" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="I14" s="46" t="inlineStr">
+        <is>
+          <t>Standard; Subgruppen-Logik Borenstein (PK)</t>
+        </is>
+      </c>
+      <c r="J14" s="46" t="inlineStr">
+        <is>
+          <t>mittel-hoch</t>
+        </is>
+      </c>
+      <c r="K14" s="46" t="inlineStr">
+        <is>
+          <t>niedrig</t>
+        </is>
+      </c>
+      <c r="L14" s="46" t="inlineStr">
+        <is>
+          <t>DEC-028</t>
+        </is>
+      </c>
+      <c r="M14" s="46" t="inlineStr">
+        <is>
+          <t>HAUPTTEXT-Satz; Rechnung Appendix</t>
+        </is>
+      </c>
+      <c r="N14" s="46" t="inlineStr">
+        <is>
+          <t>GO (RW 2026-07-04)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="46" t="inlineStr">
+        <is>
+          <t>N13</t>
+        </is>
+      </c>
+      <c r="B15" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C15" s="46" t="inlineStr">
+        <is>
+          <t>p-Curve / Evidenzwert der Post-Paris-Primärliteratur</t>
+        </is>
+      </c>
+      <c r="D15" s="46" t="inlineStr">
+        <is>
+          <t>Dreht die Beweislast komplett: Hat die Literatur, die den Post-Paris-Effekt nahelegt, überhaupt evidenziellen Wert — oder ist die positive Evidenz selbst dünn/selektiert?</t>
+        </is>
+      </c>
+      <c r="E15" s="46" t="inlineStr">
+        <is>
+          <t>Signifikante Effekte der Post-Zelle sammeln (ein p pro Studie, Regel a priori); p-Curve-Tests (Right-Skew, 33%-Power) nach Simonsohn et al.; p aus r,n rekonstruiert (Genauigkeitscaveat bei konvertierten r).</t>
+        </is>
+      </c>
+      <c r="F15" s="46" t="inlineStr">
+        <is>
+          <t>ja (p aus r,n rekonstruierbar)</t>
+        </is>
+      </c>
+      <c r="G15" s="46" t="inlineStr">
+        <is>
+          <t>Auswahlregel je Studie; MACHBARKEITSRISIKO: Post-Zelle = 11 Studien → ggf. &lt;5 signifikante p → nicht interpretierbar. Konditional: nur wenn ≥5</t>
+        </is>
+      </c>
+      <c r="H15" s="46" t="inlineStr">
+        <is>
+          <t>nein — Simonsohn et al. 2014 im PK</t>
+        </is>
+      </c>
+      <c r="I15" s="46" t="inlineStr">
+        <is>
+          <t>Simonsohn et al. 2014 (PK)</t>
+        </is>
+      </c>
+      <c r="J15" s="46" t="inlineStr">
+        <is>
+          <t>mittel (Beweislast-Umkehr), riskant</t>
+        </is>
+      </c>
+      <c r="K15" s="46" t="inlineStr">
+        <is>
+          <t>niedrig-mittel</t>
+        </is>
+      </c>
+      <c r="L15" s="46" t="inlineStr">
+        <is>
+          <t>DEC-028 (konditionale Regel a priori)</t>
+        </is>
+      </c>
+      <c r="M15" s="46" t="inlineStr">
+        <is>
+          <t>KONDITIONAL (Appendix, nur bei Machbarkeit)</t>
+        </is>
+      </c>
+      <c r="N15" s="46" t="inlineStr">
+        <is>
+          <t>GO — konditional (≥5-Regel a priori)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="46" t="inlineStr">
+        <is>
+          <t>N14</t>
+        </is>
+      </c>
+      <c r="B16" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C16" s="46" t="inlineStr">
+        <is>
+          <t>Publikations-Bias-Korrektur getrennt pre/post</t>
+        </is>
+      </c>
+      <c r="D16" s="46" t="inlineStr">
+        <is>
+          <t>Zeigt, dass der Null nicht durch asymmetrische Selektion in einer Periode erzeugt oder verdeckt wird — und ob der erwartete Post-Effekt der Literatur selbst selektionsgetrieben aussieht.</t>
+        </is>
+      </c>
+      <c r="E16" s="46" t="inlineStr">
+        <is>
+          <t>PET-PEESE (+ ggf. Selektionsmodelle) je Periode; Post-Zelle nur deskriptiv behandeln (11 Studien, Overclaim-Guard); RoBMA aus N3 deckt einen Teil modellgemittelt ab.</t>
+        </is>
+      </c>
+      <c r="F16" s="46" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G16" s="46" t="inlineStr">
+        <is>
+          <t>keine neuen; Post-Zellen-Grenzen beachten</t>
+        </is>
+      </c>
+      <c r="H16" s="46" t="inlineStr">
+        <is>
+          <t>nein — Stanley 2008/2013, Andrews-Kasy, Bartoš, van Aert alle im PK</t>
+        </is>
+      </c>
+      <c r="I16" s="46" t="inlineStr">
+        <is>
+          <t>T5-Anker (PK, mehrfach)</t>
+        </is>
+      </c>
+      <c r="J16" s="46" t="inlineStr">
+        <is>
+          <t>mittel-hoch</t>
+        </is>
+      </c>
+      <c r="K16" s="46" t="inlineStr">
+        <is>
+          <t>niedrig (T5-Maschinerie existiert)</t>
+        </is>
+      </c>
+      <c r="L16" s="46" t="inlineStr">
+        <is>
+          <t>T5-Scope-Erweiterung in DEC-028</t>
+        </is>
+      </c>
+      <c r="M16" s="46" t="inlineStr">
+        <is>
+          <t>APPENDIX; Haupttext-Satz</t>
+        </is>
+      </c>
+      <c r="N16" s="46" t="inlineStr">
+        <is>
+          <t>GO — Appendix</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="46" t="inlineStr">
+        <is>
+          <t>N15</t>
+        </is>
+      </c>
+      <c r="B17" s="46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C17" s="46" t="inlineStr">
+        <is>
+          <t>Within-Study-Paris-Kontrast (deskriptiv) — FLAGGED</t>
+        </is>
+      </c>
+      <c r="D17" s="46" t="inlineStr">
+        <is>
+          <t>Die einzige kompositionsfreie Paris-Evidenz: gleiche Studie, beide Perioden. Als deskriptive Zelle neben clean-window — kein Test.</t>
+        </is>
+      </c>
+      <c r="E17" s="46" t="inlineStr">
+        <is>
+          <t>Für die 3 Mixed-Studien (Chodnicka, Cubas, Seltzer) innerhalb der Studie Post-minus-Pre-Differenzen bilden; Punkt + Streuung deskriptiv ausweisen; explizit keine p-Werte (3 Cluster).</t>
+        </is>
+      </c>
+      <c r="F17" s="46" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G17" s="46" t="inlineStr">
+        <is>
+          <t>keine</t>
+        </is>
+      </c>
+      <c r="H17" s="46" t="inlineStr">
+        <is>
+          <t>nein</t>
+        </is>
+      </c>
+      <c r="I17" s="46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J17" s="46" t="inlineStr">
+        <is>
+          <t>niedrig-mittel (einzigartige Zelle)</t>
+        </is>
+      </c>
+      <c r="K17" s="46" t="inlineStr">
+        <is>
+          <t>sehr niedrig</t>
+        </is>
+      </c>
+      <c r="L17" s="46" t="inlineStr">
+        <is>
+          <t>ACHTUNG: DEC-008-Reopen nötig (Move 6 "dead") — nur mit explizitem Go (F19); Begründung: neue Zielsetzung Null-Battery</t>
+        </is>
+      </c>
+      <c r="M17" s="46" t="inlineStr">
+        <is>
+          <t>APPENDIX deskriptiv — nur nach Reopen-Go</t>
+        </is>
+      </c>
+      <c r="N17" s="46" t="inlineStr">
+        <is>
+          <t>GO — inkl. DEC-008-Teil-Reopen (nur deskriptiv)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4039,12 +6371,12 @@
       </c>
       <c r="F6" s="41" t="inlineStr">
         <is>
-          <t>offen · an V5/Pending-B gekoppelt</t>
+          <t>gelöst (2026-07-04, DEC-028)</t>
         </is>
       </c>
       <c r="G6" s="41" t="inlineStr">
         <is>
-          <t>method_artefacts = r-Konversions-/Extraktionsartefakt-Flag; Operationalisierung mit V5 (r-Transformations-Doku)</t>
+          <t>method_artefacts := ES_source (36 direct-r · 634 t · 570 b+SE · 66 p); §7 nutzt ES_source als 4-Level-Faktor (Ref = t-Route)</t>
         </is>
       </c>
     </row>
@@ -4392,7 +6724,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>offen (V4, vor Ch. 3)</t>
+          <t>gelöst (v9, V4)</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Flags geliefert: no_firms_source coded 593 / calculated 713 (54,6 %); autoritativ ggü. der 85 %-Arithmetik (DEC-028)</t>
         </is>
       </c>
     </row>
@@ -4422,7 +6759,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>offen (V5, vor Ch. 3)</t>
+          <t>gelöst (v9, V5; F21)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>formula-Sheet: 4 Routen dokumentiert; df≈n_obs-Konvention + pcc_df_k10/20-Sensitivität; k wird nicht nacherhoben; Pending-B geschlossen (DEC-028)</t>
         </is>
       </c>
     </row>
@@ -4483,6 +6825,11 @@
       <c r="F20" t="inlineStr">
         <is>
           <t>offen (nicht blockierend)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>None | v9/v10: Spalte L 65/65 gefüllt; Li-Waise entfernt (Lookup 65 Zeilen, Anti-Join 0/0); ES_measure-Fix (F20); Header-Typo source_verfified bleibt (Codebook-Alias); Shad-Kreuznotiz F22 in Overlap-Tabelle</t>
         </is>
       </c>
     </row>
@@ -4495,7 +6842,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4832,7 +7179,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5067,1065 +7414,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G31"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="53" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Decision-Log Index — DEC-ID-Register (Methodik-only; Pointer auf DECISION_LOG.md) (v1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>27 aktive Methodik-DECs (DEC-001..027). Volleinträge im DECISION_LOG.md (append-only).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>DEC-ID</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Datum</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Kategorie</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>Titel</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>Betrifft (#/Task)</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>Kurzfassung</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="40" customHeight="1">
-      <c r="A4" s="33" t="inlineStr">
-        <is>
-          <t>DEC-001</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Strategie</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Arbeitshypothese: Design bleibt</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>— / alle</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>FOMA CER–COD mit Paris als durchgaengiger Linse ueber alle Moderatoren.</t>
-        </is>
-      </c>
-      <c r="G4" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="40" customHeight="1">
-      <c r="A5" s="33" t="inlineStr">
-        <is>
-          <t>DEC-002</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>Dependence: 3LMA-RVE + Meta-Regression</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>#1,#2 / T1,T7</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>Multilevel/CE working model + RVE-CR2 als Headline + unified Meta-Regression — eine Pipeline, zwei Sichten.</t>
-        </is>
-      </c>
-      <c r="G5" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
-      <c r="A6" s="33" t="inlineStr">
-        <is>
-          <t>DEC-003</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>Headline-Rollenteilung</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>#1,#13 / T1,T7</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>3LMA-RVE traegt die Magnitude; Meta-Regression traegt die Identifikation (Bruch vs. Trend).</t>
-        </is>
-      </c>
-      <c r="G6" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="40" customHeight="1">
-      <c r="A7" s="33" t="inlineStr">
-        <is>
-          <t>DEC-004</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>Effektgroessen-Mischung</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>#5 / T4</t>
-        </is>
-      </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>Bivariat+partiell mischen, offenlegen, Literatur, Robustheit. Daten: nur 36 P → partial-only infeasibel, bivariat-only trivial.</t>
-        </is>
-      </c>
-      <c r="G7" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1">
-      <c r="A8" s="33" t="inlineStr">
-        <is>
-          <t>DEC-005</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>Event-Coding: Compute-then-Select</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>#3 / T2</t>
-        </is>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>Varianten rechnen (End/Median/Mean/Lags/Stringency); Headline a priori. Konkrete Headline-Wahl = Pending-A (nach T2).</t>
-        </is>
-      </c>
-      <c r="G8" s="33" t="inlineStr">
-        <is>
-          <t>aktiv (Detail offen)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="40" customHeight="1">
-      <c r="A9" s="33" t="inlineStr">
-        <is>
-          <t>DEC-006</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Framing</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>Kausalsprache abschwaechen</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>#4 / —</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>'structural break/exogenous shock' → 'temporal policy moderator'; Forschheit auf Debunking/Kontingenz umlenken.</t>
-        </is>
-      </c>
-      <c r="G9" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="40" customHeight="1">
-      <c r="A10" s="33" t="inlineStr">
-        <is>
-          <t>DEC-007</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Identifikation: 7-Move-Werkzeugkasten</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t>#13 / T8</t>
-        </is>
-      </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>Trend-Race · segm. MR · Placebo · Komposition · Diff-Exposure · Within-Study · Bounding.</t>
-        </is>
-      </c>
-      <c r="G10" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="40" customHeight="1">
-      <c r="A11" s="33" t="inlineStr">
-        <is>
-          <t>DEC-008</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Datenbefund</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>Within-Study tot; Moves 1–2 brauchen kont. Zeit</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t>#13 / T8,T0.4</t>
-        </is>
-      </c>
-      <c r="F11" s="6" t="inlineStr">
-        <is>
-          <t>Move 6 entfaellt (1–3/66 Studien ueberspannen). Identifikation ruht auf Moves 1–5; Moves 1–2 erfordern kont. Jahresvar. (T0.4).</t>
-        </is>
-      </c>
-      <c r="G11" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="40" customHeight="1">
-      <c r="A12" s="33" t="inlineStr">
-        <is>
-          <t>DEC-009</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>Moderator×Paris: Interaktion statt Subgruppen</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="inlineStr">
-        <is>
-          <t>#10 / T6,T7</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>Unified Interaktion (T7) statt genesteter Subgruppen — erzwungen durch duenne Cluster-Zellen (RVE-Mindest-Cluster unterschritten).</t>
-        </is>
-      </c>
-      <c r="G12" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="40" customHeight="1">
-      <c r="A13" s="33" t="inlineStr">
-        <is>
-          <t>DEC-010</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="inlineStr">
-        <is>
-          <t>Publikationsbias: PET-PEESE konsistent</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="inlineStr">
-        <is>
-          <t>#6 / T5</t>
-        </is>
-      </c>
-      <c r="F13" s="6" t="inlineStr">
-        <is>
-          <t>PET-PEESE-Entscheidungsregel ueber ALLE Subgruppen; PET n.s. → kein Effekt jenseits Bias. Industrie/No-pricing-Claims tempern.</t>
-        </is>
-      </c>
-      <c r="G13" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="40" customHeight="1">
-      <c r="A14" s="33" t="inlineStr">
-        <is>
-          <t>DEC-011</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Framing</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>Novelty: Zarea/Witte zitieren + abgrenzen</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr">
-        <is>
-          <t>#7 / —</t>
-        </is>
-      </c>
-      <c r="F14" s="6" t="inlineStr">
-        <is>
-          <t>'erste mit Paris' tot (Zarea H5). Novelty auf Debt-Kanal + Kanal-Dekomposition (Bank/Bond/CDS/Rating). Self-Overlap mit COE-Sibling adressieren.</t>
-        </is>
-      </c>
-      <c r="G14" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="40" customHeight="1">
-      <c r="A15" s="33" t="inlineStr">
-        <is>
-          <t>DEC-012</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Oekonomische Signifikanz in Basispunkten</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t>#8 / —</t>
-        </is>
-      </c>
-      <c r="F15" s="6" t="inlineStr">
-        <is>
-          <t>r → bp Credit-Spread; ehrliche Magnitude (r=−0,020 unter 0,07-Schwelle, Doucouliagos 2011); ~5× kleiner als Zarea.</t>
-        </is>
-      </c>
-      <c r="G15" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="40" customHeight="1">
-      <c r="A16" s="33" t="inlineStr">
-        <is>
-          <t>DEC-013</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>Outlier: 2 Extremwerte verifizieren statt winsorisieren</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>#9 / T0.4,T4</t>
-        </is>
-      </c>
-      <c r="F16" s="6" t="inlineStr">
-        <is>
-          <t>Drago (−0,998) + Devalle (+0,9998) als Kodierfehler-Verdacht an der Quelle pruefen; rstudent.rma.mv + drop-refit statt blankem Winsorizing.</t>
-        </is>
-      </c>
-      <c r="G16" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="40" customHeight="1">
-      <c r="A17" s="33" t="inlineStr">
-        <is>
-          <t>DEC-014</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
-        <is>
-          <t>Cluster-robuste Bias-/Meta-Regression (CR2)</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>#14,#6 / T5,T7</t>
-        </is>
-      </c>
-      <c r="F17" s="6" t="inlineStr">
-        <is>
-          <t>FAT-PET-PEESE &amp; Meta-Reg mit CR2-SE (geclustert auf study, Satterthwaite-df); 1.306 abh. ES nicht als unabhaengig. Tab. 7/8 neu.</t>
-        </is>
-      </c>
-      <c r="G17" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="40" customHeight="1">
-      <c r="A18" s="33" t="inlineStr">
-        <is>
-          <t>DEC-015</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>Korrelations-Small-Sample-Bias / UWLS+3</t>
-        </is>
-      </c>
-      <c r="E18" s="5" t="inlineStr">
-        <is>
-          <t>#15,#1,#5 / T4,T0.4</t>
-        </is>
-      </c>
-      <c r="F18" s="6" t="inlineStr">
-        <is>
-          <t>Fisher-z behalten (Stanley 2024/25: r-IVW rest-verzerrt, 37% n&lt;200); WLS/RVE-Headline begruenden; UWLS+3/HS-Robustheit; n-Verteilung; PCC-df (n−k−3); Bivariat-only.</t>
-        </is>
-      </c>
-      <c r="G18" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="40" customHeight="1">
-      <c r="A19" s="33" t="inlineStr">
-        <is>
-          <t>DEC-016</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Selektionsmodell sekundaer (3PSM/p-uniform*)</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="inlineStr">
-        <is>
-          <t>#16,#6 / T5</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>3PSM/p-uniform* (van Aert &amp; van Assen 2026) sekundaer auf Studienebene (k=66); PET-PEESE bleibt primaer (Stanley 2025). Triangulation.</t>
-        </is>
-      </c>
-      <c r="G19" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="40" customHeight="1">
-      <c r="A20" s="33" t="inlineStr">
-        <is>
-          <t>DEC-017</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>rho working correlation (CE/CHE-Kovarianz)</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="inlineStr">
-        <is>
-          <t>#1 / T1,T4</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>rho=0,6 default, Sensitivitaet 0,4/0,6/0,8; operationalisiert DEC-002. impute_covariance_matrix(r=0.6); CR2 macht Punktschaetzer rho-robust. spec rho_0.4/rho_0.8 in T4.</t>
-        </is>
-      </c>
-      <c r="G20" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="40" customHeight="1">
-      <c r="A21" s="33" t="inlineStr">
-        <is>
-          <t>DEC-018</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>2026-06-30</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>Interim-Zeitachse pub_year (E8)</t>
-        </is>
-      </c>
-      <c r="E21" s="5" t="inlineStr">
-        <is>
-          <t>#13 / T0.4,T8</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>Kont. Zeit fehlt im Datensatz; pub_year aus study geparst (alle 66, 2010-2024) als PROVISORISCHE Interim-Achse. Sample-Jahr (Datenagenda #10) ersetzt sie. T8 re-zentriert aus rohem pub_year.</t>
-        </is>
-      </c>
-      <c r="G21" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="40" customHeight="1">
-      <c r="A22" s="33" t="inlineStr">
-        <is>
-          <t>DEC-019</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="inlineStr">
-        <is>
-          <t>n-Definition = no_firms (headline)</t>
-        </is>
-      </c>
-      <c r="E22" s="5" t="inlineStr">
-        <is>
-          <t>T1,T4</t>
-        </is>
-      </c>
-      <c r="F22" s="6" t="inlineStr">
-        <is>
-          <t>no_firms als Gewichts-Basis; no_firm-years + study-level = Robustheit. [E14]</t>
-        </is>
-      </c>
-      <c r="G22" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="40" customHeight="1">
-      <c r="A23" s="33" t="inlineStr">
-        <is>
-          <t>DEC-020</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="inlineStr">
-        <is>
-          <t>Pre/Post-Operationalisierung + Headline-Cut</t>
-        </is>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
-        <is>
-          <t>T1,T4,T8</t>
-        </is>
-      </c>
-      <c r="F23" s="6" t="inlineStr">
-        <is>
-          <t>Suite (share/mid/end/start/median/tertil/window_class); Headline mid/kont., end→Robustheit (81% Kontamination); Cut-Entscheidung an Fable-5. Löst DEC-005-end ab.</t>
-        </is>
-      </c>
-      <c r="G23" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="40" customHeight="1">
-      <c r="A24" s="33" t="inlineStr">
-        <is>
-          <t>DEC-021</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="inlineStr">
-        <is>
-          <t>sample_mid = Zeitachse (löst DEC-018 ab)</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t>T8</t>
-        </is>
-      </c>
-      <c r="F24" s="6" t="inlineStr">
-        <is>
-          <t>Sample-Jahre vorhanden → sample_mid statt pub_year; Datenagenda #10 gelöst.</t>
-        </is>
-      </c>
-      <c r="G24" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="40" customHeight="1">
-      <c r="A25" s="33" t="inlineStr">
-        <is>
-          <t>DEC-022</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>Country-Moderatoren (region/dev/culture/legal)</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>T7</t>
-        </is>
-      </c>
-      <c r="F25" s="6" t="inlineStr">
-        <is>
-          <t>IMF Advanced · DST Western · La Porta common/civil · Region; parse-homogen → NCE; dominant gestrichen (E21).</t>
-        </is>
-      </c>
-      <c r="G25" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="40" customHeight="1">
-      <c r="A26" s="33" t="inlineStr">
-        <is>
-          <t>DEC-023</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>Quality-Moderatoren (status/VHB/JIF/field)</t>
-        </is>
-      </c>
-      <c r="E26" s="5" t="inlineStr">
-        <is>
-          <t>T7</t>
-        </is>
-      </c>
-      <c r="F26" s="6" t="inlineStr">
-        <is>
-          <t>source_lookup; CIT gestrichen. Offen: VHB/JIF für 536 Working Paper.</t>
-        </is>
-      </c>
-      <c r="G26" s="33" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>DEC-024</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>DEC-025</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Quality-Moderatoren konsolidiert; q_JIF gestrichen</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>T7</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>q_status + q_VHB (published-only, Referenzzellen-Kodierung); univariate VHB-Panels nur published; JIF analytisch tot (Roh im Lookup); DEC-023-Offenpunkt geschlossen</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>DEC-026</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Daten</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Publikationsstatus-Korrektur + Versions-Regel + Voll-Audit</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>source_lookup / T5,T7</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>7 Studien (229 Eff.) → published (Stand 2026-07-03); Effekte bleiben as-coded (Triage: keine materiellen Abweichungen); 66-Zeilen-Audit; spec status_as_extracted; Feld-Semantik journal/year=as coded, reference_verified=VoR</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>DEC-027</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Methodik</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>n-Definition validiert; E14 → n_obs</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>#1 / T1,T2,T4</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>no_firms bestätigt (konservativ; CR2-working-weights); Ableitungsregel round(n_obs/T) dokumentiert (85% konsistent, alle 9 n&lt;10); E14 umbenannt n_obs (81 Eff./3 Studien sub-annual/loan-level)</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>aktiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="33" t="inlineStr">
-        <is>
-          <t>Pending/Conditional DECs (im DECISION_LOG.md): Pending-A GELÖST → DEC-024 (2026-07-03) · Pending-B r-from-regression-Transformation (offen, V5) · Pending-C A-vs-C-Framing (offen, nach T8).</t>
-        </is>
-      </c>
-      <c r="B31" s="36" t="n"/>
-      <c r="C31" s="36" t="n"/>
-      <c r="D31" s="36" t="n"/>
-      <c r="E31" s="36" t="n"/>
-      <c r="F31" s="36" t="n"/>
-      <c r="G31" s="35" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A27:G27"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Extraction procedure: DEC-032 logged; codebook v1 frozen (F34a-f codified); production prompt + staging template; blind-pilot gate defined
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -13,10 +13,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aufgaben" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysen" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Null_Battery" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datenagenda" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifikation" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key_Results" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DecisionLog_Index" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Scoping" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datenagenda" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifikation" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key_Results" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DecisionLog_Index" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1322,7 +1323,244 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Key Results — Headline-Zahlen je abgeschlossener Analyse (v1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Digest-Layer (SOMA-Analog). Wird bei jedem Lauf gefuellt; verlinkt auf die Per-Lauf-Results-xls bzw. output-CSV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Analysis</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 — Core (T1–T3)</t>
+        </is>
+      </c>
+      <c r="B4" s="36" t="n"/>
+      <c r="C4" s="35" t="n"/>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>T1 · Hauptanalyse CER–COD (gepoolt, 3LMA-RVE)</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>output/T1_results.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="26" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>T1 · Pre/Post-Paris (Headline-Coding)</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>output/T1_results.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>T3 · Heterogenitaet (σ²_within/between, ICC, I²)</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>output/T3_results.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 — Identifikation &amp; Robustheit (T2, T8, T5, T4)</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="n"/>
+      <c r="C8" s="35" t="n"/>
+    </row>
+    <row r="9" ht="26" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>T2 · Event-Coding-Vergleich (Headline-Wahl)</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>output/T2_results.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="26" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>T8 · Identifikation Bruch vs. Trend (Verdict)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>output/T8_results.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="26" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>T5 · Publikationsbias (FAT-PET-PEESE)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>output/T5_results.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>T4 · Robustheit (Verdict)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>output/T4_results.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 — Moderatoren (T6, T7)</t>
+        </is>
+      </c>
+      <c r="B13" s="36" t="n"/>
+      <c r="C13" s="35" t="n"/>
+    </row>
+    <row r="14" ht="26" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>T6 · Moderatoren × Paris</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>output/T6_results.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="26" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>T7 · Unified Meta-Regression (Paris×Moderator)</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>output/T7_results.csv</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2440,6 +2678,30 @@
       <c r="E33" s="36" t="n"/>
       <c r="F33" s="36" t="n"/>
       <c r="G33" s="35" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>DEC-030</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Formales PRISMA-Suchupdate beschlossen (rule-based, pre-T1); CER-Gate kodifiziert (F32v2); 4-Engine-Scoping dokumentiert (~41+10 Kandidaten); Renumbering: Battery-Inputs → DEC-031</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>DEC-032</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>AI-Extraktion mit Rollen-Inversion (Claude extrahiert, Volker verifiziert 100% der Statistikfelder); Codebook v1 frozen (F34a-f kodifiziert; 13/13 Kalibrier-Effekte zellengenau reproduziert); Blind-Pilot-Gate ≥95% Konkordanz vor Produktion</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2605,7 +2867,7 @@
       </c>
       <c r="D5" s="41" t="inlineStr">
         <is>
-          <t>Re-prep (R/01_prep.R) gegen CER-COD_data_v10.xlsx; Verifier erweitert um DEC-024..028-Checks (pp_start≥2016, Identitäten, Lookup-Anti-Join, ES_source×ES_measure-Diagonale, Formel-Spotcheck, df-Berechnung Transfer-Regel). Vorab: DEC-029-Battery-Inputs fixieren (SESOI, Priors, Faktorraum, Grids). Öffnet das T1-Gate.</t>
+          <t>Re-prep (R/01_prep.R) gegen CER-COD_data_v10.xlsx; Verifier erweitert um DEC-024..028-Checks (pp_start≥2016, Identitäten, Lookup-Anti-Join, ES_source×ES_measure-Diagonale, Formel-Spotcheck, df-Berechnung Transfer-Regel). Vorab: DEC-029-Battery-Inputs fixieren (SESOI, Priors, Faktorraum, Grids). Öffnet das T1-Gate. — ERWEITERT [DEC-030]: zusätzlich erst v11 (Suchupdate) abwarten.</t>
         </is>
       </c>
       <c r="E5" s="41" t="inlineStr">
@@ -6216,7 +6478,3774 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:I85"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>KONSOLIDIERTE SCREENING-LISTE (4 Engines: Claude=C, ChatGPT=G, Perplexity-Base=P1/P2, Perplexity-Agent=A) — DEC-030. Klassen: P1=Download publiziert · P1-WP=Download Working Paper · B=Konstrukt-/Record-Check vor Download · D=raus per F32v2/Outcome (Ch.2-Kontext) · E=im Korpus/Dedup · F28=prä-Fenster-Exklusionsdoku (Volker) · R2=Runde-2-Preview. Suchinstrument bleibt Volkers DB-Re-Run (DEC-030); diese Liste = dokumentierte Supplementärsuche + Recall-Messlatte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="45" t="inlineStr">
+        <is>
+          <t>Nr</t>
+        </is>
+      </c>
+      <c r="B2" s="45" t="inlineStr">
+        <is>
+          <t>Klasse</t>
+        </is>
+      </c>
+      <c r="C2" s="45" t="inlineStr">
+        <is>
+          <t>Referenz</t>
+        </is>
+      </c>
+      <c r="D2" s="45" t="inlineStr">
+        <is>
+          <t>Konstrukt</t>
+        </is>
+      </c>
+      <c r="E2" s="45" t="inlineStr">
+        <is>
+          <t>Outcome</t>
+        </is>
+      </c>
+      <c r="F2" s="45" t="inlineStr">
+        <is>
+          <t>Fenster/Region</t>
+        </is>
+      </c>
+      <c r="G2" s="45" t="inlineStr">
+        <is>
+          <t>Engines</t>
+        </is>
+      </c>
+      <c r="H2" s="45" t="inlineStr">
+        <is>
+          <t>Aktion</t>
+        </is>
+      </c>
+      <c r="I2" s="45" t="inlineStr">
+        <is>
+          <t>Notiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="46" t="inlineStr">
+        <is>
+          <t>P1-01</t>
+        </is>
+      </c>
+      <c r="B3" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C3" s="46" t="inlineStr">
+        <is>
+          <t>Owolabi, Mousavi, Gozgor &amp; Li (2024). Energy Economics 139, 107925. DOI 10.1016/j.eneco.2024.107925</t>
+        </is>
+      </c>
+      <c r="D3" s="46" t="inlineStr">
+        <is>
+          <t>Carbon Risk</t>
+        </is>
+      </c>
+      <c r="E3" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F3" s="46" t="inlineStr">
+        <is>
+          <t>2011-20 G7</t>
+        </is>
+      </c>
+      <c r="G3" s="46" t="inlineStr">
+        <is>
+          <t>C,G,P1,P2,A</t>
+        </is>
+      </c>
+      <c r="H3" s="46" t="inlineStr">
+        <is>
+          <t>Download + PK (F29)</t>
+        </is>
+      </c>
+      <c r="I3" s="46" t="inlineStr">
+        <is>
+          <t>Paris-Design · N12-formal · Gold-OA</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="46" t="inlineStr">
+        <is>
+          <t>P1-02</t>
+        </is>
+      </c>
+      <c r="B4" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C4" s="46" t="inlineStr">
+        <is>
+          <t>Ehlers, Packer &amp; de Greiff (2022). JBF 136, 106180</t>
+        </is>
+      </c>
+      <c r="D4" s="46" t="inlineStr">
+        <is>
+          <t>Carbon-Intensität (Scope 1)</t>
+        </is>
+      </c>
+      <c r="E4" s="46" t="inlineStr">
+        <is>
+          <t>Synd. Loans</t>
+        </is>
+      </c>
+      <c r="F4" s="46" t="inlineStr">
+        <is>
+          <t>2014-18 global</t>
+        </is>
+      </c>
+      <c r="G4" s="46" t="inlineStr">
+        <is>
+          <t>C,G,P2,A</t>
+        </is>
+      </c>
+      <c r="H4" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I4" s="46" t="inlineStr">
+        <is>
+          <t>BIS WP 946 = OA-Route</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="46" t="inlineStr">
+        <is>
+          <t>P1-03</t>
+        </is>
+      </c>
+      <c r="B5" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C5" s="46" t="inlineStr">
+        <is>
+          <t>Al-Fakir Al Rabab'a, Rashid &amp; Shams (2023). IRFA 88, 102641</t>
+        </is>
+      </c>
+      <c r="D5" s="46" t="inlineStr">
+        <is>
+          <t>Carbon Performance (CDP)</t>
+        </is>
+      </c>
+      <c r="E5" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F5" s="46" t="inlineStr">
+        <is>
+          <t>2003-18 APAC</t>
+        </is>
+      </c>
+      <c r="G5" s="46" t="inlineStr">
+        <is>
+          <t>C,G,P2,A</t>
+        </is>
+      </c>
+      <c r="H5" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I5" s="46" t="inlineStr">
+        <is>
+          <t>Art.-Nr. 102641 (2:1 vs. 102651)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="46" t="inlineStr">
+        <is>
+          <t>P1-04</t>
+        </is>
+      </c>
+      <c r="B6" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C6" s="46" t="inlineStr">
+        <is>
+          <t>Cumming, Duppati, Fernando, Singh &amp; Tiwari (2025). BAR 57(2), 101353. DOI 10.1016/j.bar.2024.101353</t>
+        </is>
+      </c>
+      <c r="D6" s="46" t="inlineStr">
+        <is>
+          <t>Carbon Risk</t>
+        </is>
+      </c>
+      <c r="E6" s="46" t="inlineStr">
+        <is>
+          <t>CoD/Leverage-Adj.</t>
+        </is>
+      </c>
+      <c r="F6" s="46" t="inlineStr">
+        <is>
+          <t>2006-20</t>
+        </is>
+      </c>
+      <c r="G6" s="46" t="inlineStr">
+        <is>
+          <t>G,A</t>
+        </is>
+      </c>
+      <c r="H6" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I6" s="46" t="inlineStr">
+        <is>
+          <t>2x Perplexity-Blindstelle · via DOI ziehen</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="46" t="inlineStr">
+        <is>
+          <t>P1-05</t>
+        </is>
+      </c>
+      <c r="B7" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C7" s="46" t="inlineStr">
+        <is>
+          <t>Ho &amp; Wong (2021/2023). HKMA RM06-2021 [PDF frei] / EMR 55 prüfen</t>
+        </is>
+      </c>
+      <c r="D7" s="46" t="inlineStr">
+        <is>
+          <t>GHG-Intensität, Brown-Flag</t>
+        </is>
+      </c>
+      <c r="E7" s="46" t="inlineStr">
+        <is>
+          <t>Synd. Loans (AISD)</t>
+        </is>
+      </c>
+      <c r="F7" s="46" t="inlineStr">
+        <is>
+          <t>2010-21 APAC</t>
+        </is>
+      </c>
+      <c r="G7" s="46" t="inlineStr">
+        <is>
+          <t>P1,G,A</t>
+        </is>
+      </c>
+      <c r="H7" s="46" t="inlineStr">
+        <is>
+          <t>Download Memo + EMR-Verify</t>
+        </is>
+      </c>
+      <c r="I7" s="46" t="inlineStr">
+        <is>
+          <t>Koeffizienten liegen vor (+44.59***) · Publikations-Check am Record</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="46" t="inlineStr">
+        <is>
+          <t>P1-06</t>
+        </is>
+      </c>
+      <c r="B8" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C8" s="46" t="inlineStr">
+        <is>
+          <t>Ali, Nadeem, Pandey &amp; Bhabra (2023). BSE 32(6), 3417-3431. DOI 10.1002/bse.3308</t>
+        </is>
+      </c>
+      <c r="D8" s="46" t="inlineStr">
+        <is>
+          <t>Env. Performance</t>
+        </is>
+      </c>
+      <c r="E8" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F8" s="46" t="inlineStr"/>
+      <c r="G8" s="46" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H8" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I8" s="46" t="inlineStr">
+        <is>
+          <t>BSE-Fit-Beleg 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="46" t="inlineStr">
+        <is>
+          <t>P1-07</t>
+        </is>
+      </c>
+      <c r="B9" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C9" s="46" t="inlineStr">
+        <is>
+          <t>Kleimeier &amp; Viehs (2021). Economics Letters 205, 109936</t>
+        </is>
+      </c>
+      <c r="D9" s="46" t="inlineStr">
+        <is>
+          <t>Carbon Disclosure/Pricing</t>
+        </is>
+      </c>
+      <c r="E9" s="46" t="inlineStr">
+        <is>
+          <t>Loans</t>
+        </is>
+      </c>
+      <c r="F9" s="46" t="inlineStr"/>
+      <c r="G9" s="46" t="inlineStr">
+        <is>
+          <t>C,G</t>
+        </is>
+      </c>
+      <c r="H9" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I9" s="46" t="inlineStr">
+        <is>
+          <t>Supersession des 2016/18-WP per Fussnote pruefen</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="46" t="inlineStr">
+        <is>
+          <t>P1-08</t>
+        </is>
+      </c>
+      <c r="B10" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C10" s="46" t="inlineStr">
+        <is>
+          <t>Dumrose &amp; Höck (2023). FRL 51, 103414</t>
+        </is>
+      </c>
+      <c r="D10" s="46" t="inlineStr">
+        <is>
+          <t>Carbon-Mgmt (CDP) + Exposure</t>
+        </is>
+      </c>
+      <c r="E10" s="46" t="inlineStr">
+        <is>
+          <t>Credit Spreads</t>
+        </is>
+      </c>
+      <c r="F10" s="46" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="G10" s="46" t="inlineStr">
+        <is>
+          <t>C,P2,A</t>
+        </is>
+      </c>
+      <c r="H10" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I10" s="46" t="inlineStr">
+        <is>
+          <t>Mgmt-Schätzer extrahieren (Exposure-Teil = F32v2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="46" t="inlineStr">
+        <is>
+          <t>P1-09</t>
+        </is>
+      </c>
+      <c r="B11" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C11" s="46" t="inlineStr">
+        <is>
+          <t>Mahmoudian et al. (2023). JIAAT 52</t>
+        </is>
+      </c>
+      <c r="D11" s="46" t="inlineStr">
+        <is>
+          <t>Carbon</t>
+        </is>
+      </c>
+      <c r="E11" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F11" s="46" t="inlineStr"/>
+      <c r="G11" s="46" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H11" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I11" s="46" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="46" t="inlineStr">
+        <is>
+          <t>P1-10</t>
+        </is>
+      </c>
+      <c r="B12" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C12" s="46" t="inlineStr">
+        <is>
+          <t>González Sánchez et al. (2026). CSREM 33(1), 1230-1248. DOI 10.1002/csr.70220</t>
+        </is>
+      </c>
+      <c r="D12" s="46" t="inlineStr">
+        <is>
+          <t>Env.</t>
+        </is>
+      </c>
+      <c r="E12" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F12" s="46" t="inlineStr"/>
+      <c r="G12" s="46" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H12" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I12" s="46" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="46" t="inlineStr">
+        <is>
+          <t>P1-11</t>
+        </is>
+      </c>
+      <c r="B13" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C13" s="46" t="inlineStr">
+        <is>
+          <t>Wang, Chang &amp; Wu (2025). CSREM 32(1), 465-480. DOI 10.1002/csr.2953</t>
+        </is>
+      </c>
+      <c r="D13" s="46" t="inlineStr">
+        <is>
+          <t>Env.</t>
+        </is>
+      </c>
+      <c r="E13" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F13" s="46" t="inlineStr"/>
+      <c r="G13" s="46" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H13" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I13" s="46" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="46" t="inlineStr">
+        <is>
+          <t>P1-12</t>
+        </is>
+      </c>
+      <c r="B14" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C14" s="46" t="inlineStr">
+        <is>
+          <t>Lin et al. (2025). CSREM. DOI 10.1002/csr.70087</t>
+        </is>
+      </c>
+      <c r="D14" s="46" t="inlineStr">
+        <is>
+          <t>Env.</t>
+        </is>
+      </c>
+      <c r="E14" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F14" s="46" t="inlineStr"/>
+      <c r="G14" s="46" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H14" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I14" s="46" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="46" t="inlineStr">
+        <is>
+          <t>P1-13</t>
+        </is>
+      </c>
+      <c r="B15" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C15" s="46" t="inlineStr">
+        <is>
+          <t>Safiullah et al. (2025). A&amp;F 65(2), 2173-2210. DOI 10.1111/acfi.70000</t>
+        </is>
+      </c>
+      <c r="D15" s="46" t="inlineStr">
+        <is>
+          <t>Env.</t>
+        </is>
+      </c>
+      <c r="E15" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F15" s="46" t="inlineStr"/>
+      <c r="G15" s="46" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H15" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I15" s="46" t="inlineStr">
+        <is>
+          <t>NEUES Paper (≠ Korpus-Safiullah 2021)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="46" t="inlineStr">
+        <is>
+          <t>P1-14</t>
+        </is>
+      </c>
+      <c r="B16" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C16" s="46" t="inlineStr">
+        <is>
+          <t>Nasih et al. (2024). SAGE Open 14(4), 21582440241292134</t>
+        </is>
+      </c>
+      <c r="D16" s="46" t="inlineStr">
+        <is>
+          <t>Carbon-Disclosure</t>
+        </is>
+      </c>
+      <c r="E16" s="46" t="inlineStr">
+        <is>
+          <t>CoD (Zins)</t>
+        </is>
+      </c>
+      <c r="F16" s="46" t="inlineStr">
+        <is>
+          <t>2015-19 Indonesien</t>
+        </is>
+      </c>
+      <c r="G16" s="46" t="inlineStr">
+        <is>
+          <t>C,A</t>
+        </is>
+      </c>
+      <c r="H16" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I16" s="46" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="46" t="inlineStr">
+        <is>
+          <t>P1-15</t>
+        </is>
+      </c>
+      <c r="B17" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C17" s="46" t="inlineStr">
+        <is>
+          <t>Cicchini, De Luca, Principale &amp; Signore (2026). BSE Early View. DOI 10.1002/bse.70550</t>
+        </is>
+      </c>
+      <c r="D17" s="46" t="inlineStr">
+        <is>
+          <t>GHG</t>
+        </is>
+      </c>
+      <c r="E17" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F17" s="46" t="inlineStr">
+        <is>
+          <t>2021-24 Europa</t>
+        </is>
+      </c>
+      <c r="G17" s="46" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H17" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I17" s="46" t="inlineStr">
+        <is>
+          <t>BSE-Fit 2 · reines Post-Paris-Fenster!</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="46" t="inlineStr">
+        <is>
+          <t>P1-16</t>
+        </is>
+      </c>
+      <c r="B18" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C18" s="46" t="inlineStr">
+        <is>
+          <t>Boubaker et al. (2026). IREF 106, 104910</t>
+        </is>
+      </c>
+      <c r="D18" s="46" t="inlineStr">
+        <is>
+          <t>Env. Practices</t>
+        </is>
+      </c>
+      <c r="E18" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F18" s="46" t="inlineStr">
+        <is>
+          <t>2015-23 Europa</t>
+        </is>
+      </c>
+      <c r="G18" s="46" t="inlineStr">
+        <is>
+          <t>G,P2</t>
+        </is>
+      </c>
+      <c r="H18" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I18" s="46" t="inlineStr">
+        <is>
+          <t>Autoren am PDF klären (P2-Garble: Chouaibi/Hamza)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="46" t="inlineStr">
+        <is>
+          <t>P1-17</t>
+        </is>
+      </c>
+      <c r="B19" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C19" s="46" t="inlineStr">
+        <is>
+          <t>Ali, Farooq &amp; Al-Jabri (2026). CSREM. DOI 10.1002/csr.70643</t>
+        </is>
+      </c>
+      <c r="D19" s="46" t="inlineStr">
+        <is>
+          <t>Carbon</t>
+        </is>
+      </c>
+      <c r="E19" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F19" s="46" t="inlineStr"/>
+      <c r="G19" s="46" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H19" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I19" s="46" t="inlineStr">
+        <is>
+          <t>Board-Gender-Lead ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="46" t="inlineStr">
+        <is>
+          <t>P1-18</t>
+        </is>
+      </c>
+      <c r="B20" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C20" s="46" t="inlineStr">
+        <is>
+          <t>Attig, Rahaman &amp; Trabelsi (2025). CGIR 33(2), 202-230. DOI 10.1111/corg.12599</t>
+        </is>
+      </c>
+      <c r="D20" s="46" t="inlineStr">
+        <is>
+          <t>Env.</t>
+        </is>
+      </c>
+      <c r="E20" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F20" s="46" t="inlineStr"/>
+      <c r="G20" s="46" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H20" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I20" s="46" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="46" t="inlineStr">
+        <is>
+          <t>P1-19</t>
+        </is>
+      </c>
+      <c r="B21" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C21" s="46" t="inlineStr">
+        <is>
+          <t>Borsuk &amp; Shrimali (2026). Energy Economics 158, 109315</t>
+        </is>
+      </c>
+      <c r="D21" s="46" t="inlineStr">
+        <is>
+          <t>Env.</t>
+        </is>
+      </c>
+      <c r="E21" s="46" t="inlineStr">
+        <is>
+          <t>Ratings</t>
+        </is>
+      </c>
+      <c r="F21" s="46" t="inlineStr">
+        <is>
+          <t>Indien</t>
+        </is>
+      </c>
+      <c r="G21" s="46" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H21" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I21" s="46" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="46" t="inlineStr">
+        <is>
+          <t>P1-20</t>
+        </is>
+      </c>
+      <c r="B22" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C22" s="46" t="inlineStr">
+        <is>
+          <t>Brinette, Abidi Perier &amp; Sener Tournus (2026). FRL 98, 109835</t>
+        </is>
+      </c>
+      <c r="D22" s="46" t="inlineStr">
+        <is>
+          <t>Waste Mgmt</t>
+        </is>
+      </c>
+      <c r="E22" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F22" s="46" t="inlineStr">
+        <is>
+          <t>STOXX600</t>
+        </is>
+      </c>
+      <c r="G22" s="46" t="inlineStr">
+        <is>
+          <t>G,P1</t>
+        </is>
+      </c>
+      <c r="H22" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I22" s="46">
+        <f> VoR des Waste-WP SSRN 5553376 (nur FRL ziehen)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="46" t="inlineStr">
+        <is>
+          <t>P1-21</t>
+        </is>
+      </c>
+      <c r="B23" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C23" s="46" t="inlineStr">
+        <is>
+          <t>Almutairi (2026). IJFS 14(5), 123</t>
+        </is>
+      </c>
+      <c r="D23" s="46" t="inlineStr">
+        <is>
+          <t>Env.-Disclosure</t>
+        </is>
+      </c>
+      <c r="E23" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F23" s="46" t="inlineStr">
+        <is>
+          <t>Ägypten</t>
+        </is>
+      </c>
+      <c r="G23" s="46" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H23" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I23" s="46" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="46" t="inlineStr">
+        <is>
+          <t>P1-22</t>
+        </is>
+      </c>
+      <c r="B24" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C24" s="46" t="inlineStr">
+        <is>
+          <t>Bahloul &amp; Wali (2026). EuroMed JB. DOI 10.1108/EMJB-07-2025-0254</t>
+        </is>
+      </c>
+      <c r="D24" s="46" t="inlineStr">
+        <is>
+          <t>Env. Emissions</t>
+        </is>
+      </c>
+      <c r="E24" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F24" s="46" t="inlineStr"/>
+      <c r="G24" s="46" t="inlineStr">
+        <is>
+          <t>G,P1</t>
+        </is>
+      </c>
+      <c r="H24" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I24" s="46" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="46" t="inlineStr">
+        <is>
+          <t>P1-23</t>
+        </is>
+      </c>
+      <c r="B25" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C25" s="46" t="inlineStr">
+        <is>
+          <t>Tan et al. (2026). Int. Review of Finance 26(1), e70064</t>
+        </is>
+      </c>
+      <c r="D25" s="46" t="inlineStr">
+        <is>
+          <t>Klimarisiko-DISCLOSURE</t>
+        </is>
+      </c>
+      <c r="E25" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F25" s="46" t="inlineStr"/>
+      <c r="G25" s="46" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H25" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I25" s="46" t="inlineStr">
+        <is>
+          <t>Disclosure = Conduct ✓ (≠ Exposure)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="46" t="inlineStr">
+        <is>
+          <t>P1-24</t>
+        </is>
+      </c>
+      <c r="B26" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C26" s="46" t="inlineStr">
+        <is>
+          <t>Kim &amp; Pouget (2026). JCF 97, 102932</t>
+        </is>
+      </c>
+      <c r="D26" s="46" t="inlineStr">
+        <is>
+          <t>Carbon</t>
+        </is>
+      </c>
+      <c r="E26" s="46" t="inlineStr">
+        <is>
+          <t>Bond Spreads (primär/sekundär)</t>
+        </is>
+      </c>
+      <c r="F26" s="46" t="inlineStr">
+        <is>
+          <t>2005-22 USA</t>
+        </is>
+      </c>
+      <c r="G26" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H26" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I26" s="46" t="inlineStr">
+        <is>
+          <t>Claude-Lead 1 ✓ · stats confirmed</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="46" t="inlineStr">
+        <is>
+          <t>P1-25</t>
+        </is>
+      </c>
+      <c r="B27" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C27" s="46" t="inlineStr">
+        <is>
+          <t>Okimoto &amp; Takaoka (2024). Energy Economics 133, 107504</t>
+        </is>
+      </c>
+      <c r="D27" s="46" t="inlineStr">
+        <is>
+          <t>Carbon</t>
+        </is>
+      </c>
+      <c r="E27" s="46" t="inlineStr">
+        <is>
+          <t>CDS</t>
+        </is>
+      </c>
+      <c r="F27" s="46" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="G27" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H27" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I27" s="46" t="inlineStr">
+        <is>
+          <t>ZWEITPAPER (≠ Korpus-O&amp;T = IRFA 91, 103052)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="46" t="inlineStr">
+        <is>
+          <t>P1-26</t>
+        </is>
+      </c>
+      <c r="B28" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C28" s="46" t="inlineStr">
+        <is>
+          <t>D'Arcangelo, Kruse, Pisu &amp; Tomasi (2025). JEM 387, 125866</t>
+        </is>
+      </c>
+      <c r="D28" s="46" t="inlineStr">
+        <is>
+          <t>Emissionsintensität + Green Patents</t>
+        </is>
+      </c>
+      <c r="E28" s="46" t="inlineStr">
+        <is>
+          <t>Synd. Loans</t>
+        </is>
+      </c>
+      <c r="F28" s="46" t="inlineStr">
+        <is>
+          <t>40 Länder</t>
+        </is>
+      </c>
+      <c r="G28" s="46" t="inlineStr">
+        <is>
+          <t>P2,A</t>
+        </is>
+      </c>
+      <c r="H28" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I28" s="46" t="inlineStr">
+        <is>
+          <t>ex-OECD WP 1757</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="46" t="inlineStr">
+        <is>
+          <t>P1-27</t>
+        </is>
+      </c>
+      <c r="B29" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C29" s="46" t="inlineStr">
+        <is>
+          <t>Ma et al. (2022). J. Int. Fin. Mgmt &amp; Accounting 33(3), 480-504. DOI 10.1111/jifm.12154</t>
+        </is>
+      </c>
+      <c r="D29" s="46" t="inlineStr">
+        <is>
+          <t>Umwelt-Violations</t>
+        </is>
+      </c>
+      <c r="E29" s="46" t="inlineStr">
+        <is>
+          <t>Bondkosten</t>
+        </is>
+      </c>
+      <c r="F29" s="46" t="inlineStr">
+        <is>
+          <t>2008-20 China</t>
+        </is>
+      </c>
+      <c r="G29" s="46" t="inlineStr">
+        <is>
+          <t>P2,A</t>
+        </is>
+      </c>
+      <c r="H29" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I29" s="46" t="inlineStr">
+        <is>
+          <t>P2-Journal-Garble korrigiert · Autorenliste am PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="46" t="inlineStr">
+        <is>
+          <t>P1-28</t>
+        </is>
+      </c>
+      <c r="B30" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C30" s="46" t="inlineStr">
+        <is>
+          <t>Duong, Kalev, Kalimipalli &amp; Trivedi (2025). JCF 94, 102843</t>
+        </is>
+      </c>
+      <c r="D30" s="46" t="inlineStr">
+        <is>
+          <t>Carbon-Risk-MANAGEMENT (CDP)</t>
+        </is>
+      </c>
+      <c r="E30" s="46" t="inlineStr">
+        <is>
+          <t>CDS</t>
+        </is>
+      </c>
+      <c r="F30" s="46" t="inlineStr">
+        <is>
+          <t>2009-18 USA</t>
+        </is>
+      </c>
+      <c r="G30" s="46" t="inlineStr">
+        <is>
+          <t>A,P2</t>
+        </is>
+      </c>
+      <c r="H30" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I30" s="46" t="inlineStr">
+        <is>
+          <t>P2 hatte Javadi&amp;Al-Masum konflatiert</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="46" t="inlineStr">
+        <is>
+          <t>P1-29</t>
+        </is>
+      </c>
+      <c r="B31" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C31" s="46" t="inlineStr">
+        <is>
+          <t>Wang, Ding, Yang &amp; Wu (2025). IRFA 106</t>
+        </is>
+      </c>
+      <c r="D31" s="46" t="inlineStr">
+        <is>
+          <t>Env. Performance</t>
+        </is>
+      </c>
+      <c r="E31" s="46" t="inlineStr">
+        <is>
+          <t>Bond Spreads</t>
+        </is>
+      </c>
+      <c r="F31" s="46" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="G31" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H31" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I31" s="46" t="inlineStr">
+        <is>
+          <t>Art.-Nr. am Record</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="46" t="inlineStr">
+        <is>
+          <t>P1-30</t>
+        </is>
+      </c>
+      <c r="B32" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C32" s="46" t="inlineStr">
+        <is>
+          <t>Wang &amp; Wijethilake (2026). BSE 35(7). DOI 10.1002/bse.71126</t>
+        </is>
+      </c>
+      <c r="D32" s="46" t="inlineStr">
+        <is>
+          <t>Carbon-Disclosure-Qualität</t>
+        </is>
+      </c>
+      <c r="E32" s="46" t="inlineStr">
+        <is>
+          <t>Green-Bond-Kosten</t>
+        </is>
+      </c>
+      <c r="F32" s="46" t="inlineStr">
+        <is>
+          <t>2014-24 China</t>
+        </is>
+      </c>
+      <c r="G32" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H32" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I32" s="46" t="inlineStr">
+        <is>
+          <t>BSE-Fit 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="46" t="inlineStr">
+        <is>
+          <t>P1-31</t>
+        </is>
+      </c>
+      <c r="B33" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C33" s="46" t="inlineStr">
+        <is>
+          <t>Xiang &amp; Gong (2026). FRL 103, 110156</t>
+        </is>
+      </c>
+      <c r="D33" s="46" t="inlineStr">
+        <is>
+          <t>TCFD-Klima-Disclosure</t>
+        </is>
+      </c>
+      <c r="E33" s="46" t="inlineStr">
+        <is>
+          <t>Bond Spreads</t>
+        </is>
+      </c>
+      <c r="F33" s="46" t="inlineStr">
+        <is>
+          <t>2008-23 China</t>
+        </is>
+      </c>
+      <c r="G33" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H33" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I33" s="46" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="46" t="inlineStr">
+        <is>
+          <t>P1-32</t>
+        </is>
+      </c>
+      <c r="B34" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C34" s="46" t="inlineStr">
+        <is>
+          <t>Ririmasse, Tsitsianis &amp; Mitrou (2026). EMFT 62(9), 2966-2984</t>
+        </is>
+      </c>
+      <c r="D34" s="46" t="inlineStr">
+        <is>
+          <t>Carbon-Intensität/Reporting</t>
+        </is>
+      </c>
+      <c r="E34" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F34" s="46" t="inlineStr">
+        <is>
+          <t>dev+EM</t>
+        </is>
+      </c>
+      <c r="G34" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H34" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I34" s="46" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="46" t="inlineStr">
+        <is>
+          <t>P1-33</t>
+        </is>
+      </c>
+      <c r="B35" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C35" s="46" t="inlineStr">
+        <is>
+          <t>Shi, Zhou &amp; Wang (2025). JEM 389, 126152</t>
+        </is>
+      </c>
+      <c r="D35" s="46" t="inlineStr">
+        <is>
+          <t>Env.-Performance-Ratings</t>
+        </is>
+      </c>
+      <c r="E35" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F35" s="46" t="inlineStr">
+        <is>
+          <t>2018-20</t>
+        </is>
+      </c>
+      <c r="G35" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H35" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I35" s="46" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="46" t="inlineStr">
+        <is>
+          <t>P1-34</t>
+        </is>
+      </c>
+      <c r="B36" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C36" s="46" t="inlineStr">
+        <is>
+          <t>Hu, Lazar, Pan &amp; Wang (2024). IRFA 96, 103635</t>
+        </is>
+      </c>
+      <c r="D36" s="46" t="inlineStr">
+        <is>
+          <t>Env. Performance</t>
+        </is>
+      </c>
+      <c r="E36" s="46" t="inlineStr">
+        <is>
+          <t>Credit Ratings</t>
+        </is>
+      </c>
+      <c r="F36" s="46" t="inlineStr">
+        <is>
+          <t>US/EU</t>
+        </is>
+      </c>
+      <c r="G36" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H36" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I36" s="46" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="46" t="inlineStr">
+        <is>
+          <t>P1-35</t>
+        </is>
+      </c>
+      <c r="B37" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C37" s="46" t="inlineStr">
+        <is>
+          <t>Yang, Wen &amp; Li (2024). J. Applied Economics 27(1), 2301280</t>
+        </is>
+      </c>
+      <c r="D37" s="46" t="inlineStr">
+        <is>
+          <t>Env.-Info-Disclosure</t>
+        </is>
+      </c>
+      <c r="E37" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F37" s="46" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="G37" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H37" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I37" s="46" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="46" t="inlineStr">
+        <is>
+          <t>P1-36</t>
+        </is>
+      </c>
+      <c r="B38" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C38" s="46" t="inlineStr">
+        <is>
+          <t>Tang, Wang, Pan &amp; Li (2023). Energy Economics 126, 107008</t>
+        </is>
+      </c>
+      <c r="D38" s="46" t="inlineStr">
+        <is>
+          <t>Env.-Disclosure-Qualität</t>
+        </is>
+      </c>
+      <c r="E38" s="46" t="inlineStr">
+        <is>
+          <t>Green-Bond-Spread</t>
+        </is>
+      </c>
+      <c r="F38" s="46" t="inlineStr">
+        <is>
+          <t>2016-20 China</t>
+        </is>
+      </c>
+      <c r="G38" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H38" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I38" s="46" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="46" t="inlineStr">
+        <is>
+          <t>P1-37</t>
+        </is>
+      </c>
+      <c r="B39" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C39" s="46" t="inlineStr">
+        <is>
+          <t>Liu, Chen &amp; Deng (2023). PBFJ 80, 102055</t>
+        </is>
+      </c>
+      <c r="D39" s="46" t="inlineStr">
+        <is>
+          <t>Staatl. Umwelt-Ratings</t>
+        </is>
+      </c>
+      <c r="E39" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F39" s="46" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="G39" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H39" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I39" s="46" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="46" t="inlineStr">
+        <is>
+          <t>P1-38</t>
+        </is>
+      </c>
+      <c r="B40" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C40" s="46" t="inlineStr">
+        <is>
+          <t>Zhang, Liu &amp; Wang (2023). ESPR 30(34), 82696-82716</t>
+        </is>
+      </c>
+      <c r="D40" s="46" t="inlineStr">
+        <is>
+          <t>Carbon</t>
+        </is>
+      </c>
+      <c r="E40" s="46" t="inlineStr">
+        <is>
+          <t>CDS</t>
+        </is>
+      </c>
+      <c r="F40" s="46" t="inlineStr">
+        <is>
+          <t>2007-20 USA</t>
+        </is>
+      </c>
+      <c r="G40" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H40" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I40" s="46" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="46" t="inlineStr">
+        <is>
+          <t>P1-39</t>
+        </is>
+      </c>
+      <c r="B41" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C41" s="46" t="inlineStr">
+        <is>
+          <t>Feng &amp; Wareewanich (2024). JIPD 8(10), 7997</t>
+        </is>
+      </c>
+      <c r="D41" s="46" t="inlineStr">
+        <is>
+          <t>Carbon-Intensität</t>
+        </is>
+      </c>
+      <c r="E41" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F41" s="46" t="inlineStr">
+        <is>
+          <t>2015-22 S&amp;P500</t>
+        </is>
+      </c>
+      <c r="G41" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H41" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I41" s="46" t="inlineStr">
+        <is>
+          <t>Venue-Tier im Screening</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="46" t="inlineStr">
+        <is>
+          <t>P1-40</t>
+        </is>
+      </c>
+      <c r="B42" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C42" s="46" t="inlineStr">
+        <is>
+          <t>Kozak (2021). Energies 14(24), 8361</t>
+        </is>
+      </c>
+      <c r="D42" s="46" t="inlineStr">
+        <is>
+          <t>CO2-Intensität</t>
+        </is>
+      </c>
+      <c r="E42" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F42" s="46" t="inlineStr">
+        <is>
+          <t>2018-21 EU</t>
+        </is>
+      </c>
+      <c r="G42" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H42" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I42" s="46" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="46" t="inlineStr">
+        <is>
+          <t>P1-41</t>
+        </is>
+      </c>
+      <c r="B43" s="46" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C43" s="46" t="inlineStr">
+        <is>
+          <t>Ratajczak &amp; Mikołajewicz (2021). EBR 7(2), 74-96</t>
+        </is>
+      </c>
+      <c r="D43" s="46" t="inlineStr">
+        <is>
+          <t>E-Dimension (separat)</t>
+        </is>
+      </c>
+      <c r="E43" s="46" t="inlineStr">
+        <is>
+          <t>CoD kurz/lang</t>
+        </is>
+      </c>
+      <c r="F43" s="46" t="inlineStr"/>
+      <c r="G43" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H43" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I43" s="46" t="inlineStr">
+        <is>
+          <t>E-Pillar-Separierung am PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="46" t="inlineStr">
+        <is>
+          <t>W-01</t>
+        </is>
+      </c>
+      <c r="B44" s="46" t="inlineStr">
+        <is>
+          <t>P1-WP</t>
+        </is>
+      </c>
+      <c r="C44" s="46" t="inlineStr">
+        <is>
+          <t>Owolabi et al. (2025). SSRN 5205230</t>
+        </is>
+      </c>
+      <c r="D44" s="46" t="inlineStr">
+        <is>
+          <t>Carbon</t>
+        </is>
+      </c>
+      <c r="E44" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F44" s="46" t="inlineStr">
+        <is>
+          <t>2010-20, 8 Asian EM</t>
+        </is>
+      </c>
+      <c r="G44" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H44" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I44" s="46" t="inlineStr">
+        <is>
+          <t>Sequel: Paris × Accounting Conservatism · Ch.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="46" t="inlineStr">
+        <is>
+          <t>W-02</t>
+        </is>
+      </c>
+      <c r="B45" s="46" t="inlineStr">
+        <is>
+          <t>P1-WP</t>
+        </is>
+      </c>
+      <c r="C45" s="46" t="inlineStr">
+        <is>
+          <t>Zhou, Williams &amp; Shrimali (2024, rev. 2025). SSRN 4957523</t>
+        </is>
+      </c>
+      <c r="D45" s="46" t="inlineStr">
+        <is>
+          <t>Netto-Null-Ziele/Disclosure</t>
+        </is>
+      </c>
+      <c r="E45" s="46" t="inlineStr">
+        <is>
+          <t>Synd. Loans</t>
+        </is>
+      </c>
+      <c r="F45" s="46" t="inlineStr">
+        <is>
+          <t>Energie/Utilities global</t>
+        </is>
+      </c>
+      <c r="G45" s="46" t="inlineStr">
+        <is>
+          <t>G,P1,P2</t>
+        </is>
+      </c>
+      <c r="H45" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I45" s="46" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="46" t="inlineStr">
+        <is>
+          <t>W-03</t>
+        </is>
+      </c>
+      <c r="B46" s="46" t="inlineStr">
+        <is>
+          <t>P1-WP</t>
+        </is>
+      </c>
+      <c r="C46" s="46" t="inlineStr">
+        <is>
+          <t>Hansen &amp; Marcet (2025). SSRN 5293084</t>
+        </is>
+      </c>
+      <c r="D46" s="46" t="inlineStr">
+        <is>
+          <t>Umwelt-Violations (EPA)</t>
+        </is>
+      </c>
+      <c r="E46" s="46" t="inlineStr">
+        <is>
+          <t>CoD + CoE</t>
+        </is>
+      </c>
+      <c r="F46" s="46" t="inlineStr">
+        <is>
+          <t>2000-19 USA</t>
+        </is>
+      </c>
+      <c r="G46" s="46" t="inlineStr">
+        <is>
+          <t>C,G,P2</t>
+        </is>
+      </c>
+      <c r="H46" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I46" s="46" t="inlineStr">
+        <is>
+          <t>ersetzt SSRN 5030796/EFMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="46" t="inlineStr">
+        <is>
+          <t>W-04</t>
+        </is>
+      </c>
+      <c r="B47" s="46" t="inlineStr">
+        <is>
+          <t>P1-WP</t>
+        </is>
+      </c>
+      <c r="C47" s="46" t="inlineStr">
+        <is>
+          <t>Dong, Hengge, Valencia &amp; Varghese (2025). IMF WP 2025/250</t>
+        </is>
+      </c>
+      <c r="D47" s="46" t="inlineStr">
+        <is>
+          <t>Carbon + Commitments</t>
+        </is>
+      </c>
+      <c r="E47" s="46" t="inlineStr">
+        <is>
+          <t>Loan Pricing</t>
+        </is>
+      </c>
+      <c r="F47" s="46" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G47" s="46" t="inlineStr">
+        <is>
+          <t>G,P2,A</t>
+        </is>
+      </c>
+      <c r="H47" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I47" s="46" t="inlineStr">
+        <is>
+          <t>Autoren 2:1 bestätigt (P2-Garble)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="46" t="inlineStr">
+        <is>
+          <t>W-05</t>
+        </is>
+      </c>
+      <c r="B48" s="46" t="inlineStr">
+        <is>
+          <t>P1-WP</t>
+        </is>
+      </c>
+      <c r="C48" s="46" t="inlineStr">
+        <is>
+          <t>Boermans, Bun &amp; van der Straten (2024). DNB WP 797 / SSRN 4696871</t>
+        </is>
+      </c>
+      <c r="D48" s="46" t="inlineStr">
+        <is>
+          <t>Scope-1+2-Intensität + Patente</t>
+        </is>
+      </c>
+      <c r="E48" s="46" t="inlineStr">
+        <is>
+          <t>Bond Spreads</t>
+        </is>
+      </c>
+      <c r="F48" s="46" t="inlineStr">
+        <is>
+          <t>2016-21</t>
+        </is>
+      </c>
+      <c r="G48" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H48" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I48" s="46" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="46" t="inlineStr">
+        <is>
+          <t>W-06</t>
+        </is>
+      </c>
+      <c r="B49" s="46" t="inlineStr">
+        <is>
+          <t>P1-WP</t>
+        </is>
+      </c>
+      <c r="C49" s="46" t="inlineStr">
+        <is>
+          <t>Altavilla, Boucinha, Pagano &amp; Polo (2024). ECB WP 2969</t>
+        </is>
+      </c>
+      <c r="D49" s="46" t="inlineStr">
+        <is>
+          <t>Emissionen + Commitments</t>
+        </is>
+      </c>
+      <c r="E49" s="46" t="inlineStr">
+        <is>
+          <t>Loan Rates</t>
+        </is>
+      </c>
+      <c r="F49" s="46" t="inlineStr">
+        <is>
+          <t>Euroraum</t>
+        </is>
+      </c>
+      <c r="G49" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H49" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I49" s="46" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="46" t="inlineStr">
+        <is>
+          <t>W-07</t>
+        </is>
+      </c>
+      <c r="B50" s="46" t="inlineStr">
+        <is>
+          <t>P1-WP</t>
+        </is>
+      </c>
+      <c r="C50" s="46" t="inlineStr">
+        <is>
+          <t>Panjwani, Melin &amp; Mercereau (2022). SSRN 4205875</t>
+        </is>
+      </c>
+      <c r="D50" s="46" t="inlineStr">
+        <is>
+          <t>Scope-3-Emissionen/Disclosure</t>
+        </is>
+      </c>
+      <c r="E50" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F50" s="46" t="inlineStr"/>
+      <c r="G50" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H50" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I50" s="46" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="46" t="inlineStr">
+        <is>
+          <t>W-08</t>
+        </is>
+      </c>
+      <c r="B51" s="46" t="inlineStr">
+        <is>
+          <t>P1-WP</t>
+        </is>
+      </c>
+      <c r="C51" s="46" t="inlineStr">
+        <is>
+          <t>Li &amp; Qiu (2025). SSRN 5078106</t>
+        </is>
+      </c>
+      <c r="D51" s="46" t="inlineStr">
+        <is>
+          <t>Industrielle Emissionen</t>
+        </is>
+      </c>
+      <c r="E51" s="46" t="inlineStr">
+        <is>
+          <t>Credit Spreads</t>
+        </is>
+      </c>
+      <c r="F51" s="46" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G51" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H51" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I51" s="46" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="46" t="inlineStr">
+        <is>
+          <t>W-09</t>
+        </is>
+      </c>
+      <c r="B52" s="46" t="inlineStr">
+        <is>
+          <t>P1-WP</t>
+        </is>
+      </c>
+      <c r="C52" s="46" t="inlineStr">
+        <is>
+          <t>Kacperczyk &amp; Peydró. SSRN 3915486</t>
+        </is>
+      </c>
+      <c r="D52" s="46" t="inlineStr">
+        <is>
+          <t>Carbon</t>
+        </is>
+      </c>
+      <c r="E52" s="46" t="inlineStr">
+        <is>
+          <t>Bank Lending</t>
+        </is>
+      </c>
+      <c r="F52" s="46" t="inlineStr"/>
+      <c r="G52" s="46" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H52" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I52" s="46" t="inlineStr">
+        <is>
+          <t>Publikations-Recheck vor Freeze</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="46" t="inlineStr">
+        <is>
+          <t>W-10</t>
+        </is>
+      </c>
+      <c r="B53" s="46" t="inlineStr">
+        <is>
+          <t>P1-WP</t>
+        </is>
+      </c>
+      <c r="C53" s="46" t="inlineStr">
+        <is>
+          <t>Trinh, Trinh, Nguyen &amp; Phung (2024). St Andrews WP 24-019</t>
+        </is>
+      </c>
+      <c r="D53" s="46" t="inlineStr">
+        <is>
+          <t>Eco-Innovation</t>
+        </is>
+      </c>
+      <c r="E53" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F53" s="46" t="inlineStr">
+        <is>
+          <t>G7</t>
+        </is>
+      </c>
+      <c r="G53" s="46" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="H53" s="46" t="inlineStr">
+        <is>
+          <t>Download</t>
+        </is>
+      </c>
+      <c r="I53" s="46" t="inlineStr">
+        <is>
+          <t>sauberer Narrow-E-Fit</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="46" t="inlineStr">
+        <is>
+          <t>B-01</t>
+        </is>
+      </c>
+      <c r="B54" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C54" s="46" t="inlineStr">
+        <is>
+          <t>Ren, Li, Duan &amp; Urquhart (2025). JIMF 153, 103294</t>
+        </is>
+      </c>
+      <c r="D54" s="46" t="inlineStr">
+        <is>
+          <t>Carbon Risk</t>
+        </is>
+      </c>
+      <c r="E54" s="46" t="inlineStr">
+        <is>
+          <t>primär Leverage/Debt-Volumen, CoD sekundär</t>
+        </is>
+      </c>
+      <c r="F54" s="46" t="inlineStr">
+        <is>
+          <t>2010-20, 24 Länder</t>
+        </is>
+      </c>
+      <c r="G54" s="46" t="inlineStr">
+        <is>
+          <t>C,G,P2,A</t>
+        </is>
+      </c>
+      <c r="H54" s="46" t="inlineStr">
+        <is>
+          <t>Outcome-Check am PDF</t>
+        </is>
+      </c>
+      <c r="I54" s="46" t="inlineStr">
+        <is>
+          <t>3 Engines uneins über DV</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="46" t="inlineStr">
+        <is>
+          <t>B-02</t>
+        </is>
+      </c>
+      <c r="B55" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C55" s="46" t="inlineStr">
+        <is>
+          <t>Boccaletti, Gucciardi &amp; Ruberti (2026). RIBAF 83, 103267</t>
+        </is>
+      </c>
+      <c r="D55" s="46" t="inlineStr">
+        <is>
+          <t>EU-Taxonomie + ESG-Signale</t>
+        </is>
+      </c>
+      <c r="E55" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F55" s="46" t="inlineStr">
+        <is>
+          <t>2007-22 Europa</t>
+        </is>
+      </c>
+      <c r="G55" s="46" t="inlineStr">
+        <is>
+          <t>P1,P2,A</t>
+        </is>
+      </c>
+      <c r="H55" s="46" t="inlineStr">
+        <is>
+          <t>Konstrukt-Check</t>
+        </is>
+      </c>
+      <c r="I55" s="46" t="inlineStr">
+        <is>
+          <t>Taxonomie-Klassifikation vs. Firmenverhalten</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="46" t="inlineStr">
+        <is>
+          <t>B-03</t>
+        </is>
+      </c>
+      <c r="B56" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C56" s="46" t="inlineStr">
+        <is>
+          <t>Hoepner, Schiemann, Schneider &amp; Tietmeyer (2025). IRFA 106, 104478</t>
+        </is>
+      </c>
+      <c r="D56" s="46" t="inlineStr">
+        <is>
+          <t>ESG-Disclosure (E-Pillar enthalten)</t>
+        </is>
+      </c>
+      <c r="E56" s="46" t="inlineStr">
+        <is>
+          <t>Bond Spreads</t>
+        </is>
+      </c>
+      <c r="F56" s="46" t="inlineStr">
+        <is>
+          <t>2009-17 USA</t>
+        </is>
+      </c>
+      <c r="G56" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H56" s="46" t="inlineStr">
+        <is>
+          <t>E-Pillar-Separat-Check</t>
+        </is>
+      </c>
+      <c r="I56" s="46" t="inlineStr">
+        <is>
+          <t>≠ Korpus-Hoepner 2016</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="46" t="inlineStr">
+        <is>
+          <t>B-04</t>
+        </is>
+      </c>
+      <c r="B57" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C57" s="46" t="inlineStr">
+        <is>
+          <t>Wang, Zhang &amp; Zhou (2022). IJERPH 19(6), 3584</t>
+        </is>
+      </c>
+      <c r="D57" s="46" t="inlineStr">
+        <is>
+          <t>Luftverschmutzung + Violation-RISK</t>
+        </is>
+      </c>
+      <c r="E57" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F57" s="46" t="inlineStr">
+        <is>
+          <t>2014-18 China</t>
+        </is>
+      </c>
+      <c r="G57" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H57" s="46" t="inlineStr">
+        <is>
+          <t>Konstrukt-Check</t>
+        </is>
+      </c>
+      <c r="I57" s="46" t="inlineStr">
+        <is>
+          <t>Violation-Risk = Exposure?</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="46" t="inlineStr">
+        <is>
+          <t>B-05</t>
+        </is>
+      </c>
+      <c r="B58" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C58" s="46" t="inlineStr">
+        <is>
+          <t>Beyer &amp; Nobile (2025). ECB WP 3087</t>
+        </is>
+      </c>
+      <c r="D58" s="46" t="inlineStr">
+        <is>
+          <t>Klima-LITIGATION-Risk × Env-Performance</t>
+        </is>
+      </c>
+      <c r="E58" s="46" t="inlineStr">
+        <is>
+          <t>Synd. Loans</t>
+        </is>
+      </c>
+      <c r="F58" s="46" t="inlineStr">
+        <is>
+          <t>2006-21 global</t>
+        </is>
+      </c>
+      <c r="G58" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H58" s="46" t="inlineStr">
+        <is>
+          <t>Konstrukt-Check</t>
+        </is>
+      </c>
+      <c r="I58" s="46" t="inlineStr">
+        <is>
+          <t>Env-Perf-Hauptterm ggf. extrahierbar</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="46" t="inlineStr">
+        <is>
+          <t>B-06</t>
+        </is>
+      </c>
+      <c r="B59" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C59" s="46" t="inlineStr">
+        <is>
+          <t>Dong, Liu, Wang &amp; Zhang (2024). SSRN 4761221</t>
+        </is>
+      </c>
+      <c r="D59" s="46" t="inlineStr">
+        <is>
+          <t>Transition Risk / Carbon Gap</t>
+        </is>
+      </c>
+      <c r="E59" s="46" t="inlineStr">
+        <is>
+          <t>Bond Spreads</t>
+        </is>
+      </c>
+      <c r="F59" s="46" t="inlineStr">
+        <is>
+          <t>2008-18 China</t>
+        </is>
+      </c>
+      <c r="G59" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H59" s="46" t="inlineStr">
+        <is>
+          <t>Konstrukt-Check</t>
+        </is>
+      </c>
+      <c r="I59" s="46" t="inlineStr">
+        <is>
+          <t>Carbon Gap = Soll-Ist-Verhalten?</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="46" t="inlineStr">
+        <is>
+          <t>B-07</t>
+        </is>
+      </c>
+      <c r="B60" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C60" s="46" t="inlineStr">
+        <is>
+          <t>N.N. (2025). SSRN 5448774 [Guedhami et al. lt. ChatGPT]</t>
+        </is>
+      </c>
+      <c r="D60" s="46" t="inlineStr">
+        <is>
+          <t>Umwelt-Strafen (administrativ)</t>
+        </is>
+      </c>
+      <c r="E60" s="46" t="inlineStr">
+        <is>
+          <t>Bond Pricing</t>
+        </is>
+      </c>
+      <c r="F60" s="46" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="G60" s="46" t="inlineStr">
+        <is>
+          <t>G,P1,P2</t>
+        </is>
+      </c>
+      <c r="H60" s="46" t="inlineStr">
+        <is>
+          <t>Autoren verifizieren, dann Download</t>
+        </is>
+      </c>
+      <c r="I60" s="46" t="inlineStr">
+        <is>
+          <t>Merge zweier Sweep-Einträge</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="46" t="inlineStr">
+        <is>
+          <t>B-08</t>
+        </is>
+      </c>
+      <c r="B61" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C61" s="46" t="inlineStr">
+        <is>
+          <t>Kempa &amp; Moslener (2025). SSRN 4274711</t>
+        </is>
+      </c>
+      <c r="D61" s="46" t="inlineStr">
+        <is>
+          <t>Emissionen × Policy-Stringenz</t>
+        </is>
+      </c>
+      <c r="E61" s="46" t="inlineStr">
+        <is>
+          <t>Spreads/Ratings</t>
+        </is>
+      </c>
+      <c r="F61" s="46" t="inlineStr">
+        <is>
+          <t>EU/global</t>
+        </is>
+      </c>
+      <c r="G61" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H61" s="46" t="inlineStr">
+        <is>
+          <t>Konstrukt-Check</t>
+        </is>
+      </c>
+      <c r="I61" s="46" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="46" t="inlineStr">
+        <is>
+          <t>B-09</t>
+        </is>
+      </c>
+      <c r="B62" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C62" s="46" t="inlineStr">
+        <is>
+          <t>Arian &amp; Sands (2024)</t>
+        </is>
+      </c>
+      <c r="D62" s="46" t="inlineStr">
+        <is>
+          <t>Carbon</t>
+        </is>
+      </c>
+      <c r="E62" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F62" s="46" t="inlineStr"/>
+      <c r="G62" s="46" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H62" s="46" t="inlineStr">
+        <is>
+          <t>Record nachziehen</t>
+        </is>
+      </c>
+      <c r="I62" s="46" t="inlineStr">
+        <is>
+          <t>nur Serien-Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="46" t="inlineStr">
+        <is>
+          <t>B-10</t>
+        </is>
+      </c>
+      <c r="B63" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C63" s="46" t="inlineStr">
+        <is>
+          <t>Siwela &amp; Ngwakwe (2024)</t>
+        </is>
+      </c>
+      <c r="D63" s="46" t="inlineStr">
+        <is>
+          <t>Env.</t>
+        </is>
+      </c>
+      <c r="E63" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F63" s="46" t="inlineStr"/>
+      <c r="G63" s="46" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H63" s="46" t="inlineStr">
+        <is>
+          <t>Record nachziehen</t>
+        </is>
+      </c>
+      <c r="I63" s="46" t="inlineStr">
+        <is>
+          <t>nur Serien-Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="46" t="inlineStr">
+        <is>
+          <t>B-11</t>
+        </is>
+      </c>
+      <c r="B64" s="46" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C64" s="46" t="inlineStr">
+        <is>
+          <t>Ballester, González-Urteaga &amp; Martínez (2025). IREF 99, 104057</t>
+        </is>
+      </c>
+      <c r="D64" s="46" t="inlineStr">
+        <is>
+          <t>Green-Bond-Emission</t>
+        </is>
+      </c>
+      <c r="E64" s="46" t="inlineStr">
+        <is>
+          <t>Credit Risk</t>
+        </is>
+      </c>
+      <c r="F64" s="46" t="inlineStr"/>
+      <c r="G64" s="46" t="inlineStr">
+        <is>
+          <t>C,G</t>
+        </is>
+      </c>
+      <c r="H64" s="46" t="inlineStr">
+        <is>
+          <t>Konstrukt+Outcome-Check</t>
+        </is>
+      </c>
+      <c r="I64" s="46" t="inlineStr">
+        <is>
+          <t>Emittenten-Verhalten vs. Instrument</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="46" t="inlineStr">
+        <is>
+          <t>D-01</t>
+        </is>
+      </c>
+      <c r="B65" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C65" s="46" t="inlineStr">
+        <is>
+          <t>Trinh, Trinh, Li &amp; Vo (2024). JFS 74, 101315</t>
+        </is>
+      </c>
+      <c r="D65" s="46" t="inlineStr">
+        <is>
+          <t>Klima-Exposure (textbasiert)</t>
+        </is>
+      </c>
+      <c r="E65" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F65" s="46" t="inlineStr">
+        <is>
+          <t>2001-20 EU</t>
+        </is>
+      </c>
+      <c r="G65" s="46" t="inlineStr">
+        <is>
+          <t>C,G,P2,A</t>
+        </is>
+      </c>
+      <c r="H65" s="46" t="inlineStr">
+        <is>
+          <t>raus (F32v2)</t>
+        </is>
+      </c>
+      <c r="I65" s="46" t="inlineStr">
+        <is>
+          <t>nur re-checken falls Emissions-Submass separat</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="46" t="inlineStr">
+        <is>
+          <t>D-02</t>
+        </is>
+      </c>
+      <c r="B66" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C66" s="46" t="inlineStr">
+        <is>
+          <t>Demetriades &amp; Politsidis (2025). JFS 76, 101349</t>
+        </is>
+      </c>
+      <c r="D66" s="46" t="inlineStr">
+        <is>
+          <t>Fossil-Branchenstatus</t>
+        </is>
+      </c>
+      <c r="E66" s="46" t="inlineStr">
+        <is>
+          <t>Loan Spreads</t>
+        </is>
+      </c>
+      <c r="F66" s="46" t="inlineStr">
+        <is>
+          <t>2001-21</t>
+        </is>
+      </c>
+      <c r="G66" s="46" t="inlineStr">
+        <is>
+          <t>C,G,P2,A</t>
+        </is>
+      </c>
+      <c r="H66" s="46" t="inlineStr">
+        <is>
+          <t>raus (F32v2)</t>
+        </is>
+      </c>
+      <c r="I66" s="46" t="inlineStr">
+        <is>
+          <t>Ch.2-Kontext</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="46" t="inlineStr">
+        <is>
+          <t>D-03</t>
+        </is>
+      </c>
+      <c r="B67" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C67" s="46" t="inlineStr">
+        <is>
+          <t>Lu, Zeng, Huang &amp; Wu (2025). JIMF 153</t>
+        </is>
+      </c>
+      <c r="D67" s="46" t="inlineStr">
+        <is>
+          <t>Mgmt-Klimarisiko-Wahrnehmung</t>
+        </is>
+      </c>
+      <c r="E67" s="46" t="inlineStr">
+        <is>
+          <t>Bond Spreads</t>
+        </is>
+      </c>
+      <c r="F67" s="46" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="G67" s="46" t="inlineStr">
+        <is>
+          <t>C,A</t>
+        </is>
+      </c>
+      <c r="H67" s="46" t="inlineStr">
+        <is>
+          <t>raus (F32v2)</t>
+        </is>
+      </c>
+      <c r="I67" s="46" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="46" t="inlineStr">
+        <is>
+          <t>D-04</t>
+        </is>
+      </c>
+      <c r="B68" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C68" s="46" t="inlineStr">
+        <is>
+          <t>Cang &amp; Li (2024). FRL 67, 105741</t>
+        </is>
+      </c>
+      <c r="D68" s="46" t="inlineStr">
+        <is>
+          <t>Klimarisiko-Indikator</t>
+        </is>
+      </c>
+      <c r="E68" s="46" t="inlineStr">
+        <is>
+          <t>Bond Spreads</t>
+        </is>
+      </c>
+      <c r="F68" s="46" t="inlineStr">
+        <is>
+          <t>2007-22 China</t>
+        </is>
+      </c>
+      <c r="G68" s="46" t="inlineStr">
+        <is>
+          <t>C,A</t>
+        </is>
+      </c>
+      <c r="H68" s="46" t="inlineStr">
+        <is>
+          <t>raus (F32v2)</t>
+        </is>
+      </c>
+      <c r="I68" s="46" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="46" t="inlineStr">
+        <is>
+          <t>D-05</t>
+        </is>
+      </c>
+      <c r="B69" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C69" s="46" t="inlineStr">
+        <is>
+          <t>He, Ren, Wang &amp; Lei (2025). JIMF 154, 103297</t>
+        </is>
+      </c>
+      <c r="D69" s="46" t="inlineStr">
+        <is>
+          <t>Physisches Klimarisiko</t>
+        </is>
+      </c>
+      <c r="E69" s="46" t="inlineStr">
+        <is>
+          <t>Bond Spreads</t>
+        </is>
+      </c>
+      <c r="F69" s="46" t="inlineStr">
+        <is>
+          <t>2008-23 China</t>
+        </is>
+      </c>
+      <c r="G69" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H69" s="46" t="inlineStr">
+        <is>
+          <t>raus (F32v2)</t>
+        </is>
+      </c>
+      <c r="I69" s="46" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="46" t="inlineStr">
+        <is>
+          <t>D-06</t>
+        </is>
+      </c>
+      <c r="B70" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C70" s="46" t="inlineStr">
+        <is>
+          <t>Zhou, Caldecott, Shrimali &amp; Zhang (2025). EnEco 144, 108323</t>
+        </is>
+      </c>
+      <c r="D70" s="46" t="inlineStr">
+        <is>
+          <t>Policy-Risk/Energie-Exposure</t>
+        </is>
+      </c>
+      <c r="E70" s="46" t="inlineStr">
+        <is>
+          <t>Loan Spreads</t>
+        </is>
+      </c>
+      <c r="F70" s="46" t="inlineStr">
+        <is>
+          <t>Energie</t>
+        </is>
+      </c>
+      <c r="G70" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H70" s="46" t="inlineStr">
+        <is>
+          <t>raus (F32v2)</t>
+        </is>
+      </c>
+      <c r="I70" s="46" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="46" t="inlineStr">
+        <is>
+          <t>D-07</t>
+        </is>
+      </c>
+      <c r="B71" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C71" s="46" t="inlineStr">
+        <is>
+          <t>Hu, Zhong, Cao &amp; Wang (2024). A&amp;F 64(4), 3495-3533</t>
+        </is>
+      </c>
+      <c r="D71" s="46" t="inlineStr">
+        <is>
+          <t>Luftverschmutzung (ambient)</t>
+        </is>
+      </c>
+      <c r="E71" s="46" t="inlineStr">
+        <is>
+          <t>Bond Yields</t>
+        </is>
+      </c>
+      <c r="F71" s="46" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="G71" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H71" s="46" t="inlineStr">
+        <is>
+          <t>raus (F32v2)</t>
+        </is>
+      </c>
+      <c r="I71" s="46" t="inlineStr">
+        <is>
+          <t>Stadt-Exposure ≠ Firmenverhalten</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="46" t="inlineStr">
+        <is>
+          <t>D-08</t>
+        </is>
+      </c>
+      <c r="B72" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C72" s="46" t="inlineStr">
+        <is>
+          <t>Zhai et al. (2024). SETP 44(11)</t>
+        </is>
+      </c>
+      <c r="D72" s="46" t="inlineStr">
+        <is>
+          <t>Klimapolitik-Unsicherheit</t>
+        </is>
+      </c>
+      <c r="E72" s="46" t="inlineStr">
+        <is>
+          <t>Bondkosten</t>
+        </is>
+      </c>
+      <c r="F72" s="46" t="inlineStr">
+        <is>
+          <t>2009-20 China</t>
+        </is>
+      </c>
+      <c r="G72" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H72" s="46" t="inlineStr">
+        <is>
+          <t>raus (F32v2)</t>
+        </is>
+      </c>
+      <c r="I72" s="46" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="46" t="inlineStr">
+        <is>
+          <t>D-09</t>
+        </is>
+      </c>
+      <c r="B73" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C73" s="46" t="inlineStr">
+        <is>
+          <t>Batoon &amp; Rroji (2024). Risks 12(1), 16</t>
+        </is>
+      </c>
+      <c r="D73" s="46" t="inlineStr">
+        <is>
+          <t>CDS-implizierter Carbon-Faktor</t>
+        </is>
+      </c>
+      <c r="E73" s="46" t="inlineStr">
+        <is>
+          <t>CDS</t>
+        </is>
+      </c>
+      <c r="F73" s="46" t="inlineStr">
+        <is>
+          <t>2020-23 Europa</t>
+        </is>
+      </c>
+      <c r="G73" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H73" s="46" t="inlineStr">
+        <is>
+          <t>raus (F32v2)</t>
+        </is>
+      </c>
+      <c r="I73" s="46" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="46" t="inlineStr">
+        <is>
+          <t>D-10</t>
+        </is>
+      </c>
+      <c r="B74" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C74" s="46" t="inlineStr">
+        <is>
+          <t>Blasberg, Kiesel &amp; Taschini (2024). SSRN 4257215</t>
+        </is>
+      </c>
+      <c r="D74" s="46" t="inlineStr">
+        <is>
+          <t>CDS-implizierter Faktor</t>
+        </is>
+      </c>
+      <c r="E74" s="46" t="inlineStr">
+        <is>
+          <t>CDS</t>
+        </is>
+      </c>
+      <c r="F74" s="46" t="inlineStr">
+        <is>
+          <t>EU/NA</t>
+        </is>
+      </c>
+      <c r="G74" s="46" t="inlineStr">
+        <is>
+          <t>P1,P2,A</t>
+        </is>
+      </c>
+      <c r="H74" s="46" t="inlineStr">
+        <is>
+          <t>raus (F32v2)</t>
+        </is>
+      </c>
+      <c r="I74" s="46" t="inlineStr">
+        <is>
+          <t>CESifo-10016-Attribution strittig (vs. Barth et al.) — Ch.2-Fussnote</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="46" t="inlineStr">
+        <is>
+          <t>D-11</t>
+        </is>
+      </c>
+      <c r="B75" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C75" s="46" t="inlineStr">
+        <is>
+          <t>Javadi &amp; Masum (2021). JCF 69, 102019</t>
+        </is>
+      </c>
+      <c r="D75" s="46" t="inlineStr">
+        <is>
+          <t>Physisches Klimarisiko</t>
+        </is>
+      </c>
+      <c r="E75" s="46" t="inlineStr">
+        <is>
+          <t>Bank Loans</t>
+        </is>
+      </c>
+      <c r="F75" s="46" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="G75" s="46" t="inlineStr">
+        <is>
+          <t>P2-Konflation</t>
+        </is>
+      </c>
+      <c r="H75" s="46" t="inlineStr">
+        <is>
+          <t>raus (F32v2)</t>
+        </is>
+      </c>
+      <c r="I75" s="46" t="inlineStr">
+        <is>
+          <t>von Duong-Eintrag getrennt</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="46" t="inlineStr">
+        <is>
+          <t>D-12</t>
+        </is>
+      </c>
+      <c r="B76" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C76" s="46" t="inlineStr">
+        <is>
+          <t>Hrazdil et al. (2024) · Ren/Derouiche (2024) · Ren/Boubaker (2023) · Jiao (2025)</t>
+        </is>
+      </c>
+      <c r="D76" s="46" t="inlineStr">
+        <is>
+          <t>Klima-Reputation/ETS-/Event-Exposure</t>
+        </is>
+      </c>
+      <c r="E76" s="46" t="inlineStr">
+        <is>
+          <t>div.</t>
+        </is>
+      </c>
+      <c r="F76" s="46" t="inlineStr"/>
+      <c r="G76" s="46" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H76" s="46" t="inlineStr">
+        <is>
+          <t>raus (F32v2)</t>
+        </is>
+      </c>
+      <c r="I76" s="46" t="inlineStr">
+        <is>
+          <t>Sammelzeile · Ch.2-Kontext</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="46" t="inlineStr">
+        <is>
+          <t>D-13</t>
+        </is>
+      </c>
+      <c r="B77" s="46" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C77" s="46" t="inlineStr">
+        <is>
+          <t>Tan, Chan &amp; Chen (2022). BSE 31(1), 464-482</t>
+        </is>
+      </c>
+      <c r="D77" s="46" t="inlineStr">
+        <is>
+          <t>Luftverschmutzung (PM2.5, ambient)</t>
+        </is>
+      </c>
+      <c r="E77" s="46" t="inlineStr">
+        <is>
+          <t>Bond Spreads</t>
+        </is>
+      </c>
+      <c r="F77" s="46" t="inlineStr">
+        <is>
+          <t>2013-18 China</t>
+        </is>
+      </c>
+      <c r="G77" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H77" s="46" t="inlineStr">
+        <is>
+          <t>raus (F32v2) + Korpus-Dedup</t>
+        </is>
+      </c>
+      <c r="I77" s="46" t="inlineStr">
+        <is>
+          <t>ggf. VoR von Korpus-Tan 2021 — Spalte-L-Check</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="46" t="inlineStr">
+        <is>
+          <t>E-01</t>
+        </is>
+      </c>
+      <c r="B78" s="46" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C78" s="46" t="inlineStr">
+        <is>
+          <t>Sze et al. (2021). SSRN 3995764</t>
+        </is>
+      </c>
+      <c r="D78" s="46" t="inlineStr">
+        <is>
+          <t>ESG-E</t>
+        </is>
+      </c>
+      <c r="E78" s="46" t="inlineStr">
+        <is>
+          <t>Bonds EMEAP</t>
+        </is>
+      </c>
+      <c r="F78" s="46" t="inlineStr"/>
+      <c r="G78" s="46" t="inlineStr">
+        <is>
+          <t>P2,A</t>
+        </is>
+      </c>
+      <c r="H78" s="46" t="inlineStr">
+        <is>
+          <t>— (Korpus)</t>
+        </is>
+      </c>
+      <c r="I78" s="46" t="inlineStr">
+        <is>
+          <t>P2 hatte Ho&amp;Wong-Fragment hierauf fehlgemappt</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="46" t="inlineStr">
+        <is>
+          <t>E-02</t>
+        </is>
+      </c>
+      <c r="B79" s="46" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C79" s="46" t="inlineStr">
+        <is>
+          <t>Okimoto &amp; Takaoka (2024). IRFA 91, 103052</t>
+        </is>
+      </c>
+      <c r="D79" s="46" t="inlineStr">
+        <is>
+          <t>ESG/E</t>
+        </is>
+      </c>
+      <c r="E79" s="46" t="inlineStr">
+        <is>
+          <t>Spreads Japan</t>
+        </is>
+      </c>
+      <c r="F79" s="46" t="inlineStr"/>
+      <c r="G79" s="46" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H79" s="46" t="inlineStr">
+        <is>
+          <t>— (Korpus-VoR)</t>
+        </is>
+      </c>
+      <c r="I79" s="46" t="inlineStr">
+        <is>
+          <t>Art.-Nr. 103052 → Spalte L ergänzen</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="46" t="inlineStr">
+        <is>
+          <t>E-03</t>
+        </is>
+      </c>
+      <c r="B80" s="46" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C80" s="46" t="inlineStr">
+        <is>
+          <t>Palea &amp; Drogo (2020) · Maaloul &amp; Wegener (2021) · Zhu &amp; Zhao (2022) · Jung et al. (2016)</t>
+        </is>
+      </c>
+      <c r="D80" s="46" t="inlineStr">
+        <is>
+          <t>Carbon/Env</t>
+        </is>
+      </c>
+      <c r="E80" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F80" s="46" t="inlineStr"/>
+      <c r="G80" s="46" t="inlineStr">
+        <is>
+          <t>div.</t>
+        </is>
+      </c>
+      <c r="H80" s="46" t="inlineStr">
+        <is>
+          <t>— (Korpus)</t>
+        </is>
+      </c>
+      <c r="I80" s="46" t="inlineStr">
+        <is>
+          <t>Gate-Belege</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="46" t="inlineStr">
+        <is>
+          <t>E-04</t>
+        </is>
+      </c>
+      <c r="B81" s="46" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="C81" s="46" t="inlineStr">
+        <is>
+          <t>Ding et al. (2023). IRFA 86</t>
+        </is>
+      </c>
+      <c r="D81" s="46" t="inlineStr">
+        <is>
+          <t>Env.</t>
+        </is>
+      </c>
+      <c r="E81" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F81" s="46" t="inlineStr"/>
+      <c r="G81" s="46" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="H81" s="46" t="inlineStr">
+        <is>
+          <t>Pflicht-Dedup</t>
+        </is>
+      </c>
+      <c r="I81" s="46" t="inlineStr">
+        <is>
+          <t>vs. Korpus-Ding 2022 (mutmasslich VoR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="46" t="inlineStr">
+        <is>
+          <t>F28-01</t>
+        </is>
+      </c>
+      <c r="B82" s="46" t="inlineStr">
+        <is>
+          <t>F28</t>
+        </is>
+      </c>
+      <c r="C82" s="46" t="inlineStr">
+        <is>
+          <t>Maaloul (2018). CSRM 25(6), 1407-1415</t>
+        </is>
+      </c>
+      <c r="D82" s="46" t="inlineStr">
+        <is>
+          <t>GHG</t>
+        </is>
+      </c>
+      <c r="E82" s="46" t="inlineStr">
+        <is>
+          <t>CoD Kanada</t>
+        </is>
+      </c>
+      <c r="F82" s="46" t="inlineStr">
+        <is>
+          <t>prä-Fenster</t>
+        </is>
+      </c>
+      <c r="G82" s="46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H82" s="46" t="inlineStr">
+        <is>
+          <t>Volker: Exklusionsgrund dokumentieren</t>
+        </is>
+      </c>
+      <c r="I82" s="46" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="46" t="inlineStr">
+        <is>
+          <t>F28-02</t>
+        </is>
+      </c>
+      <c r="B83" s="46" t="inlineStr">
+        <is>
+          <t>F28</t>
+        </is>
+      </c>
+      <c r="C83" s="46" t="inlineStr">
+        <is>
+          <t>Kleimeier &amp; Viehs (2016/18). SSRN 2719665</t>
+        </is>
+      </c>
+      <c r="D83" s="46" t="inlineStr">
+        <is>
+          <t>Carbon Disclosure</t>
+        </is>
+      </c>
+      <c r="E83" s="46" t="inlineStr">
+        <is>
+          <t>Loans</t>
+        </is>
+      </c>
+      <c r="F83" s="46" t="inlineStr">
+        <is>
+          <t>prä-Fenster</t>
+        </is>
+      </c>
+      <c r="G83" s="46" t="inlineStr">
+        <is>
+          <t>C,G,P2,A</t>
+        </is>
+      </c>
+      <c r="H83" s="46" t="inlineStr">
+        <is>
+          <t>Volker: Doku (konditional)</t>
+        </is>
+      </c>
+      <c r="I83" s="46" t="inlineStr">
+        <is>
+          <t>entfällt falls EL-2021-Supersession bestätigt</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="46" t="inlineStr">
+        <is>
+          <t>F28-03</t>
+        </is>
+      </c>
+      <c r="B84" s="46" t="inlineStr">
+        <is>
+          <t>F28</t>
+        </is>
+      </c>
+      <c r="C84" s="46" t="inlineStr">
+        <is>
+          <t>Caragnano, Pizzutilo, Mariani &amp; Zito (2020). IJFS 8(4), 61</t>
+        </is>
+      </c>
+      <c r="D84" s="46" t="inlineStr">
+        <is>
+          <t>Carbon/GHG</t>
+        </is>
+      </c>
+      <c r="E84" s="46" t="inlineStr">
+        <is>
+          <t>CoD Europa</t>
+        </is>
+      </c>
+      <c r="F84" s="46" t="inlineStr">
+        <is>
+          <t>prä-Fenster</t>
+        </is>
+      </c>
+      <c r="G84" s="46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H84" s="46" t="inlineStr">
+        <is>
+          <t>Volker: Exklusionsgrund dokumentieren</t>
+        </is>
+      </c>
+      <c r="I84" s="46" t="inlineStr">
+        <is>
+          <t>hochzitiert — Lücke erklären</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="46" t="inlineStr">
+        <is>
+          <t>R2-00</t>
+        </is>
+      </c>
+      <c r="B85" s="46" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="C85" s="46" t="inlineStr">
+        <is>
+          <t>ROUND-2-PREVIEW (ESG/CSR-Komposite, geparkt): Fiorillo et al. 2025 IRFA 102 · Boccaletti &amp; Gucciardi 2025 JSFI 15(3) · Cheng/He/Tang 2025 FRL 76 · Yan et al. 2025 Applied Economics 57(46) · Mathath et al. 2024 MDE 45(4) · Wong et al. 2024 IJMEF 17(1) · Shi et al. 2024 CJAR 17(4) · Prabaswara et al. 2024 IJSDP 19(11) · Gigante &amp; Manglaviti 2022 IRFA 84 · Karaman 2024 IJFE · Lian et al. 2023 IREF</t>
+        </is>
+      </c>
+      <c r="D85" s="46" t="inlineStr">
+        <is>
+          <t>ESG/CSR-Komposit</t>
+        </is>
+      </c>
+      <c r="E85" s="46" t="inlineStr">
+        <is>
+          <t>CoD</t>
+        </is>
+      </c>
+      <c r="F85" s="46" t="inlineStr">
+        <is>
+          <t>2021-26</t>
+        </is>
+      </c>
+      <c r="G85" s="46" t="inlineStr">
+        <is>
+          <t>G,A</t>
+        </is>
+      </c>
+      <c r="H85" s="46" t="inlineStr">
+        <is>
+          <t>Runde 2</t>
+        </is>
+      </c>
+      <c r="I85" s="46" t="inlineStr">
+        <is>
+          <t>Aslan-Fragment final tot (Aslan/Poppe/Posch 2021 = Default-Outcome)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6833,6 +10862,86 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>18</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Formales Suchupdate: DB-Re-Run (10 DBs + GS), identische Kriterien, Enddatum=Ausführung, zweistufiger PRISMA-Flow → Extraktion → v11 [DEC-030]</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>19</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Kandidaten-Downloads lt. Update_Scoping (P1: 41 publ. + 10 WP; B nach Checks) via WU-Zugang; Owolabi zusätzlich ins PK [F29]</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Robert</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>20</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Blind-Pilot Extraktion: 2 Bestandspaper (nicht kalibriert; Vorschlag Devalle 2017 + 1 Loan-Paper) — PDFs hochladen, Claude extrahiert blind, Diff + Konkordanzmaß [DEC-032 §9]</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Robert + Claude</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>21</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Produktions-Extraktion 51 Kandidaten (Cowork-Batch, eigenes Projekt: Codebook v1 + Prompt + Template im PK) + Volker-Verifikation 100% Statistikfelder → Staging → v11</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Robert/Claude + Volker</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>nach Pilot-PASS</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
@@ -6842,7 +10951,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7177,241 +11286,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Key Results — Headline-Zahlen je abgeschlossener Analyse (v1)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Digest-Layer (SOMA-Analog). Wird bei jedem Lauf gefuellt; verlinkt auf die Per-Lauf-Results-xls bzw. output-CSV.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Analysis</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="17" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Phase 2 — Core (T1–T3)</t>
-        </is>
-      </c>
-      <c r="B4" s="36" t="n"/>
-      <c r="C4" s="35" t="n"/>
-    </row>
-    <row r="5" ht="26" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>T1 · Hauptanalyse CER–COD (gepoolt, 3LMA-RVE)</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>output/T1_results.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="26" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>T1 · Pre/Post-Paris (Headline-Coding)</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>output/T1_results.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="26" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>T3 · Heterogenitaet (σ²_within/between, ICC, I²)</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>output/T3_results.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Phase 2 — Identifikation &amp; Robustheit (T2, T8, T5, T4)</t>
-        </is>
-      </c>
-      <c r="B8" s="36" t="n"/>
-      <c r="C8" s="35" t="n"/>
-    </row>
-    <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>T2 · Event-Coding-Vergleich (Headline-Wahl)</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>output/T2_results.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>T8 · Identifikation Bruch vs. Trend (Verdict)</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>output/T8_results.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>T5 · Publikationsbias (FAT-PET-PEESE)</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>output/T5_results.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>T4 · Robustheit (Verdict)</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>output/T4_results.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="17" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Phase 2 — Moderatoren (T6, T7)</t>
-        </is>
-      </c>
-      <c r="B13" s="36" t="n"/>
-      <c r="C13" s="35" t="n"/>
-    </row>
-    <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>T6 · Moderatoren × Paris</t>
-        </is>
-      </c>
-      <c r="B14" s="6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>output/T6_results.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>T7 · Unified Meta-Regression (Paris×Moderator)</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>output/T7_results.csv</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Codebook v1.2 rebuilt as self-contained edition
- Delta edition (34 lines) referenced v1.1 sections, but v1.1 was removed
  from the extraction project's knowledge per swap instruction -> rule text
  was unreachable at extraction time
- Full rule set now inline (83 lines): construct gate, all-models rule,
  sign two-step, closed lists, supplementary fields, Annex A
- Same filename and version pin; prompt, template, instructions unchanged
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1560,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2700,6 +2700,30 @@
       <c r="B35" t="inlineStr">
         <is>
           <t>AI-Extraktion mit Rollen-Inversion (Claude extrahiert, Volker verifiziert 100% der Statistikfelder); Codebook v1 frozen (F34a-f kodifiziert; 13/13 Kalibrier-Effekte zellengenau reproduziert); Blind-Pilot-Gate ≥95% Konkordanz vor Produktion</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DEC-033</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Option C: Vollkorpus-Re-Extraktion unter Codebook v1.1 (Cowork); neue Extraktion = kanonisch für v11; v10 = unabhängige Doppelkodierung; Exact-Match = wechselseitig verifiziert, nur Diffs+Neu-Zeilen zu Volker; Capelle-Blancard raus (unit of analysis, 66-&gt;65); Segment-Flag bleibt</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>DEC-034</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Sechs Zusatzfelder (copy-level, purpose-tagged, result-blind): x_lag, estimation_method, se_clustering, subsample_dimension/value, subsample_start/end (Effekt-Ebene), n_obs_by_year (Studien-Ebene); Codebook v1.2; Headline-Definitionen unverändert (DEC-024); Pilot-Stagings invalidiert (Batch-Uniformität)</t>
         </is>
       </c>
     </row>
@@ -10245,7 +10269,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10908,7 +10932,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Blind-Pilot Extraktion: 2 Bestandspaper (nicht kalibriert; Vorschlag Devalle 2017 + 1 Loan-Paper) — PDFs hochladen, Claude extrahiert blind, Diff + Konkordanzmaß [DEC-032 §9]</t>
+          <t>Blind-Pilot Extraktion: 2 Bestandspaper (nicht kalibriert; Vorschlag Devalle 2017 + 1 Loan-Paper) — PDFs hochladen, Claude extrahiert blind, Diff + Konkordanzmaß [DEC-032 §9] — ERGEBNIS: 4 Paper blind extrahiert; 0 Extraktor-Fehler auf Statistik-Kernfeldern; PASS. Report: docs/pilot_concordance_report.md</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -10918,7 +10942,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (PASS, 2026-07-05)</t>
         </is>
       </c>
     </row>
@@ -10928,7 +10952,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Produktions-Extraktion 51 Kandidaten (Cowork-Batch, eigenes Projekt: Codebook v1 + Prompt + Template im PK) + Volker-Verifikation 100% Statistikfelder → Staging → v11</t>
+          <t>Produktions-Extraktion VOLLKORPUS [DEC-033, Option C]: 65 Legacy-Paper + alle gescreenten Update-Kandidaten via Cowork-Batch (1 Paper/Run; staging_&lt;study&gt;.csv + log_&lt;study&gt;.md + Manifest); Maschinen-Diff vs v10; Volker adjudiziert nur Diffs + Neu-Zeilen (Exact-Match = wechselseitig verifiziert); 4 Pilot-Extraktionen wiederverwendbar (Yilmaz-Regulation per F36b nachkodieren) — UPDATE [DEC-034]: Batch läuft unter Codebook v1.2 (6 Zusatzfelder); VOR Volllauf die 4 Pilot-Stagings aus staging\ löschen (Resume-Regel!), damit alle Paper uniform v1.2 laufen</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -10938,7 +10962,47 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>nach Pilot-PASS</t>
+          <t>bereit — Batch-Start</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Erratum-/Verifikationsliste F35 a-f aus Pilot (u.a. Devalle Zeile 409: r=+0.9998 aus OR-Misprint — HIGH, vor erstem Analyselauf fixen; Atif-Regulation; Atif CER_measure; Capelle 21/20; Sovereign-Scope-Note; Breitenbefund + Segment-Dummy-Empfehlung) — Korrekturen landen in v11 via Prep + DEC — ÜBERFÜHRT in DEC-033-Adjudikation (Teil der Diff-Liste)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>in Adjudikation (DEC-033)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Capelle-Blancard: harmonization-stage exclusion dokumentieren (unit of analysis: sovereign; R2.1/F36h) — PRISMA-Note + Drop-one-Sensitivitätsnotiz; Korpus 66-&gt;65, Effekte 1306-&gt;1305 (Legacy-Basis) [DEC-033]</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Robert + Volker</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>offen</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mid-batch gate rulings: DEC-035 logged; codebook v1.3+v1.4 committed while governing
- F38: Delis stays (reserves = embedded-emissions conduct; boundary formula)
- F39a: Fard exits (country-level policy stringency; corpus 64->63, -46 effects)
- F39b: KLD climate-concern = conduct (v1.4); Bauer&Hann re-run mandated,
  Chava FLAG rows resolve at adjudication
- Version-evolution defense: additive deltas + targeted re-runs
- Status: index +DEC-035; Datenagenda #24 (Fard doc); Cumming -> D
- .gitignore: work/ (local derivatives)
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1560,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2724,6 +2724,18 @@
       <c r="B37" t="inlineStr">
         <is>
           <t>Sechs Zusatzfelder (copy-level, purpose-tagged, result-blind): x_lag, estimation_method, se_clustering, subsample_dimension/value, subsample_start/end (Effekt-Ebene), n_obs_by_year (Studien-Ebene); Codebook v1.2; Headline-Definitionen unverändert (DEC-024); Pilot-Stagings invalidiert (Batch-Uniformität)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>DEC-035</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Mid-Batch-Gate-Rulings: F38 (Delis bleibt; Reserven=Conduct; Grenzformel) · F39a Fard-Exit (64-&gt;63, -46 Eff.) · F39b KLD-Concern=Conduct (v1.4; B&amp;H-Re-Run; Chava via Adjudikation) · F39c-e Adjudikation · F39f Fix; Versions-Verteidigung: additive Deltas + gezielte Re-Runs = single-rule-set-äquivalent</t>
         </is>
       </c>
     </row>
@@ -6719,7 +6731,7 @@
       </c>
       <c r="B6" s="46" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C6" s="46" t="inlineStr">
@@ -6754,7 +6766,7 @@
       </c>
       <c r="I6" s="46" t="inlineStr">
         <is>
-          <t>2x Perplexity-Blindstelle · via DOI ziehen</t>
+          <t>2x Perplexity-Blindstelle · via DOI ziehen — RE-KLASSIFIZIERT [DEC-035]: 0 qualifizierende Effekte (X=Exposure-Komposit; DV=Leverage, kein COD) -&gt; raus</t>
         </is>
       </c>
     </row>
@@ -10269,7 +10281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11001,6 +11013,26 @@
         </is>
       </c>
       <c r="D26" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Fard et al (2020): harmonization-stage exclusion dokumentieren (Länder-Policy-Stringenz = Exposure; F39a/DEC-035) — PRISMA-Note + Drop-one-Sensitivität; Legacy-Basis -46 Effekte, Korpus 64-&gt;63</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Robert + Volker</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
         <is>
           <t>offen</t>
         </is>

</xml_diff>

<commit_message>
F40 construct micro-rulings: DEC-036 logged; codebook v1.5
- Own-measure dummies, awareness-as-disclosure, Heckman-outcome equations,
  gologit thresholds, consumption-based measures: all additive, conduct-side
- No re-extractions: case papers carry included+FLAGged rows -> adjudication
- Instructions pin -> v1.5; DEC-037 reserved for adjudication + v11
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1560,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2736,6 +2736,18 @@
       <c r="B38" t="inlineStr">
         <is>
           <t>Mid-Batch-Gate-Rulings: F38 (Delis bleibt; Reserven=Conduct; Grenzformel) · F39a Fard-Exit (64-&gt;63, -46 Eff.) · F39b KLD-Concern=Conduct (v1.4; B&amp;H-Re-Run; Chava via Adjudikation) · F39c-e Adjudikation · F39f Fix; Versions-Verteidigung: additive Deltas + gezielte Re-Runs = single-rule-set-äquivalent</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>DEC-036</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>F40 a-e kodifiziert (v1.5): Eigen-Mass-Dummies, Awareness-als-Disclosure, Heckman-Outcome-Gleichungen, Gologit-Thresholds, Verbrauchsmasse — additive Mikro-Rulings; keine Re-Runs (Adjudikation löst FLAGs); DEC-037 reserviert für Adjudikation+v11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
F41 rulings: DEC-037 logged; codebook v1.6
- Koelbel stays: disclosure-channel boundary (own reporting instruments =
  conduct; call/media-derived = exposure); re-extraction mandated
- System-estimator line per Lemma precedent (external-IV out, 3SLS in);
  Mahmoudian re-run; no Lemma re-run
- CECE ratings = conduct; spread components in; stars-only ES_source label
- Maaloul source identity resolved (M&W 2022 GHG paper; lookup erratum ->
  F35); Maaloul 2018 stays out (F28, pre-window)
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1560,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2748,6 +2748,18 @@
       <c r="B39" t="inlineStr">
         <is>
           <t>F40 a-e kodifiziert (v1.5): Eigen-Mass-Dummies, Awareness-als-Disclosure, Heckman-Outcome-Gleichungen, Gologit-Thresholds, Verbrauchsmasse — additive Mikro-Rulings; keine Re-Runs (Adjudikation löst FLAGs); DEC-037 reserviert für Adjudikation+v11</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DEC-037</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>F41 a-e (v1.6): Kölbel bleibt (Disclosure-Kanal-Grenze; Re-Run) · Systemschätzer-Linie (Lemma-Präzedenz; Mahmoudian-Re-Run; kein Lemma-Re-Run) · CECE=Conduct · Spread-Komponenten rein · Stars-only-Label; Maaloul-Quellidentität geklärt (Lookup-Erratum -&gt; F35; M&amp;W-2022 = Korpusquelle; Maaloul-2018 bleibt F28/raus)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Post-batch bundle: DEC-038 logged
- F42/F44/F45/F46 rulings booked (slope in; Zhu&Zhao in with firm-weight
  boundary; Trinh=performance; Wang-e split COD/estimator; Weber exit)
- Corpus ledger corrected: 66 keys -> 61 legacy studies / 1,239 rows base
- Hui (2024) retagged to update segment; Zhou gap closed (22 rows;
  Spearman hypothesis queued for the 62->22 delta and Cubas)
- Evidence-based crosswalk (Fonseka orientation via permutation test)
- Rescreen mandate: 20 papers + K&V-2021 identity check, segment=rescreen
- Datenagenda #25 (rescreen) / #26 (Pass-2b + adjudication package)
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1560,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2760,6 +2760,18 @@
       <c r="B40" t="inlineStr">
         <is>
           <t>F41 a-e (v1.6): Kölbel bleibt (Disclosure-Kanal-Grenze; Re-Run) · Systemschätzer-Linie (Lemma-Präzedenz; Mahmoudian-Re-Run; kein Lemma-Re-Run) · CECE=Conduct · Spread-Komponenten rein · Stars-only-Label; Maaloul-Quellidentität geklärt (Lookup-Erratum -&gt; F35; M&amp;W-2022 = Korpusquelle; Maaloul-2018 bleibt F28/raus)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>DEC-038</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Post-Batch-Bündel: F42/F44/F45/F46 verbucht (Slope rein; Zhu&amp;Zhao rein mit Firm-Gewichts-Grenze; Trinh=performance; Wang-e zweigeteilt; Weber-Exit) · Ledger korrigiert 66-&gt;61 Legacy / 1239 Zeilen · Hui-&gt;update-Retag · Zhou-Gap zu (22 Zeilen; Spearman-Hypothese für 62-&gt;22) · Crosswalk evidenzbasiert · Rescreen-Mandat 20+1 (segment=rescreen; Wang-2020/K&amp;V-2018 retroaktiv)</t>
         </is>
       </c>
     </row>
@@ -10305,7 +10317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11059,6 +11071,46 @@
       <c r="D27" t="inlineStr">
         <is>
           <t>offen</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Rescreen-Tranche [DEC-038]: 20 Paper + K&amp;V-2021-Identitätscheck aus inbox_rescreen -&gt; papers -&gt; v1.6-Kickoff; 0-Zeilen-Läufe = retroaktive PRISMA-Ausschlussdoku; nicht beschaffbare als not-retrievable dokumentieren</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Robert</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>bereit</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Pass-2b + Adjudikationspaket [DEC-038]: Ursachen-Etiketten je 727 Posten; Resolutions-Vorbefüllung (Slope 48, Trinh 104, Zhu&amp;Zhao 28, prod_inno 12, Wang 28, F37d); B&amp;H-Block-Adjudikation (N-Zuordnung); Spearman-Hypothese Zhou/Cubas; Kalibrier-Delta-3; dann Volker-Gespräch (Paket + Sandra/Ofogbe + F35-Errata)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Claude -&gt; Volker</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>in Arbeit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Adjudication package v1 committed; F47a author-approved (K&V cluster)
- 6-sheet handover: 797 cause-labeled items, live-counted FLAG resolutions,
  study concordance, evidence-based crosswalk, special cases
- K&V ruling: one study cluster; 2018 WP row set canonical, EL 2021 =
  citable VoR (9/10 rows reproduced); Volker confirms in adjudication call
- Status: Datenagenda #26 delivered, #27 Volker adjudication meeting opened
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -10317,7 +10317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11100,7 +11100,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Pass-2b + Adjudikationspaket [DEC-038]: Ursachen-Etiketten je 727 Posten; Resolutions-Vorbefüllung (Slope 48, Trinh 104, Zhu&amp;Zhao 28, prod_inno 12, Wang 28, F37d); B&amp;H-Block-Adjudikation (N-Zuordnung); Spearman-Hypothese Zhou/Cubas; Kalibrier-Delta-3; dann Volker-Gespräch (Paket + Sandra/Ofogbe + F35-Errata)</t>
+          <t>Pass-2b + Adjudikationspaket [DEC-038]: Ursachen-Etiketten je 727 Posten; Resolutions-Vorbefüllung (Slope 48, Trinh 104, Zhu&amp;Zhao 28, prod_inno 12, Wang 28, F37d); B&amp;H-Block-Adjudikation (N-Zuordnung); Spearman-Hypothese Zhou/Cubas; Kalibrier-Delta-3; dann Volker-Gespräch (Paket + Sandra/Ofogbe + F35-Errata) — GELIEFERT: docs/adjudication_package_v1.xlsx (6 Sheets; 797 Posten mit Ursache-Klasse; Prefills live gezählt; K&amp;V-Ruling F47a autor-ok)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -11110,7 +11110,27 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>in Arbeit</t>
+          <t>erledigt (2026-07-07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Volker-Adjudikationsgespräch: Paket-Walkthrough in Agenda-Reihenfolge (Rahmen -&gt; Block-Entscheide [B&amp;H-N, strukturell, Versionsdrift, F37d] -&gt; Einzelprüfungen 343 -&gt; Sonderfälle [F35a, Sandra/Ofogbe, K&amp;V, Zhou/Cubas-Prüfaufträge, Spot-Checks] -&gt; Rescreen-Story); Rückläufer an Claude -&gt; DEC-039/v11</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Robert + Volker</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>offen — terminieren</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ruling layer closed: DEC-039 logged (R1-R8, K1-K4)
- Unit boundary codified: firm and below qualifies; above the firm does not
  (Eichholtz stays, 36 rows; sovereign exits unchanged)
- Two study clusters: Sandra/Ofogbe (duplicate cell counts once) and K&V
  (WP canonical + EL-unique row added, source=EL2021; 29 rows)
- Devalle sign regime: printed scale governs; row 409 corrected via z-route
- Delis price-valued variants tagged in; industry-sensitive operationalized
  (incl. new mixed label); K4 withdrawn on file evidence
- cluster_id mechanic reserved for v11 assembly; DEC-040 reserved
- Package: new sheet Rulings_Verdikte; dossier carries the verdict block
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1560,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2772,6 +2772,18 @@
       <c r="B41" t="inlineStr">
         <is>
           <t>Post-Batch-Bündel: F42/F44/F45/F46 verbucht (Slope rein; Zhu&amp;Zhao rein mit Firm-Gewichts-Grenze; Trinh=performance; Wang-e zweigeteilt; Weber-Exit) · Ledger korrigiert 66-&gt;61 Legacy / 1239 Zeilen · Hui-&gt;update-Retag · Zhou-Gap zu (22 Zeilen; Spearman-Hypothese für 62-&gt;22) · Crosswalk evidenzbasiert · Rescreen-Mandat 20+1 (segment=rescreen; Wang-2020/K&amp;V-2018 retroaktiv)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>DEC-039</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Ruling-Layer geschlossen (R1-R8, K1-K4): Unit-Grenze "Firma und darunter"; Devalle-Vorzeichenregime; 2 Studien-Cluster (Sandra/Ofogbe, K&amp;V inkl. EL-Zeile); Delis-Preisvarianten getaggt rein; industry-Operationalisierung + mixed; K4 zurückgezogen (Datei-Beweis); cluster_id-Mechanik für v11; DEC-040 reserviert (Adjudikationsergebnisse + v11)</t>
         </is>
       </c>
     </row>
@@ -10317,7 +10329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -11100,7 +11112,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Pass-2b + Adjudikationspaket [DEC-038]: Ursachen-Etiketten je 727 Posten; Resolutions-Vorbefüllung (Slope 48, Trinh 104, Zhu&amp;Zhao 28, prod_inno 12, Wang 28, F37d); B&amp;H-Block-Adjudikation (N-Zuordnung); Spearman-Hypothese Zhou/Cubas; Kalibrier-Delta-3; dann Volker-Gespräch (Paket + Sandra/Ofogbe + F35-Errata) — GELIEFERT: docs/adjudication_package_v1.xlsx (6 Sheets; 797 Posten mit Ursache-Klasse; Prefills live gezählt; K&amp;V-Ruling F47a autor-ok)</t>
+          <t>Pass-2b + Adjudikationspaket [DEC-038]: Ursachen-Etiketten je 727 Posten; Resolutions-Vorbefüllung (Slope 48, Trinh 104, Zhu&amp;Zhao 28, prod_inno 12, Wang 28, F37d); B&amp;H-Block-Adjudikation (N-Zuordnung); Spearman-Hypothese Zhou/Cubas; Kalibrier-Delta-3; dann Volker-Gespräch (Paket + Sandra/Ofogbe + F35-Errata)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -11110,27 +11122,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>erledigt (2026-07-07)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>27</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Volker-Adjudikationsgespräch: Paket-Walkthrough in Agenda-Reihenfolge (Rahmen -&gt; Block-Entscheide [B&amp;H-N, strukturell, Versionsdrift, F37d] -&gt; Einzelprüfungen 343 -&gt; Sonderfälle [F35a, Sandra/Ofogbe, K&amp;V, Zhou/Cubas-Prüfaufträge, Spot-Checks] -&gt; Rescreen-Story); Rückläufer an Claude -&gt; DEC-039/v11</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Robert + Volker</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>offen — terminieren</t>
+          <t>in Arbeit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DEC-040: adjudication booked as study-level dispositions; v11 spec issued
- 1b Lesart (i): 208 structural v10-only rows stay out; 95 adoptions
  without cause attribution (N1: F37c conjecture); 51 version-drift
  adoptions with numeric dedup (documented DEC-026 exception)
- Zhou/Cubas source waiver (N2); lookup 61/61 verified (web-enabled run)
- Quality moderator = VHB only; JIF dormant (resolves DEC-023)
- v11 balance ~2,853; preliminary now, freeze = DEC-041 after DB re-run
- Agenda: #28 assembly build (review-gated), #29 JIF top-up, #30 moderators
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1560,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2784,6 +2784,18 @@
       <c r="B42" t="inlineStr">
         <is>
           <t>Ruling-Layer geschlossen (R1-R8, K1-K4): Unit-Grenze "Firma und darunter"; Devalle-Vorzeichenregime; 2 Studien-Cluster (Sandra/Ofogbe, K&amp;V inkl. EL-Zeile); Delis-Preisvarianten getaggt rein; industry-Operationalisierung + mixed; K4 zurückgezogen (Datei-Beweis); cluster_id-Mechanik für v11; DEC-040 reserviert (Adjudikationsergebnisse + v11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>DEC-040</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Adjudikation als Studien-Level-Dispositionen verbucht (1b Lesart i: 208 strukturell draußen; 95 Adoptionen ohne Ursache [N1: F37c-Vermutung]; 51 Versionsdrift-Adoptionen [DEC-026-Ausnahme]; Zhou/Cubas-Waiver [N2]); Lookup 61/61 verifiziert; q-Moderator=VHB-only, JIF ruhend (löst DEC-023); v11-Spec erlassen; Bilanz ~2853; preliminary jetzt, Freeze=DEC-041 nach DB-Re-Run</t>
         </is>
       </c>
     </row>
@@ -10329,7 +10341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10962,7 +10974,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>terminiert: Ende dieser Woche (Volker)</t>
         </is>
       </c>
     </row>
@@ -11123,6 +11135,66 @@
       <c r="D29" t="inlineStr">
         <is>
           <t>in Arbeit</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>v11-preliminary bauen [DEC-040]: Assembly-Skript + Verifier nach Spec (docs/v11_assembly_spec.md); FOUNDATIONAL -&gt; Pre-Execution-Diff-Review durch Robert; danach Prep-Spec/T1-Entwicklung gegen preliminary</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Claude -&gt; Robert (Review)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Spec liegt vor</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>JIF-Nachtrag alle Journals (b1, ruhendes Feld) — im DB-Re-Run-Slot via Cowork</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Robert (Cowork)</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>offen — mit #18</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Moderator-Block Neuzugänge (country/regulation/industry per F36/R4) — Skript parst Logs; Restliste an Volker</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Claude -&gt; Volker</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>mit #28</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DEC-041: v11 DATA FREEZE (2,852 rows / 2,730 usable / 120 studies; verifier 26/26)
- Native DEC-024 derivation grid + moderators populated corpus-wide
  (industry R4, regulation E1-E4, country_econ via extended country_lookup)
- Scope cutoff 2026-07-10: author decision B; reviewer dissent (A) documented
  with mitigation package (result-blind, catalogued 593, validation framing,
  ~1-week revision contingency)
- Rulings formalized: session S1-S19, blankets B1-B4, gap-run E1-E8
- Ledger correction: 65 v10 keys (not 66); Python/R tooling boundary codified
- Search & screening protocol shipped (3 DBs, recall 43/60, 1,720 screened)
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1560,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2796,6 +2796,18 @@
       <c r="B43" t="inlineStr">
         <is>
           <t>Adjudikation als Studien-Level-Dispositionen verbucht (1b Lesart i: 208 strukturell draußen; 95 Adoptionen ohne Ursache [N1: F37c-Vermutung]; 51 Versionsdrift-Adoptionen [DEC-026-Ausnahme]; Zhou/Cubas-Waiver [N2]); Lookup 61/61 verifiziert; q-Moderator=VHB-only, JIF ruhend (löst DEC-023); v11-Spec erlassen; Bilanz ~2853; preliminary jetzt, Freeze=DEC-041 nach DB-Re-Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>DEC-041</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>v11 DATA FREEZE: 2.852 Zeilen/2.730 usable/120 Studien; natives DEC-024-Grid + Moderatoren korpusweit (Verifier 26/26); Scope-Cutoff 2026-07-10 (Autor: B; Reviewer-Dissens A dokumentiert; Mitigation: result-blind, Katalog 593, Validierungs-Framing, Revisions-Kontingenz ~1 Woche); Rulings S1-S19/B1-B4/E1-E8 formalisiert; Ledger-Korrektur 65 v10-Keys; Sprachgrenze Python/R kodifiziert</t>
         </is>
       </c>
     </row>
@@ -10341,7 +10353,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10974,7 +10986,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>terminiert: Ende dieser Woche (Volker)</t>
+          <t>erledigt (2026-07-10, DEC-041)</t>
         </is>
       </c>
     </row>
@@ -11154,7 +11166,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Spec liegt vor</t>
+          <t>erledigt (2026-07-10, DEC-041)</t>
         </is>
       </c>
     </row>
@@ -11174,7 +11186,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>offen — mit #18</t>
+          <t>erledigt (2026-07-10, DEC-041)</t>
         </is>
       </c>
     </row>
@@ -11194,7 +11206,87 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>mit #28</t>
+          <t>erledigt (2026-07-10, DEC-041)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Screening-Katalog/Appendix: 593er-Liste als identified-not-extracted aufbereiten (optional Präzisions-Pass als Doku-Layer)</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Claude</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>offen (Manuskriptphase)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Manuskript-Fixes: Paris-Coding-Absatz -&gt; DEC-024-Architektur; Sensitive-Industry-Liste -&gt; R4; PRISMA-Sektion neu; Search-Absatz um 2026-Layer; Konkurrenz-Paper #1139 (CER/Policy Stringency/Debt Cost Europe 2026) lesen &amp; positionieren</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Robert/Claude</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Original-2021-Suchmetadaten (Daten/Ns je DB) im Archiv suchen; sonst Waiver</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>verschoben</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>DEC-031 (Analyse-Batterie, SESOI 0.070) -&gt; T0.4 Prep -&gt; T1</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Claude -&gt; Robert (Review-Gates)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>NÄCHSTER SCHRITT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
DEC-031a: battery walk-through amendments + Status workbook Analyse_Batterie sheet
- Moderator inventory recut (narrative C-panel: CER/COD/industry/regulation/4x country; technical checks -> G; q_status -> D grey-literature panel); corpus_segment and cluster_study removed (on-demand retention); new specs one_per_cluster_median, outlier_mad, trim_1_99; trim-and-fill/SD-rules/SAMD excluded with citations; two pre-registered conditional upgrades adjudicated by design_quantities_v12.csv; figure inventory and G reporting principle fixed

- Status: new Analyse_Batterie tracking sheet (63 analyses A1-H11, per-analysis status/reference/result columns); Ablauf/Index/Null_Battery updated
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -11,13 +11,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ablauf" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Roadmap" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aufgaben" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysen" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Null_Battery" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Scoping" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datenagenda" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifikation" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key_Results" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DecisionLog_Index" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analyse_Batterie" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysen" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Null_Battery" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Update_Scoping" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datenagenda" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Identifikation" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Key_Results" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DecisionLog_Index" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -216,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -345,6 +346,12 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1323,6 +1330,343 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Identifikation: Bruch vs. Trend — Werkzeugkasten gegen den Saekulartrend-Confound (#13 / T8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Problem: Pre/Post-Dummy trennt Bruch nicht von Drift. Daten zeigen Drift (Pre-median r=−0,025 vs. Post r=−0,019). Strategie: Trend modellieren, Paris muss DARUEBER HINAUS liefern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Move</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Staerke-Tier</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Was es testet / leistet</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>Methode</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>Datenabhaengigkeit</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>Praezedenz / Anker</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="84" customHeight="1">
+      <c r="A4" s="27" t="inlineStr">
+        <is>
+          <t>1. Trend-vs-Bruch-Wettrennen</t>
+        </is>
+      </c>
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Tier 1 — essenziell, sofort</t>
+        </is>
+      </c>
+      <c r="C4" s="27" t="inlineStr">
+        <is>
+          <t>Trennt glatte Drift vom diskreten Level-Sprung. Dummy weg → nur Drift; ueberlebt → echte Diskontinuitaet</t>
+        </is>
+      </c>
+      <c r="D4" s="27" t="inlineStr">
+        <is>
+          <t>Kont. Zeit (zentr. Midpoint) + Paris-Dummy im SELBEN sparsamen Modell</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>Sofort — sobald T0.4 kont. Zeit liefert</t>
+        </is>
+      </c>
+      <c r="F4" s="27" t="inlineStr">
+        <is>
+          <t>Huang 2020 (pub-year-Control neben GFC)</t>
+        </is>
+      </c>
+      <c r="G4" s="27" t="inlineStr">
+        <is>
+          <t>OFFEN (T0.4-abh.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="84" customHeight="1">
+      <c r="A5" s="27" t="inlineStr">
+        <is>
+          <t>2. Segmentierte Meta-Regression (ITS)</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>Tier 1 — essenziell, sofort</t>
+        </is>
+      </c>
+      <c r="C5" s="27" t="inlineStr">
+        <is>
+          <t>β₂ Level-Sprung, β₃ Slope-Aenderung. Nistet reinen Trend vs. Bruch als testbare Spezialfaelle</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>effect ~ β₀+β₁·Zeit+β₂·post+β₃·(Zeit×post); RVE</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>Sofort — T0.4-abh.</t>
+        </is>
+      </c>
+      <c r="F5" s="27" t="inlineStr">
+        <is>
+          <t>ITS-Standard; COVID-Wellen-Analogon</t>
+        </is>
+      </c>
+      <c r="G5" s="27" t="inlineStr">
+        <is>
+          <t>OFFEN (T0.4-abh.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="84" customHeight="1">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>3. Placebo-/Falsifikations-Bruchdaten</t>
+        </is>
+      </c>
+      <c r="B6" s="30" t="inlineStr">
+        <is>
+          <t>Tier 2 — stark</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="inlineStr">
+        <is>
+          <t>Bruch an Nicht-Paris-Jahren (2012/13/17/18). Ueberall → kein Paris-Bruch; nur 2015/16 → echt. DEUTET LAG1–3 ZU FALSIFIKATION UM</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="inlineStr">
+        <is>
+          <t>Bruch-Magnitude je Cutoff; Lokalisierungs-Vergleich</t>
+        </is>
+      </c>
+      <c r="E6" s="29" t="inlineStr">
+        <is>
+          <t>Sofort — T0.4-abh.</t>
+        </is>
+      </c>
+      <c r="F6" s="29" t="inlineStr">
+        <is>
+          <t>Placebo-Test-Standard</t>
+        </is>
+      </c>
+      <c r="G6" s="29" t="inlineStr">
+        <is>
+          <t>OFFEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="84" customHeight="1">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>4. Kompositions-Kontrolle</t>
+        </is>
+      </c>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>Tier 2 — stark, sofort</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>Haelt Studien-/Laender-/Instrument-Mix konstant; Within-Stratum-Check. Nur im Aggregat → kompositorisch</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="inlineStr">
+        <is>
+          <t>Paris-Term + Moderatoren als Kovariaten (= T7); Within-Stratum</t>
+        </is>
+      </c>
+      <c r="E7" s="29" t="inlineStr">
+        <is>
+          <t>Sofort (= T7)</t>
+        </is>
+      </c>
+      <c r="F7" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G7" s="29" t="inlineStr">
+        <is>
+          <t>OFFEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="84" customHeight="1">
+      <c r="A8" s="29" t="inlineStr">
+        <is>
+          <t>5. Differential-Exposure (DiD-artig)</t>
+        </is>
+      </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>Tier 2 — stark</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>(post−pre) High-Exposure minus (post−pre) Low: gemeinsamer Trend differenziert sich heraus</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="inlineStr">
+        <is>
+          <t>post × High-Exposure (carbon-intensiv / Carbon-Pricing); Pre-Trend-Check</t>
+        </is>
+      </c>
+      <c r="E8" s="29" t="inlineStr">
+        <is>
+          <t>Sofort; Pre-Trend datenabh.</t>
+        </is>
+      </c>
+      <c r="F8" s="29" t="inlineStr">
+        <is>
+          <t>DiD-Logik. CAVEAT: Parallel-Trends unpruefbar</t>
+        </is>
+      </c>
+      <c r="G8" s="29" t="inlineStr">
+        <is>
+          <t>OFFEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="84" customHeight="1">
+      <c r="A9" s="31" t="inlineStr">
+        <is>
+          <t>6. Within-Study-Identifikation</t>
+        </is>
+      </c>
+      <c r="B9" s="32" t="inlineStr">
+        <is>
+          <t>Tier 3 — Goldstandard, DATENBEDINGT TOT</t>
+        </is>
+      </c>
+      <c r="C9" s="31" t="inlineStr">
+        <is>
+          <t>Studien, die Bruch SELBST ueberspannen + separate Pre/Post. Haelt alle between-Confounder konstant</t>
+        </is>
+      </c>
+      <c r="D9" s="31" t="inlineStr">
+        <is>
+          <t>Within-Study-Pre/Post-Kontrast</t>
+        </is>
+      </c>
+      <c r="E9" s="31" t="inlineStr">
+        <is>
+          <t>NICHT VERFUEGBAR — nur 1–3/66 Studien ueberspannen</t>
+        </is>
+      </c>
+      <c r="F9" s="31" t="inlineStr">
+        <is>
+          <t>COVID within-cohort (Sun, Robinson)</t>
+        </is>
+      </c>
+      <c r="G9" s="31" t="inlineStr">
+        <is>
+          <t>ENTFAELLT (Datenbefund T0.3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="84" customHeight="1">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>7. Sensitivitaets-Schranke (Bounding)</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Tier 4 — Schlussklammer</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>Wie gross muesste ein Trend sein, um verbleibenden Paris-Dummy zu erklaeren. Begrenzt Confound explizit</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>Oster-Bounds / E-Value auf finales Modell</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>Sofort (nach Hauptmodell)</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="inlineStr">
+        <is>
+          <t>Oster 2019; E-Value (VanderWeele 2017)</t>
+        </is>
+      </c>
+      <c r="G10" s="17" t="inlineStr">
+        <is>
+          <t>OFFEN</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1554,13 +1898,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1582,7 +1926,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>29 aktive Methodik-DECs (DEC-001..029). Volleinträge im DECISION_LOG.md (append-only).</t>
+          <t>43 Methodik-DECs (DEC-001..029 + 030..042 + 031/031a; Reihenfolge im Log = chronologisch/append-only). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -2808,6 +3152,42 @@
       <c r="B44" t="inlineStr">
         <is>
           <t>v11 DATA FREEZE: 2.852 Zeilen/2.730 usable/120 Studien; natives DEC-024-Grid + Moderatoren korpusweit (Verifier 26/26); Scope-Cutoff 2026-07-10 (Autor: B; Reviewer-Dissens A dokumentiert; Mitigation: result-blind, Katalog 593, Validierungs-Framing, Revisions-Kontingenz ~1 Woche); Rulings S1-S19/B1-B4/E1-E8 formalisiert; Ledger-Korrektur 65 v10-Keys; Sprachgrenze Python/R kodifiziert</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>DEC-042</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>v12 kanonisch: Moderatorschicht komplett, Formel-Architektur, Row-Level-Country, Integritäts-Audit (31 Checks)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>DEC-031</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Finale Analyse-Batterie auf v12 fixiert; a-priori Inputs (Seeds/Grids/SESOI); Pending-D geöffnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>DEC-031a</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Walk-through-Amendments: Moderator-Inventar neu geschnitten, Katalog final, konditionale Upgrades, Figuren</t>
         </is>
       </c>
     </row>
@@ -2827,7 +3207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2847,83 +3227,53 @@
       </c>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="40" t="inlineStr">
+      <c r="A2" s="45" t="inlineStr">
+        <is>
+          <t>STAND 2026-07-10: Datenphase abgeschlossen (v12 kanonisch, DEC-042) · Batterie fixiert (DEC-031/031a) · Schritt 2 = T0.4-Prep (Review-Gate) als Nächstes · Detailplan je Analyse: Sheet "Analyse_Batterie"</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="46" customHeight="1">
+      <c r="A3" s="40" t="inlineStr">
         <is>
           <t>Nr</t>
         </is>
       </c>
-      <c r="B2" s="40" t="inlineStr">
+      <c r="B3" s="40" t="inlineStr">
         <is>
           <t>Block</t>
         </is>
       </c>
-      <c r="C2" s="40" t="inlineStr">
+      <c r="C3" s="40" t="inlineStr">
         <is>
           <t>Schritt</t>
         </is>
       </c>
-      <c r="D2" s="40" t="inlineStr">
+      <c r="D3" s="40" t="inlineStr">
         <is>
           <t>Kurzbeschreibung</t>
         </is>
       </c>
-      <c r="E2" s="40" t="inlineStr">
+      <c r="E3" s="40" t="inlineStr">
         <is>
           <t>Gate / Abhängigkeit</t>
         </is>
       </c>
-      <c r="F2" s="40" t="inlineStr">
+      <c r="F3" s="40" t="inlineStr">
         <is>
           <t>Ort</t>
         </is>
       </c>
-      <c r="G2" s="40" t="inlineStr">
+      <c r="G3" s="40" t="inlineStr">
         <is>
           <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="46" customHeight="1">
-      <c r="A3" s="41" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="B3" s="41" t="inlineStr">
-        <is>
-          <t>Daten &amp; Methodik</t>
-        </is>
-      </c>
-      <c r="C3" s="41" t="inlineStr">
-        <is>
-          <t>Volker-Daten-Audit</t>
-        </is>
-      </c>
-      <c r="D3" s="41" t="inlineStr">
-        <is>
-          <t>Volkers Lieferung gegen Datenagenda prüfen (kritisch: 1 n-Regel, 2 Regulierung, 10 Sample-Jahre; Klärung: 4/5/7) + COE-Overlap (#11). Ergebnis: was gelöst / offen / ändert Methodik. [ERLEDIGT: v4 final, DEC-019–023; Lookups country+source; Headline-Cut + VHB/JIF-WP offen für Step 1]</t>
-        </is>
-      </c>
-      <c r="E3" s="41" t="inlineStr">
-        <is>
-          <t>Volker-Daten erhalten ✓</t>
-        </is>
-      </c>
-      <c r="F3" s="41" t="inlineStr">
-        <is>
-          <t>dieser Chat</t>
-        </is>
-      </c>
-      <c r="G3" s="41" t="inlineStr">
-        <is>
-          <t>erledigt</t>
         </is>
       </c>
     </row>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="41" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="B4" s="41" t="inlineStr">
@@ -2933,22 +3283,22 @@
       </c>
       <c r="C4" s="41" t="inlineStr">
         <is>
-          <t>Methodik finalisieren</t>
+          <t>Volker-Daten-Audit</t>
         </is>
       </c>
       <c r="D4" s="41" t="inlineStr">
         <is>
-          <t>Geplante Methodik (DEC-001..018) gegen Audit-Ergebnis validieren + offene Items schließen. [ERLEDIGT 2026-07-03: DEC-024–027 geloggt; Pending-A gelöst; Headline pp_share_lag0 + Inference-Transfer-Regel; q_JIF gestrichen; Status-Korrektur 7 Studien; n validiert/E14→n_obs; Datenbasis v8; #11/#12 geschlossen]</t>
+          <t>Volkers Lieferung gegen Datenagenda prüfen (kritisch: 1 n-Regel, 2 Regulierung, 10 Sample-Jahre; Klärung: 4/5/7) + COE-Overlap (#11). Ergebnis: was gelöst / offen / ändert Methodik. [ERLEDIGT: v4 final, DEC-019–023; Lookups country+source; Headline-Cut + VHB/JIF-WP offen für Step 1]</t>
         </is>
       </c>
       <c r="E4" s="41" t="inlineStr">
         <is>
-          <t>Schritt 0</t>
+          <t>Volker-Daten erhalten ✓</t>
         </is>
       </c>
       <c r="F4" s="41" t="inlineStr">
         <is>
-          <t>neuer Chat · Fable 5</t>
+          <t>dieser Chat</t>
         </is>
       </c>
       <c r="G4" s="41" t="inlineStr">
@@ -2960,7 +3310,7 @@
     <row r="5" ht="46" customHeight="1">
       <c r="A5" s="41" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B5" s="41" t="inlineStr">
@@ -2970,54 +3320,54 @@
       </c>
       <c r="C5" s="41" t="inlineStr">
         <is>
-          <t>Finales Datenset bauen</t>
+          <t>Methodik finalisieren</t>
         </is>
       </c>
       <c r="D5" s="41" t="inlineStr">
         <is>
-          <t>Re-prep (R/01_prep.R) gegen CER-COD_data_v10.xlsx; Verifier erweitert um DEC-024..028-Checks (pp_start≥2016, Identitäten, Lookup-Anti-Join, ES_source×ES_measure-Diagonale, Formel-Spotcheck, df-Berechnung Transfer-Regel). Vorab: DEC-029-Battery-Inputs fixieren (SESOI, Priors, Faktorraum, Grids). Öffnet das T1-Gate. — ERWEITERT [DEC-030]: zusätzlich erst v11 (Suchupdate) abwarten.</t>
+          <t>Geplante Methodik (DEC-001..018) gegen Audit-Ergebnis validieren + offene Items schließen. [ERLEDIGT 2026-07-03: DEC-024–027 geloggt; Pending-A gelöst; Headline pp_share_lag0 + Inference-Transfer-Regel; q_JIF gestrichen; Status-Korrektur 7 Studien; n validiert/E14→n_obs; Datenbasis v8; #11/#12 geschlossen]</t>
         </is>
       </c>
       <c r="E5" s="41" t="inlineStr">
         <is>
-          <t>Schritt 1 ✓</t>
+          <t>Schritt 0</t>
         </is>
       </c>
       <c r="F5" s="41" t="inlineStr">
         <is>
-          <t>CC / RStudio</t>
+          <t>neuer Chat · Fable 5</t>
         </is>
       </c>
       <c r="G5" s="41" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt</t>
         </is>
       </c>
     </row>
     <row r="6" ht="46" customHeight="1">
       <c r="A6" s="41" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B6" s="41" t="inlineStr">
         <is>
-          <t>Analysen</t>
+          <t>Daten &amp; Methodik</t>
         </is>
       </c>
       <c r="C6" s="41" t="inlineStr">
         <is>
-          <t>Alle Analysen</t>
+          <t>Finales Datenset bauen</t>
         </is>
       </c>
       <c r="D6" s="41" t="inlineStr">
         <is>
-          <t>T1 (3LMA-RVE) · T4 (Robustheit) · T5 (Pub-Bias) · T7 (unified MR) · T8 (Identifikation). Je Skript + Verifier.</t>
+          <t>Re-prep (R/01_prep.R) gegen CER-COD_data_v10.xlsx; Verifier erweitert um DEC-024..028-Checks (pp_start≥2016, Identitäten, Lookup-Anti-Join, ES_source×ES_measure-Diagonale, Formel-Spotcheck, df-Berechnung Transfer-Regel). Vorab: DEC-029-Battery-Inputs fixieren (SESOI, Priors, Faktorraum, Grids). Öffnet das T1-Gate. — ERWEITERT [DEC-030]: zusätzlich erst v11 (Suchupdate) abwarten.</t>
         </is>
       </c>
       <c r="E6" s="41" t="inlineStr">
         <is>
-          <t>finales Datenset (Schritt 2)</t>
+          <t>Schritt 1 ✓</t>
         </is>
       </c>
       <c r="F6" s="41" t="inlineStr">
@@ -3027,14 +3377,14 @@
       </c>
       <c r="G6" s="41" t="inlineStr">
         <is>
-          <t>gated</t>
+          <t>offen</t>
         </is>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
       <c r="A7" s="41" t="inlineStr">
         <is>
-          <t>3b</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B7" s="41" t="inlineStr">
@@ -3044,22 +3394,22 @@
       </c>
       <c r="C7" s="41" t="inlineStr">
         <is>
-          <t>Ergebnisse + A-vs-C entscheiden</t>
+          <t>Alle Analysen</t>
         </is>
       </c>
       <c r="D7" s="41" t="inlineStr">
         <is>
-          <t>Finalen Paris-Befund interpretieren; strategische Weiche Pfad A (Nullbefund/Debunking) vs. C (kontingenter Effekt). Determiniert 4–6.</t>
+          <t>T1 (3LMA-RVE) · T4 (Robustheit) · T5 (Pub-Bias) · T7 (unified MR) · T8 (Identifikation). Je Skript + Verifier.</t>
         </is>
       </c>
       <c r="E7" s="41" t="inlineStr">
         <is>
-          <t>Schritt 3</t>
+          <t>finales Datenset (Schritt 2)</t>
         </is>
       </c>
       <c r="F7" s="41" t="inlineStr">
         <is>
-          <t>dieser Chat</t>
+          <t>CC / RStudio</t>
         </is>
       </c>
       <c r="G7" s="41" t="inlineStr">
@@ -3071,27 +3421,27 @@
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="41" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3b</t>
         </is>
       </c>
       <c r="B8" s="41" t="inlineStr">
         <is>
-          <t>Positionierung</t>
+          <t>Analysen</t>
         </is>
       </c>
       <c r="C8" s="41" t="inlineStr">
         <is>
-          <t>Narrativer roter Faden</t>
+          <t>Ergebnisse + A-vs-C entscheiden</t>
         </is>
       </c>
       <c r="D8" s="41" t="inlineStr">
         <is>
-          <t>Intro→RQ→Beitrag; Claim–Evidence-Abgleich (Paris-Framing an Befund). GEKOPPELT mit 5/6, iterativ.</t>
+          <t>Finalen Paris-Befund interpretieren; strategische Weiche Pfad A (Nullbefund/Debunking) vs. C (kontingenter Effekt). Determiniert 4–6.</t>
         </is>
       </c>
       <c r="E8" s="41" t="inlineStr">
         <is>
-          <t>A-vs-C (3b)</t>
+          <t>Schritt 3</t>
         </is>
       </c>
       <c r="F8" s="41" t="inlineStr">
@@ -3108,7 +3458,7 @@
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="41" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B9" s="41" t="inlineStr">
@@ -3118,12 +3468,12 @@
       </c>
       <c r="C9" s="41" t="inlineStr">
         <is>
-          <t>Hypothesen</t>
+          <t>Narrativer roter Faden</t>
         </is>
       </c>
       <c r="D9" s="41" t="inlineStr">
         <is>
-          <t>H2/H3-Renumber, RQ↔H-Mapping, Formulierung an A-vs-C. GEKOPPELT mit 4/6.</t>
+          <t>Intro→RQ→Beitrag; Claim–Evidence-Abgleich (Paris-Framing an Befund). GEKOPPELT mit 5/6, iterativ.</t>
         </is>
       </c>
       <c r="E9" s="41" t="inlineStr">
@@ -3145,7 +3495,7 @@
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="41" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B10" s="41" t="inlineStr">
@@ -3155,12 +3505,12 @@
       </c>
       <c r="C10" s="41" t="inlineStr">
         <is>
-          <t>Theorie / Konstrukt</t>
+          <t>Hypothesen</t>
         </is>
       </c>
       <c r="D10" s="41" t="inlineStr">
         <is>
-          <t>Transition-Risk-Repricing als integrierende Klammer; Theorie-Architektur an Befund. GEKOPPELT mit 4/5.</t>
+          <t>H2/H3-Renumber, RQ↔H-Mapping, Formulierung an A-vs-C. GEKOPPELT mit 4/6.</t>
         </is>
       </c>
       <c r="E10" s="41" t="inlineStr">
@@ -3182,27 +3532,27 @@
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="41" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B11" s="41" t="inlineStr">
         <is>
-          <t>Schreiben</t>
+          <t>Positionierung</t>
         </is>
       </c>
       <c r="C11" s="41" t="inlineStr">
         <is>
-          <t>Ch 2 — Literatur &amp; Hypothesen</t>
+          <t>Theorie / Konstrukt</t>
         </is>
       </c>
       <c r="D11" s="41" t="inlineStr">
         <is>
-          <t>Schreiben/finalisieren; Novelty/Positionierung (Zarea/Witte, COE-Abgrenzung DEC-011).</t>
+          <t>Transition-Risk-Repricing als integrierende Klammer; Theorie-Architektur an Befund. GEKOPPELT mit 4/5.</t>
         </is>
       </c>
       <c r="E11" s="41" t="inlineStr">
         <is>
-          <t>Positionierung (4–6)</t>
+          <t>A-vs-C (3b)</t>
         </is>
       </c>
       <c r="F11" s="41" t="inlineStr">
@@ -3219,7 +3569,7 @@
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="41" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B12" s="41" t="inlineStr">
@@ -3229,17 +3579,17 @@
       </c>
       <c r="C12" s="41" t="inlineStr">
         <is>
-          <t>Ch 3 — Methodik</t>
+          <t>Ch 2 — Literatur &amp; Hypothesen</t>
         </is>
       </c>
       <c r="D12" s="41" t="inlineStr">
         <is>
-          <t>Schreiben/finalisieren gegen finale Methodik + Analysen.</t>
+          <t>Schreiben/finalisieren; Novelty/Positionierung (Zarea/Witte, COE-Abgrenzung DEC-011).</t>
         </is>
       </c>
       <c r="E12" s="41" t="inlineStr">
         <is>
-          <t>Schritt 1 + 3</t>
+          <t>Positionierung (4–6)</t>
         </is>
       </c>
       <c r="F12" s="41" t="inlineStr">
@@ -3256,7 +3606,7 @@
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="41" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B13" s="41" t="inlineStr">
@@ -3266,17 +3616,17 @@
       </c>
       <c r="C13" s="41" t="inlineStr">
         <is>
-          <t>Ch 4 — Results &amp; Diskussion</t>
+          <t>Ch 3 — Methodik</t>
         </is>
       </c>
       <c r="D13" s="41" t="inlineStr">
         <is>
-          <t>Schreiben/finalisieren gegen Analysen + A-vs-C.</t>
+          <t>Schreiben/finalisieren gegen finale Methodik + Analysen.</t>
         </is>
       </c>
       <c r="E13" s="41" t="inlineStr">
         <is>
-          <t>Schritt 3 + 3b</t>
+          <t>Schritt 1 + 3</t>
         </is>
       </c>
       <c r="F13" s="41" t="inlineStr">
@@ -3293,7 +3643,7 @@
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="41" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B14" s="41" t="inlineStr">
@@ -3303,17 +3653,17 @@
       </c>
       <c r="C14" s="41" t="inlineStr">
         <is>
-          <t>Ch 1 — Einleitung</t>
+          <t>Ch 4 — Results &amp; Diskussion</t>
         </is>
       </c>
       <c r="D14" s="41" t="inlineStr">
         <is>
-          <t>Schreiben/finalisieren zuletzt, aus finalem Framing.</t>
+          <t>Schreiben/finalisieren gegen Analysen + A-vs-C.</t>
         </is>
       </c>
       <c r="E14" s="41" t="inlineStr">
         <is>
-          <t>Ch 2–4 (7–9)</t>
+          <t>Schritt 3 + 3b</t>
         </is>
       </c>
       <c r="F14" s="41" t="inlineStr">
@@ -3330,77 +3680,115 @@
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="41" t="inlineStr">
         <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B15" s="41" t="inlineStr">
+        <is>
+          <t>Schreiben</t>
+        </is>
+      </c>
+      <c r="C15" s="41" t="inlineStr">
+        <is>
+          <t>Ch 1 — Einleitung</t>
+        </is>
+      </c>
+      <c r="D15" s="41" t="inlineStr">
+        <is>
+          <t>Schreiben/finalisieren zuletzt, aus finalem Framing.</t>
+        </is>
+      </c>
+      <c r="E15" s="41" t="inlineStr">
+        <is>
+          <t>Ch 2–4 (7–9)</t>
+        </is>
+      </c>
+      <c r="F15" s="41" t="inlineStr">
+        <is>
+          <t>dieser Chat</t>
+        </is>
+      </c>
+      <c r="G15" s="41" t="inlineStr">
+        <is>
+          <t>gated</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="41" t="inlineStr">
+        <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B15" s="41" t="inlineStr">
+      <c r="B16" s="41" t="inlineStr">
         <is>
           <t>Schreiben</t>
         </is>
       </c>
-      <c r="C15" s="41" t="inlineStr">
+      <c r="C16" s="41" t="inlineStr">
         <is>
           <t>Ch 5 — Conclusion + Abstract</t>
         </is>
       </c>
-      <c r="D15" s="41" t="inlineStr">
+      <c r="D16" s="41" t="inlineStr">
         <is>
           <t>Schreiben/finalisieren; Abstract ganz am Ende.</t>
         </is>
       </c>
-      <c r="E15" s="41" t="inlineStr">
+      <c r="E16" s="41" t="inlineStr">
         <is>
           <t>Ch 1–4</t>
         </is>
       </c>
-      <c r="F15" s="41" t="inlineStr">
+      <c r="F16" s="41" t="inlineStr">
         <is>
           <t>dieser Chat</t>
         </is>
       </c>
-      <c r="G15" s="41" t="inlineStr">
+      <c r="G16" s="41" t="inlineStr">
         <is>
           <t>gated</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="43" t="inlineStr">
+    <row r="17"/>
+    <row r="18" ht="30" customHeight="1">
+      <c r="A18" s="43" t="inlineStr">
         <is>
           <t>Guardrails / Hinweise</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="41" t="inlineStr">
-        <is>
-          <t>G1 — PK vor Schritt 1 aktuell: DEC-018, analysis_plan.md, Status-xlsx, data_dictionary.md — und die T0.4-Skripte (01_prep.R, 01_verify_outputs.R) mit hochladen, damit Fable 5 die reale Prep-Logik sieht, nicht nur die Spec.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="41" t="inlineStr">
         <is>
-          <t>G2 — Scope in Fable-5 binden: offene Items schließen + Plan validieren; die 18 DECs NICHT grundlos neu aufrollen (verteidigte Entscheidungen → sonst Churn).</t>
+          <t>G1 — PK vor Schritt 1 aktuell: DEC-018, analysis_plan.md, Status-xlsx, data_dictionary.md — und die T0.4-Skripte (01_prep.R, 01_verify_outputs.R) mit hochladen, damit Fable 5 die reale Prep-Logik sieht, nicht nur die Spec.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="41" t="inlineStr">
         <is>
-          <t>G3 — Fordert Fable 5 einen DEC heraus: auf Merit prüfen + loggen — weder automatisch übernehmen noch abtun. Begründete Kritik bleibt, bis entkräftet.</t>
+          <t>G2 — Scope in Fable-5 binden: offene Items schließen + Plan validieren; die 18 DECs NICHT grundlos neu aufrollen (verteidigte Entscheidungen → sonst Churn).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="41" t="inlineStr">
         <is>
-          <t>G4 — Schritte 4–6 sind ein gekoppelter, iterativer Positionierungs-Block (Primärordnung Narrativ→Hyp→Theorie), kein starrer Einmal-Lock.</t>
+          <t>G3 — Fordert Fable 5 einen DEC heraus: auf Merit prüfen + loggen — weder automatisch übernehmen noch abtun. Begründete Kritik bleibt, bis entkräftet.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="41" t="inlineStr">
+        <is>
+          <t>G4 — Schritte 4–6 sind ein gekoppelter, iterativer Positionierungs-Block (Primärordnung Narrativ→Hyp→Theorie), kein starrer Einmal-Lock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="41" t="inlineStr">
         <is>
           <t>G5 — COE-Selbstüberlappung (#11) ist Desk-Reject-Risiko: klären im Audit (0) oder spätestens bei Ch 2 (7).</t>
         </is>
@@ -4963,7 +5351,1829 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:G74"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Analyse-Batterie — CER–COD FOMA (per DEC-031 + DEC-031a, 2026-07-10; result-blind bis Gates T0.4/T1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="45" t="inlineStr">
+        <is>
+          <t>Nr</t>
+        </is>
+      </c>
+      <c r="B3" s="45" t="inlineStr">
+        <is>
+          <t>Titel</t>
+        </is>
+      </c>
+      <c r="C3" s="45" t="inlineStr">
+        <is>
+          <t>Kurzbeschreibung</t>
+        </is>
+      </c>
+      <c r="D3" s="45" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E3" s="45" t="inlineStr">
+        <is>
+          <t>Referenz</t>
+        </is>
+      </c>
+      <c r="F3" s="45" t="inlineStr">
+        <is>
+          <t>Anmerkung Ergebnis</t>
+        </is>
+      </c>
+      <c r="G3" s="45" t="inlineStr">
+        <is>
+          <t>Anmerkung allgemein</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="47" t="inlineStr">
+        <is>
+          <t>— Block A — Kern (T1)</t>
+        </is>
+      </c>
+      <c r="B4" s="48" t="inlineStr"/>
+      <c r="C4" s="46" t="inlineStr"/>
+      <c r="D4" s="48" t="inlineStr"/>
+      <c r="E4" s="48" t="inlineStr"/>
+      <c r="F4" s="46" t="inlineStr"/>
+      <c r="G4" s="46" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="48" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="B5" s="48" t="inlineStr">
+        <is>
+          <t>Headline 3LMA-RVE</t>
+        </is>
+      </c>
+      <c r="C5" s="46" t="inlineStr">
+        <is>
+          <t>Gepoolter Gesamteffekt: Drei-Ebenen-MA über 2.714 Effekte, Fisher-z-PCC (van Aert 2023), rho=0,6, CR2 auf cluster_id</t>
+        </is>
+      </c>
+      <c r="D5" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E5" s="48" t="inlineStr"/>
+      <c r="F5" s="46" t="inlineStr"/>
+      <c r="G5" s="46" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="48" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B6" s="48" t="inlineStr">
+        <is>
+          <t>Varianzzerlegung</t>
+        </is>
+      </c>
+      <c r="C6" s="46" t="inlineStr">
+        <is>
+          <t>tau² zwischen vs. innerhalb Studien (+Cluster-Ebene wo schätzbar)</t>
+        </is>
+      </c>
+      <c r="D6" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E6" s="48" t="inlineStr"/>
+      <c r="F6" s="46" t="inlineStr"/>
+      <c r="G6" s="46" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="48" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="B7" s="48" t="inlineStr">
+        <is>
+          <t>Prädiktionsintervall</t>
+        </is>
+      </c>
+      <c r="C7" s="46" t="inlineStr">
+        <is>
+          <t>Erwarteter Effektbereich einer neuen Studie</t>
+        </is>
+      </c>
+      <c r="D7" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E7" s="48" t="inlineStr"/>
+      <c r="F7" s="46" t="inlineStr"/>
+      <c r="G7" s="46" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="48" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="B8" s="48" t="inlineStr">
+        <is>
+          <t>rho-Sensitivität</t>
+        </is>
+      </c>
+      <c r="C8" s="46" t="inlineStr">
+        <is>
+          <t>Headline mit rho=0,4 und 0,8</t>
+        </is>
+      </c>
+      <c r="D8" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E8" s="48" t="inlineStr"/>
+      <c r="F8" s="46" t="inlineStr"/>
+      <c r="G8" s="46" t="inlineStr">
+        <is>
+          <t>Register-Zeilen in G-Langtabelle</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="48" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="B9" s="48" t="inlineStr">
+        <is>
+          <t>Schätzer-Robustheit</t>
+        </is>
+      </c>
+      <c r="C9" s="46" t="inlineStr">
+        <is>
+          <t>One-effect-per-cluster (rho-Aggregation) · UWLS+3 · HS+WAAP (Appendix)</t>
+        </is>
+      </c>
+      <c r="D9" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E9" s="48" t="inlineStr"/>
+      <c r="F9" s="46" t="inlineStr"/>
+      <c r="G9" s="46" t="inlineStr">
+        <is>
+          <t>FE/RE-Dichotomie im Text adressiert, nicht als Zeile (DEC-031a.4e)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="48" t="inlineStr">
+        <is>
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="B10" s="48" t="inlineStr">
+        <is>
+          <t>Ökonomische Übersetzung</t>
+        </is>
+      </c>
+      <c r="C10" s="46" t="inlineStr">
+        <is>
+          <t>Gepoolter Effekt in Basispunkte COD (DEC-012)</t>
+        </is>
+      </c>
+      <c r="D10" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E10" s="48" t="inlineStr"/>
+      <c r="F10" s="46" t="inlineStr"/>
+      <c r="G10" s="46" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="48" t="inlineStr">
+        <is>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="B11" s="48" t="inlineStr">
+        <is>
+          <t>Caterpillar-Plot</t>
+        </is>
+      </c>
+      <c r="C11" s="46" t="inlineStr">
+        <is>
+          <t>Alle 120 Cluster-Aggregate sortiert, ohne Labels, Pooled+PI-Referenzlinien (Appendix)</t>
+        </is>
+      </c>
+      <c r="D11" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E11" s="48" t="inlineStr"/>
+      <c r="F11" s="46" t="inlineStr"/>
+      <c r="G11" s="46" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="48" t="inlineStr">
+        <is>
+          <t>A8</t>
+        </is>
+      </c>
+      <c r="B12" s="48" t="inlineStr">
+        <is>
+          <t>Forest-Plot Studienebene</t>
+        </is>
+      </c>
+      <c r="C12" s="46" t="inlineStr">
+        <is>
+          <t>120 beschriftete Studien-Aggregate mit CI, gepoolte Referenzlinie (Appendix, ganzseitig)</t>
+        </is>
+      </c>
+      <c r="D12" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E12" s="48" t="inlineStr"/>
+      <c r="F12" s="46" t="inlineStr"/>
+      <c r="G12" s="46" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="47" t="inlineStr">
+        <is>
+          <t>— Block B — Paris-Identifikation (T2/T8)</t>
+        </is>
+      </c>
+      <c r="B13" s="48" t="inlineStr"/>
+      <c r="C13" s="46" t="inlineStr"/>
+      <c r="D13" s="48" t="inlineStr"/>
+      <c r="E13" s="48" t="inlineStr"/>
+      <c r="F13" s="46" t="inlineStr"/>
+      <c r="G13" s="46" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="48" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="B14" s="48" t="inlineStr">
+        <is>
+          <t>Paris Headline binär</t>
+        </is>
+      </c>
+      <c r="C14" s="46" t="inlineStr">
+        <is>
+          <t>Post- vs. Prä-mehrheitliche Fenster via pp_mid_lag0 (≡ share_2016 ≥ 0,5, ties→Post); Transfer-Regel: df&lt;4–5 → deskriptiv, Inferenz wandert zu B2</t>
+        </is>
+      </c>
+      <c r="D14" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E14" s="48" t="inlineStr"/>
+      <c r="F14" s="46" t="inlineStr"/>
+      <c r="G14" s="46" t="inlineStr">
+        <is>
+          <t>df aus design_quantities_v12.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="48" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="B15" s="48" t="inlineStr">
+        <is>
+          <t>Dosis-Modell (kontinuierlich)</t>
+        </is>
+      </c>
+      <c r="C15" s="46" t="inlineStr">
+        <is>
+          <t>zi ~ sample_mid_c + pp_share_lag0; vorhergesagte Effekte bei 0/0,6/1 Post-Anteil; Quadrat-Check; Identifikations-Kern</t>
+        </is>
+      </c>
+      <c r="D15" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E15" s="48" t="inlineStr"/>
+      <c r="F15" s="46" t="inlineStr"/>
+      <c r="G15" s="46" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="48" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B16" s="48" t="inlineStr">
+        <is>
+          <t>Kodierungs-Sensitivitäten</t>
+        </is>
+      </c>
+      <c r="C16" s="46" t="inlineStr">
+        <is>
+          <t>tie_break (pp_median_lag0) · end_any_exposure (pp_end_lag0) · Share-Lags 2017/18/19 · End-Lags (Appendix) · clean-window deskriptiv</t>
+        </is>
+      </c>
+      <c r="D16" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E16" s="48" t="inlineStr"/>
+      <c r="F16" s="46" t="inlineStr"/>
+      <c r="G16" s="46" t="inlineStr">
+        <is>
+          <t>Upgrade-Bedingung: clean-window → volle Inferenz falls df≥5 auf v12 (DEC-031a.5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="48" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B17" s="48" t="inlineStr">
+        <is>
+          <t>Trend-vs-Bruch + Placebos</t>
+        </is>
+      </c>
+      <c r="C17" s="46" t="inlineStr">
+        <is>
+          <t>Bruch 2016 gegen glatten Zeittrend; Placebo-Bruchjahre 2008–2015; segmentierte MR</t>
+        </is>
+      </c>
+      <c r="D17" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E17" s="48" t="inlineStr"/>
+      <c r="F17" s="46" t="inlineStr"/>
+      <c r="G17" s="46" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="48" t="inlineStr">
+        <is>
+          <t>B5</t>
+        </is>
+      </c>
+      <c r="B18" s="48" t="inlineStr">
+        <is>
+          <t>Kompositions-Kontrolle</t>
+        </is>
+      </c>
+      <c r="C18" s="46" t="inlineStr">
+        <is>
+          <t>Prüft ob Zeiteffekt = veränderte Studienkomposition post-2016 (Move 4, core)</t>
+        </is>
+      </c>
+      <c r="D18" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E18" s="48" t="inlineStr"/>
+      <c r="F18" s="46" t="inlineStr"/>
+      <c r="G18" s="46" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="48" t="inlineStr">
+        <is>
+          <t>B6</t>
+        </is>
+      </c>
+      <c r="B19" s="48" t="inlineStr">
+        <is>
+          <t>Post-Zellen-LOSO</t>
+        </is>
+      </c>
+      <c r="C19" s="46" t="inlineStr">
+        <is>
+          <t>Leave-one-study-out speziell für die Post-Zelle; Dominanzanteile</t>
+        </is>
+      </c>
+      <c r="D19" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E19" s="48" t="inlineStr"/>
+      <c r="F19" s="46" t="inlineStr"/>
+      <c r="G19" s="46" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="48" t="inlineStr">
+        <is>
+          <t>B7</t>
+        </is>
+      </c>
+      <c r="B20" s="48" t="inlineStr">
+        <is>
+          <t>Disclosures</t>
+        </is>
+      </c>
+      <c r="C20" s="46" t="inlineStr">
+        <is>
+          <t>Attenuation / Knife-edge / Panel-Drift, re-computed auf v12 (Methods-Sätze)</t>
+        </is>
+      </c>
+      <c r="D20" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E20" s="48" t="inlineStr"/>
+      <c r="F20" s="46" t="inlineStr"/>
+      <c r="G20" s="46" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="47" t="inlineStr">
+        <is>
+          <t>— Block C — Narrative Moderatoren (T7 Stufe 1)</t>
+        </is>
+      </c>
+      <c r="B21" s="48" t="inlineStr"/>
+      <c r="C21" s="46" t="inlineStr"/>
+      <c r="D21" s="48" t="inlineStr"/>
+      <c r="E21" s="48" t="inlineStr"/>
+      <c r="F21" s="46" t="inlineStr"/>
+      <c r="G21" s="46" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="48" t="inlineStr">
+        <is>
+          <t>C0</t>
+        </is>
+      </c>
+      <c r="B22" s="48" t="inlineStr">
+        <is>
+          <t>Country-Korrelationsmatrix</t>
+        </is>
+      </c>
+      <c r="C22" s="46" t="inlineStr">
+        <is>
+          <t>Assoziationsmatrix region/econ/culture/legal inkl. Regulation-Überlappung</t>
+        </is>
+      </c>
+      <c r="D22" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E22" s="48" t="inlineStr"/>
+      <c r="F22" s="46" t="inlineStr"/>
+      <c r="G22" s="46" t="inlineStr">
+        <is>
+          <t>NUR Hintergrund (r15), nicht Manuskript; Input für Pending-D</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="48" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B23" s="48" t="inlineStr">
+        <is>
+          <t>Moderator CER_measure</t>
+        </is>
+      </c>
+      <c r="C23" s="46" t="inlineStr">
+        <is>
+          <t>Performance vs. Disclosure: Haupteffekt- + Paris-Interaktions-Modell, F-Test</t>
+        </is>
+      </c>
+      <c r="D23" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E23" s="48" t="inlineStr"/>
+      <c r="F23" s="46" t="inlineStr"/>
+      <c r="G23" s="46" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="48" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B24" s="48" t="inlineStr">
+        <is>
+          <t>Moderator COD_instrument</t>
+        </is>
+      </c>
+      <c r="C24" s="46" t="inlineStr">
+        <is>
+          <t>loan / bond / CDS / rating</t>
+        </is>
+      </c>
+      <c r="D24" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E24" s="48" t="inlineStr"/>
+      <c r="F24" s="46" t="inlineStr"/>
+      <c r="G24" s="46" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="48" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B25" s="48" t="inlineStr">
+        <is>
+          <t>Moderator industry</t>
+        </is>
+      </c>
+      <c r="C25" s="46" t="inlineStr">
+        <is>
+          <t>sensitiv / nicht-sensitiv / 99_NCE</t>
+        </is>
+      </c>
+      <c r="D25" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E25" s="48" t="inlineStr"/>
+      <c r="F25" s="46" t="inlineStr"/>
+      <c r="G25" s="46" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="48" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B26" s="48" t="inlineStr">
+        <is>
+          <t>Moderator regulation3</t>
+        </is>
+      </c>
+      <c r="C26" s="46" t="inlineStr">
+        <is>
+          <t>mit / ohne ETS-CT / 99_NCE</t>
+        </is>
+      </c>
+      <c r="D26" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E26" s="48" t="inlineStr"/>
+      <c r="F26" s="46" t="inlineStr"/>
+      <c r="G26" s="46" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="48" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B27" s="48" t="inlineStr">
+        <is>
+          <t>Moderator country_region</t>
+        </is>
+      </c>
+      <c r="C27" s="46" t="inlineStr">
+        <is>
+          <t>1_US / 2_Europe / 3_AsiaPac / 99_NCE</t>
+        </is>
+      </c>
+      <c r="D27" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E27" s="48" t="inlineStr"/>
+      <c r="F27" s="46" t="inlineStr"/>
+      <c r="G27" s="46" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="48" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B28" s="48" t="inlineStr">
+        <is>
+          <t>Moderator country_econ</t>
+        </is>
+      </c>
+      <c r="C28" s="46" t="inlineStr">
+        <is>
+          <t>developed / developing / 99_NCE</t>
+        </is>
+      </c>
+      <c r="D28" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E28" s="48" t="inlineStr"/>
+      <c r="F28" s="46" t="inlineStr"/>
+      <c r="G28" s="46" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="48" t="inlineStr">
+        <is>
+          <t>C7</t>
+        </is>
+      </c>
+      <c r="B29" s="48" t="inlineStr">
+        <is>
+          <t>Moderator country_culture</t>
+        </is>
+      </c>
+      <c r="C29" s="46" t="inlineStr">
+        <is>
+          <t>western / non-western / 99_NCE</t>
+        </is>
+      </c>
+      <c r="D29" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E29" s="48" t="inlineStr"/>
+      <c r="F29" s="46" t="inlineStr"/>
+      <c r="G29" s="46" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="48" t="inlineStr">
+        <is>
+          <t>C8</t>
+        </is>
+      </c>
+      <c r="B30" s="48" t="inlineStr">
+        <is>
+          <t>Moderator country_legal</t>
+        </is>
+      </c>
+      <c r="C30" s="46" t="inlineStr">
+        <is>
+          <t>common law / civil law / 99_NCE</t>
+        </is>
+      </c>
+      <c r="D30" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E30" s="48" t="inlineStr"/>
+      <c r="F30" s="46" t="inlineStr"/>
+      <c r="G30" s="46" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="48" t="inlineStr">
+        <is>
+          <t>C9</t>
+        </is>
+      </c>
+      <c r="B31" s="48" t="inlineStr">
+        <is>
+          <t>Unified model(s)</t>
+        </is>
+      </c>
+      <c r="C31" s="46" t="inlineStr">
+        <is>
+          <t>Komposition offen — Pending-D-Session nach T0.4, vor T7; ggf. Varianten V1..Vk, alle berichtet</t>
+        </is>
+      </c>
+      <c r="D31" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E31" s="48" t="inlineStr"/>
+      <c r="F31" s="46" t="inlineStr"/>
+      <c r="G31" s="46" t="inlineStr">
+        <is>
+          <t>Resolves als DEC-043; Inputs: Zellgrößen v12 + C0</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="47" t="inlineStr">
+        <is>
+          <t>— Block D — Publication Bias (T5)</t>
+        </is>
+      </c>
+      <c r="B32" s="48" t="inlineStr"/>
+      <c r="C32" s="46" t="inlineStr"/>
+      <c r="D32" s="48" t="inlineStr"/>
+      <c r="E32" s="48" t="inlineStr"/>
+      <c r="F32" s="46" t="inlineStr"/>
+      <c r="G32" s="46" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="48" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B33" s="48" t="inlineStr">
+        <is>
+          <t>FAT-PET-PEESE</t>
+        </is>
+      </c>
+      <c r="C33" s="46" t="inlineStr">
+        <is>
+          <t>Funnel-Asymmetrie-Regression, CR2/cluster_id; PEESE nur falls PET-Intercept signifikant (Regel fix)</t>
+        </is>
+      </c>
+      <c r="D33" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E33" s="48" t="inlineStr"/>
+      <c r="F33" s="46" t="inlineStr"/>
+      <c r="G33" s="46" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="48" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B34" s="48" t="inlineStr">
+        <is>
+          <t>Selektionsmodelle</t>
+        </is>
+      </c>
+      <c r="C34" s="46" t="inlineStr">
+        <is>
+          <t>3PSM (steps 0,025) + p-uniform* auf One-per-Cluster-Aggregaten</t>
+        </is>
+      </c>
+      <c r="D34" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E34" s="48" t="inlineStr"/>
+      <c r="F34" s="46" t="inlineStr"/>
+      <c r="G34" s="46" t="inlineStr">
+        <is>
+          <t>Trim-and-Fill begründet ausgeschlossen (Carter et al. 2019; DEC-031a.4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="48" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B35" s="48" t="inlineStr">
+        <is>
+          <t>RoBMA</t>
+        </is>
+      </c>
+      <c r="C35" s="46" t="inlineStr">
+        <is>
+          <t>Bayesianisches Modell-Averaging, Bayes-Faktor; Priors per Annex H</t>
+        </is>
+      </c>
+      <c r="D35" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E35" s="48" t="inlineStr"/>
+      <c r="F35" s="46" t="inlineStr"/>
+      <c r="G35" s="46" t="inlineStr">
+        <is>
+          <t>Zarea-Prior: Extraktion PENDING</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="48" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B36" s="48" t="inlineStr">
+        <is>
+          <t>Prä/Post-Bias-Split</t>
+        </is>
+      </c>
+      <c r="C36" s="46" t="inlineStr">
+        <is>
+          <t>FAT-PET-PEESE getrennt vor/nach Paris (Appendix)</t>
+        </is>
+      </c>
+      <c r="D36" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E36" s="48" t="inlineStr"/>
+      <c r="F36" s="46" t="inlineStr"/>
+      <c r="G36" s="46" t="inlineStr">
+        <is>
+          <t>Upgrade: 3PSM/p-uniform* in den Split falls Post-Zelle ≥20 Studien (DEC-031a.5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="48" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
+      <c r="B37" s="48" t="inlineStr">
+        <is>
+          <t>Grey-Literature-Panel</t>
+        </is>
+      </c>
+      <c r="C37" s="46" t="inlineStr">
+        <is>
+          <t>q_status published vs. WP als direkter Selektions-Check</t>
+        </is>
+      </c>
+      <c r="D37" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E37" s="48" t="inlineStr"/>
+      <c r="F37" s="46" t="inlineStr"/>
+      <c r="G37" s="46" t="inlineStr">
+        <is>
+          <t>aus C verschoben (DEC-031a.1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="48" t="inlineStr">
+        <is>
+          <t>D6</t>
+        </is>
+      </c>
+      <c r="B38" s="48" t="inlineStr">
+        <is>
+          <t>Triangulations-Statement</t>
+        </is>
+      </c>
+      <c r="C38" s="46" t="inlineStr">
+        <is>
+          <t>Konvergenz/Divergenz der Bias-Verfahren; füttert A-vs-C-Framing (Pending-C)</t>
+        </is>
+      </c>
+      <c r="D38" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E38" s="48" t="inlineStr"/>
+      <c r="F38" s="46" t="inlineStr"/>
+      <c r="G38" s="46" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="47" t="inlineStr">
+        <is>
+          <t>— Block E — Äquivalenztests (N1)</t>
+        </is>
+      </c>
+      <c r="B39" s="48" t="inlineStr"/>
+      <c r="C39" s="46" t="inlineStr"/>
+      <c r="D39" s="48" t="inlineStr"/>
+      <c r="E39" s="48" t="inlineStr"/>
+      <c r="F39" s="46" t="inlineStr"/>
+      <c r="G39" s="46" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="48" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="B40" s="48" t="inlineStr">
+        <is>
+          <t>TOST Gesamteffekt</t>
+        </is>
+      </c>
+      <c r="C40" s="46" t="inlineStr">
+        <is>
+          <t>Zwei einseitige Tests gegen SESOI |r|=0,070 (primär) und 0,05 (sekundär)</t>
+        </is>
+      </c>
+      <c r="D40" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E40" s="48" t="inlineStr"/>
+      <c r="F40" s="46" t="inlineStr"/>
+      <c r="G40" s="46" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="48" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="B41" s="48" t="inlineStr">
+        <is>
+          <t>TOST Paris-Kontrast</t>
+        </is>
+      </c>
+      <c r="C41" s="46" t="inlineStr">
+        <is>
+          <t>Äquivalenz des Prä/Post-Unterschieds; bei Transfer auf Dosis-Kontrast 0→0,6</t>
+        </is>
+      </c>
+      <c r="D41" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E41" s="48" t="inlineStr"/>
+      <c r="F41" s="46" t="inlineStr"/>
+      <c r="G41" s="46" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="48" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="B42" s="48" t="inlineStr">
+        <is>
+          <t>Evidence-of-Absence-Sprachregelung</t>
+        </is>
+      </c>
+      <c r="C42" s="46" t="inlineStr">
+        <is>
+          <t>E1/E2 + D3-BF fixieren die zulässige Formulierung (Pending-C-Input)</t>
+        </is>
+      </c>
+      <c r="D42" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E42" s="48" t="inlineStr"/>
+      <c r="F42" s="46" t="inlineStr"/>
+      <c r="G42" s="46" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="47" t="inlineStr">
+        <is>
+          <t>— Block F — Ausreißer &amp; Einfluss (T4)</t>
+        </is>
+      </c>
+      <c r="B43" s="48" t="inlineStr"/>
+      <c r="C43" s="46" t="inlineStr"/>
+      <c r="D43" s="48" t="inlineStr"/>
+      <c r="E43" s="48" t="inlineStr"/>
+      <c r="F43" s="46" t="inlineStr"/>
+      <c r="G43" s="46" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="48" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B44" s="48" t="inlineStr">
+        <is>
+          <t>Identifikation rstudent</t>
+        </is>
+      </c>
+      <c r="C44" s="46" t="inlineStr">
+        <is>
+          <t>Studentisierte deleted residuals aus dem 3-Ebenen-Modell; Set vollständig berichtet</t>
+        </is>
+      </c>
+      <c r="D44" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E44" s="48" t="inlineStr"/>
+      <c r="F44" s="46" t="inlineStr"/>
+      <c r="G44" s="46" t="inlineStr">
+        <is>
+          <t>Devalle/Drago: geprüft-und-behalten per DEC-013</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="48" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="B45" s="48" t="inlineStr">
+        <is>
+          <t>Drop-and-Refit</t>
+        </is>
+      </c>
+      <c r="C45" s="46" t="inlineStr">
+        <is>
+          <t>Hauptmodell ohne geflaggte Effekte (prominente Robustheitszeile)</t>
+        </is>
+      </c>
+      <c r="D45" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E45" s="48" t="inlineStr"/>
+      <c r="F45" s="46" t="inlineStr"/>
+      <c r="G45" s="46" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="48" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="B46" s="48" t="inlineStr">
+        <is>
+          <t>Winsor/Unwinsor</t>
+        </is>
+      </c>
+      <c r="C46" s="46" t="inlineStr">
+        <is>
+          <t>1./99. Perzentil gestutzt; Sensitivitätspaar, nie primär</t>
+        </is>
+      </c>
+      <c r="D46" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E46" s="48" t="inlineStr"/>
+      <c r="F46" s="46" t="inlineStr"/>
+      <c r="G46" s="46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="48" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="B47" s="48" t="inlineStr">
+        <is>
+          <t>Cluster-LOO</t>
+        </is>
+      </c>
+      <c r="C47" s="46" t="inlineStr">
+        <is>
+          <t>Gesamteffekt je ohne einen der 120 Cluster</t>
+        </is>
+      </c>
+      <c r="D47" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E47" s="48" t="inlineStr"/>
+      <c r="F47" s="46" t="inlineStr"/>
+      <c r="G47" s="46" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="48" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="B48" s="48" t="inlineStr">
+        <is>
+          <t>Einfluss-Diagnostik</t>
+        </is>
+      </c>
+      <c r="C48" s="46" t="inlineStr">
+        <is>
+          <t>Cooks Distance / Hat-Werte (deskriptiver Appendix)</t>
+        </is>
+      </c>
+      <c r="D48" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E48" s="48" t="inlineStr"/>
+      <c r="F48" s="46" t="inlineStr"/>
+      <c r="G48" s="46" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="48" t="inlineStr">
+        <is>
+          <t>F6</t>
+        </is>
+      </c>
+      <c r="B49" s="48" t="inlineStr">
+        <is>
+          <t>MAD-Zweitidentifikation</t>
+        </is>
+      </c>
+      <c r="C49" s="46" t="inlineStr">
+        <is>
+          <t>Leys-konforme MAD-Regel als zweite Identifikationsmethode (outlier_mad)</t>
+        </is>
+      </c>
+      <c r="D49" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E49" s="48" t="inlineStr"/>
+      <c r="F49" s="46" t="inlineStr"/>
+      <c r="G49" s="46" t="inlineStr">
+        <is>
+          <t>±SD und SAMD begründet ausgeschlossen (Leys 2013; DEC-031a.4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="48" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+      <c r="B50" s="48" t="inlineStr">
+        <is>
+          <t>Trimming 1/99</t>
+        </is>
+      </c>
+      <c r="C50" s="46" t="inlineStr">
+        <is>
+          <t>Symmetrisches Trimmen als Gegenstück zum Winsorizing (trim_1_99)</t>
+        </is>
+      </c>
+      <c r="D50" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E50" s="48" t="inlineStr"/>
+      <c r="F50" s="46" t="inlineStr"/>
+      <c r="G50" s="46" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="47" t="inlineStr">
+        <is>
+          <t>— Block G — Zusätzliche Robustheit (Register: Langtabelle vollständig, Text nur Zusätzliches)</t>
+        </is>
+      </c>
+      <c r="B51" s="48" t="inlineStr"/>
+      <c r="C51" s="46" t="inlineStr"/>
+      <c r="D51" s="48" t="inlineStr"/>
+      <c r="E51" s="48" t="inlineStr"/>
+      <c r="F51" s="46" t="inlineStr"/>
+      <c r="G51" s="46" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="48" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="B52" s="48" t="inlineStr">
+        <is>
+          <t>no_starbound</t>
+        </is>
+      </c>
+      <c r="C52" s="46" t="inlineStr">
+        <is>
+          <t>Headline ohne die 99 star-bound-Zeilen (11 Studien)</t>
+        </is>
+      </c>
+      <c r="D52" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E52" s="48" t="inlineStr"/>
+      <c r="F52" s="46" t="inlineStr"/>
+      <c r="G52" s="46" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="48" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="B53" s="48" t="inlineStr">
+        <is>
+          <t>no_nobs_proxyfill</t>
+        </is>
+      </c>
+      <c r="C53" s="46" t="inlineStr">
+        <is>
+          <t>Headline ohne die 297 Proxy-n-Zeilen (inkl. 134 FLAG-basierte, R-19)</t>
+        </is>
+      </c>
+      <c r="D53" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E53" s="48" t="inlineStr"/>
+      <c r="F53" s="46" t="inlineStr"/>
+      <c r="G53" s="46" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="48" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="B54" s="48" t="inlineStr">
+        <is>
+          <t>n_firms_variance</t>
+        </is>
+      </c>
+      <c r="C54" s="46" t="inlineStr">
+        <is>
+          <t>Varianz-/Gewichtungsbasis n_firms statt firm-years (Autor r02f2)</t>
+        </is>
+      </c>
+      <c r="D54" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E54" s="48" t="inlineStr"/>
+      <c r="F54" s="46" t="inlineStr"/>
+      <c r="G54" s="46" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="48" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
+      <c r="B55" s="48" t="inlineStr">
+        <is>
+          <t>direct_r_only</t>
+        </is>
+      </c>
+      <c r="C55" s="46" t="inlineStr">
+        <is>
+          <t>Nur direkt berichtete Korrelationen</t>
+        </is>
+      </c>
+      <c r="D55" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E55" s="48" t="inlineStr"/>
+      <c r="F55" s="46" t="inlineStr"/>
+      <c r="G55" s="46" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="48" t="inlineStr">
+        <is>
+          <t>G5</t>
+        </is>
+      </c>
+      <c r="B56" s="48" t="inlineStr">
+        <is>
+          <t>pcc_df_k10 / k20</t>
+        </is>
+      </c>
+      <c r="C56" s="46" t="inlineStr">
+        <is>
+          <t>Alternative df-Konventionen der PCC-Varianz</t>
+        </is>
+      </c>
+      <c r="D56" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E56" s="48" t="inlineStr"/>
+      <c r="F56" s="46" t="inlineStr"/>
+      <c r="G56" s="46" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="48" t="inlineStr">
+        <is>
+          <t>G6</t>
+        </is>
+      </c>
+      <c r="B57" s="48" t="inlineStr">
+        <is>
+          <t>one_per_cluster_median</t>
+        </is>
+      </c>
+      <c r="C57" s="46" t="inlineStr">
+        <is>
+          <t>Median-Aggregation je Cluster als annahmefreier Zweitcheck</t>
+        </is>
+      </c>
+      <c r="D57" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E57" s="48" t="inlineStr"/>
+      <c r="F57" s="46" t="inlineStr"/>
+      <c r="G57" s="46" t="inlineStr">
+        <is>
+          <t>neu per DEC-031a.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="48" t="inlineStr">
+        <is>
+          <t>G7</t>
+        </is>
+      </c>
+      <c r="B58" s="48" t="inlineStr">
+        <is>
+          <t>Technisches Panel q_VHB</t>
+        </is>
+      </c>
+      <c r="C58" s="46" t="inlineStr">
+        <is>
+          <t>high / low / 99_NCE Subgruppen (Regel D31.4)</t>
+        </is>
+      </c>
+      <c r="D58" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E58" s="48" t="inlineStr"/>
+      <c r="F58" s="46" t="inlineStr"/>
+      <c r="G58" s="46" t="inlineStr">
+        <is>
+          <t>aus C verschoben (DEC-031a.1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="48" t="inlineStr">
+        <is>
+          <t>G8</t>
+        </is>
+      </c>
+      <c r="B59" s="48" t="inlineStr">
+        <is>
+          <t>Technisches Panel field</t>
+        </is>
+      </c>
+      <c r="C59" s="46" t="inlineStr">
+        <is>
+          <t>fin-acc-econ / sust / mgmt</t>
+        </is>
+      </c>
+      <c r="D59" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E59" s="48" t="inlineStr"/>
+      <c r="F59" s="46" t="inlineStr"/>
+      <c r="G59" s="46" t="inlineStr">
+        <is>
+          <t>aus C verschoben</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="48" t="inlineStr">
+        <is>
+          <t>G9</t>
+        </is>
+      </c>
+      <c r="B60" s="48" t="inlineStr">
+        <is>
+          <t>Technisches Panel ES_measure</t>
+        </is>
+      </c>
+      <c r="C60" s="46" t="inlineStr">
+        <is>
+          <t>partiell vs. bivariat</t>
+        </is>
+      </c>
+      <c r="D60" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E60" s="48" t="inlineStr"/>
+      <c r="F60" s="46" t="inlineStr"/>
+      <c r="G60" s="46" t="inlineStr">
+        <is>
+          <t>aus C verschoben</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="48" t="inlineStr">
+        <is>
+          <t>G10</t>
+        </is>
+      </c>
+      <c r="B61" s="48" t="inlineStr">
+        <is>
+          <t>Technisches Panel es_method</t>
+        </is>
+      </c>
+      <c r="C61" s="46" t="inlineStr">
+        <is>
+          <t>Konversionsroute (Methoden-Artefakt-Check); in Unified-Varianten nur Haupteffekt</t>
+        </is>
+      </c>
+      <c r="D61" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E61" s="48" t="inlineStr"/>
+      <c r="F61" s="46" t="inlineStr"/>
+      <c r="G61" s="46" t="inlineStr">
+        <is>
+          <t>aus C verschoben</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="48" t="inlineStr">
+        <is>
+          <t>G11</t>
+        </is>
+      </c>
+      <c r="B62" s="48" t="inlineStr">
+        <is>
+          <t>Spec-Langtabelle (CSV)</t>
+        </is>
+      </c>
+      <c r="C62" s="46" t="inlineStr">
+        <is>
+          <t>Eine Zeile pro Spezifikation (~25), Querverweis-Spalte "reported in §x.y"; Appendix vollständig</t>
+        </is>
+      </c>
+      <c r="D62" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E62" s="48" t="inlineStr"/>
+      <c r="F62" s="46" t="inlineStr"/>
+      <c r="G62" s="46" t="inlineStr">
+        <is>
+          <t>corpus_segment + cluster_study + Provenienz-Specs gestrichen; on-demand hinterlegt</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="47" t="inlineStr">
+        <is>
+          <t>— Block H — Null-Batterie</t>
+        </is>
+      </c>
+      <c r="B63" s="48" t="inlineStr"/>
+      <c r="C63" s="46" t="inlineStr"/>
+      <c r="D63" s="48" t="inlineStr"/>
+      <c r="E63" s="48" t="inlineStr"/>
+      <c r="F63" s="46" t="inlineStr"/>
+      <c r="G63" s="46" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="48" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="B64" s="48" t="inlineStr">
+        <is>
+          <t>MDE-Simulation (N2)</t>
+        </is>
+      </c>
+      <c r="C64" s="46" t="inlineStr">
+        <is>
+          <t>Design-basiert: welche Effektgröße war entdeckbar? tau²-Grid ×{0,5/1/2}, B=5.000, Seed 20260710</t>
+        </is>
+      </c>
+      <c r="D64" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E64" s="48" t="inlineStr"/>
+      <c r="F64" s="46" t="inlineStr"/>
+      <c r="G64" s="46" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="48" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="B65" s="48" t="inlineStr">
+        <is>
+          <t>RoBMA/BF Zarea-informiert (N3)</t>
+        </is>
+      </c>
+      <c r="C65" s="46" t="inlineStr">
+        <is>
+          <t>Bayes-Faktor pro/contra Null; PSMA-Defaults + Zarea-Prior</t>
+        </is>
+      </c>
+      <c r="D65" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E65" s="48" t="inlineStr"/>
+      <c r="F65" s="46" t="inlineStr"/>
+      <c r="G65" s="46" t="inlineStr">
+        <is>
+          <t>PENDING: Zarea-Extraktion (einziger externer Input)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="48" t="inlineStr">
+        <is>
+          <t>H3</t>
+        </is>
+      </c>
+      <c r="B66" s="48" t="inlineStr">
+        <is>
+          <t>Multiverse/Spec-Curve (N5)</t>
+        </is>
+      </c>
+      <c r="C66" s="46" t="inlineStr">
+        <is>
+          <t>~1.400 Spezifikations-Kombinationen; Permutations-Gesamtinferenz B=500</t>
+        </is>
+      </c>
+      <c r="D66" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E66" s="48" t="inlineStr"/>
+      <c r="F66" s="46" t="inlineStr"/>
+      <c r="G66" s="46" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="48" t="inlineStr">
+        <is>
+          <t>H4</t>
+        </is>
+      </c>
+      <c r="B67" s="48" t="inlineStr">
+        <is>
+          <t>Sup-Break (N6)</t>
+        </is>
+      </c>
+      <c r="C67" s="46" t="inlineStr">
+        <is>
+          <t>Stärkster Strukturbruch über Kandidatenjahre 2008–2019 (sup-Wald)</t>
+        </is>
+      </c>
+      <c r="D67" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E67" s="48" t="inlineStr"/>
+      <c r="F67" s="46" t="inlineStr"/>
+      <c r="G67" s="46" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="48" t="inlineStr">
+        <is>
+          <t>H5</t>
+        </is>
+      </c>
+      <c r="B68" s="48" t="inlineStr">
+        <is>
+          <t>Permutations-Inferenz (N7)</t>
+        </is>
+      </c>
+      <c r="C68" s="46" t="inlineStr">
+        <is>
+          <t>Cluster-Label-Permutation B=2.000, Seed 20260710; p_perm neben p_CR2</t>
+        </is>
+      </c>
+      <c r="D68" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E68" s="48" t="inlineStr"/>
+      <c r="F68" s="46" t="inlineStr"/>
+      <c r="G68" s="46" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="48" t="inlineStr">
+        <is>
+          <t>H6</t>
+        </is>
+      </c>
+      <c r="B69" s="48" t="inlineStr">
+        <is>
+          <t>Zarea-Transplantation (N8)</t>
+        </is>
+      </c>
+      <c r="C69" s="46" t="inlineStr">
+        <is>
+          <t>Unsere Daten unter Zarea-Operationalisierung (Mittelpunkt-Regel, Tie-Exklusion)</t>
+        </is>
+      </c>
+      <c r="D69" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E69" s="48" t="inlineStr"/>
+      <c r="F69" s="46" t="inlineStr"/>
+      <c r="G69" s="46" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="48" t="inlineStr">
+        <is>
+          <t>H7</t>
+        </is>
+      </c>
+      <c r="B70" s="48" t="inlineStr">
+        <is>
+          <t>Kumulative MA (N10)</t>
+        </is>
+      </c>
+      <c r="C70" s="46" t="inlineStr">
+        <is>
+          <t>Chronologisch aufkumulierter Effekt — Haupttext-Zeitgrafik</t>
+        </is>
+      </c>
+      <c r="D70" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E70" s="48" t="inlineStr"/>
+      <c r="F70" s="46" t="inlineStr"/>
+      <c r="G70" s="46" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="48" t="inlineStr">
+        <is>
+          <t>H8</t>
+        </is>
+      </c>
+      <c r="B71" s="48" t="inlineStr">
+        <is>
+          <t>Rollierendes Fenster (N11)</t>
+        </is>
+      </c>
+      <c r="C71" s="46" t="inlineStr">
+        <is>
+          <t>Breite 6 J., Schritt 1 J., min. 5 Cluster je Fenster</t>
+        </is>
+      </c>
+      <c r="D71" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E71" s="48" t="inlineStr"/>
+      <c r="F71" s="46" t="inlineStr"/>
+      <c r="G71" s="46" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="48" t="inlineStr">
+        <is>
+          <t>H9</t>
+        </is>
+      </c>
+      <c r="B72" s="48" t="inlineStr">
+        <is>
+          <t>Externer Differenztest (N12)</t>
+        </is>
+      </c>
+      <c r="C72" s="46" t="inlineStr">
+        <is>
+          <t>Vergleich gegen COE-Companion-Effekt (ein Satz)</t>
+        </is>
+      </c>
+      <c r="D72" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E72" s="48" t="inlineStr"/>
+      <c r="F72" s="46" t="inlineStr"/>
+      <c r="G72" s="46" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="48" t="inlineStr">
+        <is>
+          <t>H10</t>
+        </is>
+      </c>
+      <c r="B73" s="48" t="inlineStr">
+        <is>
+          <t>p-Curve konditional (N13)</t>
+        </is>
+      </c>
+      <c r="C73" s="46" t="inlineStr">
+        <is>
+          <t>Nur falls ≥5 signifikante Post-Studien; sonst "infeasible" berichtet</t>
+        </is>
+      </c>
+      <c r="D73" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E73" s="48" t="inlineStr"/>
+      <c r="F73" s="46" t="inlineStr"/>
+      <c r="G73" s="46" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="48" t="inlineStr">
+        <is>
+          <t>H11</t>
+        </is>
+      </c>
+      <c r="B74" s="48" t="inlineStr">
+        <is>
+          <t>Within-Study-Display (N15)</t>
+        </is>
+      </c>
+      <c r="C74" s="46" t="inlineStr">
+        <is>
+          <t>Studien mit eigenen Prä- UND Post-Effekten deskriptiv nebeneinander</t>
+        </is>
+      </c>
+      <c r="D74" s="48" t="inlineStr">
+        <is>
+          <t>offen</t>
+        </is>
+      </c>
+      <c r="E74" s="48" t="inlineStr"/>
+      <c r="F74" s="46" t="inlineStr"/>
+      <c r="G74" s="46" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -4979,50 +7189,40 @@
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="44" t="inlineStr">
+      <c r="A2" s="45" t="inlineStr">
+        <is>
+          <t>SUPERSEDED 2026-07-10: aktueller Analyse-Plan + Tracking im Sheet "Analyse_Batterie" (per DEC-031/031a). Diese Übersicht (Daten-Status v4) bleibt als Archiv.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="44" t="inlineStr">
         <is>
           <t>Block / Analyse</t>
         </is>
       </c>
-      <c r="B2" s="44" t="inlineStr">
+      <c r="B3" s="44" t="inlineStr">
         <is>
           <t>Split</t>
         </is>
       </c>
-      <c r="C2" s="44" t="inlineStr">
+      <c r="C3" s="44" t="inlineStr">
         <is>
           <t>Status (Daten v4)</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="43" t="inlineStr">
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="43" t="inlineStr">
         <is>
           <t>1 — Main</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="41" t="inlineStr">
-        <is>
-          <t>Forest Plot</t>
-        </is>
-      </c>
-      <c r="B4" s="41" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C4" s="41" t="inlineStr">
-        <is>
-          <t>ready</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
       <c r="A5" s="41" t="inlineStr">
         <is>
-          <t>Overall</t>
+          <t>Forest Plot</t>
         </is>
       </c>
       <c r="B5" s="41" t="inlineStr">
@@ -5039,48 +7239,48 @@
     <row r="6" ht="28" customHeight="1">
       <c r="A6" s="41" t="inlineStr">
         <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="B6" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C6" s="41" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="41" t="inlineStr">
+        <is>
           <t>Overall Pre/Post</t>
         </is>
       </c>
-      <c r="B6" s="41" t="inlineStr">
+      <c r="B7" s="41" t="inlineStr">
         <is>
           <t>pre/post</t>
         </is>
       </c>
-      <c r="C6" s="41" t="inlineStr">
+      <c r="C7" s="41" t="inlineStr">
         <is>
           <t>ready</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="43" t="inlineStr">
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="43" t="inlineStr">
         <is>
           <t>2 — Robustheit: Parametrisierung</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="41" t="inlineStr">
-        <is>
-          <t>Pre/Post Lag 1/2/3</t>
-        </is>
-      </c>
-      <c r="B8" s="41" t="inlineStr">
-        <is>
-          <t>pre/post</t>
-        </is>
-      </c>
-      <c r="C8" s="41" t="inlineStr">
-        <is>
-          <t>ready (pp_share_lag1–3)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
       <c r="A9" s="41" t="inlineStr">
         <is>
-          <t>Event-Cut: median / end / start</t>
+          <t>Pre/Post Lag 1/2/3</t>
         </is>
       </c>
       <c r="B9" s="41" t="inlineStr">
@@ -5090,14 +7290,14 @@
       </c>
       <c r="C9" s="41" t="inlineStr">
         <is>
-          <t>ready (pp_median/end/start)</t>
+          <t>ready (pp_share_lag1–3)</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
       <c r="A10" s="41" t="inlineStr">
         <is>
-          <t>Outlier: drop-outliers/-contributors · cap · SAMD(2×,3×) · SD · winsor · trim</t>
+          <t>Event-Cut: median / end / start</t>
         </is>
       </c>
       <c r="B10" s="41" t="inlineStr">
@@ -5107,14 +7307,14 @@
       </c>
       <c r="C10" s="41" t="inlineStr">
         <is>
-          <t>ready (R)</t>
+          <t>ready (pp_median/end/start)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
       <c r="A11" s="41" t="inlineStr">
         <is>
-          <t>Effektgröße: drop bivariate</t>
+          <t>Outlier: drop-outliers/-contributors · cap · SAMD(2×,3×) · SD · winsor · trim</t>
         </is>
       </c>
       <c r="B11" s="41" t="inlineStr">
@@ -5124,14 +7324,14 @@
       </c>
       <c r="C11" s="41" t="inlineStr">
         <is>
-          <t>ready (ES_measure)</t>
+          <t>ready (R)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="41" t="inlineStr">
         <is>
-          <t>Modell-Spez. (FE/RE/…)</t>
+          <t>Effektgröße: drop bivariate</t>
         </is>
       </c>
       <c r="B12" s="41" t="inlineStr">
@@ -5141,14 +7341,14 @@
       </c>
       <c r="C12" s="41" t="inlineStr">
         <is>
-          <t>ready (R)</t>
+          <t>ready (ES_measure)</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="41" t="inlineStr">
         <is>
-          <t>Study-Level</t>
+          <t>Modell-Spez. (FE/RE/…)</t>
         </is>
       </c>
       <c r="B13" s="41" t="inlineStr">
@@ -5158,14 +7358,14 @@
       </c>
       <c r="C13" s="41" t="inlineStr">
         <is>
-          <t>ready (R-Aggregation)</t>
+          <t>ready (R)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="A14" s="41" t="inlineStr">
         <is>
-          <t>Firm-Years</t>
+          <t>Study-Level</t>
         </is>
       </c>
       <c r="B14" s="41" t="inlineStr">
@@ -5175,14 +7375,14 @@
       </c>
       <c r="C14" s="41" t="inlineStr">
         <is>
-          <t>ready (no_firm-years)</t>
+          <t>ready (R-Aggregation)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="28" customHeight="1">
       <c r="A15" s="41" t="inlineStr">
         <is>
-          <t>Quality: Status / VHB / JIF / Field</t>
+          <t>Firm-Years</t>
         </is>
       </c>
       <c r="B15" s="41" t="inlineStr">
@@ -5192,103 +7392,103 @@
       </c>
       <c r="C15" s="41" t="inlineStr">
         <is>
-          <t>ready (v4)</t>
+          <t>ready (no_firm-years)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="28" customHeight="1">
       <c r="A16" s="41" t="inlineStr">
         <is>
+          <t>Quality: Status / VHB / JIF / Field</t>
+        </is>
+      </c>
+      <c r="B16" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C16" s="41" t="inlineStr">
+        <is>
+          <t>ready (v4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="41" t="inlineStr">
+        <is>
           <t>Quality: CIT</t>
         </is>
       </c>
-      <c r="B16" s="41" t="inlineStr">
+      <c r="B17" s="41" t="inlineStr">
         <is>
           <t>pre/post</t>
         </is>
       </c>
-      <c r="C16" s="41" t="inlineStr">
+      <c r="C17" s="41" t="inlineStr">
         <is>
           <t>GESTRICHEN (DEC-023)</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="43" t="inlineStr">
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="43" t="inlineStr">
         <is>
           <t>3 — Robustheit: Underlying Trend (T8)</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="41" t="inlineStr">
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="41" t="inlineStr">
         <is>
           <t>Secular-Trend / Identifikation</t>
         </is>
       </c>
-      <c r="B18" s="41" t="inlineStr">
+      <c r="B19" s="41" t="inlineStr">
         <is>
           <t>kont. Zeit</t>
         </is>
       </c>
-      <c r="C18" s="41" t="inlineStr">
+      <c r="C19" s="41" t="inlineStr">
         <is>
           <t>ready (sample_mid, DEC-021)</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="43" t="inlineStr">
+    <row r="20" ht="28" customHeight="1">
+      <c r="A20" s="43" t="inlineStr">
         <is>
           <t>4 — Publication Bias</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="28" customHeight="1">
-      <c r="A20" s="41" t="inlineStr">
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="41" t="inlineStr">
         <is>
           <t>Funnel · FAT-PET-PEESE · Trim&amp;Fill · 3PSM · p-curve/p-uniform · RoBMA</t>
         </is>
       </c>
-      <c r="B20" s="41" t="inlineStr">
+      <c r="B21" s="41" t="inlineStr">
         <is>
           <t>overall/subgruppen</t>
         </is>
       </c>
-      <c r="C20" s="41" t="inlineStr">
+      <c r="C21" s="41" t="inlineStr">
         <is>
           <t>ready (R; RoBMA-Paket)</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="43" t="inlineStr">
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="43" t="inlineStr">
         <is>
           <t>5 — Moderatoren</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="41" t="inlineStr">
-        <is>
-          <t>CER-Measure (perf/discl)</t>
-        </is>
-      </c>
-      <c r="B22" s="41" t="inlineStr">
-        <is>
-          <t>pre/post</t>
-        </is>
-      </c>
-      <c r="C22" s="41" t="inlineStr">
-        <is>
-          <t>ready</t>
         </is>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="41" t="inlineStr">
         <is>
-          <t>COD-Instrument (loan/rating/bond/deriv)</t>
+          <t>CER-Measure (perf/discl)</t>
         </is>
       </c>
       <c r="B23" s="41" t="inlineStr">
@@ -5305,7 +7505,7 @@
     <row r="24" ht="28" customHeight="1">
       <c r="A24" s="41" t="inlineStr">
         <is>
-          <t>Industrie (sensitive/non-sensitive)</t>
+          <t>COD-Instrument (loan/rating/bond/deriv)</t>
         </is>
       </c>
       <c r="B24" s="41" t="inlineStr">
@@ -5322,7 +7522,7 @@
     <row r="25" ht="28" customHeight="1">
       <c r="A25" s="41" t="inlineStr">
         <is>
-          <t>Country: Region · Development · Culture · Legal</t>
+          <t>Industrie (sensitive/non-sensitive)</t>
         </is>
       </c>
       <c r="B25" s="41" t="inlineStr">
@@ -5332,46 +7532,63 @@
       </c>
       <c r="C25" s="41" t="inlineStr">
         <is>
-          <t>ready (v4, 4 Schemata + NCE)</t>
+          <t>ready</t>
         </is>
       </c>
     </row>
     <row r="26" ht="28" customHeight="1">
       <c r="A26" s="41" t="inlineStr">
         <is>
+          <t>Country: Region · Development · Culture · Legal</t>
+        </is>
+      </c>
+      <c r="B26" s="41" t="inlineStr">
+        <is>
+          <t>pre/post</t>
+        </is>
+      </c>
+      <c r="C26" s="41" t="inlineStr">
+        <is>
+          <t>ready (v4, 4 Schemata + NCE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="41" t="inlineStr">
+        <is>
           <t>Regulierung (ETS/CT)</t>
         </is>
       </c>
-      <c r="B26" s="41" t="inlineStr">
+      <c r="B27" s="41" t="inlineStr">
         <is>
           <t>pre/post</t>
         </is>
       </c>
-      <c r="C26" s="41" t="inlineStr">
+      <c r="C27" s="41" t="inlineStr">
         <is>
           <t>ready</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="43" t="inlineStr">
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="43" t="inlineStr">
         <is>
           <t>6 — Regression (T7)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="41" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="41" t="inlineStr">
         <is>
           <t>Unified Meta-Regression</t>
         </is>
       </c>
-      <c r="B28" s="41" t="inlineStr">
+      <c r="B29" s="41" t="inlineStr">
         <is>
           <t>kont. + Interaktionen</t>
         </is>
       </c>
-      <c r="C28" s="41" t="inlineStr">
+      <c r="C29" s="41" t="inlineStr">
         <is>
           <t>ready</t>
         </is>
@@ -5391,13 +7608,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -6575,12 +8792,19 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-10: Alle N-Inputs a priori fixiert per DEC-031 Annex H (Seeds 20260710, B-Werte, Grids, SESOI 0,070/0,05, N13-Regel). Einziger externer Pending: Zarea-Prior (N3). Tracking: Sheet "Analyse_Batterie", Block H.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10347,7 +12571,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11297,341 +13521,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Identifikation: Bruch vs. Trend — Werkzeugkasten gegen den Saekulartrend-Confound (#13 / T8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Problem: Pre/Post-Dummy trennt Bruch nicht von Drift. Daten zeigen Drift (Pre-median r=−0,025 vs. Post r=−0,019). Strategie: Trend modellieren, Paris muss DARUEBER HINAUS liefern.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>Move</t>
-        </is>
-      </c>
-      <c r="B3" s="8" t="inlineStr">
-        <is>
-          <t>Staerke-Tier</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Was es testet / leistet</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
-          <t>Methode</t>
-        </is>
-      </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>Datenabhaengigkeit</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>Praezedenz / Anker</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="84" customHeight="1">
-      <c r="A4" s="27" t="inlineStr">
-        <is>
-          <t>1. Trend-vs-Bruch-Wettrennen</t>
-        </is>
-      </c>
-      <c r="B4" s="28" t="inlineStr">
-        <is>
-          <t>Tier 1 — essenziell, sofort</t>
-        </is>
-      </c>
-      <c r="C4" s="27" t="inlineStr">
-        <is>
-          <t>Trennt glatte Drift vom diskreten Level-Sprung. Dummy weg → nur Drift; ueberlebt → echte Diskontinuitaet</t>
-        </is>
-      </c>
-      <c r="D4" s="27" t="inlineStr">
-        <is>
-          <t>Kont. Zeit (zentr. Midpoint) + Paris-Dummy im SELBEN sparsamen Modell</t>
-        </is>
-      </c>
-      <c r="E4" s="27" t="inlineStr">
-        <is>
-          <t>Sofort — sobald T0.4 kont. Zeit liefert</t>
-        </is>
-      </c>
-      <c r="F4" s="27" t="inlineStr">
-        <is>
-          <t>Huang 2020 (pub-year-Control neben GFC)</t>
-        </is>
-      </c>
-      <c r="G4" s="27" t="inlineStr">
-        <is>
-          <t>OFFEN (T0.4-abh.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="84" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
-        <is>
-          <t>2. Segmentierte Meta-Regression (ITS)</t>
-        </is>
-      </c>
-      <c r="B5" s="28" t="inlineStr">
-        <is>
-          <t>Tier 1 — essenziell, sofort</t>
-        </is>
-      </c>
-      <c r="C5" s="27" t="inlineStr">
-        <is>
-          <t>β₂ Level-Sprung, β₃ Slope-Aenderung. Nistet reinen Trend vs. Bruch als testbare Spezialfaelle</t>
-        </is>
-      </c>
-      <c r="D5" s="27" t="inlineStr">
-        <is>
-          <t>effect ~ β₀+β₁·Zeit+β₂·post+β₃·(Zeit×post); RVE</t>
-        </is>
-      </c>
-      <c r="E5" s="27" t="inlineStr">
-        <is>
-          <t>Sofort — T0.4-abh.</t>
-        </is>
-      </c>
-      <c r="F5" s="27" t="inlineStr">
-        <is>
-          <t>ITS-Standard; COVID-Wellen-Analogon</t>
-        </is>
-      </c>
-      <c r="G5" s="27" t="inlineStr">
-        <is>
-          <t>OFFEN (T0.4-abh.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="84" customHeight="1">
-      <c r="A6" s="29" t="inlineStr">
-        <is>
-          <t>3. Placebo-/Falsifikations-Bruchdaten</t>
-        </is>
-      </c>
-      <c r="B6" s="30" t="inlineStr">
-        <is>
-          <t>Tier 2 — stark</t>
-        </is>
-      </c>
-      <c r="C6" s="29" t="inlineStr">
-        <is>
-          <t>Bruch an Nicht-Paris-Jahren (2012/13/17/18). Ueberall → kein Paris-Bruch; nur 2015/16 → echt. DEUTET LAG1–3 ZU FALSIFIKATION UM</t>
-        </is>
-      </c>
-      <c r="D6" s="29" t="inlineStr">
-        <is>
-          <t>Bruch-Magnitude je Cutoff; Lokalisierungs-Vergleich</t>
-        </is>
-      </c>
-      <c r="E6" s="29" t="inlineStr">
-        <is>
-          <t>Sofort — T0.4-abh.</t>
-        </is>
-      </c>
-      <c r="F6" s="29" t="inlineStr">
-        <is>
-          <t>Placebo-Test-Standard</t>
-        </is>
-      </c>
-      <c r="G6" s="29" t="inlineStr">
-        <is>
-          <t>OFFEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="84" customHeight="1">
-      <c r="A7" s="29" t="inlineStr">
-        <is>
-          <t>4. Kompositions-Kontrolle</t>
-        </is>
-      </c>
-      <c r="B7" s="30" t="inlineStr">
-        <is>
-          <t>Tier 2 — stark, sofort</t>
-        </is>
-      </c>
-      <c r="C7" s="29" t="inlineStr">
-        <is>
-          <t>Haelt Studien-/Laender-/Instrument-Mix konstant; Within-Stratum-Check. Nur im Aggregat → kompositorisch</t>
-        </is>
-      </c>
-      <c r="D7" s="29" t="inlineStr">
-        <is>
-          <t>Paris-Term + Moderatoren als Kovariaten (= T7); Within-Stratum</t>
-        </is>
-      </c>
-      <c r="E7" s="29" t="inlineStr">
-        <is>
-          <t>Sofort (= T7)</t>
-        </is>
-      </c>
-      <c r="F7" s="29" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G7" s="29" t="inlineStr">
-        <is>
-          <t>OFFEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="84" customHeight="1">
-      <c r="A8" s="29" t="inlineStr">
-        <is>
-          <t>5. Differential-Exposure (DiD-artig)</t>
-        </is>
-      </c>
-      <c r="B8" s="30" t="inlineStr">
-        <is>
-          <t>Tier 2 — stark</t>
-        </is>
-      </c>
-      <c r="C8" s="29" t="inlineStr">
-        <is>
-          <t>(post−pre) High-Exposure minus (post−pre) Low: gemeinsamer Trend differenziert sich heraus</t>
-        </is>
-      </c>
-      <c r="D8" s="29" t="inlineStr">
-        <is>
-          <t>post × High-Exposure (carbon-intensiv / Carbon-Pricing); Pre-Trend-Check</t>
-        </is>
-      </c>
-      <c r="E8" s="29" t="inlineStr">
-        <is>
-          <t>Sofort; Pre-Trend datenabh.</t>
-        </is>
-      </c>
-      <c r="F8" s="29" t="inlineStr">
-        <is>
-          <t>DiD-Logik. CAVEAT: Parallel-Trends unpruefbar</t>
-        </is>
-      </c>
-      <c r="G8" s="29" t="inlineStr">
-        <is>
-          <t>OFFEN</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="84" customHeight="1">
-      <c r="A9" s="31" t="inlineStr">
-        <is>
-          <t>6. Within-Study-Identifikation</t>
-        </is>
-      </c>
-      <c r="B9" s="32" t="inlineStr">
-        <is>
-          <t>Tier 3 — Goldstandard, DATENBEDINGT TOT</t>
-        </is>
-      </c>
-      <c r="C9" s="31" t="inlineStr">
-        <is>
-          <t>Studien, die Bruch SELBST ueberspannen + separate Pre/Post. Haelt alle between-Confounder konstant</t>
-        </is>
-      </c>
-      <c r="D9" s="31" t="inlineStr">
-        <is>
-          <t>Within-Study-Pre/Post-Kontrast</t>
-        </is>
-      </c>
-      <c r="E9" s="31" t="inlineStr">
-        <is>
-          <t>NICHT VERFUEGBAR — nur 1–3/66 Studien ueberspannen</t>
-        </is>
-      </c>
-      <c r="F9" s="31" t="inlineStr">
-        <is>
-          <t>COVID within-cohort (Sun, Robinson)</t>
-        </is>
-      </c>
-      <c r="G9" s="31" t="inlineStr">
-        <is>
-          <t>ENTFAELLT (Datenbefund T0.3)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="84" customHeight="1">
-      <c r="A10" s="17" t="inlineStr">
-        <is>
-          <t>7. Sensitivitaets-Schranke (Bounding)</t>
-        </is>
-      </c>
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>Tier 4 — Schlussklammer</t>
-        </is>
-      </c>
-      <c r="C10" s="17" t="inlineStr">
-        <is>
-          <t>Wie gross muesste ein Trend sein, um verbleibenden Paris-Dummy zu erklaeren. Begrenzt Confound explizit</t>
-        </is>
-      </c>
-      <c r="D10" s="17" t="inlineStr">
-        <is>
-          <t>Oster-Bounds / E-Value auf finales Modell</t>
-        </is>
-      </c>
-      <c r="E10" s="17" t="inlineStr">
-        <is>
-          <t>Sofort (nach Hauptmodell)</t>
-        </is>
-      </c>
-      <c r="F10" s="17" t="inlineStr">
-        <is>
-          <t>Oster 2019; E-Value (VanderWeele 2017)</t>
-        </is>
-      </c>
-      <c r="G10" s="17" t="inlineStr">
-        <is>
-          <t>OFFEN</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Status hotfix: estimation-set counts in active rows (2,713; 115 studies/114 clusters in A1/A7/A8/F4), Move-6 reference cell canonical (73/72/1), Datenagenda #36 (COE overlap refresh on final corpus)
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -5145,7 +5145,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="45" t="inlineStr">
         <is>
@@ -5209,7 +5208,7 @@
       </c>
       <c r="C5" s="46" t="inlineStr">
         <is>
-          <t>Gepoolter Gesamteffekt: Drei-Ebenen-MA über 2.714 Effekte, Fisher-z-PCC (van Aert 2023), rho=0,6, CR2 auf cluster_id</t>
+          <t>Gepoolter Gesamteffekt: Drei-Ebenen-MA über 2.713 Effekte (115 Studien / 114 Cluster), Fisher-z-PCC (van Aert 2023), rho=0,6, CR2 auf cluster_id</t>
         </is>
       </c>
       <c r="D5" s="48" t="inlineStr">
@@ -5367,7 +5366,7 @@
       </c>
       <c r="C11" s="46" t="inlineStr">
         <is>
-          <t>Alle 120 Cluster-Aggregate sortiert, ohne Labels, Pooled+PI-Referenzlinien (Appendix)</t>
+          <t>Alle 114 Cluster-Aggregate sortiert, ohne Labels, Pooled+PI-Referenzlinien (Appendix)</t>
         </is>
       </c>
       <c r="D11" s="48" t="inlineStr">
@@ -5392,7 +5391,7 @@
       </c>
       <c r="C12" s="46" t="inlineStr">
         <is>
-          <t>120 beschriftete Studien-Aggregate mit CI, gepoolte Referenzlinie (Appendix, ganzseitig)</t>
+          <t>115 beschriftete Studien-Aggregate mit CI, gepoolte Referenzlinie (Appendix, ganzseitig)</t>
         </is>
       </c>
       <c r="D12" s="48" t="inlineStr">
@@ -6271,7 +6270,7 @@
       </c>
       <c r="C48" s="46" t="inlineStr">
         <is>
-          <t>Gesamteffekt je ohne einen der 120 Cluster</t>
+          <t>Gesamteffekt je ohne einen der 114 Cluster</t>
         </is>
       </c>
       <c r="D48" s="48" t="inlineStr">
@@ -11958,7 +11957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -12914,6 +12913,28 @@
       <c r="F37" t="inlineStr">
         <is>
           <t>geparkt (Manuskriptphase; Pending-C-Input); Zahlen kanonisch (T0.4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>COE-Overlap-Refresh auf finalem 120er-Korpus: Overlap-Disclosure (DEC-031b-Note, N12) basiert auf 5/66-Analyse (DEC-026); mit 54 Neuzugängen gegen die 75 COE-Studien neu prüfen (Studien- und ES-Ebene)</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Claude -&gt; Robert</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>offen (vor Manuskript-Methods; billig, deterministisch aus beiden Studienlisten)</t>
         </is>
       </c>
     </row>
@@ -13210,7 +13231,7 @@
       </c>
       <c r="E10" s="31" t="inlineStr">
         <is>
-          <t>NICHT VERFUEGBAR — nur 1–3/66 Studien ueberspannen</t>
+          <t>NICHT VERFÜGBAR als Identifikation — kanonisch (T0.4): 73/115 Studien überspannen den Bruch, 72 poolen darüber, genau 1 splittet (Li et al 2022) → N15/H11 = Ein-Studien-Exhibit; Intro-Baustein #35</t>
         </is>
       </c>
       <c r="F10" s="31" t="inlineStr">

</xml_diff>

<commit_message>
T1 complete: canonical run (verifier 21/21) + Block A results workbook (SOMA template, 13 tabs) + manuscript/T1.md + status tracker update
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -734,7 +734,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Update 2026-07-12: v12 kanonisch (DEC-042, Commit 63356a7) · Analyse-Batterie fixiert (DEC-031/031a; 031b/042a pending im T0.4-Paket) · T0.4 in Ausführung (Gate 1 bestanden). Alte v4-Zeile ersetzt.</t>
+          <t>Update 2026-07-12: v12 kanonisch (DEC-042, Commit 63356a7) · Analyse-Batterie fixiert (DEC-031/031a; 031b/042a pending im T0.4-Paket) · T0.4 in Ausführung (Gate 1 bestanden). Alte v4-Zeile ersetzt. · Update 2026-07-13: T1/Block A abgeschlossen (CC kanonisch, Verifier 21/21; DEC-012a + DEC-042b geloggt; F53–F57 geschlossen); Results-Workbook-Template etabliert (13 Tabs, SOMA-Muster); Konvention bestaetigt: EIN Workbook je LAUF (Block B =&gt; T2- und T8-Workbook getrennt).</t>
         </is>
       </c>
     </row>
@@ -1419,12 +1419,12 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>r = -0,059 [-0,086; -0,031]; PI [-0,390; +0,287]; df 111,7; p &lt; 0,0001; 2.713 ES / 115 St. / 114 Cluster</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>output/T1_results.csv</t>
+          <t>output/T1_results.csv; output/T1_results_workbook.xlsx</t>
         </is>
       </c>
     </row>
@@ -1436,23 +1436,31 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>prae -0,060 [-0,098; -0,022] (1.994 ES/83 St.) · post -0,049 [-0,066; -0,031] (711 ES/31 St.); deskriptiv, Test = B1; 8 ES ohne Fenster raus [DEC-042b]</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>output/T1_results.csv</t>
+          <t>output/T1_results.csv; output/T1_results_workbook.xlsx Tab 8</t>
         </is>
       </c>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>T3 · Heterogenitaet (σ²_within/between, ICC, I²)</t>
-        </is>
-      </c>
-      <c r="B8" s="36" t="n"/>
-      <c r="C8" s="35" t="n"/>
+          <t>T1/A2 · Heterogenitaet (sigma2 je Ebene, Anteile)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>62,3% Cluster / ~0% Studie (Boundary) / 37,5% ES / 0,1% Sampling</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>output/T1_results.csv (A2); Workbook Tab 7</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
@@ -1567,10 +1575,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A8:C8"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
@@ -1584,7 +1591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1606,7 +1613,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>45 Methodik-DECs (append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>47 Methodik-DECs (append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -2892,6 +2899,80 @@
       <c r="B49" t="inlineStr">
         <is>
           <t>Volker-Liste E1–E4 geschlossen; Schätzmenge 2.713 fixiert; R-19 final</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>DEC-012a</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Oekonomische Uebersetzung operationalisiert (Instrument-Mediane)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>#9 / T1,A6</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Extraktionsregel fixiert: Median-SD(COD) je Instrument (loan/bond/CDS) via Volker-Task; Grid-Platzhalter PENDING; Ratio-Zeile konstantenfrei</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>aktiv (Konstanten pending)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>DEC-042b</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Daten/Design</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Perioden-Zellen-Domaene: 8 ES / 2 Studien ohne Fenster</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>T1/A3; Block B</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>NA = Design-Fakt; listenweise nur aus Perioden-/Dosis-Zellen (prae+post = 2.705); Schaetzmenge 2.713 unveraendert</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>aktiv</t>
         </is>
       </c>
     </row>
@@ -2933,7 +3014,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="45" t="inlineStr">
         <is>
-          <t>STAND 2026-07-10: Datenphase abgeschlossen (v12 kanonisch, DEC-042) · Batterie fixiert (DEC-031/031a) · Schritt 2 = T0.4-Prep (Review-Gate) als Nächstes · Detailplan je Analyse: Sheet "Analyse_Batterie"</t>
+          <t>STAND 2026-07-10: Datenphase abgeschlossen (v12 kanonisch, DEC-042) · Batterie fixiert (DEC-031/031a) · Schritt 2 = T0.4-Prep (Review-Gate) als Nächstes · Detailplan je Analyse: Sheet "Analyse_Batterie" · STAND 2026-07-13: T1/Block A abgeschlossen (Verifier 21/21; DEC-012a/042b; F53–F57)</t>
         </is>
       </c>
     </row>
@@ -3066,7 +3147,7 @@
       </c>
       <c r="D6" s="41" t="inlineStr">
         <is>
-          <t>Prep R/00_prep.R gegen data/CER-COD_data_v12.xlsx; Verifier v2 (28 Checks); design_quantities_v12.csv — IN AUSFÜHRUNG (Gate 1 bestanden, kanonischer CC-Lauf läuft)</t>
+          <t>Prep R/00_prep.R gegen data/CER-COD_data_v12.xlsx; Verifier v2 (28 Checks); design_quantities_v12.csv — ERLEDIGT (kanonisch 2026-07-12, Verifier 28/28)</t>
         </is>
       </c>
       <c r="E6" s="41" t="inlineStr">
@@ -3081,7 +3162,7 @@
       </c>
       <c r="G6" s="41" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt</t>
         </is>
       </c>
     </row>
@@ -3118,7 +3199,7 @@
       </c>
       <c r="G7" s="41" t="inlineStr">
         <is>
-          <t>gated</t>
+          <t>in Ausführung (Block A/T1 erledigt 2026-07-13; B–H offen)</t>
         </is>
       </c>
     </row>
@@ -3455,6 +3536,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="43" t="inlineStr">
         <is>
@@ -4693,22 +4775,22 @@
       </c>
       <c r="H8" s="25" t="inlineStr">
         <is>
-          <t>OFFEN</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="I8" s="26" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DONE 2026-07-13: kanonischer CC-Lauf, Verifier 21/21 (nach 2 spec-konformen STOPs: S2-&gt;DEC-042b, S3-&gt;F57); Rulings F53-F57 geschlossen; DEC-012a geloggt (Konstanten pending); Ergebnisse: Analyse_Batterie A1-A8 + Key_Results; Commit-Hash nachtragen</t>
         </is>
       </c>
       <c r="J8" s="26" t="inlineStr">
         <is>
-          <t>R/NN_t1_main + R/NN_verify · output/T1_results.csv · manuscript/T1.md</t>
+          <t>R/01_core.R + R/01_verify_outputs.R · output/T1_results.csv · output/T1_results_workbook.xlsx · manuscript/T1.md · docs/cc_prompt_T1.md</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>NÄCHSTER SCHRITT (Gate 2: Diff-Review)</t>
+          <t>erledigt (21/21, 2026-07-13)</t>
         </is>
       </c>
     </row>
@@ -5213,11 +5295,19 @@
       </c>
       <c r="D5" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E5" s="48" t="inlineStr"/>
-      <c r="F5" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-13, Verifier 21/21)</t>
+        </is>
+      </c>
+      <c r="E5" s="48" t="inlineStr">
+        <is>
+          <t>output/T1_results.csv; output/T1_results_workbook.xlsx Tab 6; R/01_core.R; manuscript/T1.md</t>
+        </is>
+      </c>
+      <c r="F5" s="46" t="inlineStr">
+        <is>
+          <t>r = -0,059 [-0,086; -0,031], df 111,7, p &lt; 0,0001; 0,84x Doucouliagos-small</t>
+        </is>
+      </c>
       <c r="G5" s="46" t="inlineStr"/>
     </row>
     <row r="6">
@@ -5238,11 +5328,19 @@
       </c>
       <c r="D6" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E6" s="48" t="inlineStr"/>
-      <c r="F6" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-13, Verifier 21/21)</t>
+        </is>
+      </c>
+      <c r="E6" s="48" t="inlineStr">
+        <is>
+          <t>output/T1_results_workbook.xlsx Tab 7</t>
+        </is>
+      </c>
+      <c r="F6" s="46" t="inlineStr">
+        <is>
+          <t>62,3% Cluster / ~0% Studie (Boundary) / 37,5% ES / 0,1% Sampling; typ. v 4,3e-05</t>
+        </is>
+      </c>
       <c r="G6" s="46" t="inlineStr"/>
     </row>
     <row r="7">
@@ -5263,12 +5361,24 @@
       </c>
       <c r="D7" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E7" s="48" t="inlineStr"/>
-      <c r="F7" s="46" t="inlineStr"/>
-      <c r="G7" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-13, Verifier 21/21)</t>
+        </is>
+      </c>
+      <c r="E7" s="48" t="inlineStr">
+        <is>
+          <t>output/T1_results_workbook.xlsx Tab 8</t>
+        </is>
+      </c>
+      <c r="F7" s="46" t="inlineStr">
+        <is>
+          <t>PI gesamt [-0,390; +0,287] (vorzeicheninklusiv); prae -0,060 (83 St.) vs. post -0,049 (31 St.), deskriptiv</t>
+        </is>
+      </c>
+      <c r="G7" s="46" t="inlineStr">
+        <is>
+          <t>8 ES / 2 Studien ohne Fenster listenweise nur aus Periodenzellen [DEC-042b]; Test = B1</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="48" t="inlineStr">
@@ -5288,11 +5398,19 @@
       </c>
       <c r="D8" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E8" s="48" t="inlineStr"/>
-      <c r="F8" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-13, Verifier 21/21)</t>
+        </is>
+      </c>
+      <c r="E8" s="48" t="inlineStr">
+        <is>
+          <t>output/T1_results_workbook.xlsx Tab 9</t>
+        </is>
+      </c>
+      <c r="F8" s="46" t="inlineStr">
+        <is>
+          <t>rho 0,4/0,8: -0,059/-0,058 -- invariant</t>
+        </is>
+      </c>
       <c r="G8" s="46" t="inlineStr">
         <is>
           <t>Register-Zeilen in G-Langtabelle</t>
@@ -5317,14 +5435,22 @@
       </c>
       <c r="D9" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E9" s="48" t="inlineStr"/>
-      <c r="F9" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-13, Verifier 21/21)</t>
+        </is>
+      </c>
+      <c r="E9" s="48" t="inlineStr">
+        <is>
+          <t>output/T1_results_workbook.xlsx Tab 9</t>
+        </is>
+      </c>
+      <c r="F9" s="46" t="inlineStr">
+        <is>
+          <t>OPC -0,062 (KnHa df 113); UWLS+3 -0,031; HS -0,022; WAAP -0,031 (704/2.713 powered, 26%)</t>
+        </is>
+      </c>
       <c r="G9" s="46" t="inlineStr">
         <is>
-          <t>FE/RE-Dichotomie im Text adressiert, nicht als Zeile (DEC-031a.4e)</t>
+          <t>FE/RE-Dichotomie im Text adressiert, nicht als Zeile (DEC-031a.4e) · F57: UWLS/WAAP df 2,3/2,2 disclosed (Top-Cluster 37,9% Gewicht); CIs unter df 4 unzuverlaessig (Tipton)</t>
         </is>
       </c>
     </row>
@@ -5346,12 +5472,24 @@
       </c>
       <c r="D10" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E10" s="48" t="inlineStr"/>
-      <c r="F10" s="46" t="inlineStr"/>
-      <c r="G10" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-13, Verifier 21/21)</t>
+        </is>
+      </c>
+      <c r="E10" s="48" t="inlineStr">
+        <is>
+          <t>output/T1_results_workbook.xlsx Tab 10</t>
+        </is>
+      </c>
+      <c r="F10" s="46" t="inlineStr">
+        <is>
+          <t>Platzhalter-Grid: -5,9/-8,8/-11,7 bp je 1 SD CER (SD 100/150/200); Ratio 0,84x small (konstantenfrei)</t>
+        </is>
+      </c>
+      <c r="G10" s="46" t="inlineStr">
+        <is>
+          <t>Manuskriptzeile BLOCKED bis DEC-012a-Konstanten (Volker-Extraktion, Instrument-Mediane)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="48" t="inlineStr">
@@ -5371,11 +5509,19 @@
       </c>
       <c r="D11" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E11" s="48" t="inlineStr"/>
-      <c r="F11" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-13, Verifier 21/21)</t>
+        </is>
+      </c>
+      <c r="E11" s="48" t="inlineStr">
+        <is>
+          <t>output/figures/T1_A7_caterpillar_cluster.pdf|.png</t>
+        </is>
+      </c>
+      <c r="F11" s="46" t="inlineStr">
+        <is>
+          <t>erstellt (Appendix; Pooled- + PI-Linien)</t>
+        </is>
+      </c>
       <c r="G11" s="46" t="inlineStr"/>
     </row>
     <row r="12">
@@ -5396,11 +5542,19 @@
       </c>
       <c r="D12" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E12" s="48" t="inlineStr"/>
-      <c r="F12" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-13, Verifier 21/21)</t>
+        </is>
+      </c>
+      <c r="E12" s="48" t="inlineStr">
+        <is>
+          <t>output/figures/T1_A8_forest_study.pdf</t>
+        </is>
+      </c>
+      <c r="F12" s="46" t="inlineStr">
+        <is>
+          <t>erstellt (Appendix, A4-ganzseitig, 115 Studien)</t>
+        </is>
+      </c>
       <c r="G12" s="46" t="inlineStr"/>
     </row>
     <row r="13">
@@ -11957,7 +12111,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -12885,7 +13039,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>T0.4 ERLEDIGT (kanonisch 2026-07-12); NÄCHSTER SCHRITT: T1-Dry-Run (Gate 2)</t>
+          <t>T0.4 ERLEDIGT (kanonisch 2026-07-12); T1 ERLEDIGT (21/21, 2026-07-13); weiter blockweise (B als Naechstes)</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -12935,6 +13089,28 @@
       <c r="F38" t="inlineStr">
         <is>
           <t>offen (vor Manuskript-Methods; billig, deterministisch aus beiden Studienlisten)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>DEC-012a-Extraktion: SD(COD)-Benchmarks je Instrument (loan/bond/CDS) -- Median ueber alle Korpus-Studien mit berichteter SD in bp-konvertierbaren Einheiten (Regel fixiert; Task-Text in DEC-012a)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Volker</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>offen (entsperrt Manuskript-A6-Zeile / TB-08)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T2 complete: Paris moderation = precise null (diff_z +0.010, p=0.582; 10 codings, 31 LOSO, disclosures) + results workbook + manuscript/T2.md + status update incl. T1 hash back-fill
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -734,7 +734,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Update 2026-07-12: v12 kanonisch (DEC-042, Commit 63356a7) · Analyse-Batterie fixiert (DEC-031/031a; 031b/042a pending im T0.4-Paket) · T0.4 in Ausführung (Gate 1 bestanden). Alte v4-Zeile ersetzt. · Update 2026-07-13: T1/Block A abgeschlossen (CC kanonisch, Verifier 21/21; DEC-012a + DEC-042b geloggt; F53–F57 geschlossen); Results-Workbook-Template etabliert (13 Tabs, SOMA-Muster); Konvention bestaetigt: EIN Workbook je LAUF (Block B =&gt; T2- und T8-Workbook getrennt).</t>
+          <t>Update 2026-07-12: v12 kanonisch (DEC-042, Commit 63356a7) · Analyse-Batterie fixiert (DEC-031/031a; 031b/042a pending im T0.4-Paket) · T0.4 in Ausführung (Gate 1 bestanden). Alte v4-Zeile ersetzt. · Update 2026-07-13: T1/Block A abgeschlossen (CC kanonisch, Verifier 21/21; DEC-012a + DEC-042b geloggt; F53–F57 geschlossen); Results-Workbook-Template etabliert (13 Tabs, SOMA-Muster); Konvention bestaetigt: EIN Workbook je LAUF (Block B =&gt; T2- und T8-Workbook getrennt). · Update 2026-07-14: T2 abgeschlossen (Standard-Loop bewaehrt: S4-Erratum-Fang F58, Audit 0 Findings, 17/17); T1-Hashes nachgetragen (ce5d80b ff.).</t>
         </is>
       </c>
     </row>
@@ -1479,12 +1479,12 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>B1 diff_z = +0,010 [-0,028; +0,049], p=0,582 (df 15,0) -- Paris-Moderation null; alle 10 Kodierungen null (max |diff| 0,040 ns); clean_window -0,013 ns; LOSO-Range 0,011; Panjwani 22,8%/23,9% disclosed</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>output/T2_results.csv</t>
+          <t>output/T2_results.csv; output/T2_results_workbook.xlsx</t>
         </is>
       </c>
     </row>
@@ -1576,9 +1576,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A13:C13"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A13:C13"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3014,7 +3014,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="45" t="inlineStr">
         <is>
-          <t>STAND 2026-07-10: Datenphase abgeschlossen (v12 kanonisch, DEC-042) · Batterie fixiert (DEC-031/031a) · Schritt 2 = T0.4-Prep (Review-Gate) als Nächstes · Detailplan je Analyse: Sheet "Analyse_Batterie" · STAND 2026-07-13: T1/Block A abgeschlossen (Verifier 21/21; DEC-012a/042b; F53–F57)</t>
+          <t>STAND 2026-07-10: Datenphase abgeschlossen (v12 kanonisch, DEC-042) · Batterie fixiert (DEC-031/031a) · Schritt 2 = T0.4-Prep (Review-Gate) als Nächstes · Detailplan je Analyse: Sheet "Analyse_Batterie" · STAND 2026-07-13: T1/Block A abgeschlossen (Verifier 21/21; DEC-012a/042b; F53–F57) · STAND 2026-07-14: T2 abgeschlossen (17/17; Paris-Moderation = praeziser Null); naechster Schritt T8 (Gate 2)</t>
         </is>
       </c>
     </row>
@@ -3536,7 +3536,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="43" t="inlineStr">
         <is>
@@ -4780,7 +4779,7 @@
       </c>
       <c r="I8" s="26" t="inlineStr">
         <is>
-          <t>DONE 2026-07-13: kanonischer CC-Lauf, Verifier 21/21 (nach 2 spec-konformen STOPs: S2-&gt;DEC-042b, S3-&gt;F57); Rulings F53-F57 geschlossen; DEC-012a geloggt (Konstanten pending); Ergebnisse: Analyse_Batterie A1-A8 + Key_Results; Commit-Hash nachtragen</t>
+          <t>DONE 2026-07-13: kanonischer CC-Lauf, Verifier 21/21 (nach 2 spec-konformen STOPs: S2-&gt;DEC-042b, S3-&gt;F57); Rulings F53-F57 geschlossen; DEC-012a geloggt (Konstanten pending); Ergebnisse: Analyse_Batterie A1-A8 + Key_Results; Commits: a054e29/6e34f06/5075ddb (Skripte+DECs), ce5d80b (Outputs+Workbook+Status)</t>
         </is>
       </c>
       <c r="J8" s="26" t="inlineStr">
@@ -4812,7 +4811,7 @@
       </c>
       <c r="D9" s="26" t="inlineStr">
         <is>
-          <t>End · Median@2015/16 · Mean · Lags · (opt.) Stringency in EINEM Driver → Long-CSV mit spec-Spalte; Headline fixieren.</t>
+          <t>Paris-Kodierungsschicht per Batterie B1/B3/B6/B7 [DEC-024/031a.9; ersetzt Alt-Beschreibung End/Median/Mean/Stringency]: pp_mid headline · tie_break · end_any · Share-Recuts 17-19 · End-Lags 1-3 (Appendix) · clean_window (volle Inferenz) · Post-LOSO 31 · Dominanz · 3 Disclosures</t>
         </is>
       </c>
       <c r="E9" s="25" t="inlineStr">
@@ -4832,22 +4831,22 @@
       </c>
       <c r="H9" s="25" t="inlineStr">
         <is>
-          <t>OFFEN</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="I9" s="26" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>DONE 2026-07-14: CC Standard-Loop (Build aus docs/T2_spec.md Rev. 2026-07-13b, F58-Erratum vorab via STOP S4; 7-Agenten-Konformitaets-Audit 0 Findings), Verifier 17/17; Paris-Moderation = praeziser Null (diff_z +0,010, p=0,582); P1-P5-Pins empirisch bestaetigt; Commit-Hash nachtragen</t>
         </is>
       </c>
       <c r="J9" s="26" t="inlineStr">
         <is>
-          <t>R/NN_t2_eventcode + _verify · output/T2_results.csv · manuscript/T2.md</t>
+          <t>R/02_paris.R + R/02_verify_outputs.R · output/T2_results.csv · output/T2_results_workbook.xlsx · manuscript/T2.md · docs/T2_spec.md · docs/cc_prompt_T2.md</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (17/17, 2026-07-14)</t>
         </is>
       </c>
     </row>
@@ -5227,6 +5226,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="45" t="inlineStr">
         <is>
@@ -5588,14 +5588,22 @@
       </c>
       <c r="D14" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E14" s="48" t="inlineStr"/>
-      <c r="F14" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-14, Verifier 17/17)</t>
+        </is>
+      </c>
+      <c r="E14" s="48" t="inlineStr">
+        <is>
+          <t>output/T2_results_workbook.xlsx Tab 6; output/T2_results.csv; R/02_paris.R; manuscript/T2.md</t>
+        </is>
+      </c>
+      <c r="F14" s="46" t="inlineStr">
+        <is>
+          <t>diff_z = +0,010 [-0,028; +0,049], t(15,0)=0,56, p=0,582 -- praeziser Null; Zellen: prae r=-0,062 (1.994/83), post r=-0,051 (711/31)</t>
+        </is>
+      </c>
       <c r="G14" s="46" t="inlineStr">
         <is>
-          <t>df(pp_mid)=31,9 → Transfer-Regel greift NICHT, Binär trägt volle Inferenz; Post-Zelle 31 Studien (kanonisch bestätigt, T0.4 v2 28/28, 2026-07-12)</t>
+          <t>df(pp_mid)=31,9 → Transfer-Regel greift NICHT, Binär trägt volle Inferenz; Post-Zelle 31 Studien (kanonisch bestätigt, T0.4 v2 28/28, 2026-07-12) · realisierte Kontrast-df 15,0 vs. Design-df 31,9 (disclosed; beide &gt; Tipton-Boden); Zellmittel vs. A3 = Estimanden-Unterschied (gemeinsames Modell)</t>
         </is>
       </c>
     </row>
@@ -5642,14 +5650,22 @@
       </c>
       <c r="D16" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E16" s="48" t="inlineStr"/>
-      <c r="F16" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-14, Verifier 17/17)</t>
+        </is>
+      </c>
+      <c r="E16" s="48" t="inlineStr">
+        <is>
+          <t>output/T2_results_workbook.xlsx Tab 7</t>
+        </is>
+      </c>
+      <c r="F16" s="46" t="inlineStr">
+        <is>
+          <t>alle 9 Varianten null: tie +0,010 · Recuts 17/18/19 +0,008/+0,003/+0,004 · end-Familie -0,019..+0,040 (Appendix-Lags) · clean_window -0,013 [-0,049;+0,023], df 23,5 (volle Inferenz)</t>
+        </is>
+      </c>
       <c r="G16" s="46" t="inlineStr">
         <is>
-          <t>Upgrade GEFEUERT (kanonisch): clean-window df=12,3 ≥ 5 → volle Inferenz (DEC-031a.5; design_quantities_v12.csv)</t>
+          <t>Upgrade GEFEUERT (kanonisch): clean-window df=12,3 ≥ 5 → volle Inferenz (DEC-031a.5; design_quantities_v12.csv) · kein Kollaps ('collapse = finding' verneint); Vorzeichen-Heterogenitaet um null = kein systematischer Shift; end-Familie durch 66%-Kontamination erklaert (B7)</t>
         </is>
       </c>
     </row>
@@ -5721,11 +5737,19 @@
       </c>
       <c r="D19" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E19" s="48" t="inlineStr"/>
-      <c r="F19" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-14, Verifier 17/17)</t>
+        </is>
+      </c>
+      <c r="E19" s="48" t="inlineStr">
+        <is>
+          <t>output/T2_results_workbook.xlsx Tabs 8-9</t>
+        </is>
+      </c>
+      <c r="F19" s="46" t="inlineStr">
+        <is>
+          <t>LOSO-Range 0,011 z (alle 31 Diffs +0,002..+0,014, alle ns; min: drop Li 2022, max: drop Brinette 2026); Dominanz: Panjwani 22,8% Gewicht / 23,9% ES (Memo bestaetigt), Top-3 ~44%</t>
+        </is>
+      </c>
       <c r="G19" s="46" t="inlineStr"/>
     </row>
     <row r="20">
@@ -5746,12 +5770,24 @@
       </c>
       <c r="D20" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E20" s="48" t="inlineStr"/>
-      <c r="F20" s="46" t="inlineStr"/>
-      <c r="G20" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-14, Verifier 17/17)</t>
+        </is>
+      </c>
+      <c r="E20" s="48" t="inlineStr">
+        <is>
+          <t>output/T2_results_workbook.xlsx Tab 10</t>
+        </is>
+      </c>
+      <c r="F20" s="46" t="inlineStr">
+        <is>
+          <t>Attenuation end 66,0% (1.383/2.094 ES; 56 St.; vorher ~81%) · knife-edge 2,9% (79 ES/5 St. = Tie-Menge) · panel drift +0,015 (0,358 vs 0,343)</t>
+        </is>
+      </c>
+      <c r="G20" s="46" t="inlineStr">
+        <is>
+          <t>v12-kanonisch; traegt Kodierungs-Verteidigung (TB-16/17/18)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">

</xml_diff>

<commit_message>
T8 complete (verifier 27/27 @ 76074a2): canonical outputs + results workbook (TB-20..28) + manuscript/T8.md; status B2/B4/B5/B8 done, DecisionLog-Index +4, 20a4e90 backfills; cc_prompt output-contract fix
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1591,7 +1591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1613,7 +1613,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>47 Methodik-DECs (append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>51 Methodik-DECs (append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -2971,6 +2971,154 @@
         </is>
       </c>
       <c r="G51" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>DEC-024a</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Placebo-Recode-Regel share_Y 2008–2015 (schließt F60)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>T8 / B4</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Kanonische share_Y-Formel, ties→Post; 2016-Identity-Gate; Zellen als Konstanten gepinnt</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>DEC-031c</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Pre-Trend-Guard Move 5: M-pre einziger präreg. Zusatz (schließt F59; Ruling R2)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>T7 / C3,C4</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>M-full + Stratum-Segmentierung on-demand; D31.5-Panelform unangetastet; C4-df-Schutz</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>DEC-031d</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>B5-Kovariatenset = 3 kategoriale von 5 §6-Drifts (schließt F61)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>T8 / B5,B8</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>{region, instrument, CER}; Kanal-Zuweisung window/n; Oster-Paar race/trend_comp; Read-out Δβ+CI vs SESOI</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>DEC-031e</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>T8-Execution-Amendment: break_only Cell-Means; fit3l ~1 (schließt S5-Halt)</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>T8 / B4</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>nlminb-Falschkonvergenz an σ²_study-Boundary; T2/B1-Konvention; Zertifikate in run_meta; F62 eröffnet</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
         <is>
           <t>aktiv</t>
         </is>
@@ -5226,7 +5374,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="45" t="inlineStr">
         <is>
@@ -5593,7 +5740,7 @@
       </c>
       <c r="E14" s="48" t="inlineStr">
         <is>
-          <t>output/T2_results_workbook.xlsx Tab 6; output/T2_results.csv; R/02_paris.R; manuscript/T2.md</t>
+          <t>output/T2_results_workbook.xlsx Tab 6; output/T2_results.csv; R/02_paris.R; manuscript/T2.md @ 20a4e90</t>
         </is>
       </c>
       <c r="F14" s="46" t="inlineStr">
@@ -5625,12 +5772,24 @@
       </c>
       <c r="D15" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E15" s="48" t="inlineStr"/>
-      <c r="F15" s="46" t="inlineStr"/>
-      <c r="G15" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-15, Verifier 27/27)</t>
+        </is>
+      </c>
+      <c r="E15" s="48" t="inlineStr">
+        <is>
+          <t>output/T8_results_workbook.xlsx Tabs 7–10; output/T8_results.csv @ 76074a2</t>
+        </is>
+      </c>
+      <c r="F15" s="46" t="inlineStr">
+        <is>
+          <t>Slope +0,052 (p=,271); Kontrast 0→0,6 +0,031 [−0,026;+0,088]; Quadrat p=,332; Joint p=,207 — kein Dosis-Gradient</t>
+        </is>
+      </c>
+      <c r="G15" s="46" t="inlineStr">
+        <is>
+          <t>z̄ bei 2015,5: −0,087→−0,035; corr(mid,share)=0,8146 (A.9/D2); Joint-Support-Caveat z̄(1); Bewertung via Offset (CENTER=2012,258)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="48" t="inlineStr">
@@ -5655,7 +5814,7 @@
       </c>
       <c r="E16" s="48" t="inlineStr">
         <is>
-          <t>output/T2_results_workbook.xlsx Tab 7</t>
+          <t>output/T2_results_workbook.xlsx Tab 7 @ 20a4e90</t>
         </is>
       </c>
       <c r="F16" s="46" t="inlineStr">
@@ -5687,12 +5846,24 @@
       </c>
       <c r="D17" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E17" s="48" t="inlineStr"/>
-      <c r="F17" s="46" t="inlineStr"/>
-      <c r="G17" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-15, Verifier 27/27)</t>
+        </is>
+      </c>
+      <c r="E17" s="48" t="inlineStr">
+        <is>
+          <t>output/T8_results_workbook.xlsx Tabs 7–10; output/T8_results.csv @ 76074a2</t>
+        </is>
+      </c>
+      <c r="F17" s="46" t="inlineStr">
+        <is>
+          <t>Race Doppel-Null: Trend −0,0024/J (p=,113), Bruch +0,026 [−0,026;+0,079] (p=,306); Placebo-Rang 2016 = 7/9 (|b| 2009–11: 0,033–0,040); Segment-Joint p=,525</t>
+        </is>
+      </c>
+      <c r="G17" s="46" t="inlineStr">
+        <is>
+          <t>break_only Cell-Means per DEC-031e (O15-Identität ~1e-16); realisierte df 15,0 vs Design 31,9; Race-CI-Rand +0,079 &gt; SESOI — Präzisionsgrenze offengelegt (F61-P3)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="48" t="inlineStr">
@@ -5712,12 +5883,24 @@
       </c>
       <c r="D18" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E18" s="48" t="inlineStr"/>
-      <c r="F18" s="46" t="inlineStr"/>
-      <c r="G18" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-15, Verifier 27/27)</t>
+        </is>
+      </c>
+      <c r="E18" s="48" t="inlineStr">
+        <is>
+          <t>output/T8_results_workbook.xlsx Tabs 7–10; output/T8_results.csv @ 76074a2</t>
+        </is>
+      </c>
+      <c r="F18" s="46" t="inlineStr">
+        <is>
+          <t>Δβ = +0,002; adj. pp +0,012 [−0,025;+0,050] (df 14,2) bzw. +0,014 [−0,024;+0,052] (df 19,2); Komp.-Walds p≈,3</t>
+        </is>
+      </c>
+      <c r="G18" s="46" t="inlineStr">
+        <is>
+          <t>Set {region, instrument, CER} per DEC-031d; Read-out Δβ+CI vs SESOI-Band (F61-P3); beide CIs in ±0,070; trend_comp-Rand +0,052 marginal über ±0,05</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="48" t="inlineStr">
@@ -5742,7 +5925,7 @@
       </c>
       <c r="E19" s="48" t="inlineStr">
         <is>
-          <t>output/T2_results_workbook.xlsx Tabs 8-9</t>
+          <t>output/T2_results_workbook.xlsx Tabs 8-9 @ 20a4e90</t>
         </is>
       </c>
       <c r="F19" s="46" t="inlineStr">
@@ -5775,7 +5958,7 @@
       </c>
       <c r="E20" s="48" t="inlineStr">
         <is>
-          <t>output/T2_results_workbook.xlsx Tab 10</t>
+          <t>output/T2_results_workbook.xlsx Tab 10 @ 20a4e90</t>
         </is>
       </c>
       <c r="F20" s="46" t="inlineStr">
@@ -5807,13 +5990,22 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="F21" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-15, Verifier 27/27)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>output/T8_results_workbook.xlsx Tabs 7–10; output/T8_results.csv @ 76074a2</t>
+        </is>
+      </c>
+      <c r="F21" s="46" t="inlineStr">
+        <is>
+          <t>β*(δ=1)=+0,012; δ*=9,28 (Caveat: nahe Null instabil); E-Values Punkt 1,19 · CI-Rand 1,43 · Mask 1,42/1,53; R²u=−0,015/R²c=+0,010</t>
+        </is>
+      </c>
       <c r="G21" s="46" t="inlineStr">
         <is>
-          <t>Schlussklammer der T8-Verteidigung; läuft nach dem Hauptmodell</t>
+          <t>Oster-Paar race vs trend_composition (F61-P1); pseudo-R² negativ möglich (REML); Schlussklammer — Gewicht liegt auf Race+Placebos+Komposition</t>
         </is>
       </c>
     </row>
@@ -5932,7 +6124,11 @@
       </c>
       <c r="E26" s="48" t="inlineStr"/>
       <c r="F26" s="46" t="inlineStr"/>
-      <c r="G26" s="46" t="inlineStr"/>
+      <c r="G26" s="46" t="inlineStr">
+        <is>
+          <t>DEC-031c: M-pre (Pre-Trend-Guard) präregistriert; M-full/Stratum-Seg. on-demand — expected-descriptive (3 Post-Cl)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="48" t="inlineStr">
@@ -5957,7 +6153,11 @@
       </c>
       <c r="E27" s="48" t="inlineStr"/>
       <c r="F27" s="46" t="inlineStr"/>
-      <c r="G27" s="46" t="inlineStr"/>
+      <c r="G27" s="46" t="inlineStr">
+        <is>
+          <t>DEC-031c: M-pre (Pre-Trend-Guard) präregistriert; M-full/Stratum-Seg. on-demand — Move-5-Gewicht hier (14/6/11 Post-Cl)</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="48" t="inlineStr">

</xml_diff>

<commit_message>
T5 (Block D komplett): Ergebnisse + 13-Tab-Workbook (recalced) + Status-Touch (Z11/Z12, Index 53, D-Zeilen, D3->H2) + ERROR_LOG #1-#9; refs DEC-031g/031f/031a.5/016/010
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1496,12 +1496,12 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>Trend −0,0024/J (p=0,113) · Bruch 2016 +0,026 [−0,026; +0,079] (p=0,306) · Placebo-Rang 2016: 7/9 (|b| 2009–11: 0,033–0,040) · Segment-Joint p=0,525 · Dosis: Slope +0,052 (p=0,271), Kontrast 0→0,6 +0,031 [−0,026; +0,088], Joint p=0,207 · Komposition: Δβ +0,002, adj. pp +0,012 [−0,025; +0,050] · Bounding: β*(δ=1)=+0,012, δ*=9,28, E-Value 1,19/CI-Rand 1,43, Masks 1,42/1,53 — Verdict-Text: Pending-C</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>output/T8_results.csv</t>
+          <t>output/T8_results.csv; output/T8_results_workbook.xlsx @ 62d80d4</t>
         </is>
       </c>
     </row>
@@ -1513,12 +1513,12 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>PET −0,043 [−0,076; −0,010] (p=0,011) → Regel: PEESE −0,055 [−0,084; −0,027] (p=0,0002) · FAT −0,64 (p=0,050) · 3PSM μ +0,012 [−0,071; +0,094] (δ=0,49, LRT p=0,025) · p-uniform* +0,012 [−0,069; +0,098] · Prä/Post-PEESE −0,058/−0,045 · Grey-Kontrast +0,002 (p=0,928) — Verdict-Text: Pending-C</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>output/T5_results.csv</t>
+          <t>output/T5_results.csv; output/T5_results_workbook.xlsx (Lauf-Basis @ 6bf40b1)</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1613,7 +1613,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>51 Methodik-DECs (append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>53 Methodik-DECs (append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -3121,6 +3121,70 @@
       <c r="G55" t="inlineStr">
         <is>
           <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>DEC-031f</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Konvergenzprotokoll 3L-RVE-Spine: Optimizer-Ladder, Zertifikate, R6-Kontrollfit (schließt F62)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>alle Spine-Läufe</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>nlminb→BFGS→Nelder-Mead, first-certified-wins; Fallback-Flags; Toleranzen 1e-5/1e-6; Addendum A.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>DEC-031g</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>T5/Block-D-Execution-Spec: 3PSM-Basis RE/ML (F63), puniform-Lockfile (F64), A5-Anker-Protokoll (F65), D5-Zellen-Pin, D3→H</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>T5 / D1,D2,D4,D5,D6</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>P-T5-1..5; Richtungs-Pins less/left; not_estimable-Signaturliste; A.12; F-Register leer (nächste F66)</t>
         </is>
       </c>
     </row>
@@ -6319,11 +6383,19 @@
       </c>
       <c r="D34" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E34" s="48" t="inlineStr"/>
-      <c r="F34" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-19, Verifier 27/27)</t>
+        </is>
+      </c>
+      <c r="E34" s="48" t="inlineStr">
+        <is>
+          <t>output/T5_results_workbook.xlsx Tab 6; output/T5_results.csv @ 6bf40b1 (Lauf-Basis)</t>
+        </is>
+      </c>
+      <c r="F34" s="46" t="inlineStr">
+        <is>
+          <t>PET −0,043 [−0,076; −0,010] (p=,011) → Regel: PEESE −0,055 [−0,084; −0,027] (p=,0002); FAT −0,64 (p=,050 — Grenze); r(PEESE) −0,055</t>
+        </is>
+      </c>
       <c r="G34" s="46" t="inlineStr"/>
     </row>
     <row r="35">
@@ -6344,11 +6416,19 @@
       </c>
       <c r="D35" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E35" s="48" t="inlineStr"/>
-      <c r="F35" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-19, Verifier 27/27)</t>
+        </is>
+      </c>
+      <c r="E35" s="48" t="inlineStr">
+        <is>
+          <t>output/T5_results_workbook.xlsx Tab 7; output/T5_results.csv @ 6bf40b1 (Lauf-Basis)</t>
+        </is>
+      </c>
+      <c r="F35" s="46" t="inlineStr">
+        <is>
+          <t>3PSM μ +0,012 [−0,071; +0,094] (δ=0,49; LRT p=,025); p-uniform* +0,012 [−0,069; +0,098]; τ² ~0,069; unadj. −0,062; Anker OPC −0,062 (df 113) repliziert (O13–O15)</t>
+        </is>
+      </c>
       <c r="G35" s="46" t="inlineStr">
         <is>
           <t>Trim-and-Fill begründet ausgeschlossen (Carter et al. 2019; DEC-031a.4)</t>
@@ -6373,7 +6453,7 @@
       </c>
       <c r="D36" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>offen (→ H2 per DEC-031g)</t>
         </is>
       </c>
       <c r="E36" s="48" t="inlineStr"/>
@@ -6402,11 +6482,19 @@
       </c>
       <c r="D37" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E37" s="48" t="inlineStr"/>
-      <c r="F37" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-19, Verifier 27/27)</t>
+        </is>
+      </c>
+      <c r="E37" s="48" t="inlineStr">
+        <is>
+          <t>output/T5_results_workbook.xlsx Tab 8; output/T5_results.csv @ 6bf40b1 (Lauf-Basis)</t>
+        </is>
+      </c>
+      <c r="F37" s="46" t="inlineStr">
+        <is>
+          <t>Regel → PEESE beidseitig: prä −0,058 (PET p=,0497 — knife-edge) · post −0,045 (PET p=,0098); FAT prä p=,162 / post −1,24 (p=,0047); 3PSM prä −0,022 (LRT p=,309) / post −0,006 (LRT p=,080)</t>
+        </is>
+      </c>
       <c r="G37" s="46" t="inlineStr">
         <is>
           <t>Upgrade GEFEUERT (kanonisch): Post-Zelle 31 ≥ 20 Studien → 3PSM/p-uniform* im Split (DEC-031a.5)</t>
@@ -6431,11 +6519,19 @@
       </c>
       <c r="D38" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E38" s="48" t="inlineStr"/>
-      <c r="F38" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-19, Verifier 27/27)</t>
+        </is>
+      </c>
+      <c r="E38" s="48" t="inlineStr">
+        <is>
+          <t>output/T5_results_workbook.xlsx Tab 9; output/T5_results.csv @ 6bf40b1 (Lauf-Basis)</t>
+        </is>
+      </c>
+      <c r="F38" s="46" t="inlineStr">
+        <is>
+          <t>Kontrast NP−P +0,002 [−0,054; +0,059], t(17,1), p=,928 — präziser Null; Zellen publ. −0,059 (2.033/101/100) vs. WP −0,057 (680/14/14)</t>
+        </is>
+      </c>
       <c r="G38" s="46" t="inlineStr">
         <is>
           <t>aus C verschoben (DEC-031a.1)</t>
@@ -6460,11 +6556,19 @@
       </c>
       <c r="D39" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E39" s="48" t="inlineStr"/>
-      <c r="F39" s="46" t="inlineStr"/>
+          <t>DRAFT (2026-07-19) — RoBMA-Zeile BLOCKED bis H2</t>
+        </is>
+      </c>
+      <c r="E39" s="48" t="inlineStr">
+        <is>
+          <t>output/T5_results_workbook.xlsx Tab 10</t>
+        </is>
+      </c>
+      <c r="F39" s="46" t="inlineStr">
+        <is>
+          <t>mechanisch: unadj. −0,062 · PET −0,043 · PEESE −0,055 · 3PSM +0,012 · p-uni* +0,012 · Grey-Null; alle korrigierten Punkte im SESOI-Band |r|=0,070; RoBMA ausstehend (H2) — Einordnung Pending-C</t>
+        </is>
+      </c>
       <c r="G39" s="46" t="inlineStr"/>
     </row>
     <row r="40">

</xml_diff>

<commit_message>
DEC-044 (Pending-C resolved: Framing A): Claim-Leiter + N1/N3-Sprach-Gate; Status: Kurzerklaerung-Spalte, Index 54, Z11/Z12- und D6-Verdicts; refs DEC-044/031g/031/005
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1496,7 +1496,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Trend −0,0024/J (p=0,113) · Bruch 2016 +0,026 [−0,026; +0,079] (p=0,306) · Placebo-Rang 2016: 7/9 (|b| 2009–11: 0,033–0,040) · Segment-Joint p=0,525 · Dosis: Slope +0,052 (p=0,271), Kontrast 0→0,6 +0,031 [−0,026; +0,088], Joint p=0,207 · Komposition: Δβ +0,002, adj. pp +0,012 [−0,025; +0,050] · Bounding: β*(δ=1)=+0,012, δ*=9,28, E-Value 1,19/CI-Rand 1,43, Masks 1,42/1,53 — Verdict-Text: Pending-C</t>
+          <t>Trend −0,0024/J (p=0,113) · Bruch 2016 +0,026 [−0,026; +0,079] (p=0,306) · Placebo-Rang 2016: 7/9 (|b| 2009–11: 0,033–0,040) · Segment-Joint p=0,525 · Dosis: Slope +0,052 (p=0,271), Kontrast 0→0,6 +0,031 [−0,026; +0,088], Joint p=0,207 · Komposition: Δβ +0,002, adj. pp +0,012 [−0,025; +0,050] · Bounding: β*(δ=1)=+0,012, δ*=9,28, E-Value 1,19/CI-Rand 1,43, Masks 1,42/1,53 — Verdict: A per DEC-044 (Sprachkalibrierung nach N1/N3)</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>PET −0,043 [−0,076; −0,010] (p=0,011) → Regel: PEESE −0,055 [−0,084; −0,027] (p=0,0002) · FAT −0,64 (p=0,050) · 3PSM μ +0,012 [−0,071; +0,094] (δ=0,49, LRT p=0,025) · p-uniform* +0,012 [−0,069; +0,098] · Prä/Post-PEESE −0,058/−0,045 · Grey-Kontrast +0,002 (p=0,928) — Verdict-Text: Pending-C</t>
+          <t>PET −0,043 [−0,076; −0,010] (p=0,011) → Regel: PEESE −0,055 [−0,084; −0,027] (p=0,0002) · FAT −0,64 (p=0,050) · 3PSM μ +0,012 [−0,071; +0,094] (δ=0,49, LRT p=0,025) · p-uniform* +0,012 [−0,069; +0,098] · Prä/Post-PEESE −0,058/−0,045 · Grey-Kontrast +0,002 (p=0,928) — Verdict: A per DEC-044 (Sprachkalibrierung nach N1/N3)</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1591,7 +1591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1613,7 +1613,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>53 Methodik-DECs (append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>54 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -3185,6 +3185,38 @@
       <c r="F57" t="inlineStr">
         <is>
           <t>P-T5-1..5; Richtungs-Pins less/left; not_estimable-Signaturliste; A.12; F-Register leer (nächste F66)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>DEC-044</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Framing</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Pending-C resolved: Framing A (null/debunking) mit zweistufiger Claim-Leiter; Sprach-Gate N1/N3</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Manuskript / Ablauf 3b</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Paris-Null hart; Pooled "negligible, not null" (CI-Rand &gt; SESOI); C -&gt; Boundary-Conditions; T7 = Heterogenitäts-Exploration in A</t>
         </is>
       </c>
     </row>
@@ -5419,7 +5451,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5429,6 +5461,7 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
     <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="72" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5472,6 +5505,11 @@
       <c r="G3" s="45" t="inlineStr">
         <is>
           <t>Anmerkung allgemein</t>
+        </is>
+      </c>
+      <c r="H3" s="45" t="inlineStr">
+        <is>
+          <t>Kurzerklärung (einfach)</t>
         </is>
       </c>
     </row>
@@ -5520,6 +5558,11 @@
         </is>
       </c>
       <c r="G5" s="46" t="inlineStr"/>
+      <c r="H5" s="46" t="inlineStr">
+        <is>
+          <t>Über alle Studien ist der Zusammenhang negativ, aber sehr klein (r=−0,059) — unter der Schwelle für ökonomische Bedeutsamkeit (0,07). Statistisch nachweisbar, praktisch nahe null. Zwischen den Studien schwankt der Effekt allerdings stark.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="48" t="inlineStr">
@@ -5553,6 +5596,11 @@
         </is>
       </c>
       <c r="G6" s="46" t="inlineStr"/>
+      <c r="H6" s="46" t="inlineStr">
+        <is>
+          <t>Die Unterschiede liegen fast komplett zwischen den Studien-Clustern (62 %) und innerhalb von Studien (38 %), kaum im Zufallsrauschen. Heißt: Die Studien messen wirklich Unterschiedliches — was das erklärt, prüfen die Moderator-Analysen.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="48" t="inlineStr">
@@ -5590,6 +5638,11 @@
           <t>8 ES / 2 Studien ohne Fenster listenweise nur aus Periodenzellen [DEC-042b]; Test = B1</t>
         </is>
       </c>
+      <c r="H7" s="46" t="inlineStr">
+        <is>
+          <t>Das Vorhersageintervall reicht von deutlich negativ bis deutlich positiv [−0,39; +0,29]: Eine einzelne neue Studie kann jedes Vorzeichen finden. Prä (−0,060) und post (−0,049) unterscheiden sich kaum.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="48" t="inlineStr">
@@ -5627,6 +5680,11 @@
           <t>Register-Zeilen in G-Langtabelle</t>
         </is>
       </c>
+      <c r="H8" s="46" t="inlineStr">
+        <is>
+          <t>Die technische Annahme, wie stark Ergebnisse innerhalb eines Clusters zusammenhängen (ρ), ändert praktisch nichts: −0,059 vs. −0,058. Das Hauptergebnis ist gegen diese Stellschraube robust.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="48" t="inlineStr">
@@ -5664,6 +5722,11 @@
           <t>FE/RE-Dichotomie im Text adressiert, nicht als Zeile (DEC-031a.4e) · F57: UWLS/WAAP df 2,3/2,2 disclosed (Top-Cluster 37,9% Gewicht); CIs unter df 4 unzuverlaessig (Tipton)</t>
         </is>
       </c>
+      <c r="H9" s="46" t="inlineStr">
+        <is>
+          <t>Alternative Schätzverfahren liefern dasselbe Bild: zwischen −0,022 und −0,062, alle klein. Egal wie man rechnet — der Effekt bleibt nahe null.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="48" t="inlineStr">
@@ -5701,6 +5764,11 @@
           <t>Manuskriptzeile BLOCKED bis DEC-012a-Konstanten (Volker-Extraktion, Instrument-Mediane)</t>
         </is>
       </c>
+      <c r="H10" s="46" t="inlineStr">
+        <is>
+          <t>In Basispunkten: je nach angenommener Streuung grob 6–12 bp niedrigere Fremdkapitalkosten pro 1 SD besserer Umweltleistung (Platzhalter; finale Umrechnung wartet auf DEC-012a-Benchmarks). Größenordnung: spürbar klein.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="48" t="inlineStr">
@@ -5734,6 +5802,11 @@
         </is>
       </c>
       <c r="G11" s="46" t="inlineStr"/>
+      <c r="H11" s="46" t="inlineStr">
+        <is>
+          <t>Anhangs-Grafik: alle Cluster-Effekte einzeln mit Gesamtmittel und Vorhersageintervall — macht die große Streuung auf einen Blick sichtbar.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="48" t="inlineStr">
@@ -5767,6 +5840,11 @@
         </is>
       </c>
       <c r="G12" s="46" t="inlineStr"/>
+      <c r="H12" s="46" t="inlineStr">
+        <is>
+          <t>Anhangs-Grafik (A4-ganzseitig): alle 115 Studien im Forest-Plot — Transparenz über die komplette Evidenzbasis.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="47" t="inlineStr">
@@ -5817,6 +5895,11 @@
           <t>df(pp_mid)=31,9 → Transfer-Regel greift NICHT, Binär trägt volle Inferenz; Post-Zelle 31 Studien (kanonisch bestätigt, T0.4 v2 28/28, 2026-07-12) · realisierte Kontrast-df 15,0 vs. Design-df 31,9 (disclosed; beide &gt; Tipton-Boden); Zellmittel vs. A3 = Estimanden-Unterschied (gemeinsames Modell)</t>
         </is>
       </c>
+      <c r="H14" s="46" t="inlineStr">
+        <is>
+          <t>Der Unterschied zwischen prä- und post-Paris ist winzig (+0,010) und klar nicht signifikant (p=0,58). Das Konfidenzintervall schließt auch kleine Effekte weitgehend aus. Heißt: Das Paris-Abkommen hat den CER-COD-Zusammenhang nicht messbar verändert.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="48" t="inlineStr">
@@ -5854,6 +5937,11 @@
           <t>z̄ bei 2015,5: −0,087→−0,035; corr(mid,share)=0,8146 (A.9/D2); Joint-Support-Caveat z̄(1); Bewertung via Offset (CENTER=2012,258)</t>
         </is>
       </c>
+      <c r="H15" s="46" t="inlineStr">
+        <is>
+          <t>Auch als 'Dosis' gerechnet (Anteil des Studienfensters nach Paris) zeigt sich kein Muster: Steigung ns, nicht-linear ebenfalls nichts (Joint p=0,21). Mehr Paris-Anteil heißt nicht anderer Effekt.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="48" t="inlineStr">
@@ -5891,6 +5979,11 @@
           <t>Upgrade GEFEUERT (kanonisch): clean-window df=12,3 ≥ 5 → volle Inferenz (DEC-031a.5; design_quantities_v12.csv) · kein Kollaps ('collapse = finding' verneint); Vorzeichen-Heterogenitaet um null = kein systematischer Shift; end-Familie durch 66%-Kontamination erklaert (B7)</t>
         </is>
       </c>
+      <c r="H16" s="46" t="inlineStr">
+        <is>
+          <t>Neun alternative Kodierungen des Paris-Schnitts ändern nichts — alle Differenzen bleiben winzig und ns. Das Null-Ergebnis hängt nicht an einer Kodier-Entscheidung.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="48" t="inlineStr">
@@ -5928,6 +6021,11 @@
           <t>break_only Cell-Means per DEC-031e (O15-Identität ~1e-16); realisierte df 15,0 vs Design 31,9; Race-CI-Rand +0,079 &gt; SESOI — Präzisionsgrenze offengelegt (F61-P3)</t>
         </is>
       </c>
+      <c r="H17" s="46" t="inlineStr">
+        <is>
+          <t>Weder ein allmählicher Zeittrend noch ein Bruch 2016 ist nachweisbar (beide ns); der 2016er-Schnitt ist nur Rang 7 von 9 möglichen Jahren. Wäre Paris ein echter Wendepunkt, müsste 2016 herausstechen — tut es nicht.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="48" t="inlineStr">
@@ -5965,6 +6063,11 @@
           <t>Set {region, instrument, CER} per DEC-031d; Read-out Δβ+CI vs SESOI-Band (F61-P3); beide CIs in ±0,070; trend_comp-Rand +0,052 marginal über ±0,05</t>
         </is>
       </c>
+      <c r="H18" s="46" t="inlineStr">
+        <is>
+          <t>Kontrolliert man Unterschiede in Länderregion, COD-Messung und CER-Messung, ändert sich der Paris-Koeffizient um +0,002 — praktisch gar nicht. Das Null liegt nicht an verschobener Studienzusammensetzung.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="48" t="inlineStr">
@@ -5998,6 +6101,11 @@
         </is>
       </c>
       <c r="G19" s="46" t="inlineStr"/>
+      <c r="H19" s="46" t="inlineStr">
+        <is>
+          <t>Kein Einzelstudien-Effekt: Lässt man jede Studie einmal weg, bleibt die Differenz zwischen +0,002 und +0,014, immer ns. Auch die gewichtigste Studie (≈23 %) treibt nichts.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="48" t="inlineStr">
@@ -6035,6 +6143,11 @@
           <t>v12-kanonisch; traegt Kodierungs-Verteidigung (TB-16/17/18)</t>
         </is>
       </c>
+      <c r="H20" s="46" t="inlineStr">
+        <is>
+          <t>Die Kodierwahl ist belastbar: Nur 2,9 % der Effekte sind Kipp-Fälle, und die alte End-Jahr-Kodierung hätte zwei Drittel der Post-Zelle mit überwiegend Prä-Daten verwässert.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -6070,6 +6183,11 @@
       <c r="G21" s="46" t="inlineStr">
         <is>
           <t>Oster-Paar race vs trend_composition (F61-P1); pseudo-R² negativ möglich (REML); Schlussklammer — Gewicht liegt auf Race+Placebos+Komposition</t>
+        </is>
+      </c>
+      <c r="H21" s="46" t="inlineStr">
+        <is>
+          <t>Rechnet man unbeobachtete Störgrößen ein, bleibt der Bruch bei ~+0,01; allerdings würden schon mäßige Störfaktoren genügen, um einen echten kleinen Effekt zu verdecken. Der Null-Befund stützt sich daher auf die Gesamtbatterie, nicht auf diesen einen Test.</t>
         </is>
       </c>
     </row>
@@ -6397,6 +6515,11 @@
         </is>
       </c>
       <c r="G34" s="46" t="inlineStr"/>
+      <c r="H34" s="46" t="inlineStr">
+        <is>
+          <t>Kleine Studien berichten etwas negativere Effekte (Asymmetrie exakt an der Signifikanzgrenze). Korrigiert man dafür, bleibt ein kleiner negativer Effekt (−0,04 bis −0,06) — weiter unter der Bedeutsamkeitsschwelle.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="48" t="inlineStr">
@@ -6432,6 +6555,11 @@
       <c r="G35" s="46" t="inlineStr">
         <is>
           <t>Trim-and-Fill begründet ausgeschlossen (Carter et al. 2019; DEC-031a.4)</t>
+        </is>
+      </c>
+      <c r="H35" s="46" t="inlineStr">
+        <is>
+          <t>Nach Korrektur für selektives Publizieren schrumpft der Effekt auf praktisch null (+0,01, ns) — zwei unabhängige Verfahren landen fast identisch dort. Zudem gibt es ein Signal, dass nicht-signifikante Ergebnisse seltener publiziert wurden (p=0,025). Der kleine negative Literatur-Durchschnitt ist also teils ein Publikations-Artefakt.</t>
         </is>
       </c>
     </row>
@@ -6463,6 +6591,11 @@
           <t>Prior-Quelle = COE-Companion (Witte et al., BSE) per DEC-031b — kein externes Pending; gleiche RoBMA-Maschinerie wie H2</t>
         </is>
       </c>
+      <c r="H36" s="46" t="inlineStr">
+        <is>
+          <t>Läuft in der H-Session: Bayesianisches Modell-Averaging (RoBMA) als zusätzliche Bias-Korrektur; Ergebnis fließt in die D6-Gesamtschau ein.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="48" t="inlineStr">
@@ -6500,6 +6633,11 @@
           <t>Upgrade GEFEUERT (kanonisch): Post-Zelle 31 ≥ 20 Studien → 3PSM/p-uniform* im Split (DEC-031a.5)</t>
         </is>
       </c>
+      <c r="H37" s="46" t="inlineStr">
+        <is>
+          <t>Das Bias-Bild ist vor und nach Paris ähnlich: Korrekturen bleiben klein bzw. gehen Richtung null; auffällige Klein-Studien-Asymmetrie erst in der Post-Zelle. Für die Paris-Frage ändert das nichts.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="48" t="inlineStr">
@@ -6537,6 +6675,11 @@
           <t>aus C verschoben (DEC-031a.1)</t>
         </is>
       </c>
+      <c r="H38" s="46" t="inlineStr">
+        <is>
+          <t>Publizierte und unpublizierte Studien finden praktisch denselben Effekt (−0,059 vs. −0,057; Differenz ns). Der Publikationsstatus verzerrt im gefundenen Korpus also nicht — die Selektion wirkt über die Signifikanz (siehe D2).</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="48" t="inlineStr">
@@ -6566,10 +6709,15 @@
       </c>
       <c r="F39" s="46" t="inlineStr">
         <is>
-          <t>mechanisch: unadj. −0,062 · PET −0,043 · PEESE −0,055 · 3PSM +0,012 · p-uni* +0,012 · Grey-Null; alle korrigierten Punkte im SESOI-Band |r|=0,070; RoBMA ausstehend (H2) — Einordnung Pending-C</t>
+          <t>mechanisch: unadj. −0,062 · PET −0,043 · PEESE −0,055 · 3PSM +0,012 · p-uni* +0,012 · Grey-Null; alle korrigierten Punkte im SESOI-Band |r|=0,070; RoBMA ausstehend (H2) — Einordnung: A per DEC-044; RoBMA-Zeile weiter BLOCKED (H2)</t>
         </is>
       </c>
       <c r="G39" s="46" t="inlineStr"/>
+      <c r="H39" s="46" t="inlineStr">
+        <is>
+          <t>Zusammenschau (Entwurf): Alle Korrekturverfahren landen zwischen ~0 und −0,06 — ökonomisch durchweg vernachlässigbar; die Verfahren streiten nur darüber, ob überhaupt ein Rest bleibt. Endfassung nach RoBMA (H2).</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="47" t="inlineStr">

</xml_diff>

<commit_message>
TH-a/TH-c results (run family): canonical outputs (17/17, 19/19 PASS), 13-tab workbooks, status touch - framing-neutral pending DEC-044 gate resolution [DEC-045]; TH_c_perms.rds kept out of git per repo .rds convention, md5-pinned in run_meta + design row; ERROR_LOG #15 (commit-block status path, repeat of #5)
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1356,7 +1356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1571,6 +1571,47 @@
       <c r="C16" s="6" t="inlineStr">
         <is>
           <t>output/T7_results.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Phase 2 — Null-Batterie (Block E/H · TH-a/TH-c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>TH-a · E-Batterie + H-Schnellläufe (E1-E3, H4-Grid, H6-H11)</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>E1 TOST ±0,070 p=0,205 (Flag 0) · E2 ±0,050 p=0,022 (Flag 1; diff +0,010) · sup|t|=2,12@2009 · Zarea +0,011 (p=,574) · H7 Ende -0,059 · H8 -0,087..-0,015 (20/21 Fenster) · H9 COD -0,059 vs COE -0,039 · H10 Stouffer p=2,1e-119, Flatness pp=1,000 · H11 within +0,036 — Verdict-Text: Gate offen [DEC-044]</t>
+        </is>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>output/TH_a_results.csv; output/TH_a_results_workbook.xlsx (Familien-Commit, Basis dafd95e)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>TH-c · Simulation/Permutation (H1, H3, H4-Perm, H5)</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>MDE80 own x1/x2=NA (&gt;0,08; Power@0,08 0,730/0,448), x0,5=0,063; COE-LB 0,010-0,018; Kalibrierung 0,765 · H3 Kern 0/10, Vollkurve 1/1.260, p_perm 1,000/0,854 · H4 p_perm=0,341 · H5 p_perm=0,401 · eff_B 500/500/500; Counter 11.500/92/0 · 540/3/0 · 200/2/0 — Verdict-Text: Gate offen [DEC-044]</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>output/TH_c_results.csv; output/TH_c_results_workbook.xlsx (Familien-Commit, Basis dafd95e)</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1613,7 +1654,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>54 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>55 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -3217,6 +3258,43 @@
       <c r="F58" t="inlineStr">
         <is>
           <t>Paris-Null hart; Pooled "negligible, not null" (CI-Rand &gt; SESOI); C -&gt; Boundary-Conditions; T7 = Heterogenitäts-Exploration in A</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>DEC-045</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>E/H-Batterie-Execution-Spec: Run-Architektur TH-a/b/c, Supersessions S1-S9, TOST-Pins, H1-Precompute, Zeittranslations-Permutation, RoBMA-Prior-Paket (F66)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Block E/H / TH-a, TH-b, TH-c</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Result-blind Amendment: 10-Kodierungs-Kern (D1 verbatim aus T2); B=500 (S5); N10=113 Schritte; H8-Tiers (S6); F66 offen (einziges offenes F)</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>aktiv</t>
         </is>
       </c>
     </row>
@@ -6750,12 +6828,25 @@
       </c>
       <c r="D41" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E41" s="48" t="inlineStr"/>
-      <c r="F41" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-24, Verifier 17/17)</t>
+        </is>
+      </c>
+      <c r="E41" s="48" t="inlineStr">
+        <is>
+          <t>output/TH_a_results_workbook.xlsx Tab 6; output/TH_a_results.csv (Familien-Commit, Basis dafd95e)</t>
+        </is>
+      </c>
+      <c r="F41" s="46" t="inlineStr">
+        <is>
+          <t>TOST ±0,070: p=0,205, 90%-CI [-0,082; -0,036], Flag 0 (ex ante erwartet); ±0,050: p=0,732, Flag 0 — mechanisch; Sprachregelung: Gate offen [DEC-044]</t>
+        </is>
+      </c>
       <c r="G41" s="46" t="inlineStr"/>
+      <c r="H41" s="46" t="inlineStr">
+        <is>
+          <t>Der Gesamteffekt ist klein, aber nicht klein genug für 'praktisch null' im strengen Sinn — die endgültige Einordnung folgt nach dem Bayes-Schritt.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="48" t="inlineStr">
@@ -6775,12 +6866,25 @@
       </c>
       <c r="D42" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E42" s="48" t="inlineStr"/>
-      <c r="F42" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-24, Verifier 17/17)</t>
+        </is>
+      </c>
+      <c r="E42" s="48" t="inlineStr">
+        <is>
+          <t>output/TH_a_results_workbook.xlsx Tab 6; output/TH_a_results.csv (Familien-Commit, Basis dafd95e)</t>
+        </is>
+      </c>
+      <c r="F42" s="46" t="inlineStr">
+        <is>
+          <t>diff_z=+0,010 (p=0,582); TOST ±0,050: p=0,022, 90%-CI [-0,022; +0,042], Flag 1 — mechanisch; Gate offen [DEC-044]</t>
+        </is>
+      </c>
       <c r="G42" s="46" t="inlineStr"/>
+      <c r="H42" s="46" t="inlineStr">
+        <is>
+          <t>Der Prä/Post-Paris-Unterschied liegt vollständig im vorab festgelegten Kleinheitsband; die formale Sprachregelung folgt nach TH-b.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="48" t="inlineStr">
@@ -6800,12 +6904,25 @@
       </c>
       <c r="D43" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E43" s="48" t="inlineStr"/>
-      <c r="F43" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-24, Verifier 17/17) — AUFLÖSUNG offen (dokumentierter Schritt nach TH-b)</t>
+        </is>
+      </c>
+      <c r="E43" s="48" t="inlineStr">
+        <is>
+          <t>output/TH_a_results_workbook.xlsx Tab 6 (E3-Zeilen); output/TH_a_results.csv (Familien-Commit, Basis dafd95e)</t>
+        </is>
+      </c>
+      <c r="F43" s="46" t="inlineStr">
+        <is>
+          <t>Gate-Konfiguration fixiert: E2-PASS-Requirement + BF01-Leiter (&gt;=3 voll; 1-3 äquivalenzbasiert); Status 'resolution deferred'</t>
+        </is>
+      </c>
       <c r="G43" s="46" t="inlineStr"/>
+      <c r="H43" s="46" t="inlineStr">
+        <is>
+          <t>Regelwerk, welche Formulierung ('kein Effekt' vs. 'kein Nachweis') zulässig ist; Entscheidung fällt dokumentiert nach dem Bayes-Lauf.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="47" t="inlineStr">
@@ -7346,12 +7463,25 @@
       </c>
       <c r="D65" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E65" s="48" t="inlineStr"/>
-      <c r="F65" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-26, Verifier 19/19)</t>
+        </is>
+      </c>
+      <c r="E65" s="48" t="inlineStr">
+        <is>
+          <t>output/TH_c_results_workbook.xlsx Tab 6; output/TH_c_results.csv (Familien-Commit, Basis dafd95e)</t>
+        </is>
+      </c>
+      <c r="F65" s="46" t="inlineStr">
+        <is>
+          <t>MDE80: own x0,5=0,063; x1,0/x2,0=NA (&gt;0,08-Grid; Power@0,08=0,730/0,448); COE-Lower-Bound 0,010-0,018; Kalibrierung: Rejection 0,765, Optimismus +0,035 (200/2/0)</t>
+        </is>
+      </c>
       <c r="G65" s="46" t="inlineStr"/>
+      <c r="H65" s="46" t="inlineStr">
+        <is>
+          <t>Rechnet nach, wie groß ein Paris-Effekt hätte sein müssen, um sicher entdeckt zu werden: bei realer Streuung mehr, als das Raster zulässt — die Heterogenität, nicht die Studienzahl, ist der Engpass.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="48" t="inlineStr">
@@ -7400,12 +7530,29 @@
       </c>
       <c r="D67" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E67" s="48" t="inlineStr"/>
-      <c r="F67" s="46" t="inlineStr"/>
-      <c r="G67" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-26, Verifier 19/19)</t>
+        </is>
+      </c>
+      <c r="E67" s="48" t="inlineStr">
+        <is>
+          <t>output/TH_c_results_workbook.xlsx Tabs 7-8; output/TH_c_results.csv (Familien-Commit, Basis dafd95e)</t>
+        </is>
+      </c>
+      <c r="F67" s="46" t="inlineStr">
+        <is>
+          <t>Kern 0/10 sig.; Vollkurve 1/1.260 (end_lag2|winsor|dfE, rho 0,4: +0,018, p=,049; ~63 unter globaler Null erwartet); p_perm Share=1,000, Median-|t|=0,854 (eff_B 500); Kern-Range -0,019..+0,040, min p=,142</t>
+        </is>
+      </c>
+      <c r="G67" s="46" t="inlineStr">
+        <is>
+          <t>Faktorraum 1.260 Zellen / 10 Kodierungen per DEC-045 S2 (ersetzt die ~1.400-Formulierung der Kurzbeschreibung)</t>
+        </is>
+      </c>
+      <c r="H67" s="46" t="inlineStr">
+        <is>
+          <t>Egal wie man Paris kodiert oder das Modell variiert: praktisch keine Variante zeigt einen Effekt, und der Sammel-Test über alle Varianten ist unauffällig.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="48" t="inlineStr">
@@ -7425,12 +7572,25 @@
       </c>
       <c r="D68" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E68" s="48" t="inlineStr"/>
-      <c r="F68" s="46" t="inlineStr"/>
+          <t>erledigt (TH-a 2026-07-24 17/17 · TH-c 2026-07-26 19/19)</t>
+        </is>
+      </c>
+      <c r="E68" s="48" t="inlineStr">
+        <is>
+          <t>output/TH_a_results_workbook.xlsx Tab 7 (Grid) + output/TH_c_results_workbook.xlsx Tab 9 (Permutation); CSVs (Familien-Commit, Basis dafd95e)</t>
+        </is>
+      </c>
+      <c r="F68" s="46" t="inlineStr">
+        <is>
+          <t>sup|t|=2,12 @2009 (12 zulässige Jahre, df&gt;=5); p_perm=0,341 (eff_B 500)</t>
+        </is>
+      </c>
       <c r="G68" s="46" t="inlineStr"/>
+      <c r="H68" s="46" t="inlineStr">
+        <is>
+          <t>Sucht das auffälligste Bruchjahr 2008-2019: Selbst das stärkste Jahr (2009) ist nicht ungewöhnlicher, als Zufall es erwarten lässt.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="48" t="inlineStr">
@@ -7450,12 +7610,29 @@
       </c>
       <c r="D69" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E69" s="48" t="inlineStr"/>
-      <c r="F69" s="46" t="inlineStr"/>
-      <c r="G69" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-26, Verifier 19/19)</t>
+        </is>
+      </c>
+      <c r="E69" s="48" t="inlineStr">
+        <is>
+          <t>output/TH_c_results_workbook.xlsx Tab 10; output/TH_c_results.csv (Familien-Commit, Basis dafd95e)</t>
+        </is>
+      </c>
+      <c r="F69" s="46" t="inlineStr">
+        <is>
+          <t>p_perm(Race)=0,401 (eff_B 500); |t_race|=1,052 (Punktschätzer/p_CR2 single-home T8)</t>
+        </is>
+      </c>
+      <c r="G69" s="46" t="inlineStr">
+        <is>
+          <t>B=500 per DEC-045 S5 (Benchmark-Regel; ersetzt B=2.000 der Kurzbeschreibung)</t>
+        </is>
+      </c>
+      <c r="H69" s="46" t="inlineStr">
+        <is>
+          <t>Zufallstest mit künstlich verschobenen Studienzeitfenstern: Der echte Befund sticht aus den Zufallsvarianten nicht heraus.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="48" t="inlineStr">
@@ -7475,12 +7652,25 @@
       </c>
       <c r="D70" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E70" s="48" t="inlineStr"/>
-      <c r="F70" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-24, Verifier 17/17)</t>
+        </is>
+      </c>
+      <c r="E70" s="48" t="inlineStr">
+        <is>
+          <t>output/TH_a_results_workbook.xlsx Tab 8; output/TH_a_results.csv (Familien-Commit, Basis dafd95e)</t>
+        </is>
+      </c>
+      <c r="F70" s="46" t="inlineStr">
+        <is>
+          <t>Zarea-Operationalisierung (Midpoint + Tie-Exclusion) im eigenen 3L-RVE-Spine: diff +0,011 (t(11,6)=0,58, p=0,574); Ties 79 ES/5 Studien; Post 31-&gt;26</t>
+        </is>
+      </c>
       <c r="G70" s="46" t="inlineStr"/>
+      <c r="H70" s="46" t="inlineStr">
+        <is>
+          <t>Rechnet unsere Daten mit der Paris-Definition der Vergleichsstudie: Das Ergebnis bleibt gleich.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="48" t="inlineStr">
@@ -7500,12 +7690,25 @@
       </c>
       <c r="D71" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E71" s="48" t="inlineStr"/>
-      <c r="F71" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-24, Verifier 17/17)</t>
+        </is>
+      </c>
+      <c r="E71" s="48" t="inlineStr">
+        <is>
+          <t>output/TH_a_results_workbook.xlsx Tab 8; output/TH_a_results.csv (Familien-Commit, Basis dafd95e)</t>
+        </is>
+      </c>
+      <c r="F71" s="46" t="inlineStr">
+        <is>
+          <t>113 Schritte (Ordnung: Median-sample_mid); Floor Schritt 10 (Chen, Gao 2011); post-Floor-Range -0,095..-0,015; Endwert -0,059 [-0,087; -0,031]; step_001 not_estimable (regelkonform, #12-Guard)</t>
+        </is>
+      </c>
       <c r="G71" s="46" t="inlineStr"/>
+      <c r="H71" s="46" t="inlineStr">
+        <is>
+          <t>Baut die Meta-Analyse Studie für Studie chronologisch auf: Der negative Effekt etabliert sich früh und endet exakt beim Gesamtwert.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="48" t="inlineStr">
@@ -7525,12 +7728,25 @@
       </c>
       <c r="D72" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E72" s="48" t="inlineStr"/>
-      <c r="F72" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-24, Verifier 17/17)</t>
+        </is>
+      </c>
+      <c r="E72" s="48" t="inlineStr">
+        <is>
+          <t>output/TH_a_results_workbook.xlsx Tab 9; output/TH_a_results.csv (Familien-Commit, Basis dafd95e)</t>
+        </is>
+      </c>
+      <c r="F72" s="46" t="inlineStr">
+        <is>
+          <t>21 Fenster (Anker 1998): 20 schätzbar, 2002-2007 not_estimable (&lt;5 Cluster); Means -0,087..-0,015; Tiers per DEC-045 S6</t>
+        </is>
+      </c>
       <c r="G72" s="46" t="inlineStr"/>
+      <c r="H72" s="46" t="inlineStr">
+        <is>
+          <t>Sechs-Jahres-Fenster über die Zeit geschoben: Der Zusammenhang ist in allen schätzbaren Fenstern negativ.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="48" t="inlineStr">
@@ -7550,12 +7766,25 @@
       </c>
       <c r="D73" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E73" s="48" t="inlineStr"/>
-      <c r="F73" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-24, Verifier 17/17)</t>
+        </is>
+      </c>
+      <c r="E73" s="48" t="inlineStr">
+        <is>
+          <t>output/TH_a_results_workbook.xlsx Tab 9; output/TH_a_results.csv (Familien-Commit, Basis dafd95e)</t>
+        </is>
+      </c>
+      <c r="F73" s="46" t="inlineStr">
+        <is>
+          <t>deskriptiv: COD -0,059 vs. COE Study-Level -0,039 [-0,046; -0,032] (75 Units); kein Test (SE-Provenienz inkompatibel, N12-Scope); Overlap 6/115 Studien, 0 gemeinsame ES</t>
+        </is>
+      </c>
       <c r="G73" s="46" t="inlineStr"/>
+      <c r="H73" s="46" t="inlineStr">
+        <is>
+          <t>Vergleich mit dem Eigenkapital-Schwesterpapier: Der Fremdkapital-Effekt ist etwas größer — rein beschreibend.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="48" t="inlineStr">
@@ -7575,12 +7804,25 @@
       </c>
       <c r="D74" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E74" s="48" t="inlineStr"/>
-      <c r="F74" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-24, Verifier 17/17)</t>
+        </is>
+      </c>
+      <c r="E74" s="48" t="inlineStr">
+        <is>
+          <t>output/TH_a_results_workbook.xlsx Tab 10; output/TH_a_results.csv (Familien-Commit, Basis dafd95e)</t>
+        </is>
+      </c>
+      <c r="F74" s="46" t="inlineStr">
+        <is>
+          <t>konditional erfüllt (28/31 sig.); Rechtsschiefe: Binomial p=1,5e-6, Stouffer p=2,1e-119; Flatness pp=1,000 (NCP-Fix #11)</t>
+        </is>
+      </c>
       <c r="G74" s="46" t="inlineStr"/>
+      <c r="H74" s="46" t="inlineStr">
+        <is>
+          <t>Prüft die signifikanten Post-Paris-Studien auf p-Hacking-Muster: Die Verteilung sieht nach echter Evidenz aus, nicht nach Selektion.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="48" t="inlineStr">
@@ -7600,14 +7842,27 @@
       </c>
       <c r="D75" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E75" s="48" t="inlineStr"/>
-      <c r="F75" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-24, Verifier 17/17)</t>
+        </is>
+      </c>
+      <c r="E75" s="48" t="inlineStr">
+        <is>
+          <t>output/TH_a_results_workbook.xlsx Tab 10; output/TH_a_results.csv (Familien-Commit, Basis dafd95e)</t>
+        </is>
+      </c>
+      <c r="F75" s="46" t="inlineStr">
+        <is>
+          <t>Li et al 2022: 12 prä/5 post ES, within-diff +0,036 (deskriptiv, kein Test); 73 Straddler, davon 72 poolen über den Bruch</t>
+        </is>
+      </c>
       <c r="G75" s="46" t="inlineStr">
         <is>
           <t>N15 = 1 Studie (Li et al 2022); 73 Studien überspannen den Bruch, 72 poolen darüber → Intro-Baustein „Paris-Blindheit" (Datenagenda #35, Pending-C-Input)</t>
+        </is>
+      </c>
+      <c r="H75" s="46" t="inlineStr">
+        <is>
+          <t>Nur eine einzige Studie trennt selbst vor/nach Paris; fast alle mitteln darüber hinweg — Kernmotiv der Einleitung.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
F66 closed [DEC-046]: RoBMA stack pinned (rjags 4-17, BayesTools 0.2.23, RoBMA 3.6.1), t_RoBMA=1764.8s, y/se scale path + R/07 TH-b package (H2a/H2b RoBMA.reg, paired verifier) + ERROR_LOG #16 [DEC-045/DEC-046]
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1632,7 +1632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1654,7 +1654,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>55 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>56 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -3293,6 +3293,43 @@
         </is>
       </c>
       <c r="G59" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>DEC-046</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Methodik</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>F66-Schließung: RoBMA-Stack gepinnt (rjags 4-17, BayesTools 0.2.23, RoBMA 3.6.1, JAGS 4.3.2); y/se-Skalenpfad (Priors wirken verbatim auf z); t_RoBMA gemessen; Executor-/Leiter-Deviationen offengelegt</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>F66 / TH-b (R/07)</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Ruling A (Upstream-Repro-Guidance statt 4.0.0-Bruchrelease); effect_direction "negative" gepinnt; t_RoBMA 1764,8 s; P3-Projektion T = 3t + 3κt, GO-Check bindend; RoBMA.reg = H2b-Träger; F66 GESCHLOSSEN</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
         <is>
           <t>aktiv</t>
         </is>

</xml_diff>

<commit_message>
TH-b delivered [DEC-045/DEC-046]: canonical H2a/H2b outputs (30 rows, verifier O0-O14 PASS) + results workbook (TB-52..TB-56) + TH.md H2 update + status touch (H2/D3/D6, Key_Results); gate resolution pending [DEC-044]
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1356,7 +1356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1612,6 +1612,23 @@
       <c r="C19" s="6" t="inlineStr">
         <is>
           <t>output/TH_c_results.csv; output/TH_c_results_workbook.xlsx (Familien-Commit, Basis dafd95e)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>TH-b · RoBMA-Bayes-Batterie (H2a/H2b)</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>H2a BF01(Effekt) 7,03/2,38/1,69 (Default/COE/Wide); μ̄ −0,009…+0,008 (Spike-begrenzt); Het. saturiert; Bias BF10 94,7/11,1/16,8 · H2b BF01(Periode) 1,03/1,17/8,49 (informiert primär; Default mit Caveats); Kontrast +0,003 [−0,031; +0,045] — Verdict-Text: Gate offen [DEC-044]</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>output/TH_b_results.csv; output/TH_b_results_workbook.xlsx (Block-2-Commit)</t>
         </is>
       </c>
     </row>
@@ -1632,7 +1649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3335,6 +3352,7 @@
         </is>
       </c>
     </row>
+    <row r="61"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A27:G27"/>
@@ -6696,11 +6714,19 @@
       </c>
       <c r="D36" s="48" t="inlineStr">
         <is>
-          <t>offen (→ H2 per DEC-031g)</t>
-        </is>
-      </c>
-      <c r="E36" s="48" t="inlineStr"/>
-      <c r="F36" s="46" t="inlineStr"/>
+          <t>erledigt via H2 (2026-07-27) — Single-Home: Ergebnisse in Z66</t>
+        </is>
+      </c>
+      <c r="E36" s="48" t="inlineStr">
+        <is>
+          <t>siehe H2 (Z66): output/TH_b_results_workbook.xlsx (Block-2-Commit)</t>
+        </is>
+      </c>
+      <c r="F36" s="46" t="inlineStr">
+        <is>
+          <t>siehe H2 (Z66) — Single-Home, keine Duplikation [DEC-031g]</t>
+        </is>
+      </c>
       <c r="G36" s="46" t="inlineStr">
         <is>
           <t>Prior-Quelle = COE-Companion (Witte et al., BSE) per DEC-031b — kein externes Pending; gleiche RoBMA-Maschinerie wie H2</t>
@@ -6708,7 +6734,7 @@
       </c>
       <c r="H36" s="46" t="inlineStr">
         <is>
-          <t>Läuft in der H-Session: Bayesianisches Modell-Averaging (RoBMA) als zusätzliche Bias-Korrektur; Ergebnis fließt in die D6-Gesamtschau ein.</t>
+          <t>In der H-Session als H2 gelaufen (RoBMA); Ergebnisse und Erklärung dort (Z66). Fließt in die D6-Gesamtschau ein.</t>
         </is>
       </c>
     </row>
@@ -6814,7 +6840,7 @@
       </c>
       <c r="D39" s="48" t="inlineStr">
         <is>
-          <t>DRAFT (2026-07-19) — RoBMA-Zeile BLOCKED bis H2</t>
+          <t>DRAFT — RoBMA-Zeile jetzt befüllbar (H2 erledigt 2026-07-27); Endfassung nach Gate [DEC-044]</t>
         </is>
       </c>
       <c r="E39" s="48" t="inlineStr">
@@ -6824,13 +6850,13 @@
       </c>
       <c r="F39" s="46" t="inlineStr">
         <is>
-          <t>mechanisch: unadj. −0,062 · PET −0,043 · PEESE −0,055 · 3PSM +0,012 · p-uni* +0,012 · Grey-Null; alle korrigierten Punkte im SESOI-Band |r|=0,070; RoBMA ausstehend (H2) — Einordnung: A per DEC-044; RoBMA-Zeile weiter BLOCKED (H2)</t>
+          <t>mechanisch: unadj. −0,062 · PET −0,043 · PEESE −0,055 · 3PSM +0,012 · p-uni* +0,012 · Grey-Null; alle korrigierten Punkte im SESOI-Band |r|=0,070; RoBMA ausstehend (H2) — Einordnung: A per DEC-044; RoBMA (H2): BF01(Effekt) 7,03/2,38/1,69, μ̄ −0,009…+0,008 — mechanisch im Bild aller Korrekturverfahren (~0 bis −0,06); Endfassung nach Gate</t>
         </is>
       </c>
       <c r="G39" s="46" t="inlineStr"/>
       <c r="H39" s="46" t="inlineStr">
         <is>
-          <t>Zusammenschau (Entwurf): Alle Korrekturverfahren landen zwischen ~0 und −0,06 — ökonomisch durchweg vernachlässigbar; die Verfahren streiten nur darüber, ob überhaupt ein Rest bleibt. Endfassung nach RoBMA (H2).</t>
+          <t>Zusammenschau (Entwurf): Alle Korrekturverfahren landen zwischen ~0 und −0,06 — ökonomisch durchweg vernachlässigbar; die Verfahren streiten nur darüber, ob überhaupt ein Rest bleibt. Endfassung nach Gate-Schritt [DEC-044] — RoBMA liegt jetzt vor.</t>
         </is>
       </c>
     </row>
@@ -7538,14 +7564,27 @@
       </c>
       <c r="D66" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
-        </is>
-      </c>
-      <c r="E66" s="48" t="inlineStr"/>
-      <c r="F66" s="46" t="inlineStr"/>
+          <t>erledigt (2026-07-27, Verifier O0–O14 PASS, Lauf 3/3)</t>
+        </is>
+      </c>
+      <c r="E66" s="48" t="inlineStr">
+        <is>
+          <t>output/TH_b_results_workbook.xlsx Tabs 6–7; output/TH_b_results.csv (Block-2-Commit; Skripte @ 4cf8fe6)</t>
+        </is>
+      </c>
+      <c r="F66" s="46" t="inlineStr">
+        <is>
+          <t>H2a BF01(Effekt) = 7,03 (PSMA-Default, primär) / 2,38 (COE-informiert) / 1,69 (Wide); μ̄ −0,009 … +0,008 (Spike-begrenzte 95%-CIs); Heterogenität saturiert (BF01 = 0); Bias-Block BF10 = 94,7/11,1/16,8 · H2b BF01(Periode) = 1,03 (Kontrast-informiert N(0; 0,025), primär) / 1,17 (Wide) / 8,49 (Paket-Default, Konvergenz-Caveats offengelegt); Kontrast +0,003 z [−0,031; +0,045] — Band 1–3 ⇒ Äquivalenzregister-Input [E3]</t>
+        </is>
+      </c>
       <c r="G66" s="46" t="inlineStr">
         <is>
-          <t>Inputs vollständig fixiert (DEC-031b); Quelle Witte et al. COE-Companion, Overlap-Disclosure 5 Studien / 0 geteilte ES</t>
+          <t>Inputs vollständig fixiert (DEC-031b); Quelle Witte et al. COE-Companion, Overlap-Disclosure 5 Studien / 0 geteilte ES; Lauf-Provenienz: κ_emp 1,71–2,34 vs Pin 2,5, Wall 4 h 39 min; Läufe 1–2 = Design-Halts (ERROR_LOG #17/#18)</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Bayesianische Gesamtschau: Unter den vorab fixierten, informierten Priors ist die Moderations-Frage praktisch unentschieden (BF ≈ 1) — die Daten sprechen weder klar für noch gegen einen Paris-Effekt; der gepoolte Effekt erhält nur begrenzte Unterstützung, und die Publikations-Selektions-Komponenten werden durchgehend stark einbezogen. Einordnung und Wortlaut folgen im Gate-Schritt [DEC-044].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gate resolved [DEC-047]: Tier-1 wording = equivalence register (E2 flag 1 x BF01(period)=1.03, band 1-3; default 8.49 not claim-bearing) + status touch (E3 resolution, D6 final, DLI 57)
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1671,7 +1671,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>56 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>57 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -3352,7 +3352,43 @@
         </is>
       </c>
     </row>
-    <row r="61"/>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>DEC-047</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Framing</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Gate-Auflösung [DEC-044]: Tier-1-Wortlaut = Äquivalenzregister — E2-Flag 1 (p_TOST = ,022) × BF01(Periode) primär = 1,03 (Band 1–3) per pre-registrierter E3-Leiter; Default-BF 8,49 nicht claimtragend (nicht-primär, anders parametrisiert, Caveats)</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Gate / E3 · D6 · Manuskriptphase</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Freigegeben: "statistisch äquivalent zu null im sekundären SESOI-Band"; gesperrt: Evidence-of-Absence-Vokabular; BFs deskriptiv; Tier 2 unverändert; TB-55 + BLOCKED-TBs entsperrt (Rewrites in Manuskriptphase)</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>aktiv</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A27:G27"/>
@@ -6840,7 +6876,7 @@
       </c>
       <c r="D39" s="48" t="inlineStr">
         <is>
-          <t>DRAFT — RoBMA-Zeile jetzt befüllbar (H2 erledigt 2026-07-27); Endfassung nach Gate [DEC-044]</t>
+          <t>erledigt (2026-07-27) — Endfassung per DEC-047</t>
         </is>
       </c>
       <c r="E39" s="48" t="inlineStr">
@@ -6850,13 +6886,13 @@
       </c>
       <c r="F39" s="46" t="inlineStr">
         <is>
-          <t>mechanisch: unadj. −0,062 · PET −0,043 · PEESE −0,055 · 3PSM +0,012 · p-uni* +0,012 · Grey-Null; alle korrigierten Punkte im SESOI-Band |r|=0,070; RoBMA ausstehend (H2) — Einordnung: A per DEC-044; RoBMA (H2): BF01(Effekt) 7,03/2,38/1,69, μ̄ −0,009…+0,008 — mechanisch im Bild aller Korrekturverfahren (~0 bis −0,06); Endfassung nach Gate</t>
+          <t>mechanisch: unadj. −0,062 · PET −0,043 · PEESE −0,055 · 3PSM +0,012 · p-uni* +0,012 · Grey-Null; alle korrigierten Punkte im SESOI-Band |r|=0,070; RoBMA ausstehend (H2) — Einordnung: A per DEC-044; RoBMA (H2): BF01(Effekt) 7,03/2,38/1,69, μ̄ −0,009…+0,008 — mechanisch im Bild aller Korrekturverfahren (~0 bis −0,06); Endfassung per DEC-047: Äquivalenzregister, BFs deskriptiv</t>
         </is>
       </c>
       <c r="G39" s="46" t="inlineStr"/>
       <c r="H39" s="46" t="inlineStr">
         <is>
-          <t>Zusammenschau (Entwurf): Alle Korrekturverfahren landen zwischen ~0 und −0,06 — ökonomisch durchweg vernachlässigbar; die Verfahren streiten nur darüber, ob überhaupt ein Rest bleibt. Endfassung nach Gate-Schritt [DEC-044] — RoBMA liegt jetzt vor.</t>
+          <t>Zusammenschau: Alle Korrekturverfahren landen zwischen ~0 und −0,06 — ökonomisch durchweg vernachlässigbar; die Verfahren streiten nur darüber, ob überhaupt ein Rest bleibt. Register per DEC-047: Äquivalenz-Sprachfamilie ("praktisch null im Band"), keine Evidence-of-Absence-Formulierungen; Bayes-Faktoren deskriptiv.</t>
         </is>
       </c>
     </row>
@@ -6967,23 +7003,23 @@
       </c>
       <c r="D43" s="48" t="inlineStr">
         <is>
-          <t>erledigt (2026-07-24, Verifier 17/17) — AUFLÖSUNG offen (dokumentierter Schritt nach TH-b)</t>
+          <t>erledigt (2026-07-24, Verifier 17/17) — AUFLÖSUNG erfolgt (2026-07-27, DEC-047: Äquivalenzregister)</t>
         </is>
       </c>
       <c r="E43" s="48" t="inlineStr">
         <is>
-          <t>output/TH_a_results_workbook.xlsx Tab 6 (E3-Zeilen); output/TH_a_results.csv (Familien-Commit, Basis dafd95e)</t>
+          <t>output/TH_a_results_workbook.xlsx Tab 6 (E3-Zeilen); output/TH_a_results.csv (Familien-Commit, Basis dafd95e); DECISION_LOG.md DEC-047; output/TH_b_results_workbook.xlsx Tab 7 (BF-Inputs)</t>
         </is>
       </c>
       <c r="F43" s="46" t="inlineStr">
         <is>
-          <t>Gate-Konfiguration fixiert: E2-PASS-Requirement + BF01-Leiter (&gt;=3 voll; 1-3 äquivalenzbasiert); Status 'resolution deferred'</t>
+          <t>Gate-Konfiguration fixiert: E2-PASS-Requirement + BF01-Leiter (&gt;=3 voll; 1-3 äquivalenzbasiert); AUFLÖSUNG: E2-Flag 1 (p_TOST = ,022) × BF01(Periode) primär = 1,03 (Band 1–3) ⇒ ÄQUIVALENZREGISTER [DEC-047]; Wide 1,17 bestätigt Band; Default 8,49 nicht claimtragend (nicht-primär, meandif, Konvergenz-Caveats); BF10 &lt; 1 in allen Sets; Vokabular-Sperrliste in DEC-047</t>
         </is>
       </c>
       <c r="G43" s="46" t="inlineStr"/>
       <c r="H43" s="46" t="inlineStr">
         <is>
-          <t>Regelwerk, welche Formulierung ('kein Effekt' vs. 'kein Nachweis') zulässig ist; Entscheidung fällt dokumentiert nach dem Bayes-Lauf.</t>
+          <t>Regelwerk, welche Formulierung ('kein Effekt' vs. 'kein Nachweis') zulässig ist; Entscheidung gefallen [DEC-047]: Äquivalenzregister — "statistisch äquivalent zu null im Band", nicht "Beweis der Abwesenheit"; die Treue zur vorab festgelegten Leiter ist die Stärke des Papers.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T7 spec + package [DEC-043][DEC-048]: Block-C panels + unified ladder frozen; R/10 pair + cc prompt; A.14; ERROR #19-#21; status touch (DLI 59)
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1649,7 +1649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1671,7 +1671,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>57 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>59 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -3386,6 +3386,30 @@
       <c r="G61" t="inlineStr">
         <is>
           <t>aktiv</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>DEC-043</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>DEC-048</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
         </is>
       </c>
     </row>
@@ -6635,7 +6659,7 @@
       <c r="F32" s="46" t="inlineStr"/>
       <c r="G32" s="46" t="inlineStr">
         <is>
-          <t>Resolves als DEC-043; Inputs: Zellgrößen v12 + C0</t>
+          <t>Resolves als DEC-043; Inputs: Zellgrößen v12 + C0 | AUFGELÖST per DEC-043 (2026-07-28); Exec-Spec DEC-048 — Spec eingefroren, Lauf ausstehend</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T7 fix: PD tolerance layer + smoke hardening [DEC-049]; ERROR #23; DLI 60
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1649,7 +1649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1671,7 +1671,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>59 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>60 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -3408,6 +3408,18 @@
         </is>
       </c>
       <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>DEC-049</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>

</xml_diff>

<commit_message>
T7 fix 4: synthetic-outcome design-df (CRVE is residual-based) [DEC-049a]; ERROR #26; DLI 61
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1649,7 +1649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1671,7 +1671,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>60 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>61 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -3420,6 +3420,18 @@
         </is>
       </c>
       <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>DEC-049a</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>

</xml_diff>

<commit_message>
T7 results package [DEC-043][DEC-048][DEC-049][DEC-049a]: canonical run 7 (verifier 27/27, scripts @6e7ce03); results workbook; manuscript/T7.md; status flips C0-C9 + KR Z16; ERROR #29
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1356,7 +1356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1565,12 +1565,17 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>PASS (Verifier 27/27, Lauf 7, 2026-07-29)</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
           <t>output/T7_results.csv</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0/8 Interaktions-HTZ signifikant (min p 0,077; Holm-Min 0,616); pp konditional V1 +0,0078 (p 0,769) / V2 +0,0130 (p 0,426)</t>
         </is>
       </c>
     </row>
@@ -6439,7 +6444,7 @@
       </c>
       <c r="D23" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-29, Verifier 27/27)</t>
         </is>
       </c>
       <c r="E23" s="48" t="inlineStr"/>
@@ -6468,7 +6473,7 @@
       </c>
       <c r="D24" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-29, Verifier 27/27)</t>
         </is>
       </c>
       <c r="E24" s="48" t="inlineStr"/>
@@ -6493,7 +6498,7 @@
       </c>
       <c r="D25" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-29, Verifier 27/27)</t>
         </is>
       </c>
       <c r="E25" s="48" t="inlineStr"/>
@@ -6518,7 +6523,7 @@
       </c>
       <c r="D26" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-29, Verifier 27/27)</t>
         </is>
       </c>
       <c r="E26" s="48" t="inlineStr"/>
@@ -6547,7 +6552,7 @@
       </c>
       <c r="D27" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-29, Verifier 27/27)</t>
         </is>
       </c>
       <c r="E27" s="48" t="inlineStr"/>
@@ -6576,7 +6581,7 @@
       </c>
       <c r="D28" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-29, Verifier 27/27)</t>
         </is>
       </c>
       <c r="E28" s="48" t="inlineStr"/>
@@ -6601,7 +6606,7 @@
       </c>
       <c r="D29" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-29, Verifier 27/27)</t>
         </is>
       </c>
       <c r="E29" s="48" t="inlineStr"/>
@@ -6626,7 +6631,7 @@
       </c>
       <c r="D30" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-29, Verifier 27/27)</t>
         </is>
       </c>
       <c r="E30" s="48" t="inlineStr"/>
@@ -6651,7 +6656,7 @@
       </c>
       <c r="D31" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-29, Verifier 27/27)</t>
         </is>
       </c>
       <c r="E31" s="48" t="inlineStr"/>
@@ -6676,14 +6681,14 @@
       </c>
       <c r="D32" s="48" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-29, Verifier 27/27)</t>
         </is>
       </c>
       <c r="E32" s="48" t="inlineStr"/>
       <c r="F32" s="46" t="inlineStr"/>
       <c r="G32" s="46" t="inlineStr">
         <is>
-          <t>Resolves als DEC-043; Inputs: Zellgrößen v12 + C0 | AUFGELÖST per DEC-043 (2026-07-28); Exec-Spec DEC-048 — Spec eingefroren, Lauf ausstehend</t>
+          <t>Resolves als DEC-043; Inputs: Zellgrößen v12 + C0 | AUFGELÖST per DEC-043 (2026-07-28); Exec-Spec DEC-048 — Spec eingefroren; Kanoniklauf 7 akzeptiert (HEAD 6e7ce03, Verifier 27/27)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
TG workbook + feed + register(partial) + status [DEC-050]
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2438" uniqueCount="1737">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2441" uniqueCount="1740">
   <si>
     <t xml:space="preserve">FOMA CER–COD (Paris-Moderator) — Setup &amp; Workflow (v1, 2026-06-29)</t>
   </si>
@@ -1880,7 +1880,7 @@
     <t xml:space="preserve">Headline ohne die 99 star-bound-Zeilen (11 Studien)</t>
   </si>
   <si>
-    <t xml:space="preserve">erledigt (2026-07-29, TG 12/12, Commit folgt)</t>
+    <t xml:space="preserve">erledigt (2026-07-29, TG 12/12, c935b28)</t>
   </si>
   <si>
     <t xml:space="preserve">G2</t>
@@ -1979,7 +1979,7 @@
     <t xml:space="preserve">Eine Zeile pro Spezifikation (~25), Querverweis-Spalte "reported in §x.y"; Appendix vollständig</t>
   </si>
   <si>
-    <t xml:space="preserve">partial — F rows pending (Registerbau in W-/F-Session)</t>
+    <t xml:space="preserve">partial — F rows pending (Registerbau in W-/F-Session); register partial committed (W)</t>
   </si>
   <si>
     <t xml:space="preserve">corpus_segment + cluster_study + Provenienz-Specs gestrichen; on-demand hinterlegt</t>
@@ -4599,6 +4599,15 @@
   </si>
   <si>
     <t xml:space="preserve">output/TH_b_results.csv; output/TH_b_results_workbook.xlsx (Block-2-Commit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TG · Block-G-Robustheit (G1–G11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spine-Varianten r = -0,038…-0,062 (Headline -0,059); 7/7 Vorzeichen erhalten, 7/7 im SESOI-Band |r| &lt;= 0,070; G4-CI ueberdeckt 0 (104 ES/52 St.) · Panels HTZ p = 0,218–0,988 (deskriptiv, DEC-047) · Register 23 Zeilen partial (5 A + 11 G befuellt, 7 F-Platzhalter)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">output/TG_results.csv; output/TG_results_workbook.xlsx; output/robustness_register.csv; manuscript/TG.md</t>
   </si>
   <si>
     <t xml:space="preserve">Decision-Log Index — DEC-ID-Register (Methodik-only; Pointer auf DECISION_LOG.md) (v1)</t>
@@ -5250,7 +5259,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5343,6 +5352,12 @@
     <font>
       <sz val="9"/>
       <color rgb="FF595959"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -5489,7 +5504,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -5688,6 +5703,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -6399,7 +6418,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
@@ -6594,6 +6613,17 @@
       </c>
       <c r="C20" s="6" t="s">
         <v>1522</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="50" t="s">
+        <v>1523</v>
+      </c>
+      <c r="B21" s="50" t="s">
+        <v>1524</v>
+      </c>
+      <c r="C21" s="50" t="s">
+        <v>1525</v>
       </c>
     </row>
   </sheetData>
@@ -6632,7 +6662,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>1523</v>
+        <v>1526</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -6643,7 +6673,7 @@
     </row>
     <row r="2" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>1524</v>
+        <v>1527</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -6654,559 +6684,559 @@
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="20" t="s">
-        <v>1525</v>
+        <v>1528</v>
       </c>
       <c r="B3" s="20" t="s">
-        <v>1526</v>
+        <v>1529</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>1527</v>
+        <v>1530</v>
       </c>
       <c r="D3" s="20" t="s">
         <v>375</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>1528</v>
+        <v>1531</v>
       </c>
       <c r="F3" s="20" t="s">
-        <v>1529</v>
+        <v>1532</v>
       </c>
       <c r="G3" s="20" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="50" t="s">
-        <v>1530</v>
+      <c r="A4" s="51" t="s">
+        <v>1533</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>1531</v>
+        <v>1534</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>1532</v>
+        <v>1535</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>1533</v>
+        <v>1536</v>
       </c>
       <c r="E4" s="5" t="s">
+        <v>1537</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>1538</v>
+      </c>
+      <c r="G4" s="51" t="s">
+        <v>1539</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="51" t="s">
+        <v>194</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>1534</v>
       </c>
-      <c r="F4" s="6" t="s">
-        <v>1535</v>
-      </c>
-      <c r="G4" s="50" t="s">
-        <v>1536</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="50" t="s">
-        <v>194</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>1531</v>
-      </c>
       <c r="C5" s="5" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>1538</v>
+        <v>1541</v>
       </c>
       <c r="E5" s="5" t="s">
+        <v>1542</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>1543</v>
+      </c>
+      <c r="G5" s="51" t="s">
         <v>1539</v>
       </c>
-      <c r="F5" s="6" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="51" t="s">
+        <v>1544</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C6" s="5" t="s">
         <v>1540</v>
       </c>
-      <c r="G5" s="50" t="s">
-        <v>1536</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="50" t="s">
-        <v>1541</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>1531</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>1537</v>
-      </c>
       <c r="D6" s="6" t="s">
-        <v>1542</v>
+        <v>1545</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>1543</v>
+        <v>1546</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>1544</v>
-      </c>
-      <c r="G6" s="50" t="s">
-        <v>1536</v>
+        <v>1547</v>
+      </c>
+      <c r="G6" s="51" t="s">
+        <v>1539</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="50" t="s">
+      <c r="A7" s="51" t="s">
         <v>218</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>1531</v>
+        <v>1534</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>1545</v>
+        <v>1548</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>1546</v>
+        <v>1549</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>1547</v>
-      </c>
-      <c r="G7" s="50" t="s">
-        <v>1536</v>
+        <v>1550</v>
+      </c>
+      <c r="G7" s="51" t="s">
+        <v>1539</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="50" t="s">
+      <c r="A8" s="51" t="s">
         <v>200</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>1531</v>
+        <v>1534</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>1548</v>
+        <v>1551</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>1549</v>
+        <v>1552</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>1550</v>
-      </c>
-      <c r="G8" s="50" t="s">
-        <v>1551</v>
+        <v>1553</v>
+      </c>
+      <c r="G8" s="51" t="s">
+        <v>1554</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="50" t="s">
+      <c r="A9" s="51" t="s">
         <v>206</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>1531</v>
+        <v>1534</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>1552</v>
+        <v>1555</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>1553</v>
+        <v>1556</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>1554</v>
+        <v>1557</v>
       </c>
       <c r="F9" s="6" t="s">
+        <v>1558</v>
+      </c>
+      <c r="G9" s="51" t="s">
+        <v>1539</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="51" t="s">
+        <v>1559</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>1540</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>1560</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>1561</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>1562</v>
+      </c>
+      <c r="G10" s="51" t="s">
+        <v>1539</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="51" t="s">
+        <v>1563</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>1564</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>1565</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>1566</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>1567</v>
+      </c>
+      <c r="G11" s="51" t="s">
+        <v>1539</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="51" t="s">
+        <v>242</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>1540</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>1568</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>1569</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>1570</v>
+      </c>
+      <c r="G12" s="51" t="s">
+        <v>1539</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="51" t="s">
+        <v>1571</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>1540</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>1572</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>1573</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>1574</v>
+      </c>
+      <c r="G13" s="51" t="s">
+        <v>1539</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="51" t="s">
+        <v>229</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>1555</v>
       </c>
-      <c r="G9" s="50" t="s">
-        <v>1536</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="50" t="s">
-        <v>1556</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>1531</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>1537</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>1557</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>1558</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>1559</v>
-      </c>
-      <c r="G10" s="50" t="s">
-        <v>1536</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="50" t="s">
-        <v>1560</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>1531</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>1561</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>1562</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>1563</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>1564</v>
-      </c>
-      <c r="G11" s="50" t="s">
-        <v>1536</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="50" t="s">
-        <v>242</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>1531</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>1537</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>1565</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>1566</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>1567</v>
-      </c>
-      <c r="G12" s="50" t="s">
-        <v>1536</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="50" t="s">
-        <v>1568</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>1531</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>1537</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>1569</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>1570</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>1571</v>
-      </c>
-      <c r="G13" s="50" t="s">
-        <v>1536</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="50" t="s">
-        <v>229</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>1531</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>1552</v>
-      </c>
       <c r="D14" s="6" t="s">
-        <v>1572</v>
+        <v>1575</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>1573</v>
+        <v>1576</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>1574</v>
-      </c>
-      <c r="G14" s="50" t="s">
-        <v>1536</v>
+        <v>1577</v>
+      </c>
+      <c r="G14" s="51" t="s">
+        <v>1539</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="50" t="s">
+      <c r="A15" s="51" t="s">
         <v>233</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>1531</v>
+        <v>1534</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>1575</v>
+        <v>1578</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>1576</v>
+        <v>1579</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>1577</v>
-      </c>
-      <c r="G15" s="50" t="s">
-        <v>1536</v>
+        <v>1580</v>
+      </c>
+      <c r="G15" s="51" t="s">
+        <v>1539</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="50" t="s">
+      <c r="A16" s="51" t="s">
         <v>237</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>1531</v>
+        <v>1534</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>1578</v>
+        <v>1581</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>1579</v>
+        <v>1582</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>1580</v>
-      </c>
-      <c r="G16" s="50" t="s">
-        <v>1536</v>
+        <v>1583</v>
+      </c>
+      <c r="G16" s="51" t="s">
+        <v>1539</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="50" t="s">
+      <c r="A17" s="51" t="s">
         <v>257</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>1581</v>
+        <v>1584</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>1582</v>
+        <v>1585</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>1583</v>
+        <v>1586</v>
       </c>
       <c r="F17" s="6" t="s">
+        <v>1587</v>
+      </c>
+      <c r="G17" s="51" t="s">
+        <v>1539</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="51" t="s">
+        <v>263</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>1584</v>
       </c>
-      <c r="G17" s="50" t="s">
-        <v>1536</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="50" t="s">
-        <v>263</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>1581</v>
-      </c>
       <c r="C18" s="5" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>1585</v>
+        <v>1588</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>1586</v>
+        <v>1589</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>1587</v>
-      </c>
-      <c r="G18" s="50" t="s">
-        <v>1536</v>
+        <v>1590</v>
+      </c>
+      <c r="G18" s="51" t="s">
+        <v>1539</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="50" t="s">
+      <c r="A19" s="51" t="s">
         <v>269</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>1581</v>
+        <v>1584</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>1588</v>
+        <v>1591</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>1589</v>
+        <v>1592</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>1590</v>
-      </c>
-      <c r="G19" s="50" t="s">
-        <v>1536</v>
+        <v>1593</v>
+      </c>
+      <c r="G19" s="51" t="s">
+        <v>1539</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="50" t="s">
-        <v>1591</v>
+      <c r="A20" s="51" t="s">
+        <v>1594</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>1581</v>
+        <v>1584</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>1592</v>
+        <v>1595</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>1593</v>
+        <v>1596</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>1594</v>
-      </c>
-      <c r="G20" s="50" t="s">
-        <v>1536</v>
+        <v>1597</v>
+      </c>
+      <c r="G20" s="51" t="s">
+        <v>1539</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="50" t="s">
-        <v>1595</v>
+      <c r="A21" s="51" t="s">
+        <v>1598</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>1581</v>
+        <v>1584</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>1596</v>
+        <v>1599</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>1597</v>
+        <v>1600</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>1598</v>
-      </c>
-      <c r="G21" s="50" t="s">
-        <v>1536</v>
+        <v>1601</v>
+      </c>
+      <c r="G21" s="51" t="s">
+        <v>1539</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="50" t="s">
-        <v>1599</v>
+      <c r="A22" s="51" t="s">
+        <v>1602</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>1600</v>
+        <v>1603</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>1601</v>
+        <v>1604</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>1602</v>
+        <v>1605</v>
       </c>
       <c r="F22" s="6" t="s">
+        <v>1606</v>
+      </c>
+      <c r="G22" s="51" t="s">
+        <v>1539</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="51" t="s">
+        <v>1607</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>1603</v>
       </c>
-      <c r="G22" s="50" t="s">
-        <v>1536</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="50" t="s">
-        <v>1604</v>
-      </c>
-      <c r="B23" s="5" t="s">
-        <v>1600</v>
-      </c>
       <c r="C23" s="5" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>1605</v>
+        <v>1608</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>1606</v>
+        <v>1609</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>1607</v>
-      </c>
-      <c r="G23" s="50" t="s">
-        <v>1536</v>
+        <v>1610</v>
+      </c>
+      <c r="G23" s="51" t="s">
+        <v>1539</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="50" t="s">
-        <v>1608</v>
+      <c r="A24" s="51" t="s">
+        <v>1611</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>1600</v>
+        <v>1603</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>1609</v>
+        <v>1612</v>
       </c>
       <c r="E24" s="5" t="s">
         <v>367</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>1610</v>
-      </c>
-      <c r="G24" s="50" t="s">
-        <v>1536</v>
+        <v>1613</v>
+      </c>
+      <c r="G24" s="51" t="s">
+        <v>1539</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="50" t="s">
-        <v>1611</v>
+      <c r="A25" s="51" t="s">
+        <v>1614</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>1600</v>
+        <v>1603</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>1612</v>
+        <v>1615</v>
       </c>
       <c r="E25" s="5" t="s">
         <v>359</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>1613</v>
-      </c>
-      <c r="G25" s="50" t="s">
-        <v>1536</v>
+        <v>1616</v>
+      </c>
+      <c r="G25" s="51" t="s">
+        <v>1539</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="50" t="s">
-        <v>1614</v>
+      <c r="A26" s="51" t="s">
+        <v>1617</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>1600</v>
+        <v>1603</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>1615</v>
+        <v>1618</v>
       </c>
       <c r="E26" s="5" t="s">
         <v>359</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>1616</v>
-      </c>
-      <c r="G26" s="50" t="s">
-        <v>1536</v>
+        <v>1619</v>
+      </c>
+      <c r="G26" s="51" t="s">
+        <v>1539</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>1617</v>
+        <v>1620</v>
       </c>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -7217,71 +7247,71 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>1618</v>
+        <v>1621</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>1600</v>
+        <v>1603</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>1619</v>
+        <v>1622</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>359</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>1620</v>
+        <v>1623</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>1536</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>1621</v>
+        <v>1624</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>1600</v>
+        <v>1603</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>1352</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>1622</v>
+        <v>1625</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>1623</v>
+        <v>1626</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>1624</v>
+        <v>1627</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>1536</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>1625</v>
+        <v>1628</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>1600</v>
+        <v>1603</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>1626</v>
+        <v>1629</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>1627</v>
+        <v>1630</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>1628</v>
+        <v>1631</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>1536</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7289,50 +7319,50 @@
         <v>773</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>1629</v>
+        <v>1632</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>1352</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>1630</v>
+        <v>1633</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>1631</v>
+        <v>1634</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>1632</v>
+        <v>1635</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>1536</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>1633</v>
+        <v>1636</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>1629</v>
+        <v>1632</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>1634</v>
+        <v>1637</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>1635</v>
+        <v>1638</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>1636</v>
+        <v>1639</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>1536</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="50" t="s">
-        <v>1637</v>
+      <c r="A33" s="51" t="s">
+        <v>1640</v>
       </c>
       <c r="B33" s="49"/>
       <c r="C33" s="49"/>
@@ -7343,449 +7373,449 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>1638</v>
+        <v>1641</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>1639</v>
+        <v>1642</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>1640</v>
+        <v>1643</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>1641</v>
+        <v>1644</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>1642</v>
+        <v>1645</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>1643</v>
+        <v>1646</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>1644</v>
+        <v>1647</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>1645</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>1646</v>
+        <v>1649</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>1647</v>
+        <v>1650</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>1648</v>
+        <v>1651</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>1649</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>1650</v>
+        <v>1653</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>1651</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>1652</v>
+        <v>1655</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>1653</v>
+        <v>1656</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>1654</v>
+        <v>1657</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>1655</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>1656</v>
+        <v>1659</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>1657</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>1658</v>
+        <v>1661</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>1659</v>
+        <v>1662</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>1660</v>
+        <v>1663</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>1661</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>1662</v>
+        <v>1665</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>1663</v>
+        <v>1666</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>1664</v>
+        <v>1667</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>1665</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>1666</v>
+        <v>1669</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>1667</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>1668</v>
+        <v>1671</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>1669</v>
+        <v>1672</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>1670</v>
+        <v>1673</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>1671</v>
+        <v>1674</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>1672</v>
+        <v>1675</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>1673</v>
+        <v>1676</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>1674</v>
+        <v>1677</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>1675</v>
+        <v>1678</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>1676</v>
+        <v>1679</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>1677</v>
+        <v>1680</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>1678</v>
+        <v>1681</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>1679</v>
+        <v>1682</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>1680</v>
+        <v>1683</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>1681</v>
+        <v>1684</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>1536</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>1682</v>
+        <v>1685</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>1683</v>
+        <v>1686</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>1684</v>
+        <v>1687</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>1685</v>
+        <v>1688</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>1686</v>
+        <v>1689</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>1536</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>1687</v>
+        <v>1690</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>1688</v>
+        <v>1691</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>1689</v>
+        <v>1692</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>1690</v>
+        <v>1693</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>1691</v>
+        <v>1694</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>1536</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>1692</v>
+        <v>1695</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>1688</v>
+        <v>1691</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>1693</v>
+        <v>1696</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>1694</v>
+        <v>1697</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>1695</v>
+        <v>1698</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>1536</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>1696</v>
+        <v>1699</v>
       </c>
       <c r="B55" s="1" t="s">
+        <v>1691</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>1540</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>1700</v>
+      </c>
+      <c r="E55" s="1" t="s">
         <v>1688</v>
       </c>
-      <c r="C55" s="1" t="s">
-        <v>1537</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>1697</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>1685</v>
-      </c>
       <c r="F55" s="1" t="s">
-        <v>1698</v>
+        <v>1701</v>
       </c>
       <c r="G55" s="1" t="s">
-        <v>1536</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>1699</v>
+        <v>1702</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>1700</v>
+        <v>1703</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>1701</v>
+        <v>1704</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>1702</v>
+        <v>1705</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>1703</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>1704</v>
+        <v>1707</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>1705</v>
+        <v>1708</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>1706</v>
+        <v>1709</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>1707</v>
+        <v>1710</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>1708</v>
+        <v>1711</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>1709</v>
+        <v>1712</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>1710</v>
+        <v>1713</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>1552</v>
+        <v>1555</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>1711</v>
+        <v>1714</v>
       </c>
       <c r="E58" s="1" t="s">
-        <v>1712</v>
+        <v>1715</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>1713</v>
+        <v>1716</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>1714</v>
+        <v>1717</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>1715</v>
+        <v>1718</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>1716</v>
+        <v>1719</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>1717</v>
+        <v>1720</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>1718</v>
+        <v>1721</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>1536</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>1719</v>
+        <v>1722</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>1720</v>
+        <v>1723</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>1537</v>
+        <v>1540</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>1721</v>
+        <v>1724</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>1722</v>
+        <v>1725</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>1723</v>
+        <v>1726</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>1536</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>1724</v>
+        <v>1727</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>1720</v>
+        <v>1723</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>1552</v>
+        <v>1555</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>1725</v>
+        <v>1728</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>1726</v>
+        <v>1729</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>1727</v>
+        <v>1730</v>
       </c>
       <c r="G61" s="1" t="s">
-        <v>1536</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>1728</v>
+        <v>1731</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>1729</v>
+        <v>1732</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>1730</v>
+        <v>1733</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>1729</v>
+        <v>1732</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>1731</v>
+        <v>1734</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>1729</v>
+        <v>1732</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
+        <v>1735</v>
+      </c>
+      <c r="B65" s="1" t="s">
         <v>1732</v>
-      </c>
-      <c r="B65" s="1" t="s">
-        <v>1729</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>1733</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1736</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>1734</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1737</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>1735</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1738</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>1736</v>
+        <v>1739</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TF route fix: F1 rstudent parallel snow + worker pins 8/8 + observability [DEC-051a, ERROR #35]
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -837,8 +837,8 @@
   <dimension ref="A1:B56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="34" customWidth="1" style="52" min="1" max="1"/>
-    <col width="98" customWidth="1" style="52" min="2" max="2"/>
+    <col width="34" customWidth="1" style="102" min="1" max="1"/>
+    <col width="98" customWidth="1" style="102" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.5" customHeight="1" s="53">
@@ -1000,7 +1000,7 @@
       </c>
     </row>
     <row r="16" ht="16.5" customHeight="1" s="53">
-      <c r="A16" s="52" t="inlineStr">
+      <c r="A16" s="102" t="inlineStr">
         <is>
           <t>Prozess-Update 2026-07-12</t>
         </is>
@@ -1415,36 +1415,36 @@
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="53">
-      <c r="A54" s="52" t="inlineStr">
+      <c r="A54" s="102" t="inlineStr">
         <is>
           <t>Analyse_Batterie</t>
         </is>
       </c>
-      <c r="B54" s="52" t="inlineStr">
+      <c r="B54" s="102" t="inlineStr">
         <is>
           <t>FÜHREND: Analyse-Tracking A1–H11 (64 Analysen; Nr/Titel/Beschreibung/Status/Referenz/Ergebnis/Anmerkung) per DEC-031/031a.</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="53">
-      <c r="A55" s="52" t="inlineStr">
+      <c r="A55" s="102" t="inlineStr">
         <is>
           <t>Null_Battery</t>
         </is>
       </c>
-      <c r="B55" s="52" t="inlineStr">
+      <c r="B55" s="102" t="inlineStr">
         <is>
           <t>ARCHIV — N-Register (Prosa); operativ in Analyse_Batterie Block H.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="53">
-      <c r="A56" s="52" t="inlineStr">
+      <c r="A56" s="102" t="inlineStr">
         <is>
           <t>Update_Scoping</t>
         </is>
       </c>
-      <c r="B56" s="52" t="inlineStr">
+      <c r="B56" s="102" t="inlineStr">
         <is>
           <t>ARCHIV — Screening-Register des 2026-Updates; R2-Preview = Revisions-Kontingenz.</t>
         </is>
@@ -1478,9 +1478,9 @@
   <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="34" customWidth="1" style="52" min="1" max="1"/>
-    <col width="70" customWidth="1" style="52" min="2" max="2"/>
-    <col width="40" customWidth="1" style="52" min="3" max="3"/>
+    <col width="34" customWidth="1" style="102" min="1" max="1"/>
+    <col width="70" customWidth="1" style="102" min="2" max="2"/>
+    <col width="40" customWidth="1" style="102" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.5" customHeight="1" s="53">
@@ -1515,7 +1515,7 @@
       </c>
     </row>
     <row r="4" ht="16.5" customHeight="1" s="53">
-      <c r="A4" s="52" t="inlineStr">
+      <c r="A4" s="102" t="inlineStr">
         <is>
           <t>n=2.713 · 115 Studien/114 Cluster · Post-Zelle 31 Studien · df(pp_mid)=31,9 · beide Upgrades TRUE — kanonisch (Verifier v2 28/28, 2026-07-12)</t>
         </is>
@@ -1570,12 +1570,12 @@
           <t>T1/A2 · Heterogenitaet (sigma2 je Ebene, Anteile)</t>
         </is>
       </c>
-      <c r="B8" s="52" t="inlineStr">
+      <c r="B8" s="102" t="inlineStr">
         <is>
           <t>62,3% Cluster / ~0% Studie (Boundary) / 37,5% ES / 0,1% Sampling</t>
         </is>
       </c>
-      <c r="C8" s="52" t="inlineStr">
+      <c r="C8" s="102" t="inlineStr">
         <is>
           <t>output/T1_results.csv (A2); Workbook Tab 7</t>
         </is>
@@ -1692,7 +1692,7 @@
           <t>output/T7_results.csv</t>
         </is>
       </c>
-      <c r="D16" s="52" t="inlineStr">
+      <c r="D16" s="102" t="inlineStr">
         <is>
           <t>0/8 Interaktions-HTZ signifikant (min p 0,077; Holm-Min 0,616); pp konditional V1 +0,0078 (p 0,769) / V2 +0,0130 (p 0,426)</t>
         </is>
@@ -1792,16 +1792,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="10" customWidth="1" style="52" min="1" max="1"/>
-    <col width="12" customWidth="1" style="52" min="2" max="2"/>
-    <col width="15" customWidth="1" style="52" min="3" max="3"/>
-    <col width="30" customWidth="1" style="52" min="4" max="4"/>
-    <col width="16" customWidth="1" style="52" min="5" max="5"/>
-    <col width="53" customWidth="1" style="52" min="6" max="6"/>
-    <col width="12" customWidth="1" style="52" min="7" max="7"/>
+    <col width="10" customWidth="1" style="102" min="1" max="1"/>
+    <col width="12" customWidth="1" style="102" min="2" max="2"/>
+    <col width="15" customWidth="1" style="102" min="3" max="3"/>
+    <col width="30" customWidth="1" style="102" min="4" max="4"/>
+    <col width="16" customWidth="1" style="102" min="5" max="5"/>
+    <col width="53" customWidth="1" style="102" min="6" max="6"/>
+    <col width="12" customWidth="1" style="102" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.5" customHeight="1" s="53">
@@ -1814,7 +1814,7 @@
     <row r="2" ht="39.75" customHeight="1" s="53">
       <c r="A2" s="55" t="inlineStr">
         <is>
-          <t>66 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>67 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -2707,192 +2707,192 @@
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="53">
-      <c r="A27" s="52" t="inlineStr">
+      <c r="A27" s="102" t="inlineStr">
         <is>
           <t>DEC-024</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="53">
-      <c r="A28" s="52" t="inlineStr">
+      <c r="A28" s="102" t="inlineStr">
         <is>
           <t>DEC-025</t>
         </is>
       </c>
-      <c r="B28" s="52" t="inlineStr">
+      <c r="B28" s="102" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="C28" s="52" t="inlineStr">
+      <c r="C28" s="102" t="inlineStr">
         <is>
           <t>Methodik</t>
         </is>
       </c>
-      <c r="D28" s="52" t="inlineStr">
+      <c r="D28" s="102" t="inlineStr">
         <is>
           <t>Quality-Moderatoren konsolidiert; q_JIF gestrichen</t>
         </is>
       </c>
-      <c r="E28" s="52" t="inlineStr">
+      <c r="E28" s="102" t="inlineStr">
         <is>
           <t>T7</t>
         </is>
       </c>
-      <c r="F28" s="52" t="inlineStr">
+      <c r="F28" s="102" t="inlineStr">
         <is>
           <t>q_status + q_VHB (published-only, Referenzzellen-Kodierung); univariate VHB-Panels nur published; JIF analytisch tot (Roh im Lookup); DEC-023-Offenpunkt geschlossen</t>
         </is>
       </c>
-      <c r="G28" s="52" t="inlineStr">
+      <c r="G28" s="102" t="inlineStr">
         <is>
           <t>aktiv</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="53">
-      <c r="A29" s="52" t="inlineStr">
+      <c r="A29" s="102" t="inlineStr">
         <is>
           <t>DEC-026</t>
         </is>
       </c>
-      <c r="B29" s="52" t="inlineStr">
+      <c r="B29" s="102" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="C29" s="52" t="inlineStr">
+      <c r="C29" s="102" t="inlineStr">
         <is>
           <t>Daten</t>
         </is>
       </c>
-      <c r="D29" s="52" t="inlineStr">
+      <c r="D29" s="102" t="inlineStr">
         <is>
           <t>Publikationsstatus-Korrektur + Versions-Regel + Voll-Audit</t>
         </is>
       </c>
-      <c r="E29" s="52" t="inlineStr">
+      <c r="E29" s="102" t="inlineStr">
         <is>
           <t>source_lookup / T5,T7</t>
         </is>
       </c>
-      <c r="F29" s="52" t="inlineStr">
+      <c r="F29" s="102" t="inlineStr">
         <is>
           <t>7 Studien (229 Eff.) → published (Stand 2026-07-03); Effekte bleiben as-coded (Triage: keine materiellen Abweichungen); 66-Zeilen-Audit; spec status_as_extracted; Feld-Semantik journal/year=as coded, reference_verified=VoR</t>
         </is>
       </c>
-      <c r="G29" s="52" t="inlineStr">
+      <c r="G29" s="102" t="inlineStr">
         <is>
           <t>aktiv</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="53">
-      <c r="A30" s="52" t="inlineStr">
+      <c r="A30" s="102" t="inlineStr">
         <is>
           <t>DEC-027</t>
         </is>
       </c>
-      <c r="B30" s="52" t="inlineStr">
+      <c r="B30" s="102" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="C30" s="52" t="inlineStr">
+      <c r="C30" s="102" t="inlineStr">
         <is>
           <t>Methodik</t>
         </is>
       </c>
-      <c r="D30" s="52" t="inlineStr">
+      <c r="D30" s="102" t="inlineStr">
         <is>
           <t>n-Definition validiert; E14 → n_obs</t>
         </is>
       </c>
-      <c r="E30" s="52" t="inlineStr">
+      <c r="E30" s="102" t="inlineStr">
         <is>
           <t>#1 / T1,T2,T4</t>
         </is>
       </c>
-      <c r="F30" s="52" t="inlineStr">
+      <c r="F30" s="102" t="inlineStr">
         <is>
           <t>no_firms bestätigt (konservativ; CR2-working-weights); Ableitungsregel round(n_obs/T) dokumentiert (85% konsistent, alle 9 n&lt;10); E14 umbenannt n_obs (81 Eff./3 Studien sub-annual/loan-level)</t>
         </is>
       </c>
-      <c r="G30" s="52" t="inlineStr">
+      <c r="G30" s="102" t="inlineStr">
         <is>
           <t>aktiv</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="53">
-      <c r="A31" s="52" t="inlineStr">
+      <c r="A31" s="102" t="inlineStr">
         <is>
           <t>DEC-028</t>
         </is>
       </c>
-      <c r="B31" s="52" t="inlineStr">
+      <c r="B31" s="102" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="C31" s="52" t="inlineStr">
+      <c r="C31" s="102" t="inlineStr">
         <is>
           <t>Daten</t>
         </is>
       </c>
-      <c r="D31" s="52" t="inlineStr">
+      <c r="D31" s="102" t="inlineStr">
         <is>
           <t>Daten-Doku-Abschluss v9/v10; Pending-B gelöst</t>
         </is>
       </c>
-      <c r="E31" s="52" t="inlineStr">
+      <c r="E31" s="102" t="inlineStr">
         <is>
           <t>data/lookup · §§1/2/7/9</t>
         </is>
       </c>
-      <c r="F31" s="52" t="inlineStr">
+      <c r="F31" s="102" t="inlineStr">
         <is>
           <t>v10 kanonisch; formula-Sheet dokumentiert 4 Konversionsrouten; ES-Typ korrigiert (36 bivariat / 1.270 PCC); df≈n_obs-Konvention + pcc_df_k-Sensitivität; ES_source ersetzt es_type/method_artefacts; V4-Flags autoritativ (calculated 54,6%); Li-Key-Rename 2021→2022; Shad-Kreuznotiz (F22)</t>
         </is>
       </c>
-      <c r="G31" s="52" t="inlineStr">
+      <c r="G31" s="102" t="inlineStr">
         <is>
           <t>aktiv</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="53">
-      <c r="A32" s="52" t="inlineStr">
+      <c r="A32" s="102" t="inlineStr">
         <is>
           <t>DEC-029</t>
         </is>
       </c>
-      <c r="B32" s="52" t="inlineStr">
+      <c r="B32" s="102" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="C32" s="52" t="inlineStr">
+      <c r="C32" s="102" t="inlineStr">
         <is>
           <t>Methodik</t>
         </is>
       </c>
-      <c r="D32" s="52" t="inlineStr">
+      <c r="D32" s="102" t="inlineStr">
         <is>
           <t>Null-Battery a priori designiert (N1–N15, alle)</t>
         </is>
       </c>
-      <c r="E32" s="52" t="inlineStr">
+      <c r="E32" s="102" t="inlineStr">
         <is>
           <t>Null_Battery · §§9/13 · T1-Gate</t>
         </is>
       </c>
-      <c r="F32" s="52" t="inlineStr">
+      <c r="F32" s="102" t="inlineStr">
         <is>
           <t>Alle 15 GO; Platzierungen fixiert; N13 konditional (≥5-Regel); N15 deskriptiv mit DEC-008-Teil-Reopen; Inputs (SESOI/F18, Priors, Faktorraum, Grids, Fensterparameter) VOR T1 zu fixieren; Paper-Beschaffung: Lakens, Simonsohn 2020, WAAP</t>
         </is>
       </c>
-      <c r="G32" s="52" t="inlineStr">
+      <c r="G32" s="102" t="inlineStr">
         <is>
           <t>aktiv</t>
         </is>
@@ -2912,697 +2912,697 @@
       <c r="G33" s="61" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="53">
-      <c r="A34" s="52" t="inlineStr">
+      <c r="A34" s="102" t="inlineStr">
         <is>
           <t>DEC-030</t>
         </is>
       </c>
-      <c r="B34" s="52" t="inlineStr">
+      <c r="B34" s="102" t="inlineStr">
         <is>
           <t>Formales PRISMA-Suchupdate beschlossen (rule-based, pre-T1); CER-Gate kodifiziert (F32v2); 4-Engine-Scoping dokumentiert (~41+10 Kandidaten); Renumbering: Battery-Inputs → DEC-031</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="53">
-      <c r="A35" s="52" t="inlineStr">
+      <c r="A35" s="102" t="inlineStr">
         <is>
           <t>DEC-032</t>
         </is>
       </c>
-      <c r="B35" s="52" t="inlineStr">
+      <c r="B35" s="102" t="inlineStr">
         <is>
           <t>AI-Extraktion mit Rollen-Inversion (Claude extrahiert, Volker verifiziert 100% der Statistikfelder); Codebook v1 frozen (F34a-f kodifiziert; 13/13 Kalibrier-Effekte zellengenau reproduziert); Blind-Pilot-Gate ≥95% Konkordanz vor Produktion</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="53">
-      <c r="A36" s="52" t="inlineStr">
+      <c r="A36" s="102" t="inlineStr">
         <is>
           <t>DEC-033</t>
         </is>
       </c>
-      <c r="B36" s="52" t="inlineStr">
+      <c r="B36" s="102" t="inlineStr">
         <is>
           <t>Option C: Vollkorpus-Re-Extraktion unter Codebook v1.1 (Cowork); neue Extraktion = kanonisch für v11; v10 = unabhängige Doppelkodierung; Exact-Match = wechselseitig verifiziert, nur Diffs+Neu-Zeilen zu Volker; Capelle-Blancard raus (unit of analysis, 66-&gt;65); Segment-Flag bleibt</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="53">
-      <c r="A37" s="52" t="inlineStr">
+      <c r="A37" s="102" t="inlineStr">
         <is>
           <t>DEC-034</t>
         </is>
       </c>
-      <c r="B37" s="52" t="inlineStr">
+      <c r="B37" s="102" t="inlineStr">
         <is>
           <t>Sechs Zusatzfelder (copy-level, purpose-tagged, result-blind): x_lag, estimation_method, se_clustering, subsample_dimension/value, subsample_start/end (Effekt-Ebene), n_obs_by_year (Studien-Ebene); Codebook v1.2; Headline-Definitionen unverändert (DEC-024); Pilot-Stagings invalidiert (Batch-Uniformität)</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="53">
-      <c r="A38" s="52" t="inlineStr">
+      <c r="A38" s="102" t="inlineStr">
         <is>
           <t>DEC-035</t>
         </is>
       </c>
-      <c r="B38" s="52" t="inlineStr">
+      <c r="B38" s="102" t="inlineStr">
         <is>
           <t>Mid-Batch-Gate-Rulings: F38 (Delis bleibt; Reserven=Conduct; Grenzformel) · F39a Fard-Exit (64-&gt;63, -46 Eff.) · F39b KLD-Concern=Conduct (v1.4; B&amp;H-Re-Run; Chava via Adjudikation) · F39c-e Adjudikation · F39f Fix; Versions-Verteidigung: additive Deltas + gezielte Re-Runs = single-rule-set-äquivalent</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="53">
-      <c r="A39" s="52" t="inlineStr">
+      <c r="A39" s="102" t="inlineStr">
         <is>
           <t>DEC-036</t>
         </is>
       </c>
-      <c r="B39" s="52" t="inlineStr">
+      <c r="B39" s="102" t="inlineStr">
         <is>
           <t>F40 a-e kodifiziert (v1.5): Eigen-Mass-Dummies, Awareness-als-Disclosure, Heckman-Outcome-Gleichungen, Gologit-Thresholds, Verbrauchsmasse — additive Mikro-Rulings; keine Re-Runs (Adjudikation löst FLAGs); DEC-037 reserviert für Adjudikation+v11</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="53">
-      <c r="A40" s="52" t="inlineStr">
+      <c r="A40" s="102" t="inlineStr">
         <is>
           <t>DEC-037</t>
         </is>
       </c>
-      <c r="B40" s="52" t="inlineStr">
+      <c r="B40" s="102" t="inlineStr">
         <is>
           <t>F41 a-e (v1.6): Kölbel bleibt (Disclosure-Kanal-Grenze; Re-Run) · Systemschätzer-Linie (Lemma-Präzedenz; Mahmoudian-Re-Run; kein Lemma-Re-Run) · CECE=Conduct · Spread-Komponenten rein · Stars-only-Label; Maaloul-Quellidentität geklärt (Lookup-Erratum -&gt; F35; M&amp;W-2022 = Korpusquelle; Maaloul-2018 bleibt F28/raus)</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="53">
-      <c r="A41" s="52" t="inlineStr">
+      <c r="A41" s="102" t="inlineStr">
         <is>
           <t>DEC-038</t>
         </is>
       </c>
-      <c r="B41" s="52" t="inlineStr">
+      <c r="B41" s="102" t="inlineStr">
         <is>
           <t>Post-Batch-Bündel: F42/F44/F45/F46 verbucht (Slope rein; Zhu&amp;Zhao rein mit Firm-Gewichts-Grenze; Trinh=performance; Wang-e zweigeteilt; Weber-Exit) · Ledger korrigiert 66-&gt;61 Legacy / 1239 Zeilen · Hui-&gt;update-Retag · Zhou-Gap zu (22 Zeilen; Spearman-Hypothese für 62-&gt;22) · Crosswalk evidenzbasiert · Rescreen-Mandat 20+1 (segment=rescreen; Wang-2020/K&amp;V-2018 retroaktiv)</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="53">
-      <c r="A42" s="52" t="inlineStr">
+      <c r="A42" s="102" t="inlineStr">
         <is>
           <t>DEC-039</t>
         </is>
       </c>
-      <c r="B42" s="52" t="inlineStr">
+      <c r="B42" s="102" t="inlineStr">
         <is>
           <t>Ruling-Layer geschlossen (R1-R8, K1-K4): Unit-Grenze "Firma und darunter"; Devalle-Vorzeichenregime; 2 Studien-Cluster (Sandra/Ofogbe, K&amp;V inkl. EL-Zeile); Delis-Preisvarianten getaggt rein; industry-Operationalisierung + mixed; K4 zurückgezogen (Datei-Beweis); cluster_id-Mechanik für v11; DEC-040 reserviert (Adjudikationsergebnisse + v11)</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="53">
-      <c r="A43" s="52" t="inlineStr">
+      <c r="A43" s="102" t="inlineStr">
         <is>
           <t>DEC-040</t>
         </is>
       </c>
-      <c r="B43" s="52" t="inlineStr">
+      <c r="B43" s="102" t="inlineStr">
         <is>
           <t>Adjudikation als Studien-Level-Dispositionen verbucht (1b Lesart i: 208 strukturell draußen; 95 Adoptionen ohne Ursache [N1: F37c-Vermutung]; 51 Versionsdrift-Adoptionen [DEC-026-Ausnahme]; Zhou/Cubas-Waiver [N2]); Lookup 61/61 verifiziert; q-Moderator=VHB-only, JIF ruhend (löst DEC-023); v11-Spec erlassen; Bilanz ~2853; preliminary jetzt, Freeze=DEC-041 nach DB-Re-Run</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="53">
-      <c r="A44" s="52" t="inlineStr">
+      <c r="A44" s="102" t="inlineStr">
         <is>
           <t>DEC-041</t>
         </is>
       </c>
-      <c r="B44" s="52" t="inlineStr">
+      <c r="B44" s="102" t="inlineStr">
         <is>
           <t>v11 DATA FREEZE: 2.852 Zeilen/2.730 usable/120 Studien; natives DEC-024-Grid + Moderatoren korpusweit (Verifier 26/26); Scope-Cutoff 2026-07-10 (Autor: B; Reviewer-Dissens A dokumentiert; Mitigation: result-blind, Katalog 593, Validierungs-Framing, Revisions-Kontingenz ~1 Woche); Rulings S1-S19/B1-B4/E1-E8 formalisiert; Ledger-Korrektur 65 v10-Keys; Sprachgrenze Python/R kodifiziert</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="53">
-      <c r="A45" s="52" t="inlineStr">
+      <c r="A45" s="102" t="inlineStr">
         <is>
           <t>DEC-042</t>
         </is>
       </c>
-      <c r="B45" s="52" t="inlineStr">
+      <c r="B45" s="102" t="inlineStr">
         <is>
           <t>v12 kanonisch: Moderatorschicht komplett, Formel-Architektur, Row-Level-Country, Integritäts-Audit (31 Checks)</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="53">
-      <c r="A46" s="52" t="inlineStr">
+      <c r="A46" s="102" t="inlineStr">
         <is>
           <t>DEC-031</t>
         </is>
       </c>
-      <c r="B46" s="52" t="inlineStr">
+      <c r="B46" s="102" t="inlineStr">
         <is>
           <t>Finale Analyse-Batterie auf v12 fixiert; a-priori Inputs (Seeds/Grids/SESOI); Pending-D geöffnet</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="53">
-      <c r="A47" s="52" t="inlineStr">
+      <c r="A47" s="102" t="inlineStr">
         <is>
           <t>DEC-031a</t>
         </is>
       </c>
-      <c r="B47" s="52" t="inlineStr">
+      <c r="B47" s="102" t="inlineStr">
         <is>
           <t>Walk-through-Amendments: Moderator-Inventar neu geschnitten, Katalog final, konditionale Upgrades, Figuren</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="53">
-      <c r="A48" s="52" t="inlineStr">
+      <c r="A48" s="102" t="inlineStr">
         <is>
           <t>DEC-031b</t>
         </is>
       </c>
-      <c r="B48" s="52" t="inlineStr">
+      <c r="B48" s="102" t="inlineStr">
         <is>
           <t>N3-Prior: COE-Companion ersetzt Zarea; letztes externes Pending eliminiert</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="53">
-      <c r="A49" s="52" t="inlineStr">
+      <c r="A49" s="102" t="inlineStr">
         <is>
           <t>DEC-042a</t>
         </is>
       </c>
-      <c r="B49" s="52" t="inlineStr">
+      <c r="B49" s="102" t="inlineStr">
         <is>
           <t>Volker-Liste E1–E4 geschlossen; Schätzmenge 2.713 fixiert; R-19 final</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="53">
-      <c r="A50" s="52" t="inlineStr">
+      <c r="A50" s="102" t="inlineStr">
         <is>
           <t>DEC-012a</t>
         </is>
       </c>
-      <c r="B50" s="52" t="inlineStr">
+      <c r="B50" s="102" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="C50" s="52" t="inlineStr">
+      <c r="C50" s="102" t="inlineStr">
         <is>
           <t>Methodik</t>
         </is>
       </c>
-      <c r="D50" s="52" t="inlineStr">
+      <c r="D50" s="102" t="inlineStr">
         <is>
           <t>Oekonomische Uebersetzung operationalisiert (Instrument-Mediane)</t>
         </is>
       </c>
-      <c r="E50" s="52" t="inlineStr">
+      <c r="E50" s="102" t="inlineStr">
         <is>
           <t>#9 / T1,A6</t>
         </is>
       </c>
-      <c r="F50" s="52" t="inlineStr">
+      <c r="F50" s="102" t="inlineStr">
         <is>
           <t>Extraktionsregel fixiert: Median-SD(COD) je Instrument (loan/bond/CDS) via Volker-Task; Grid-Platzhalter PENDING; Ratio-Zeile konstantenfrei</t>
         </is>
       </c>
-      <c r="G50" s="52" t="inlineStr">
+      <c r="G50" s="102" t="inlineStr">
         <is>
           <t>aktiv (Konstanten pending)</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="53">
-      <c r="A51" s="52" t="inlineStr">
+      <c r="A51" s="102" t="inlineStr">
         <is>
           <t>DEC-042b</t>
         </is>
       </c>
-      <c r="B51" s="52" t="inlineStr">
+      <c r="B51" s="102" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="C51" s="52" t="inlineStr">
+      <c r="C51" s="102" t="inlineStr">
         <is>
           <t>Daten/Design</t>
         </is>
       </c>
-      <c r="D51" s="52" t="inlineStr">
+      <c r="D51" s="102" t="inlineStr">
         <is>
           <t>Perioden-Zellen-Domaene: 8 ES / 2 Studien ohne Fenster</t>
         </is>
       </c>
-      <c r="E51" s="52" t="inlineStr">
+      <c r="E51" s="102" t="inlineStr">
         <is>
           <t>T1/A3; Block B</t>
         </is>
       </c>
-      <c r="F51" s="52" t="inlineStr">
+      <c r="F51" s="102" t="inlineStr">
         <is>
           <t>NA = Design-Fakt; listenweise nur aus Perioden-/Dosis-Zellen (prae+post = 2.705); Schaetzmenge 2.713 unveraendert</t>
         </is>
       </c>
-      <c r="G51" s="52" t="inlineStr">
+      <c r="G51" s="102" t="inlineStr">
         <is>
           <t>aktiv</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1" s="53">
-      <c r="A52" s="52" t="inlineStr">
+      <c r="A52" s="102" t="inlineStr">
         <is>
           <t>DEC-024a</t>
         </is>
       </c>
-      <c r="B52" s="52" t="inlineStr">
+      <c r="B52" s="102" t="inlineStr">
         <is>
           <t>2026-07-14</t>
         </is>
       </c>
-      <c r="C52" s="52" t="inlineStr">
+      <c r="C52" s="102" t="inlineStr">
         <is>
           <t>Methodik</t>
         </is>
       </c>
-      <c r="D52" s="52" t="inlineStr">
+      <c r="D52" s="102" t="inlineStr">
         <is>
           <t>Placebo-Recode-Regel share_Y 2008–2015 (schließt F60)</t>
         </is>
       </c>
-      <c r="E52" s="52" t="inlineStr">
+      <c r="E52" s="102" t="inlineStr">
         <is>
           <t>T8 / B4</t>
         </is>
       </c>
-      <c r="F52" s="52" t="inlineStr">
+      <c r="F52" s="102" t="inlineStr">
         <is>
           <t>Kanonische share_Y-Formel, ties→Post; 2016-Identity-Gate; Zellen als Konstanten gepinnt</t>
         </is>
       </c>
-      <c r="G52" s="52" t="inlineStr">
+      <c r="G52" s="102" t="inlineStr">
         <is>
           <t>aktiv</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="53">
-      <c r="A53" s="52" t="inlineStr">
+      <c r="A53" s="102" t="inlineStr">
         <is>
           <t>DEC-031c</t>
         </is>
       </c>
-      <c r="B53" s="52" t="inlineStr">
+      <c r="B53" s="102" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="C53" s="52" t="inlineStr">
+      <c r="C53" s="102" t="inlineStr">
         <is>
           <t>Methodik</t>
         </is>
       </c>
-      <c r="D53" s="52" t="inlineStr">
+      <c r="D53" s="102" t="inlineStr">
         <is>
           <t>Pre-Trend-Guard Move 5: M-pre einziger präreg. Zusatz (schließt F59; Ruling R2)</t>
         </is>
       </c>
-      <c r="E53" s="52" t="inlineStr">
+      <c r="E53" s="102" t="inlineStr">
         <is>
           <t>T7 / C3,C4</t>
         </is>
       </c>
-      <c r="F53" s="52" t="inlineStr">
+      <c r="F53" s="102" t="inlineStr">
         <is>
           <t>M-full + Stratum-Segmentierung on-demand; D31.5-Panelform unangetastet; C4-df-Schutz</t>
         </is>
       </c>
-      <c r="G53" s="52" t="inlineStr">
+      <c r="G53" s="102" t="inlineStr">
         <is>
           <t>aktiv</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="53">
-      <c r="A54" s="52" t="inlineStr">
+      <c r="A54" s="102" t="inlineStr">
         <is>
           <t>DEC-031d</t>
         </is>
       </c>
-      <c r="B54" s="52" t="inlineStr">
+      <c r="B54" s="102" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="C54" s="52" t="inlineStr">
+      <c r="C54" s="102" t="inlineStr">
         <is>
           <t>Methodik</t>
         </is>
       </c>
-      <c r="D54" s="52" t="inlineStr">
+      <c r="D54" s="102" t="inlineStr">
         <is>
           <t>B5-Kovariatenset = 3 kategoriale von 5 §6-Drifts (schließt F61)</t>
         </is>
       </c>
-      <c r="E54" s="52" t="inlineStr">
+      <c r="E54" s="102" t="inlineStr">
         <is>
           <t>T8 / B5,B8</t>
         </is>
       </c>
-      <c r="F54" s="52" t="inlineStr">
+      <c r="F54" s="102" t="inlineStr">
         <is>
           <t>{region, instrument, CER}; Kanal-Zuweisung window/n; Oster-Paar race/trend_comp; Read-out Δβ+CI vs SESOI</t>
         </is>
       </c>
-      <c r="G54" s="52" t="inlineStr">
+      <c r="G54" s="102" t="inlineStr">
         <is>
           <t>aktiv</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="53">
-      <c r="A55" s="52" t="inlineStr">
+      <c r="A55" s="102" t="inlineStr">
         <is>
           <t>DEC-031e</t>
         </is>
       </c>
-      <c r="B55" s="52" t="inlineStr">
+      <c r="B55" s="102" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="C55" s="52" t="inlineStr">
+      <c r="C55" s="102" t="inlineStr">
         <is>
           <t>Methodik</t>
         </is>
       </c>
-      <c r="D55" s="52" t="inlineStr">
+      <c r="D55" s="102" t="inlineStr">
         <is>
           <t>T8-Execution-Amendment: break_only Cell-Means; fit3l ~1 (schließt S5-Halt)</t>
         </is>
       </c>
-      <c r="E55" s="52" t="inlineStr">
+      <c r="E55" s="102" t="inlineStr">
         <is>
           <t>T8 / B4</t>
         </is>
       </c>
-      <c r="F55" s="52" t="inlineStr">
+      <c r="F55" s="102" t="inlineStr">
         <is>
           <t>nlminb-Falschkonvergenz an σ²_study-Boundary; T2/B1-Konvention; Zertifikate in run_meta; F62 eröffnet</t>
         </is>
       </c>
-      <c r="G55" s="52" t="inlineStr">
+      <c r="G55" s="102" t="inlineStr">
         <is>
           <t>aktiv</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="53">
-      <c r="A56" s="52" t="inlineStr">
+      <c r="A56" s="102" t="inlineStr">
         <is>
           <t>DEC-031f</t>
         </is>
       </c>
-      <c r="B56" s="52" t="inlineStr">
+      <c r="B56" s="102" t="inlineStr">
         <is>
           <t>2026-07-16</t>
         </is>
       </c>
-      <c r="C56" s="52" t="inlineStr">
+      <c r="C56" s="102" t="inlineStr">
         <is>
           <t>Methodik</t>
         </is>
       </c>
-      <c r="D56" s="52" t="inlineStr">
+      <c r="D56" s="102" t="inlineStr">
         <is>
           <t>Konvergenzprotokoll 3L-RVE-Spine: Optimizer-Ladder, Zertifikate, R6-Kontrollfit (schließt F62)</t>
         </is>
       </c>
-      <c r="E56" s="52" t="inlineStr">
+      <c r="E56" s="102" t="inlineStr">
         <is>
           <t>alle Spine-Läufe</t>
         </is>
       </c>
-      <c r="F56" s="52" t="inlineStr">
+      <c r="F56" s="102" t="inlineStr">
         <is>
           <t>nlminb→BFGS→Nelder-Mead, first-certified-wins; Fallback-Flags; Toleranzen 1e-5/1e-6; Addendum A.11</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="53">
-      <c r="A57" s="52" t="inlineStr">
+      <c r="A57" s="102" t="inlineStr">
         <is>
           <t>DEC-031g</t>
         </is>
       </c>
-      <c r="B57" s="52" t="inlineStr">
+      <c r="B57" s="102" t="inlineStr">
         <is>
           <t>2026-07-18</t>
         </is>
       </c>
-      <c r="C57" s="52" t="inlineStr">
+      <c r="C57" s="102" t="inlineStr">
         <is>
           <t>Methodik</t>
         </is>
       </c>
-      <c r="D57" s="52" t="inlineStr">
+      <c r="D57" s="102" t="inlineStr">
         <is>
           <t>T5/Block-D-Execution-Spec: 3PSM-Basis RE/ML (F63), puniform-Lockfile (F64), A5-Anker-Protokoll (F65), D5-Zellen-Pin, D3→H</t>
         </is>
       </c>
-      <c r="E57" s="52" t="inlineStr">
+      <c r="E57" s="102" t="inlineStr">
         <is>
           <t>T5 / D1,D2,D4,D5,D6</t>
         </is>
       </c>
-      <c r="F57" s="52" t="inlineStr">
+      <c r="F57" s="102" t="inlineStr">
         <is>
           <t>P-T5-1..5; Richtungs-Pins less/left; not_estimable-Signaturliste; A.12; F-Register leer (nächste F66)</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="53">
-      <c r="A58" s="52" t="inlineStr">
+      <c r="A58" s="102" t="inlineStr">
         <is>
           <t>DEC-044</t>
         </is>
       </c>
-      <c r="B58" s="52" t="inlineStr">
+      <c r="B58" s="102" t="inlineStr">
         <is>
           <t>2026-07-19</t>
         </is>
       </c>
-      <c r="C58" s="52" t="inlineStr">
+      <c r="C58" s="102" t="inlineStr">
         <is>
           <t>Framing</t>
         </is>
       </c>
-      <c r="D58" s="52" t="inlineStr">
+      <c r="D58" s="102" t="inlineStr">
         <is>
           <t>Pending-C resolved: Framing A (null/debunking) mit zweistufiger Claim-Leiter; Sprach-Gate N1/N3</t>
         </is>
       </c>
-      <c r="E58" s="52" t="inlineStr">
+      <c r="E58" s="102" t="inlineStr">
         <is>
           <t>Manuskript / Ablauf 3b</t>
         </is>
       </c>
-      <c r="F58" s="52" t="inlineStr">
+      <c r="F58" s="102" t="inlineStr">
         <is>
           <t>Paris-Null hart; Pooled "negligible, not null" (CI-Rand &gt; SESOI); C -&gt; Boundary-Conditions; T7 = Heterogenitäts-Exploration in A</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="53">
-      <c r="A59" s="52" t="inlineStr">
+      <c r="A59" s="102" t="inlineStr">
         <is>
           <t>DEC-045</t>
         </is>
       </c>
-      <c r="B59" s="52" t="inlineStr">
+      <c r="B59" s="102" t="inlineStr">
         <is>
           <t>2026-07-22</t>
         </is>
       </c>
-      <c r="C59" s="52" t="inlineStr">
+      <c r="C59" s="102" t="inlineStr">
         <is>
           <t>Methodik</t>
         </is>
       </c>
-      <c r="D59" s="52" t="inlineStr">
+      <c r="D59" s="102" t="inlineStr">
         <is>
           <t>E/H-Batterie-Execution-Spec: Run-Architektur TH-a/b/c, Supersessions S1-S9, TOST-Pins, H1-Precompute, Zeittranslations-Permutation, RoBMA-Prior-Paket (F66)</t>
         </is>
       </c>
-      <c r="E59" s="52" t="inlineStr">
+      <c r="E59" s="102" t="inlineStr">
         <is>
           <t>Block E/H / TH-a, TH-b, TH-c</t>
         </is>
       </c>
-      <c r="F59" s="52" t="inlineStr">
+      <c r="F59" s="102" t="inlineStr">
         <is>
           <t>Result-blind Amendment: 10-Kodierungs-Kern (D1 verbatim aus T2); B=500 (S5); N10=113 Schritte; H8-Tiers (S6); F66 offen (einziges offenes F)</t>
         </is>
       </c>
-      <c r="G59" s="52" t="inlineStr">
+      <c r="G59" s="102" t="inlineStr">
         <is>
           <t>aktiv</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="53">
-      <c r="A60" s="52" t="inlineStr">
+      <c r="A60" s="102" t="inlineStr">
         <is>
           <t>DEC-046</t>
         </is>
       </c>
-      <c r="B60" s="52" t="inlineStr">
+      <c r="B60" s="102" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="C60" s="52" t="inlineStr">
+      <c r="C60" s="102" t="inlineStr">
         <is>
           <t>Methodik</t>
         </is>
       </c>
-      <c r="D60" s="52" t="inlineStr">
+      <c r="D60" s="102" t="inlineStr">
         <is>
           <t>F66-Schließung: RoBMA-Stack gepinnt (rjags 4-17, BayesTools 0.2.23, RoBMA 3.6.1, JAGS 4.3.2); y/se-Skalenpfad (Priors wirken verbatim auf z); t_RoBMA gemessen; Executor-/Leiter-Deviationen offengelegt</t>
         </is>
       </c>
-      <c r="E60" s="52" t="inlineStr">
+      <c r="E60" s="102" t="inlineStr">
         <is>
           <t>F66 / TH-b (R/07)</t>
         </is>
       </c>
-      <c r="F60" s="52" t="inlineStr">
+      <c r="F60" s="102" t="inlineStr">
         <is>
           <t>Ruling A (Upstream-Repro-Guidance statt 4.0.0-Bruchrelease); effect_direction "negative" gepinnt; t_RoBMA 1764,8 s; P3-Projektion T = 3t + 3κt, GO-Check bindend; RoBMA.reg = H2b-Träger; F66 GESCHLOSSEN</t>
         </is>
       </c>
-      <c r="G60" s="52" t="inlineStr">
+      <c r="G60" s="102" t="inlineStr">
         <is>
           <t>aktiv</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="53">
-      <c r="A61" s="52" t="inlineStr">
+      <c r="A61" s="102" t="inlineStr">
         <is>
           <t>DEC-047</t>
         </is>
       </c>
-      <c r="B61" s="52" t="inlineStr">
+      <c r="B61" s="102" t="inlineStr">
         <is>
           <t>2026-07-27</t>
         </is>
       </c>
-      <c r="C61" s="52" t="inlineStr">
+      <c r="C61" s="102" t="inlineStr">
         <is>
           <t>Framing</t>
         </is>
       </c>
-      <c r="D61" s="52" t="inlineStr">
+      <c r="D61" s="102" t="inlineStr">
         <is>
           <t>Gate-Auflösung [DEC-044]: Tier-1-Wortlaut = Äquivalenzregister — E2-Flag 1 (p_TOST = ,022) × BF01(Periode) primär = 1,03 (Band 1–3) per pre-registrierter E3-Leiter; Default-BF 8,49 nicht claimtragend (nicht-primär, anders parametrisiert, Caveats)</t>
         </is>
       </c>
-      <c r="E61" s="52" t="inlineStr">
+      <c r="E61" s="102" t="inlineStr">
         <is>
           <t>Gate / E3 · D6 · Manuskriptphase</t>
         </is>
       </c>
-      <c r="F61" s="52" t="inlineStr">
+      <c r="F61" s="102" t="inlineStr">
         <is>
           <t>Freigegeben: "statistisch äquivalent zu null im sekundären SESOI-Band"; gesperrt: Evidence-of-Absence-Vokabular; BFs deskriptiv; Tier 2 unverändert; TB-55 + BLOCKED-TBs entsperrt (Rewrites in Manuskriptphase)</t>
         </is>
       </c>
-      <c r="G61" s="52" t="inlineStr">
+      <c r="G61" s="102" t="inlineStr">
         <is>
           <t>aktiv</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="53">
-      <c r="A62" s="52" t="inlineStr">
+      <c r="A62" s="102" t="inlineStr">
         <is>
           <t>DEC-043</t>
         </is>
       </c>
-      <c r="B62" s="52" t="inlineStr">
+      <c r="B62" s="102" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="53">
-      <c r="A63" s="52" t="inlineStr">
+      <c r="A63" s="102" t="inlineStr">
         <is>
           <t>DEC-048</t>
         </is>
       </c>
-      <c r="B63" s="52" t="inlineStr">
+      <c r="B63" s="102" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="53">
-      <c r="A64" s="52" t="inlineStr">
+      <c r="A64" s="102" t="inlineStr">
         <is>
           <t>DEC-049</t>
         </is>
       </c>
-      <c r="B64" s="52" t="inlineStr">
+      <c r="B64" s="102" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="53">
-      <c r="A65" s="52" t="inlineStr">
+      <c r="A65" s="102" t="inlineStr">
         <is>
           <t>DEC-049a</t>
         </is>
       </c>
-      <c r="B65" s="52" t="inlineStr">
+      <c r="B65" s="102" t="inlineStr">
         <is>
           <t>2026-07-28</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="53">
-      <c r="A66" s="52" t="inlineStr">
+      <c r="A66" s="102" t="inlineStr">
         <is>
           <t>DEC-050 — Block-G execution spec: TG run (register G1–G10, G11 partial), F/G session split, inference conventions, dat_prep flag canonicity (2026-07-29)</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="53">
-      <c r="A67" s="52" t="inlineStr">
+      <c r="A67" s="102" t="inlineStr">
         <is>
           <t>DEC-050a — G2 count erratum: estimation-set assert 296 (297 = usable basis incl. 134 FLAG; duplicate exits at filter) (2026-07-29)</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="53">
-      <c r="A68" s="52" t="inlineStr">
+      <c r="A68" s="102" t="inlineStr">
         <is>
           <t>DEC-050b — V06 corrigendum: Gate B per DEC-048 wording, 3L refit vs. committed T1_results.csv, no hand constants (2026-07-29)</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="53">
-      <c r="A69" s="52" t="inlineStr">
+      <c r="A69" s="102" t="inlineStr">
         <is>
           <t>DEC-050c — V06 precision: label-key location analysis_id==A1; sigma2 value search unchanged (2026-07-29)</t>
         </is>
@@ -3612,6 +3612,13 @@
       <c r="A70" s="102" t="inlineStr">
         <is>
           <t>DEC-051 — Block-F execution spec: TF run (outliers &amp; influence F1–F7), register completion / G11 close, feed home manuscript\ (2026-07-29)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="102" t="inlineStr">
+        <is>
+          <t>DEC-051a — Corrigendum to DEC-051: F1 rstudent route parallel snow + toy identity probe, worker pins 8/8 (RAM-measured), runtime projection corrected; first canonical attempt aborted &gt; 10 h in the F1 pass, no outputs (2026-07-30)</t>
         </is>
       </c>
     </row>
@@ -3636,13 +3643,13 @@
   <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="5" customWidth="1" style="52" min="1" max="1"/>
-    <col width="16" customWidth="1" style="52" min="2" max="2"/>
-    <col width="27" customWidth="1" style="52" min="3" max="3"/>
-    <col width="60" customWidth="1" style="52" min="4" max="4"/>
-    <col width="24" customWidth="1" style="52" min="5" max="5"/>
-    <col width="18" customWidth="1" style="52" min="6" max="6"/>
-    <col width="9" customWidth="1" style="52" min="7" max="7"/>
+    <col width="5" customWidth="1" style="102" min="1" max="1"/>
+    <col width="16" customWidth="1" style="102" min="2" max="2"/>
+    <col width="27" customWidth="1" style="102" min="3" max="3"/>
+    <col width="60" customWidth="1" style="102" min="4" max="4"/>
+    <col width="24" customWidth="1" style="102" min="5" max="5"/>
+    <col width="18" customWidth="1" style="102" min="6" max="6"/>
+    <col width="9" customWidth="1" style="102" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" s="53">
@@ -4243,15 +4250,15 @@
   <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="5" customWidth="1" style="52" min="1" max="1"/>
-    <col width="19" customWidth="1" style="52" min="2" max="2"/>
-    <col width="5" customWidth="1" style="52" min="3" max="3"/>
-    <col width="32" customWidth="1" style="52" min="4" max="4"/>
-    <col width="42" customWidth="1" style="52" min="5" max="5"/>
-    <col width="22" customWidth="1" style="52" min="6" max="6"/>
-    <col width="15" customWidth="1" style="52" min="7" max="7"/>
-    <col width="12" customWidth="1" style="52" min="8" max="8"/>
-    <col width="9" customWidth="1" style="52" min="9" max="9"/>
+    <col width="5" customWidth="1" style="102" min="1" max="1"/>
+    <col width="19" customWidth="1" style="102" min="2" max="2"/>
+    <col width="5" customWidth="1" style="102" min="3" max="3"/>
+    <col width="32" customWidth="1" style="102" min="4" max="4"/>
+    <col width="42" customWidth="1" style="102" min="5" max="5"/>
+    <col width="22" customWidth="1" style="102" min="6" max="6"/>
+    <col width="15" customWidth="1" style="102" min="7" max="7"/>
+    <col width="12" customWidth="1" style="102" min="8" max="8"/>
+    <col width="9" customWidth="1" style="102" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.5" customHeight="1" s="53">
@@ -5070,15 +5077,15 @@
   <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="7" customWidth="1" style="52" min="1" max="1"/>
-    <col width="8" customWidth="1" style="52" min="2" max="2"/>
-    <col width="25" customWidth="1" style="52" min="3" max="3"/>
-    <col width="38" customWidth="1" style="52" min="4" max="4"/>
-    <col width="10" customWidth="1" style="52" min="5" max="5"/>
-    <col width="17" customWidth="1" style="52" min="6" max="6"/>
-    <col width="13" customWidth="1" style="52" min="7" max="8"/>
-    <col width="33" customWidth="1" style="52" min="9" max="9"/>
-    <col width="36" customWidth="1" style="52" min="10" max="10"/>
+    <col width="7" customWidth="1" style="102" min="1" max="1"/>
+    <col width="8" customWidth="1" style="102" min="2" max="2"/>
+    <col width="25" customWidth="1" style="102" min="3" max="3"/>
+    <col width="38" customWidth="1" style="102" min="4" max="4"/>
+    <col width="10" customWidth="1" style="102" min="5" max="5"/>
+    <col width="17" customWidth="1" style="102" min="6" max="6"/>
+    <col width="13" customWidth="1" style="102" min="7" max="8"/>
+    <col width="33" customWidth="1" style="102" min="9" max="9"/>
+    <col width="36" customWidth="1" style="102" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.5" customHeight="1" s="53">
@@ -5146,7 +5153,7 @@
           <t>File Reference (R-Skript + Verifier · CSV · MD)</t>
         </is>
       </c>
-      <c r="K3" s="52" t="inlineStr">
+      <c r="K3" s="102" t="inlineStr">
         <is>
           <t>Status 2026-07-10</t>
         </is>
@@ -5203,7 +5210,7 @@
           <t>docs/analysis_plan.md</t>
         </is>
       </c>
-      <c r="K4" s="52" t="inlineStr">
+      <c r="K4" s="102" t="inlineStr">
         <is>
           <t>erledigt (DEC-031 fixiert)</t>
         </is>
@@ -5260,7 +5267,7 @@
           <t>docs/analysis_plan.md</t>
         </is>
       </c>
-      <c r="K5" s="52" t="inlineStr">
+      <c r="K5" s="102" t="inlineStr">
         <is>
           <t>erledigt (DEC-031)</t>
         </is>
@@ -5317,7 +5324,7 @@
           <t>FOMA_CERCOE_Data_v1.xlsx (Tabelle1)</t>
         </is>
       </c>
-      <c r="K6" s="52" t="inlineStr">
+      <c r="K6" s="102" t="inlineStr">
         <is>
           <t>erledigt (v12/DEC-042)</t>
         </is>
@@ -5374,7 +5381,7 @@
           <t>R/01_prep.R + R/01_verify_outputs.R · docs/data_dictionary.md</t>
         </is>
       </c>
-      <c r="K7" s="52" t="inlineStr">
+      <c r="K7" s="102" t="inlineStr">
         <is>
           <t>ERLEDIGT — kanonisch (CC+Verifier v2, 28/28, 2026-07-12); Commit folgt</t>
         </is>
@@ -5431,7 +5438,7 @@
           <t>R/01_core.R + R/01_verify_outputs.R · output/T1_results.csv · output/T1_results_workbook.xlsx · manuscript/T1.md · docs/cc_prompt_T1.md</t>
         </is>
       </c>
-      <c r="K8" s="52" t="inlineStr">
+      <c r="K8" s="102" t="inlineStr">
         <is>
           <t>erledigt (21/21, 2026-07-13)</t>
         </is>
@@ -5488,7 +5495,7 @@
           <t>R/02_paris.R + R/02_verify_outputs.R · output/T2_results.csv · output/T2_results_workbook.xlsx · manuscript/T2.md · docs/T2_spec.md · docs/cc_prompt_T2.md</t>
         </is>
       </c>
-      <c r="K9" s="52" t="inlineStr">
+      <c r="K9" s="102" t="inlineStr">
         <is>
           <t>erledigt (17/17, 2026-07-14)</t>
         </is>
@@ -5545,7 +5552,7 @@
           <t>R/NN_t3_het + _verify · output/T3_results.csv · manuscript/T3.md</t>
         </is>
       </c>
-      <c r="K10" s="52" t="inlineStr">
+      <c r="K10" s="102" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
@@ -5602,7 +5609,7 @@
           <t>R/NN_t4_robust + _verify · output/T4_results.csv · manuscript/T4.md</t>
         </is>
       </c>
-      <c r="K11" s="52" t="inlineStr">
+      <c r="K11" s="102" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
@@ -5659,7 +5666,7 @@
           <t>R/NN_t5_pubbias + _verify · output/T5_results.csv · manuscript/T5.md</t>
         </is>
       </c>
-      <c r="K12" s="52" t="inlineStr">
+      <c r="K12" s="102" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
@@ -5716,7 +5723,7 @@
           <t>R/NN_t6_moderators + _verify · output/T6_results.csv · manuscript/T6.md</t>
         </is>
       </c>
-      <c r="K13" s="52" t="inlineStr">
+      <c r="K13" s="102" t="inlineStr">
         <is>
           <t>ersetzt durch T7-Interaktionen (DEC-031)</t>
         </is>
@@ -5773,7 +5780,7 @@
           <t>R/NN_t7_unified + R/NN_verify · output/T7_results.csv · manuscript/T7.md</t>
         </is>
       </c>
-      <c r="K14" s="52" t="inlineStr">
+      <c r="K14" s="102" t="inlineStr">
         <is>
           <t>offen (Pending-D vor Stufe 2)</t>
         </is>
@@ -5830,7 +5837,7 @@
           <t>R/NN_t8_identif + R/NN_verify · output/T8_results.csv · manuscript/T8.md</t>
         </is>
       </c>
-      <c r="K15" s="52" t="inlineStr">
+      <c r="K15" s="102" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
@@ -5856,18 +5863,18 @@
   <dimension ref="A1:H75"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="7" customWidth="1" style="52" min="1" max="1"/>
-    <col width="30" customWidth="1" style="52" min="2" max="2"/>
-    <col width="72" customWidth="1" style="52" min="3" max="3"/>
-    <col width="10" customWidth="1" style="52" min="4" max="4"/>
-    <col width="22" customWidth="1" style="52" min="5" max="5"/>
-    <col width="30" customWidth="1" style="52" min="6" max="6"/>
-    <col width="44" customWidth="1" style="52" min="7" max="7"/>
-    <col width="72" customWidth="1" style="52" min="8" max="8"/>
+    <col width="7" customWidth="1" style="102" min="1" max="1"/>
+    <col width="30" customWidth="1" style="102" min="2" max="2"/>
+    <col width="72" customWidth="1" style="102" min="3" max="3"/>
+    <col width="10" customWidth="1" style="102" min="4" max="4"/>
+    <col width="22" customWidth="1" style="102" min="5" max="5"/>
+    <col width="30" customWidth="1" style="102" min="6" max="6"/>
+    <col width="44" customWidth="1" style="102" min="7" max="7"/>
+    <col width="72" customWidth="1" style="102" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="53">
-      <c r="A1" s="52" t="inlineStr">
+      <c r="A1" s="102" t="inlineStr">
         <is>
           <t>Analyse-Batterie — CER–COD FOMA (per DEC-031 + DEC-031a, 2026-07-10; result-blind bis Gates T0.4/T1)</t>
         </is>
@@ -6552,12 +6559,12 @@
       </c>
     </row>
     <row r="21" ht="54.75" customHeight="1" s="53">
-      <c r="A21" s="52" t="inlineStr">
+      <c r="A21" s="102" t="inlineStr">
         <is>
           <t>B8</t>
         </is>
       </c>
-      <c r="B21" s="52" t="inlineStr">
+      <c r="B21" s="102" t="inlineStr">
         <is>
           <t>Bounding (Move 7)</t>
         </is>
@@ -6567,12 +6574,12 @@
           <t>Sensitivitäts-Schranke: wie groß müsste ein unbeobachteter Trend/Confounder sein, um einen verbleibenden Paris-Effekt zu erklären (Oster-Bounds / E-Value auf finales Modell)</t>
         </is>
       </c>
-      <c r="D21" s="52" t="inlineStr">
+      <c r="D21" s="102" t="inlineStr">
         <is>
           <t>erledigt (2026-07-15, Verifier 27/27)</t>
         </is>
       </c>
-      <c r="E21" s="52" t="inlineStr">
+      <c r="E21" s="102" t="inlineStr">
         <is>
           <t>output/T8_results_workbook.xlsx Tabs 7–10; output/T8_results.csv @ 76074a2</t>
         </is>
@@ -7851,7 +7858,7 @@
           <t>Inputs vollständig fixiert (DEC-031b); Quelle Witte et al. COE-Companion, Overlap-Disclosure 5 Studien / 0 geteilte ES; Lauf-Provenienz: κ_emp 1,71–2,34 vs Pin 2,5, Wall 4 h 39 min; Läufe 1–2 = Design-Halts (ERROR_LOG #17/#18)</t>
         </is>
       </c>
-      <c r="H66" s="52" t="inlineStr">
+      <c r="H66" s="102" t="inlineStr">
         <is>
           <t>Bayesianische Gesamtschau: Unter den vorab fixierten, informierten Priors ist die Moderations-Frage praktisch unentschieden (BF ≈ 1) — die Daten sprechen weder klar für noch gegen einen Paris-Effekt; der gepoolte Effekt erhält nur begrenzte Unterstützung, und die Publikations-Selektions-Komponenten werden durchgehend stark einbezogen. Einordnung und Wortlaut folgen im Gate-Schritt [DEC-044].</t>
         </is>
@@ -8227,24 +8234,24 @@
   <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="5" customWidth="1" style="52" min="1" max="1"/>
-    <col width="6" customWidth="1" style="52" min="2" max="2"/>
-    <col width="26" customWidth="1" style="52" min="3" max="3"/>
-    <col width="44" customWidth="1" style="52" min="4" max="4"/>
-    <col width="48" customWidth="1" style="52" min="5" max="5"/>
-    <col width="20" customWidth="1" style="52" min="6" max="6"/>
-    <col width="40" customWidth="1" style="52" min="7" max="7"/>
-    <col width="30" customWidth="1" style="52" min="8" max="8"/>
-    <col width="26" customWidth="1" style="52" min="9" max="9"/>
-    <col width="22" customWidth="1" style="52" min="10" max="10"/>
-    <col width="16" customWidth="1" style="52" min="11" max="11"/>
-    <col width="28" customWidth="1" style="52" min="12" max="12"/>
-    <col width="26" customWidth="1" style="52" min="13" max="13"/>
-    <col width="14" customWidth="1" style="52" min="14" max="14"/>
+    <col width="5" customWidth="1" style="102" min="1" max="1"/>
+    <col width="6" customWidth="1" style="102" min="2" max="2"/>
+    <col width="26" customWidth="1" style="102" min="3" max="3"/>
+    <col width="44" customWidth="1" style="102" min="4" max="4"/>
+    <col width="48" customWidth="1" style="102" min="5" max="5"/>
+    <col width="20" customWidth="1" style="102" min="6" max="6"/>
+    <col width="40" customWidth="1" style="102" min="7" max="7"/>
+    <col width="30" customWidth="1" style="102" min="8" max="8"/>
+    <col width="26" customWidth="1" style="102" min="9" max="9"/>
+    <col width="22" customWidth="1" style="102" min="10" max="10"/>
+    <col width="16" customWidth="1" style="102" min="11" max="11"/>
+    <col width="28" customWidth="1" style="102" min="12" max="12"/>
+    <col width="26" customWidth="1" style="102" min="13" max="13"/>
+    <col width="14" customWidth="1" style="102" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="53">
-      <c r="A1" s="52" t="inlineStr">
+      <c r="A1" s="102" t="inlineStr">
         <is>
           <t>Null-Battery — Kandidaten-Analysen zur Absicherung des Null-Befunds (Paris). Stand 2026-07-03. Auswahl → DEC-028 (a priori, VOR T1 zu designieren, DEC-005-Disziplin). Linien: A = Zufall/Power · B = Spezifikationsraum · C = Zeitachse · D = Benchmark/Erwartung. Kernbefund der Daten-Checks: ALLE 15 Analysen laufen auf CER-COD_data_v8.xlsx — keine neue Datenerhebung nötig. | ENTSCHEIDUNG: ALLE 15 GO per DEC-029 (2026-07-04); Inputs-Fixierung vor T1 (Battery-Prep).</t>
         </is>
@@ -9410,7 +9417,7 @@
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="53">
-      <c r="A20" s="52" t="inlineStr">
+      <c r="A20" s="102" t="inlineStr">
         <is>
           <t>2026-07-10: Alle N-Inputs a priori fixiert per DEC-031 Annex H (Seeds 20260710, B-Werte, Grids, SESOI 0,070/0,05, N13-Regel). Einziger externer Pending: Zarea-Prior (N3). Tracking: Sheet "Analyse_Batterie", Block H.</t>
         </is>
@@ -9432,18 +9439,18 @@
   <dimension ref="A1:I86"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="7" customWidth="1" style="52" min="1" max="2"/>
-    <col width="52" customWidth="1" style="52" min="3" max="3"/>
-    <col width="24" customWidth="1" style="52" min="4" max="4"/>
-    <col width="20" customWidth="1" style="52" min="5" max="5"/>
-    <col width="18" customWidth="1" style="52" min="6" max="6"/>
-    <col width="12" customWidth="1" style="52" min="7" max="7"/>
-    <col width="26" customWidth="1" style="52" min="8" max="8"/>
-    <col width="42" customWidth="1" style="52" min="9" max="9"/>
+    <col width="7" customWidth="1" style="102" min="1" max="2"/>
+    <col width="52" customWidth="1" style="102" min="3" max="3"/>
+    <col width="24" customWidth="1" style="102" min="4" max="4"/>
+    <col width="20" customWidth="1" style="102" min="5" max="5"/>
+    <col width="18" customWidth="1" style="102" min="6" max="6"/>
+    <col width="12" customWidth="1" style="102" min="7" max="7"/>
+    <col width="26" customWidth="1" style="102" min="8" max="8"/>
+    <col width="42" customWidth="1" style="102" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="53">
-      <c r="A1" s="52" t="inlineStr">
+      <c r="A1" s="102" t="inlineStr">
         <is>
           <t>KONSOLIDIERTE SCREENING-LISTE (4 Engines: Claude=C, ChatGPT=G, Perplexity-Base=P1/P2, Perplexity-Agent=A) — DEC-030. Klassen: P1=Download publiziert · P1-WP=Download Working Paper · B=Konstrukt-/Record-Check vor Download · D=raus per F32v2/Outcome (Ch.2-Kontext) · E=im Korpus/Dedup · F28=prä-Fenster-Exklusionsdoku (Volker) · R2=Runde-2-Preview. Suchinstrument bleibt Volkers DB-Re-Run (DEC-030); diese Liste = dokumentierte Supplementärsuche + Recall-Messlatte.</t>
         </is>
@@ -13207,13 +13214,13 @@
   <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="5" customWidth="1" style="52" min="1" max="1"/>
-    <col width="9" customWidth="1" style="52" min="2" max="2"/>
-    <col width="24" customWidth="1" style="52" min="3" max="3"/>
-    <col width="58" customWidth="1" style="52" min="4" max="4"/>
-    <col width="13" customWidth="1" style="52" min="5" max="5"/>
-    <col width="15" customWidth="1" style="52" min="6" max="6"/>
-    <col width="28" customWidth="1" style="52" min="7" max="7"/>
+    <col width="5" customWidth="1" style="102" min="1" max="1"/>
+    <col width="9" customWidth="1" style="102" min="2" max="2"/>
+    <col width="24" customWidth="1" style="102" min="3" max="3"/>
+    <col width="58" customWidth="1" style="102" min="4" max="4"/>
+    <col width="13" customWidth="1" style="102" min="5" max="5"/>
+    <col width="15" customWidth="1" style="102" min="6" max="6"/>
+    <col width="28" customWidth="1" style="102" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.5" customHeight="1" s="53">
@@ -13687,521 +13694,521 @@
       <c r="G16" s="67" t="n"/>
     </row>
     <row r="17" ht="15" customHeight="1" s="53">
-      <c r="A17" s="52" t="n">
+      <c r="A17" s="102" t="n">
         <v>14</v>
       </c>
-      <c r="B17" s="52" t="inlineStr">
+      <c r="B17" s="102" t="inlineStr">
         <is>
           <t>Daten</t>
         </is>
       </c>
-      <c r="C17" s="52" t="inlineStr">
+      <c r="C17" s="102" t="inlineStr">
         <is>
           <t>reported-vs-derived-Flag (no_firms)</t>
         </is>
       </c>
-      <c r="D17" s="52" t="inlineStr">
+      <c r="D17" s="102" t="inlineStr">
         <is>
           <t>Je Studie kennzeichnen: n direkt berichtet vs. round(n_obs/T) abgeleitet (DEC-027)</t>
         </is>
       </c>
-      <c r="E17" s="52" t="inlineStr">
+      <c r="E17" s="102" t="inlineStr">
         <is>
           <t>Volker</t>
         </is>
       </c>
-      <c r="F17" s="52" t="inlineStr">
+      <c r="F17" s="102" t="inlineStr">
         <is>
           <t>gelöst (v9, V4)</t>
         </is>
       </c>
-      <c r="G17" s="52" t="inlineStr">
+      <c r="G17" s="102" t="inlineStr">
         <is>
           <t>Flags geliefert: no_firms_source coded 593 / calculated 713 (54,6 %); autoritativ ggü. der 85 %-Arithmetik (DEC-028)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="53">
-      <c r="A18" s="52" t="n">
+      <c r="A18" s="102" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="52" t="inlineStr">
+      <c r="B18" s="102" t="inlineStr">
         <is>
           <t>Frage</t>
         </is>
       </c>
-      <c r="C18" s="52" t="inlineStr">
+      <c r="C18" s="102" t="inlineStr">
         <is>
           <t>r-Transformations-Doku + k der 36 PCCs</t>
         </is>
       </c>
-      <c r="D18" s="52" t="inlineStr">
+      <c r="D18" s="102" t="inlineStr">
         <is>
           <t>Exakte Konversionsformel (Peterson–Brown / t-Konversion) + k falls trivial; operationalisiert method_artefacts (#3); Pending-B</t>
         </is>
       </c>
-      <c r="E18" s="52" t="inlineStr">
+      <c r="E18" s="102" t="inlineStr">
         <is>
           <t>Volker</t>
         </is>
       </c>
-      <c r="F18" s="52" t="inlineStr">
+      <c r="F18" s="102" t="inlineStr">
         <is>
           <t>gelöst (v9, V5; F21)</t>
         </is>
       </c>
-      <c r="G18" s="52" t="inlineStr">
+      <c r="G18" s="102" t="inlineStr">
         <is>
           <t>formula-Sheet: 4 Routen dokumentiert; df≈n_obs-Konvention + pcc_df_k10/20-Sensitivität; k wird nicht nacherhoben; Pending-B geschlossen (DEC-028)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="53">
-      <c r="A19" s="52" t="n">
+      <c r="A19" s="102" t="n">
         <v>16</v>
       </c>
-      <c r="B19" s="52" t="inlineStr">
+      <c r="B19" s="102" t="inlineStr">
         <is>
           <t>Daten</t>
         </is>
       </c>
-      <c r="C19" s="52" t="inlineStr">
+      <c r="C19" s="102" t="inlineStr">
         <is>
           <t>PRISMA-Basics</t>
         </is>
       </c>
-      <c r="D19" s="52" t="inlineStr">
+      <c r="D19" s="102" t="inlineStr">
         <is>
           <t>Suchdatum, Datenbanken, Treffer-/Screening-Zahlen, Inter-Coder-Angaben (Roadmap #11)</t>
         </is>
       </c>
-      <c r="E19" s="52" t="inlineStr">
+      <c r="E19" s="102" t="inlineStr">
         <is>
           <t>Volker</t>
         </is>
       </c>
-      <c r="F19" s="52" t="inlineStr">
+      <c r="F19" s="102" t="inlineStr">
         <is>
           <t>offen (V6, vor Ch. 3)</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="53">
-      <c r="A20" s="52" t="n">
+      <c r="A20" s="102" t="n">
         <v>17</v>
       </c>
-      <c r="B20" s="52" t="inlineStr">
+      <c r="B20" s="102" t="inlineStr">
         <is>
           <t>Daten</t>
         </is>
       </c>
-      <c r="C20" s="52" t="inlineStr">
+      <c r="C20" s="102" t="inlineStr">
         <is>
           <t>Lookup-Pflege + Sharfman-Begründung</t>
         </is>
       </c>
-      <c r="D20" s="52" t="inlineStr">
+      <c r="D20" s="102" t="inlineStr">
         <is>
           <t>Shad-Jahr (Key 2022 vs ESPR 2020) · Lemma-Jahr-Konvention · Li-Doppelzeile konsolidieren · reference_verified-Header + 7 Leerzeilen · F16: Ausschlussgrund Sharfman&amp;Fernando 2008 (im COE-Korpus, berichtet COD)</t>
         </is>
       </c>
-      <c r="E20" s="52" t="inlineStr">
+      <c r="E20" s="102" t="inlineStr">
         <is>
           <t>Volker</t>
         </is>
       </c>
-      <c r="F20" s="52" t="inlineStr">
+      <c r="F20" s="102" t="inlineStr">
         <is>
           <t>offen (nicht blockierend)</t>
         </is>
       </c>
-      <c r="G20" s="52" t="inlineStr">
+      <c r="G20" s="102" t="inlineStr">
         <is>
           <t>None | v9/v10: Spalte L 65/65 gefüllt; Li-Waise entfernt (Lookup 65 Zeilen, Anti-Join 0/0); ES_measure-Fix (F20); Header-Typo source_verfified bleibt (Codebook-Alias); Shad-Kreuznotiz F22 in Overlap-Tabelle</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="53">
-      <c r="A21" s="52" t="n">
+      <c r="A21" s="102" t="n">
         <v>18</v>
       </c>
-      <c r="B21" s="52" t="inlineStr">
+      <c r="B21" s="102" t="inlineStr">
         <is>
           <t>Formales Suchupdate: DB-Re-Run (10 DBs + GS), identische Kriterien, Enddatum=Ausführung, zweistufiger PRISMA-Flow → Extraktion → v11 [DEC-030]</t>
         </is>
       </c>
-      <c r="C21" s="52" t="inlineStr">
+      <c r="C21" s="102" t="inlineStr">
         <is>
           <t>Volker</t>
         </is>
       </c>
-      <c r="D21" s="52" t="inlineStr">
+      <c r="D21" s="102" t="inlineStr">
         <is>
           <t>erledigt (2026-07-10, DEC-041)</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="53">
-      <c r="A22" s="52" t="n">
+      <c r="A22" s="102" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="52" t="inlineStr">
+      <c r="B22" s="102" t="inlineStr">
         <is>
           <t>Kandidaten-Downloads lt. Update_Scoping (P1: 41 publ. + 10 WP; B nach Checks) via WU-Zugang; Owolabi zusätzlich ins PK [F29]</t>
         </is>
       </c>
-      <c r="C22" s="52" t="inlineStr">
+      <c r="C22" s="102" t="inlineStr">
         <is>
           <t>erledigt implizit (Vollkorpus extrahiert, DEC-041)</t>
         </is>
       </c>
-      <c r="D22" s="52" t="inlineStr">
+      <c r="D22" s="102" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="53">
-      <c r="A23" s="52" t="n">
+      <c r="A23" s="102" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="52" t="inlineStr">
+      <c r="B23" s="102" t="inlineStr">
         <is>
           <t>Blind-Pilot Extraktion: 2 Bestandspaper (nicht kalibriert; Vorschlag Devalle 2017 + 1 Loan-Paper) — PDFs hochladen, Claude extrahiert blind, Diff + Konkordanzmaß [DEC-032 §9] — ERGEBNIS: 4 Paper blind extrahiert; 0 Extraktor-Fehler auf Statistik-Kernfeldern; PASS. Report: docs/pilot_concordance_report.md</t>
         </is>
       </c>
-      <c r="C23" s="52" t="inlineStr">
+      <c r="C23" s="102" t="inlineStr">
         <is>
           <t>Robert + Claude</t>
         </is>
       </c>
-      <c r="D23" s="52" t="inlineStr">
+      <c r="D23" s="102" t="inlineStr">
         <is>
           <t>erledigt (PASS, 2026-07-05)</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="53">
-      <c r="A24" s="52" t="n">
+      <c r="A24" s="102" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="52" t="inlineStr">
+      <c r="B24" s="102" t="inlineStr">
         <is>
           <t>Produktions-Extraktion VOLLKORPUS [DEC-033, Option C]: 65 Legacy-Paper + alle gescreenten Update-Kandidaten via Cowork-Batch (1 Paper/Run; staging_&lt;study&gt;.csv + log_&lt;study&gt;.md + Manifest); Maschinen-Diff vs v10; Volker adjudiziert nur Diffs + Neu-Zeilen (Exact-Match = wechselseitig verifiziert); 4 Pilot-Extraktionen wiederverwendbar (Yilmaz-Regulation per F36b nachkodieren) — UPDATE [DEC-034]: Batch läuft unter Codebook v1.2 (6 Zusatzfelder); VOR Volllauf die 4 Pilot-Stagings aus staging\ löschen (Resume-Regel!), damit alle Paper uniform v1.2 laufen</t>
         </is>
       </c>
-      <c r="C24" s="52" t="inlineStr">
+      <c r="C24" s="102" t="inlineStr">
         <is>
           <t>erledigt (Produktions-Extraktion abgeschlossen; v12/DEC-042)</t>
         </is>
       </c>
-      <c r="D24" s="52" t="inlineStr">
+      <c r="D24" s="102" t="inlineStr">
         <is>
           <t>bereit — Batch-Start</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="53">
-      <c r="A25" s="52" t="n">
+      <c r="A25" s="102" t="n">
         <v>22</v>
       </c>
-      <c r="B25" s="52" t="inlineStr">
+      <c r="B25" s="102" t="inlineStr">
         <is>
           <t>Erratum-/Verifikationsliste F35 a-f aus Pilot (u.a. Devalle Zeile 409: r=+0.9998 aus OR-Misprint — HIGH, vor erstem Analyselauf fixen; Atif-Regulation; Atif CER_measure; Capelle 21/20; Sovereign-Scope-Note; Breitenbefund + Segment-Dummy-Empfehlung) — Korrekturen landen in v11 via Prep + DEC — ÜBERFÜHRT in DEC-033-Adjudikation (Teil der Diff-Liste)</t>
         </is>
       </c>
-      <c r="C25" s="52" t="inlineStr">
+      <c r="C25" s="102" t="inlineStr">
         <is>
           <t>erledigt (Adjudikationspaket DEC-040)</t>
         </is>
       </c>
-      <c r="D25" s="52" t="inlineStr">
+      <c r="D25" s="102" t="inlineStr">
         <is>
           <t>in Adjudikation (DEC-033)</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="53">
-      <c r="A26" s="52" t="n">
+      <c r="A26" s="102" t="n">
         <v>23</v>
       </c>
-      <c r="B26" s="52" t="inlineStr">
+      <c r="B26" s="102" t="inlineStr">
         <is>
           <t>Capelle-Blancard: harmonization-stage exclusion dokumentieren (unit of analysis: sovereign; R2.1/F36h) — PRISMA-Note + Drop-one-Sensitivitätsnotiz; Korpus 66-&gt;65, Effekte 1306-&gt;1305 (Legacy-Basis) [DEC-033]</t>
         </is>
       </c>
-      <c r="C26" s="52" t="inlineStr">
+      <c r="C26" s="102" t="inlineStr">
         <is>
           <t>Robert + Volker</t>
         </is>
       </c>
-      <c r="D26" s="52" t="inlineStr">
+      <c r="D26" s="102" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="53">
-      <c r="A27" s="52" t="n">
+      <c r="A27" s="102" t="n">
         <v>24</v>
       </c>
-      <c r="B27" s="52" t="inlineStr">
+      <c r="B27" s="102" t="inlineStr">
         <is>
           <t>Fard et al (2020): harmonization-stage exclusion dokumentieren (Länder-Policy-Stringenz = Exposure; F39a/DEC-035) — PRISMA-Note + Drop-one-Sensitivität; Legacy-Basis -46 Effekte, Korpus 64-&gt;63</t>
         </is>
       </c>
-      <c r="C27" s="52" t="inlineStr">
+      <c r="C27" s="102" t="inlineStr">
         <is>
           <t>erledigt (Exclusion dokumentiert, DEC-035)</t>
         </is>
       </c>
-      <c r="D27" s="52" t="inlineStr">
+      <c r="D27" s="102" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="53">
-      <c r="A28" s="52" t="n">
+      <c r="A28" s="102" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="52" t="inlineStr">
+      <c r="B28" s="102" t="inlineStr">
         <is>
           <t>Rescreen-Tranche [DEC-038]: 20 Paper + K&amp;V-2021-Identitätscheck aus inbox_rescreen -&gt; papers -&gt; v1.6-Kickoff; 0-Zeilen-Läufe = retroaktive PRISMA-Ausschlussdoku; nicht beschaffbare als not-retrievable dokumentieren</t>
         </is>
       </c>
-      <c r="C28" s="52" t="inlineStr">
+      <c r="C28" s="102" t="inlineStr">
         <is>
           <t>erledigt (Rescreen-Segment in v12: 18 Studien)</t>
         </is>
       </c>
-      <c r="D28" s="52" t="inlineStr">
+      <c r="D28" s="102" t="inlineStr">
         <is>
           <t>bereit</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="53">
-      <c r="A29" s="52" t="n">
+      <c r="A29" s="102" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="52" t="inlineStr">
+      <c r="B29" s="102" t="inlineStr">
         <is>
           <t>Pass-2b + Adjudikationspaket [DEC-038]: Ursachen-Etiketten je 727 Posten; Resolutions-Vorbefüllung (Slope 48, Trinh 104, Zhu&amp;Zhao 28, prod_inno 12, Wang 28, F37d); B&amp;H-Block-Adjudikation (N-Zuordnung); Spearman-Hypothese Zhou/Cubas; Kalibrier-Delta-3; dann Volker-Gespräch (Paket + Sandra/Ofogbe + F35-Errata)</t>
         </is>
       </c>
-      <c r="C29" s="52" t="inlineStr">
+      <c r="C29" s="102" t="inlineStr">
         <is>
           <t>erledigt (DEC-040)</t>
         </is>
       </c>
-      <c r="D29" s="52" t="inlineStr">
+      <c r="D29" s="102" t="inlineStr">
         <is>
           <t>in Arbeit</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="53">
-      <c r="A30" s="52" t="n">
+      <c r="A30" s="102" t="n">
         <v>28</v>
       </c>
-      <c r="B30" s="52" t="inlineStr">
+      <c r="B30" s="102" t="inlineStr">
         <is>
           <t>v11-preliminary bauen [DEC-040]: Assembly-Skript + Verifier nach Spec (docs/v11_assembly_spec.md); FOUNDATIONAL -&gt; Pre-Execution-Diff-Review durch Robert; danach Prep-Spec/T1-Entwicklung gegen preliminary</t>
         </is>
       </c>
-      <c r="C30" s="52" t="inlineStr">
+      <c r="C30" s="102" t="inlineStr">
         <is>
           <t>Claude -&gt; Robert (Review)</t>
         </is>
       </c>
-      <c r="D30" s="52" t="inlineStr">
+      <c r="D30" s="102" t="inlineStr">
         <is>
           <t>erledigt (2026-07-10, DEC-041)</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="53">
-      <c r="A31" s="52" t="n">
+      <c r="A31" s="102" t="n">
         <v>29</v>
       </c>
-      <c r="B31" s="52" t="inlineStr">
+      <c r="B31" s="102" t="inlineStr">
         <is>
           <t>JIF-Nachtrag alle Journals (b1, ruhendes Feld) — im DB-Re-Run-Slot via Cowork</t>
         </is>
       </c>
-      <c r="C31" s="52" t="inlineStr">
+      <c r="C31" s="102" t="inlineStr">
         <is>
           <t>Robert (Cowork)</t>
         </is>
       </c>
-      <c r="D31" s="52" t="inlineStr">
+      <c r="D31" s="102" t="inlineStr">
         <is>
           <t>erledigt (2026-07-10, DEC-041)</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="53">
-      <c r="A32" s="52" t="n">
+      <c r="A32" s="102" t="n">
         <v>30</v>
       </c>
-      <c r="B32" s="52" t="inlineStr">
+      <c r="B32" s="102" t="inlineStr">
         <is>
           <t>Moderator-Block Neuzugänge (country/regulation/industry per F36/R4) — Skript parst Logs; Restliste an Volker</t>
         </is>
       </c>
-      <c r="C32" s="52" t="inlineStr">
+      <c r="C32" s="102" t="inlineStr">
         <is>
           <t>Claude -&gt; Volker</t>
         </is>
       </c>
-      <c r="D32" s="52" t="inlineStr">
+      <c r="D32" s="102" t="inlineStr">
         <is>
           <t>erledigt (2026-07-10, DEC-041)</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="53">
-      <c r="A33" s="52" t="n">
+      <c r="A33" s="102" t="n">
         <v>31</v>
       </c>
-      <c r="B33" s="52" t="inlineStr">
+      <c r="B33" s="102" t="inlineStr">
         <is>
           <t>Screening-Katalog/Appendix: 593er-Liste als identified-not-extracted aufbereiten (optional Präzisions-Pass als Doku-Layer)</t>
         </is>
       </c>
-      <c r="C33" s="52" t="inlineStr">
+      <c r="C33" s="102" t="inlineStr">
         <is>
           <t>Claude</t>
         </is>
       </c>
-      <c r="D33" s="52" t="inlineStr">
+      <c r="D33" s="102" t="inlineStr">
         <is>
           <t>offen (Manuskriptphase)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="53">
-      <c r="A34" s="52" t="n">
+      <c r="A34" s="102" t="n">
         <v>32</v>
       </c>
-      <c r="B34" s="52" t="inlineStr">
+      <c r="B34" s="102" t="inlineStr">
         <is>
           <t>Manuskript-Fixes: Paris-Coding-Absatz -&gt; DEC-024-Architektur; Sensitive-Industry-Liste -&gt; R4; PRISMA-Sektion neu; Search-Absatz um 2026-Layer; Konkurrenz-Paper #1139 (CER/Policy Stringency/Debt Cost Europe 2026) lesen &amp; positionieren</t>
         </is>
       </c>
-      <c r="C34" s="52" t="inlineStr">
+      <c r="C34" s="102" t="inlineStr">
         <is>
           <t>Robert/Claude</t>
         </is>
       </c>
-      <c r="D34" s="52" t="inlineStr">
+      <c r="D34" s="102" t="inlineStr">
         <is>
           <t>offen</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="53">
-      <c r="A35" s="52" t="n">
+      <c r="A35" s="102" t="n">
         <v>33</v>
       </c>
-      <c r="B35" s="52" t="inlineStr">
+      <c r="B35" s="102" t="inlineStr">
         <is>
           <t>Original-2021-Suchmetadaten (Daten/Ns je DB) im Archiv suchen; sonst Waiver</t>
         </is>
       </c>
-      <c r="C35" s="52" t="inlineStr">
+      <c r="C35" s="102" t="inlineStr">
         <is>
           <t>Volker</t>
         </is>
       </c>
-      <c r="D35" s="52" t="inlineStr">
+      <c r="D35" s="102" t="inlineStr">
         <is>
           <t>verschoben</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="53">
-      <c r="A36" s="52" t="n">
+      <c r="A36" s="102" t="n">
         <v>34</v>
       </c>
-      <c r="B36" s="52" t="inlineStr">
+      <c r="B36" s="102" t="inlineStr">
         <is>
           <t>DEC-031 (Analyse-Batterie, SESOI 0.070) -&gt; T0.4 Prep -&gt; T1</t>
         </is>
       </c>
-      <c r="C36" s="52" t="inlineStr">
+      <c r="C36" s="102" t="inlineStr">
         <is>
           <t>T0.4 ERLEDIGT (kanonisch 2026-07-12); T1 ERLEDIGT (21/21, 2026-07-13); weiter blockweise (B als Naechstes)</t>
         </is>
       </c>
-      <c r="D36" s="52" t="inlineStr">
+      <c r="D36" s="102" t="inlineStr">
         <is>
           <t>NÄCHSTER SCHRITT</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="53">
-      <c r="A37" s="52" t="inlineStr">
+      <c r="A37" s="102" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="B37" s="52" t="inlineStr">
+      <c r="B37" s="102" t="inlineStr">
         <is>
           <t>Intro-Baustein: Paris-Blindheit der Primärliteratur — 73/115 Studien überspannen den Bruch, 72 poolen darüber hinweg, 1 splittet (Li et al 2022); Gap-Argument der Einleitung, im selben Atemzug B-Batterie signalisieren (Kompositions-Konter)</t>
         </is>
       </c>
-      <c r="C37" s="52" t="inlineStr">
+      <c r="C37" s="102" t="inlineStr">
         <is>
           <t>Robert/Claude</t>
         </is>
       </c>
-      <c r="F37" s="52" t="inlineStr">
+      <c r="F37" s="102" t="inlineStr">
         <is>
           <t>geparkt (Manuskriptphase; Pending-C-Input); Zahlen kanonisch (T0.4)</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="53">
-      <c r="A38" s="52" t="inlineStr">
+      <c r="A38" s="102" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
-      <c r="B38" s="52" t="inlineStr">
+      <c r="B38" s="102" t="inlineStr">
         <is>
           <t>COE-Overlap-Refresh auf finalem 120er-Korpus: Overlap-Disclosure (DEC-031b-Note, N12) basiert auf 5/66-Analyse (DEC-026); mit 54 Neuzugängen gegen die 75 COE-Studien neu prüfen (Studien- und ES-Ebene)</t>
         </is>
       </c>
-      <c r="C38" s="52" t="inlineStr">
+      <c r="C38" s="102" t="inlineStr">
         <is>
           <t>Claude -&gt; Robert</t>
         </is>
       </c>
-      <c r="F38" s="52" t="inlineStr">
+      <c r="F38" s="102" t="inlineStr">
         <is>
           <t>offen (vor Manuskript-Methods; billig, deterministisch aus beiden Studienlisten)</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="53">
-      <c r="A39" s="52" t="inlineStr">
+      <c r="A39" s="102" t="inlineStr">
         <is>
           <t>37</t>
         </is>
       </c>
-      <c r="B39" s="52" t="inlineStr">
+      <c r="B39" s="102" t="inlineStr">
         <is>
           <t>DEC-012a-Extraktion: SD(COD)-Benchmarks je Instrument (loan/bond/CDS) -- Median ueber alle Korpus-Studien mit berichteter SD in bp-konvertierbaren Einheiten (Regel fixiert; Task-Text in DEC-012a)</t>
         </is>
       </c>
-      <c r="C39" s="52" t="inlineStr">
+      <c r="C39" s="102" t="inlineStr">
         <is>
           <t>Volker</t>
         </is>
       </c>
-      <c r="F39" s="52" t="inlineStr">
+      <c r="F39" s="102" t="inlineStr">
         <is>
           <t>offen (entsperrt Manuskript-A6-Zeile / TB-08)</t>
         </is>
@@ -14227,13 +14234,13 @@
   <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="28" customWidth="1" style="52" min="1" max="1"/>
-    <col width="22" customWidth="1" style="52" min="2" max="2"/>
-    <col width="42" customWidth="1" style="52" min="3" max="3"/>
-    <col width="40" customWidth="1" style="52" min="4" max="4"/>
-    <col width="22" customWidth="1" style="52" min="5" max="5"/>
-    <col width="30" customWidth="1" style="52" min="6" max="6"/>
-    <col width="18" customWidth="1" style="52" min="7" max="7"/>
+    <col width="28" customWidth="1" style="102" min="1" max="1"/>
+    <col width="22" customWidth="1" style="102" min="2" max="2"/>
+    <col width="42" customWidth="1" style="102" min="3" max="3"/>
+    <col width="40" customWidth="1" style="102" min="4" max="4"/>
+    <col width="22" customWidth="1" style="102" min="5" max="5"/>
+    <col width="30" customWidth="1" style="102" min="6" max="6"/>
+    <col width="18" customWidth="1" style="102" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.5" customHeight="1" s="53">

</xml_diff>

<commit_message>
TF meta fix: toJSON digits pin + deterministic reemit script [DEC-051b, ERROR #36]
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1792,7 +1792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G72"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="102" min="1" max="1"/>
@@ -1814,7 +1814,7 @@
     <row r="2" ht="39.75" customHeight="1" s="53">
       <c r="A2" s="55" t="inlineStr">
         <is>
-          <t>67 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>68 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -3619,6 +3619,13 @@
       <c r="A71" s="102" t="inlineStr">
         <is>
           <t>DEC-051a — Corrigendum to DEC-051: F1 rstudent route parallel snow + toy identity probe, worker pins 8/8 (RAM-measured), runtime projection corrected; first canonical attempt aborted &gt; 10 h in the F1 pass, no outputs (2026-07-30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="102" t="inlineStr">
+        <is>
+          <t>DEC-051b — Corrigendum to DEC-051/051a: TF_run_meta re-emission after jsonlite digits truncation (ERROR #36); value artifacts untouched, fresh verifier 12/12 = acceptance; F1 pass measured 249.4 min on 8 workers =&gt; serial ~32 h, abort confirmed ex post (2026-07-31)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
TF results package: workbook + register complete + feed + status flips / G11 close [DEC-051-051b]
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1475,7 +1475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="102" min="1" max="1"/>
@@ -1770,6 +1770,23 @@
       <c r="C21" s="100" t="inlineStr">
         <is>
           <t>output/TG_results.csv; output/TG_results_workbook.xlsx; output/robustness_register.csv; manuscript/TG.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="100" t="inlineStr">
+        <is>
+          <t>TF · Block-F-Robustheit (F1–F7 + G11-Close)</t>
+        </is>
+      </c>
+      <c r="B22" s="100" t="inlineStr">
+        <is>
+          <t>4 Handling-Varianten r = -0,032…-0,041 (Headline -0,059); 4/4 Vorzeichen + CI≠0 + SESOI; LOO 114/114 Vorzeichen + CI (est_z -0,060…-0,041), max Shift = Drago-Drop (Cook D 1,64); rstudent 13 ⊆ MAD 275; Register komplett 23×18 (|r| 0,031–0,062; 14/16 CI≠0); TB-69–71 READY, TB-65 final, TB-68 supersediert [DEC-051/051a/051b]</t>
+        </is>
+      </c>
+      <c r="C22" s="100" t="inlineStr">
+        <is>
+          <t>output/TF_results.csv; output/TF_loo.csv; output/TF_influence.csv; output/TF_results_workbook.xlsx; output/robustness_register.csv; manuscript/TF.md</t>
         </is>
       </c>
     </row>
@@ -7301,7 +7318,7 @@
       </c>
       <c r="D45" s="89" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-31, TF 12/12, 06d1eeb)</t>
         </is>
       </c>
       <c r="E45" s="89" t="n"/>
@@ -7330,7 +7347,7 @@
       </c>
       <c r="D46" s="89" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-31, TF 12/12, 06d1eeb)</t>
         </is>
       </c>
       <c r="E46" s="89" t="n"/>
@@ -7355,7 +7372,7 @@
       </c>
       <c r="D47" s="89" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-31, TF 12/12, 06d1eeb)</t>
         </is>
       </c>
       <c r="E47" s="89" t="n"/>
@@ -7380,7 +7397,7 @@
       </c>
       <c r="D48" s="89" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-31, TF 12/12, 06d1eeb)</t>
         </is>
       </c>
       <c r="E48" s="89" t="n"/>
@@ -7405,7 +7422,7 @@
       </c>
       <c r="D49" s="89" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-31, TF 12/12, 06d1eeb)</t>
         </is>
       </c>
       <c r="E49" s="89" t="n"/>
@@ -7430,7 +7447,7 @@
       </c>
       <c r="D50" s="89" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-31, TF 12/12, 06d1eeb)</t>
         </is>
       </c>
       <c r="E50" s="89" t="n"/>
@@ -7459,7 +7476,7 @@
       </c>
       <c r="D51" s="89" t="inlineStr">
         <is>
-          <t>offen</t>
+          <t>erledigt (2026-07-31, TF 12/12, 06d1eeb)</t>
         </is>
       </c>
       <c r="E51" s="89" t="n"/>
@@ -7767,7 +7784,7 @@
       </c>
       <c r="D63" s="89" t="inlineStr">
         <is>
-          <t>partial — F rows pending (Registerbau in W-/F-Session); register partial committed (W)</t>
+          <t>erledigt (2026-07-31, register complete 23×18, TF append; run 06d1eeb / verifier c1e8b6c)</t>
         </is>
       </c>
       <c r="E63" s="89" t="n"/>

</xml_diff>

<commit_message>
M3: Chapter 1 (Introduction) assembled - DEC-055
- manuscript/ch1_introduction.md v1.0 (1,961 words incl. footnote) + reference ledger

- K1 novelty scan + K2a expectation scan consolidated, hub-verified (docs/novelty_scan_K1.md)

- TB-45 placed (E-M3-1); [PENDING #37] slot mirrored from ch4; RQ4 DRAFT until M4

- ERROR #42/#43 logged; Status DLI A76; BOOTSTRAP_M4 shipped
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R_Projects\FOMA-CER-COD-Paris\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_0CC35F8561BDAF3E1EE6CA7129E063955610D683" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_0CC3FF051E9D6C311EE6CA25A1604FAD5610D7C4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2454" uniqueCount="1765">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2455" uniqueCount="1766">
   <si>
     <t>FOMA CER–COD (Paris-Moderator) — Setup &amp; Workflow (v1, 2026-06-29)</t>
   </si>
@@ -5325,6 +5325,9 @@
   </si>
   <si>
     <t>DEC-054 — M2: Chapter 4 (Results) assembled; skeleton-v2 corrigendum (hub acks 2026-08-02) + pipeline ruling, tables/figures as build artifacts (scripts/build_ch4_tables.py, R/14 ALL PASS), workbook flips TB-28/41/42/46, M-T3 variant L, reference increment, F3 resolved (2026-08-03)</t>
+  </si>
+  <si>
+    <t>DEC-055 — M3: Chapter 1 (Introduction) assembled; full rebuild per ruling register Q1-Q11/MR-1-16, K1/K2a research scans hub-verified (novelty + expectation evidence), TB-45 placed (E-M3-1), reference ledger established, ERROR #42 (2026-08-03)</t>
   </si>
 </sst>
 </file>
@@ -6618,7 +6621,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -7825,6 +7828,11 @@
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>1764</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>1765</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
M6: title/abstract/keywords finalized (DEC-058); [M6-SYNC-1] delta; Map v1.3 (appendix -> M7); TB-12 READY; ERROR #48
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\R_Projects\FOMA-CER-COD-Paris\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_0CC3DF8376418B0AB4E6CADAA1226F335710D2EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_762F7CC3C08A141AF041C95AF93E8D2D5E49EF67" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2457" uniqueCount="1768">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2458" uniqueCount="1769">
   <si>
     <t>FOMA CER–COD (Paris-Moderator) — Setup &amp; Workflow (v1, 2026-06-29)</t>
   </si>
@@ -545,7 +545,7 @@
     <t>Ch 1–4</t>
   </si>
   <si>
-    <t>in Arbeit — M5 Discussion/Conclusion erledigt (DEC-057, 2026-08-04); M6 Abstract offen (per DEC-052)</t>
+    <t>erledigt (M5 Discussion per DEC-057, 2026-08-04; M6 Abstract/Titel/Keywords per DEC-058, 2026-08-05)</t>
   </si>
   <si>
     <t>Guardrails / Hinweise</t>
@@ -4661,7 +4661,7 @@
     <t>Decision-Log Index — DEC-ID-Register (Methodik-only; Pointer auf DECISION_LOG.md) (v1)</t>
   </si>
   <si>
-    <t>74 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+    <t>75 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
   </si>
   <si>
     <t>DEC-ID</t>
@@ -5334,6 +5334,9 @@
   </si>
   <si>
     <t>DEC-057 — M5: Chapter 5 (Discussion &amp; Conclusion) assembled; eight-subsection build per ruling register M5-Q1-Q8/MR-1-28, candidate-explanations section, TB-64/TB-56 finalized + workbook flips (T7/TH_b), Formula-Reference text fix (B6/B8/B9/B11), negative a7/a8 ripple ruling, ERROR #47. FROZEN.</t>
+  </si>
+  <si>
+    <t>DEC-058 — M6: Title/abstract/keywords finalized; title T-4 (question form, R4 family), 145-word abstract (TB-12 superseded at use, T1 workbook flip READY), six keywords at BSE cap, [M6-SYNC-1] delta executed (ch5 §5.8), appendix re-docked to M7 (Map v1.3), BSE front-matter [VERIFY] closed, ERROR #48. FROZEN.</t>
   </si>
 </sst>
 </file>
@@ -6627,7 +6630,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A1:G78"/>
+  <dimension ref="A1:G79"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -7849,6 +7852,11 @@
     <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>1767</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>1768</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
M7b gate part 2: K1/K2 register (ERROR #52-#54), P3 scans ALL PASS + 4 fixes, R5/#33/#37 rulings, bootstrap v1.1, map v1.5 [DEC-060]
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1623,7 +1623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G80"/>
+  <dimension ref="A1:G81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" style="44" min="1" max="1"/>
@@ -1645,7 +1645,7 @@
     <row r="2" ht="39.75" customHeight="1" s="44">
       <c r="A2" s="45" t="inlineStr">
         <is>
-          <t>76 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>77 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3527,14 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>DEC-059 — M7a: Pre-submission gate part 1; online appendix v1.0 assembled, reference-verification pass (~30 web-verified strings), consolidated reference list (114 entries, 36 corpus asterisks per v12), five ledgers finalized, Kleimeier &amp; Viehs supersession (2018 SSRN WP; ERROR #50), version-family rule, P&amp;R-2019/S&amp;D-2014 year fixes, RQ-7a-g slots, Map v1.4. FROZEN.</t>
+          <t>DEC-059 — M7a: Pre-submission gate part 1; online appendix v1.0 assembled, reference-verification pass (~30 web-verified strings), consolidated reference list (120 entries, 36 corpus asterisks per v12), five ledgers finalized, Kleimeier &amp; Viehs supersession (2018 SSRN WP; ERROR #50), version-family rule, P&amp;R-2019/S&amp;D-2014 year fixes, RQ-7a-g slots, Map v1.4. FROZEN.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>DEC-060 — M7b: K1/K2 correction register (ERROR #52–#54; canonical count 120 = 36*/84) · P3 scans ALL PASS, 4 fixes (ch1 ×2 title-echo (c) · ch3 grid-ceiling + R5 slot) · R5 ruled scope (i) · #33 decision-by-rule (#16 dock) · #37 gate · bootstrap v1.1 · Map v1.5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
M7b close: submission-readiness register (17 items), ERROR #55, map v1.6 (M phase closed), status close touch; assembly v1.0 + reference + CC contract committed per P6.5 [DEC-060]
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1623,7 +1623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" style="44" min="1" max="1"/>
@@ -1645,7 +1645,7 @@
     <row r="2" ht="39.75" customHeight="1" s="44">
       <c r="A2" s="45" t="inlineStr">
         <is>
-          <t>77 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>78 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -3535,6 +3535,13 @@
       <c r="A81" t="inlineStr">
         <is>
           <t>DEC-060 — M7b: K1/K2 correction register (ERROR #52–#54; canonical count 120 = 36*/84) · P3 scans ALL PASS, 4 fixes (ch1 ×2 title-echo (c) · ch3 grid-ceiling + R5 slot) · R5 ruled scope (i) · #33 decision-by-rule (#16 dock) · #37 gate · bootstrap v1.1 · Map v1.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>DEC-061 — M7b/P6: Fig-3 re-render (A7 → R/14 v6.1: Fisher-z, F-CAP, ruling-Z window; ERROR #56) · verifier v5 identity checks · ch4 caption PI clause · run-path correction (ERROR #57); commit 2f3b034</t>
         </is>
       </c>
     </row>
@@ -4132,7 +4139,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>in Arbeit — M7a erledigt (Appendix v1.0, Referenz-Master, DEC-059, 2026-08-05); M7b offen (R5 · Scans · docx)</t>
+          <t>erledigt (M7b close 2026-08-06: DEC-060/DEC-061, ERROR #52–#57; P3-Scans ALL PASS; Fig-3-Re-Render; docx-Assembly v1.0 @ 2f3b034, Tag manuscript-v1.0-assembly; PENDING-external-Register → docs/SUBMISSION_READINESS.md)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
P1 Commit A: SD(COD) bp benchmarks landed [DEC-012b, DEC-062]; ERROR #41/#58/#59; A.17; readiness 5A/5B +18/+19; Status DLI 80 DECs +A83/A84
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1623,7 +1623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G82"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" style="44" min="1" max="1"/>
@@ -1645,7 +1645,7 @@
     <row r="2" ht="39.75" customHeight="1" s="44">
       <c r="A2" s="45" t="inlineStr">
         <is>
-          <t>78 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>80 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -3542,6 +3542,20 @@
       <c r="A82" t="inlineStr">
         <is>
           <t>DEC-061 — M7b/P6: Fig-3 re-render (A7 → R/14 v6.1: Fisher-z, F-CAP, ruling-Z window; ERROR #56) · verifier v5 identity checks · ch4 caption PI clause · run-path correction (ERROR #57); commit 2f3b034</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>DEC-012b — SD(COD) benchmark constants landed; two-stage median; primary loan 200.0 (k=49) / bond 150.0 (21) / CDS 168.6 (7); A6 re-key scheduled Commit B/S1</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>DEC-062 — Construct-validity screen amount-scaled COD: retain + criterion tightening + pre-declared drop-set sensitivity</t>
         </is>
       </c>
     </row>
@@ -5836,6 +5850,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="44">
       <c r="A3" s="52" t="inlineStr">
         <is>
@@ -9371,6 +9386,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20" ht="15" customHeight="1" s="44">
       <c r="A20" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
DEC-063: ERROR #58 cluster merge - v12.1 erratum (52 cells / 3 sites, CLUSTER Pizzutilo/Caragnano); audit v2 gate 33 checks 0 FAIL (+E5/E6 guards); corpus 119->118, estimation 114->113; ERROR #58 CLOSED, #60 #61 #62 registered; fingerprint pair tracked (Item 19); DLI A2=81 +A85
</commit_message>
<xml_diff>
--- a/docs/CER-COD_Status.xlsx
+++ b/docs/CER-COD_Status.xlsx
@@ -1623,7 +1623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G85"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" style="44" min="1" max="1"/>
@@ -1645,7 +1645,7 @@
     <row r="2" ht="39.75" customHeight="1" s="44">
       <c r="A2" s="45" t="inlineStr">
         <is>
-          <t>80 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
+          <t>81 DECs (Methodik + Framing; append-only; Reihenfolge chronologisch). Volleinträge im DECISION_LOG.md.</t>
         </is>
       </c>
     </row>
@@ -3556,6 +3556,13 @@
       <c r="A84" t="inlineStr">
         <is>
           <t>DEC-062 — Construct-validity screen amount-scaled COD: retain + criterion tightening + pre-declared drop-set sensitivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>DEC-063 — ERROR #58 merge executed: v12.1 erratum (52 cells / 3 sites, 'CLUSTER Pizzutilo/Caragnano'; audit v2 33 checks FAIL 0, +E5/E6 guards); corpus 119→118 / estimation 114→113; repoint register (a)/(b); Item-18 drop-set + merge bound (R-A); Commit-B carriers + design_quantities (provenance row); P2b ripple slot; ERRORs #58-CLOSED · #60 · #61 · #62</t>
         </is>
       </c>
     </row>
@@ -5850,7 +5857,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="44">
       <c r="A3" s="52" t="inlineStr">
         <is>
@@ -9386,7 +9392,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="15" customHeight="1" s="44">
       <c r="A20" t="inlineStr">
         <is>

</xml_diff>